<commit_message>
Report Suite: execute authorized full TestRail push (video edits + repairs + consolidation)
70 update_case + add_case SBC-EXP-16=C38856 + 57 delete_case, all HTTP 200 + verified;
459 active (live-verified under group 4281); R359 515->458 documented, never written;
deliverables regenerated over 459, id-map re-merged 459/459.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01AZ5XzKsK9wv7M41cSPaMyg
</commit_message>
<xml_diff>
--- a/testrail-import/Report-Suite_Inventory-Value-Report_testrail-import.xlsx
+++ b/testrail-import/Report-Suite_Inventory-Value-Report_testrail-import.xlsx
@@ -428,7 +428,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J78"/>
+  <dimension ref="A1:J69"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="50" customWidth="1" min="1" max="1"/>
@@ -633,7 +633,7 @@
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>Changing the date, location, Category, Vendor, part search, or sort reloads the rows from the server with the standard loading indicator</t>
+          <t>The report is server-paginated: one page of rows at a time, and any filter/search/sort change returns to the first page</t>
         </is>
       </c>
       <c r="B5" s="2" t="inlineStr">
@@ -648,65 +648,16 @@
       </c>
       <c r="D5" s="2" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Critical</t>
         </is>
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
           <t>1. You are signed in to the ShopView App on a desktop browser.
-2. The Inventory Value report is open with rows loaded.</t>
+2. The selected location(s) hold more in-stock parts than fit on one page (seed ZZAUTOTEST parts if needed).</t>
         </is>
       </c>
       <c r="F5" s="2" t="inlineStr">
-        <is>
-          <t>1. Change the date range and watch the data area.
-2. Change the location selection, then the Category filter, then the Vendor filter.
-3. Type in the part search, then click a column header to change the sort — watching the data area each time.</t>
-        </is>
-      </c>
-      <c r="G5" s="2" t="inlineStr">
-        <is>
-          <t>1. Each change — date range, location, Category, Vendor, part search, sort — reloads the report's rows from the server.
-2. While loading, the data area shows the standard reports loading indicator.
-3. Existing rows are replaced only when the new data returns.</t>
-        </is>
-      </c>
-      <c r="H5" s="2" t="inlineStr">
-        <is>
-          <t>specs/inventory-value.md Story 1 S1-R4; S1-R5; S1-R7</t>
-        </is>
-      </c>
-      <c r="I5" s="2" t="inlineStr"/>
-      <c r="J5" s="2" t="inlineStr"/>
-    </row>
-    <row r="6">
-      <c r="A6" s="2" t="inlineStr">
-        <is>
-          <t>The report is server-paginated: one page of rows at a time, and any filter/search/sort change returns to the first page</t>
-        </is>
-      </c>
-      <c r="B6" s="2" t="inlineStr">
-        <is>
-          <t>IV — Access &amp; Display</t>
-        </is>
-      </c>
-      <c r="C6" s="2" t="inlineStr">
-        <is>
-          <t>Functional</t>
-        </is>
-      </c>
-      <c r="D6" s="2" t="inlineStr">
-        <is>
-          <t>Critical</t>
-        </is>
-      </c>
-      <c r="E6" s="2" t="inlineStr">
-        <is>
-          <t>1. You are signed in to the ShopView App on a desktop browser.
-2. The selected location(s) hold more in-stock parts than fit on one page (seed ZZAUTOTEST parts if needed).</t>
-        </is>
-      </c>
-      <c r="F6" s="2" t="inlineStr">
         <is>
           <t>1. Open the Inventory Value report and find the pagination control.
 2. Move to page 2 (and further) and watch the rows.
@@ -714,15 +665,63 @@
 4. Repeat from a later page with a part search and with a sort change.</t>
         </is>
       </c>
-      <c r="G6" s="2" t="inlineStr">
+      <c r="G5" s="2" t="inlineStr">
         <is>
           <t>1. The server returns one page of rows at a time; the user moves through pages with the reports suite's standard pagination control.
 2. Changing any server-side filter (Date, Location, Category, Vendor), the part search, or the sort returns the FIRST page of the new result set.</t>
         </is>
       </c>
+      <c r="H5" s="2" t="inlineStr">
+        <is>
+          <t>specs/inventory-value.md Story 1 S1-R8; §2 Scale and data model</t>
+        </is>
+      </c>
+      <c r="I5" s="2" t="inlineStr"/>
+      <c r="J5" s="2" t="inlineStr"/>
+    </row>
+    <row r="6">
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t>No qualifying parts, day or location: the no-data message shows and no totals</t>
+        </is>
+      </c>
+      <c r="B6" s="2" t="inlineStr">
+        <is>
+          <t>IV — Access &amp; Display</t>
+        </is>
+      </c>
+      <c r="C6" s="2" t="inlineStr">
+        <is>
+          <t>Negative</t>
+        </is>
+      </c>
+      <c r="D6" s="2" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="E6" s="2" t="inlineStr">
+        <is>
+          <t>1. You are signed in to the ShopView App on a desktop browser.
+2. Three causes can be produced: (a) a location you can access holds no in-stock parts, (b) a past range ends entirely before nightly recording began (or its covered dates were pruned by retention), (c) the filters can be set so nothing qualifies.</t>
+        </is>
+      </c>
+      <c r="F6" s="2" t="inlineStr">
+        <is>
+          <t>1. Scope the report to the empty location and read the data area.
+2. Select a Custom range ending before nightly recording began and read the data area and the bottom of the report.
+3. Set the filters so nothing qualifies and re-read.</t>
+        </is>
+      </c>
+      <c r="G6" s="2" t="inlineStr">
+        <is>
+          <t>1. In every case the report shows the standard reports no-data message "Empty bays, endless possibilities. Get Going!" instead of rows.
+2. No totals row is shown in any of the cases.</t>
+        </is>
+      </c>
       <c r="H6" s="2" t="inlineStr">
         <is>
-          <t>specs/inventory-value.md Story 1 S1-R8; §2 Scale and data model</t>
+          <t>specs/inventory-value.md Story 1 S1-N2; Story 5 S5-N1; Story 7 S7-N2; Story 12; §7 User Feedback Summary</t>
         </is>
       </c>
       <c r="I6" s="2" t="inlineStr"/>
@@ -731,45 +730,48 @@
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>When no in-stock part exists for the selected location(s) on the resolved date, the no-data message shows instead of rows</t>
+          <t>A part appears only if not a core charge and on-hand quantity is above zero</t>
         </is>
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>IV — Access &amp; Display</t>
+          <t>IV — Row Scope</t>
         </is>
       </c>
       <c r="C7" s="2" t="inlineStr">
         <is>
-          <t>Negative</t>
+          <t>Functional</t>
         </is>
       </c>
       <c r="D7" s="2" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Critical</t>
         </is>
       </c>
       <c r="E7" s="2" t="inlineStr">
         <is>
           <t>1. You are signed in to the ShopView App on a desktop browser.
-2. A location you can access holds no in-stock parts (or the filters can be set so nothing qualifies).</t>
+2. ZZAUTOTEST parts exist at your active location: a normal part with positive on-hand quantity, a core-charge part with a positive quantity, a part with exactly zero on-hand quantity, and (if producible) one with a negative on-hand quantity.</t>
         </is>
       </c>
       <c r="F7" s="2" t="inlineStr">
         <is>
-          <t>1. Scope the report to the empty location (or filter so nothing qualifies).
-2. Read the data area.</t>
+          <t>1. Open the Inventory Value report scoped to the location.
+2. Look for the normal in-stock part.
+3. Search for the core-charge part, the zero-quantity part, and the negative-quantity part by part number; check the totals row.</t>
         </is>
       </c>
       <c r="G7" s="2" t="inlineStr">
         <is>
-          <t>1. The report shows the standard reports no-data message "Empty bays, endless possibilities. Get Going!" instead of rows.
-2. No totals row is shown.</t>
+          <t>1. The normal, positive-quantity, non-core part appears as one row.
+2. The core-charge part is never listed — even with a positive quantity — and its value is not counted in the totals row.
+3. The zero-quantity and negative-quantity parts are not listed — only quantities greater than zero are valued.
+4. Only parts meeting BOTH conditions — not a core charge, and on-hand quantity greater than zero — are listed.</t>
         </is>
       </c>
       <c r="H7" s="2" t="inlineStr">
         <is>
-          <t>specs/inventory-value.md Story 1 S1-N2; Story 12; §7 User Feedback Summary</t>
+          <t>specs/inventory-value.md Story 2 S2-R1; S2-R2; S2-N1; S2-N2; §3 Key Decisions</t>
         </is>
       </c>
       <c r="I7" s="2" t="inlineStr"/>
@@ -778,7 +780,7 @@
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>A part appears only when it is not a core charge AND its on-hand quantity is greater than zero</t>
+          <t>A part stocked at two selected locations appears as two rows (one per location), not merged — expected, do not file</t>
         </is>
       </c>
       <c r="B8" s="2" t="inlineStr">
@@ -793,31 +795,30 @@
       </c>
       <c r="D8" s="2" t="inlineStr">
         <is>
-          <t>Critical</t>
+          <t>High</t>
         </is>
       </c>
       <c r="E8" s="2" t="inlineStr">
         <is>
-          <t>1. You are signed in to the ShopView App on a desktop browser.
-2. ZZAUTOTEST parts exist at your active location: a normal part with positive on-hand quantity, and (for the negative side) a core-charge part and a zero-quantity part.</t>
+          <t>1. You are signed in to the ShopView App on a desktop browser as a user with access to at least two locations.
+2. The same ZZAUTOTEST part is in stock (positive quantity) at two of those locations.</t>
         </is>
       </c>
       <c r="F8" s="2" t="inlineStr">
         <is>
-          <t>1. Open the Inventory Value report scoped to the location.
-2. Look for the normal in-stock part.
-3. Look for the core-charge part and the zero-quantity part.</t>
+          <t>1. Open the Inventory Value report and select both locations in the Location filter.
+2. Search for the part and count its rows.</t>
         </is>
       </c>
       <c r="G8" s="2" t="inlineStr">
         <is>
-          <t>1. The normal, positive-quantity, non-core part appears as one row.
-2. Only parts meeting BOTH conditions — not a core charge, and on-hand quantity greater than zero — are listed.</t>
+          <t>1. The part appears twice — one row per location, each with that location's own quantity and values.
+2. The rows are NOT merged into one combined row; this is the documented v1 behavior.</t>
         </is>
       </c>
       <c r="H8" s="2" t="inlineStr">
         <is>
-          <t>specs/inventory-value.md Story 2 S2-R1; S2-R2; §3 Key Decisions</t>
+          <t>specs/inventory-value.md Story 2 S2-R3; §2 Known Limitations (v1)</t>
         </is>
       </c>
       <c r="I8" s="2" t="inlineStr"/>
@@ -826,7 +827,7 @@
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>A part stocked at two selected locations appears as two rows (one per location), not merged — expected, do not file</t>
+          <t>There is no dead-stock exclusion — long-sitting stock still contributes to the on-hand value</t>
         </is>
       </c>
       <c r="B9" s="2" t="inlineStr">
@@ -841,30 +842,29 @@
       </c>
       <c r="D9" s="2" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="E9" s="2" t="inlineStr">
         <is>
-          <t>1. You are signed in to the ShopView App on a desktop browser as a user with access to at least two locations.
-2. The same ZZAUTOTEST part is in stock (positive quantity) at two of those locations.</t>
+          <t>1. You are signed in to the ShopView App on a desktop browser.
+2. A part with positive, non-core stock exists that has had no movement for a long time (or the oldest-stocked part at the location is known).</t>
         </is>
       </c>
       <c r="F9" s="2" t="inlineStr">
         <is>
-          <t>1. Open the Inventory Value report and select both locations in the Location filter.
-2. Search for the part and count its rows.</t>
+          <t>1. Open the Inventory Value report scoped to the location.
+2. Search for the long-sitting part.</t>
         </is>
       </c>
       <c r="G9" s="2" t="inlineStr">
         <is>
-          <t>1. The part appears twice — one row per location, each with that location's own quantity and values.
-2. The rows are NOT merged into one combined row; this is the documented v1 behavior.</t>
+          <t>1. The long-sitting part appears and its value is counted — every part currently holding positive, non-core stock contributes to the on-hand value, however long it has sat.</t>
         </is>
       </c>
       <c r="H9" s="2" t="inlineStr">
         <is>
-          <t>specs/inventory-value.md Story 2 S2-R3; §2 Known Limitations (v1)</t>
+          <t>specs/inventory-value.md Story 2 context note (no dead-stock exclusion)</t>
         </is>
       </c>
       <c r="I9" s="2" t="inlineStr"/>
@@ -873,1191 +873,960 @@
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>A core-charge part is never shown, regardless of its quantity</t>
+          <t>Unit Sell uses the part's fixed sell price when one is set</t>
         </is>
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>IV — Row Scope</t>
+          <t>IV — Valuation &amp; Columns</t>
         </is>
       </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
-          <t>Negative</t>
+          <t>Functional</t>
         </is>
       </c>
       <c r="D10" s="2" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Critical</t>
         </is>
       </c>
       <c r="E10" s="2" t="inlineStr">
         <is>
           <t>1. You are signed in to the ShopView App on a desktop browser.
-2. A core-charge part with a positive on-hand quantity exists at the selected location.</t>
+2. A ZZAUTOTEST in-stock part exists with a known unit cost, a known FIXED sell price, and a category whose pricing-matrix markup would give a DIFFERENT figure.</t>
         </is>
       </c>
       <c r="F10" s="2" t="inlineStr">
-        <is>
-          <t>1. Open the Inventory Value report scoped to that location.
-2. Search for the core-charge part by its part number.
-3. Check the totals row for its value.</t>
-        </is>
-      </c>
-      <c r="G10" s="2" t="inlineStr">
-        <is>
-          <t>1. The core-charge part is not listed, even though its quantity is positive.
-2. Its value is not counted in the totals row.</t>
-        </is>
-      </c>
-      <c r="H10" s="2" t="inlineStr">
-        <is>
-          <t>specs/inventory-value.md Story 2 S2-N1</t>
-        </is>
-      </c>
-      <c r="I10" s="2" t="inlineStr"/>
-      <c r="J10" s="2" t="inlineStr"/>
-    </row>
-    <row r="11">
-      <c r="A11" s="2" t="inlineStr">
-        <is>
-          <t>A part with zero or negative on-hand quantity is never shown</t>
-        </is>
-      </c>
-      <c r="B11" s="2" t="inlineStr">
-        <is>
-          <t>IV — Row Scope</t>
-        </is>
-      </c>
-      <c r="C11" s="2" t="inlineStr">
-        <is>
-          <t>Negative</t>
-        </is>
-      </c>
-      <c r="D11" s="2" t="inlineStr">
-        <is>
-          <t>High</t>
-        </is>
-      </c>
-      <c r="E11" s="2" t="inlineStr">
-        <is>
-          <t>1. You are signed in to the ShopView App on a desktop browser.
-2. A part with exactly zero on-hand quantity exists at the selected location, and (if producible) one with a negative on-hand quantity.</t>
-        </is>
-      </c>
-      <c r="F11" s="2" t="inlineStr">
-        <is>
-          <t>1. Open the Inventory Value report scoped to that location.
-2. Search for the zero-quantity part by its part number.
-3. Search for the negative-quantity part if one exists.</t>
-        </is>
-      </c>
-      <c r="G11" s="2" t="inlineStr">
-        <is>
-          <t>1. The zero-quantity part is not listed.
-2. The negative-quantity part is not listed either — only quantities greater than zero are valued.</t>
-        </is>
-      </c>
-      <c r="H11" s="2" t="inlineStr">
-        <is>
-          <t>specs/inventory-value.md Story 2 S2-N2</t>
-        </is>
-      </c>
-      <c r="I11" s="2" t="inlineStr"/>
-      <c r="J11" s="2" t="inlineStr"/>
-    </row>
-    <row r="12">
-      <c r="A12" s="2" t="inlineStr">
-        <is>
-          <t>There is no dead-stock exclusion — long-sitting stock still contributes to the on-hand value</t>
-        </is>
-      </c>
-      <c r="B12" s="2" t="inlineStr">
-        <is>
-          <t>IV — Row Scope</t>
-        </is>
-      </c>
-      <c r="C12" s="2" t="inlineStr">
-        <is>
-          <t>Functional</t>
-        </is>
-      </c>
-      <c r="D12" s="2" t="inlineStr">
-        <is>
-          <t>Medium</t>
-        </is>
-      </c>
-      <c r="E12" s="2" t="inlineStr">
-        <is>
-          <t>1. You are signed in to the ShopView App on a desktop browser.
-2. A part with positive, non-core stock exists that has had no movement for a long time (or the oldest-stocked part at the location is known).</t>
-        </is>
-      </c>
-      <c r="F12" s="2" t="inlineStr">
-        <is>
-          <t>1. Open the Inventory Value report scoped to the location.
-2. Search for the long-sitting part.</t>
-        </is>
-      </c>
-      <c r="G12" s="2" t="inlineStr">
-        <is>
-          <t>1. The long-sitting part appears and its value is counted — every part currently holding positive, non-core stock contributes to the on-hand value, however long it has sat.</t>
-        </is>
-      </c>
-      <c r="H12" s="2" t="inlineStr">
-        <is>
-          <t>specs/inventory-value.md Story 2 context note (no dead-stock exclusion)</t>
-        </is>
-      </c>
-      <c r="I12" s="2" t="inlineStr"/>
-      <c r="J12" s="2" t="inlineStr"/>
-    </row>
-    <row r="13">
-      <c r="A13" s="2" t="inlineStr">
-        <is>
-          <t>Unit Sell uses the part's fixed sell price when one is set</t>
-        </is>
-      </c>
-      <c r="B13" s="2" t="inlineStr">
-        <is>
-          <t>IV — Valuation &amp; Columns</t>
-        </is>
-      </c>
-      <c r="C13" s="2" t="inlineStr">
-        <is>
-          <t>Functional</t>
-        </is>
-      </c>
-      <c r="D13" s="2" t="inlineStr">
-        <is>
-          <t>Critical</t>
-        </is>
-      </c>
-      <c r="E13" s="2" t="inlineStr">
-        <is>
-          <t>1. You are signed in to the ShopView App on a desktop browser.
-2. A ZZAUTOTEST in-stock part exists with a known unit cost, a known FIXED sell price, and a category whose pricing-matrix markup would give a DIFFERENT figure.</t>
-        </is>
-      </c>
-      <c r="F13" s="2" t="inlineStr">
         <is>
           <t>1. Open the Inventory Value report and find the part's row.
 2. Read its Unit Sell value.
 3. Compare it to the part's fixed sell price and to the figure the category markup would have produced.</t>
         </is>
       </c>
-      <c r="G13" s="2" t="inlineStr">
+      <c r="G10" s="2" t="inlineStr">
         <is>
           <t>1. Unit Sell equals the part's fixed sell price.
 2. The pricing-matrix markup is NOT applied when a fixed sell price is set — the fixed price wins.</t>
         </is>
       </c>
-      <c r="H13" s="2" t="inlineStr">
+      <c r="H10" s="2" t="inlineStr">
         <is>
           <t>specs/inventory-value.md Story 3 S3-R5 (fixed-price branch); §3 Key Decisions (unit sell resolved like the parts list)</t>
         </is>
       </c>
-      <c r="I13" s="2" t="inlineStr"/>
-      <c r="J13" s="2" t="inlineStr"/>
-    </row>
-    <row r="14">
-      <c r="A14" s="2" t="inlineStr">
+      <c r="I10" s="2" t="inlineStr"/>
+      <c r="J10" s="2" t="inlineStr"/>
+    </row>
+    <row r="11">
+      <c r="A11" s="2" t="inlineStr">
         <is>
           <t>With no fixed sell price, Unit Sell is the shop's pricing-matrix markup on cost for the part's category</t>
         </is>
       </c>
-      <c r="B14" s="2" t="inlineStr">
+      <c r="B11" s="2" t="inlineStr">
         <is>
           <t>IV — Valuation &amp; Columns</t>
         </is>
       </c>
-      <c r="C14" s="2" t="inlineStr">
-        <is>
-          <t>Functional</t>
-        </is>
-      </c>
-      <c r="D14" s="2" t="inlineStr">
+      <c r="C11" s="2" t="inlineStr">
+        <is>
+          <t>Functional</t>
+        </is>
+      </c>
+      <c r="D11" s="2" t="inlineStr">
         <is>
           <t>Critical</t>
         </is>
       </c>
-      <c r="E14" s="2" t="inlineStr">
+      <c r="E11" s="2" t="inlineStr">
         <is>
           <t>1. You are signed in to the ShopView App on a desktop browser.
 2. A ZZAUTOTEST in-stock part exists with a known unit cost, NO fixed sell price, and a category covered by the shop's pricing matrix with a known markup.</t>
         </is>
       </c>
-      <c r="F14" s="2" t="inlineStr">
+      <c r="F11" s="2" t="inlineStr">
         <is>
           <t>1. Open the Inventory Value report and find the part's row.
 2. Read its Unit Sell value.
 3. Compare it to the pricing-matrix markup applied to the part's cost for its category.</t>
         </is>
       </c>
-      <c r="G14" s="2" t="inlineStr">
+      <c r="G11" s="2" t="inlineStr">
         <is>
           <t>1. Unit Sell equals the shop's pricing-matrix markup on cost for that part's category (the same way the parts list resolves it).</t>
         </is>
       </c>
-      <c r="H14" s="2" t="inlineStr">
+      <c r="H11" s="2" t="inlineStr">
         <is>
           <t>specs/inventory-value.md Story 3 S3-R5 (matrix branch); §5 Assumptions</t>
         </is>
       </c>
-      <c r="I14" s="2" t="inlineStr"/>
-      <c r="J14" s="2" t="inlineStr"/>
-    </row>
-    <row r="15">
-      <c r="A15" s="2" t="inlineStr">
+      <c r="I11" s="2" t="inlineStr"/>
+      <c r="J11" s="2" t="inlineStr"/>
+    </row>
+    <row r="12">
+      <c r="A12" s="2" t="inlineStr">
         <is>
           <t>With no fixed sell price and no category, Unit Sell equals Unit Cost — the stock is valued at cost with a $0.00 / 0.0% margin</t>
         </is>
       </c>
-      <c r="B15" s="2" t="inlineStr">
+      <c r="B12" s="2" t="inlineStr">
         <is>
           <t>IV — Valuation &amp; Columns</t>
         </is>
       </c>
-      <c r="C15" s="2" t="inlineStr">
-        <is>
-          <t>Functional</t>
-        </is>
-      </c>
-      <c r="D15" s="2" t="inlineStr">
+      <c r="C12" s="2" t="inlineStr">
+        <is>
+          <t>Functional</t>
+        </is>
+      </c>
+      <c r="D12" s="2" t="inlineStr">
         <is>
           <t>Critical</t>
         </is>
       </c>
-      <c r="E15" s="2" t="inlineStr">
+      <c r="E12" s="2" t="inlineStr">
         <is>
           <t>1. You are signed in to the ShopView App on a desktop browser.
 2. A ZZAUTOTEST in-stock part exists with a known unit cost, NO fixed sell price, and NO category.
 3. The Margin and Total Sell columns are turned on.</t>
         </is>
       </c>
-      <c r="F15" s="2" t="inlineStr">
+      <c r="F12" s="2" t="inlineStr">
         <is>
           <t>1. Open the Inventory Value report and find the part's row.
 2. Read its Unit Sell and compare to its Unit Cost.
 3. Read its Margin and Margin % cells.</t>
         </is>
       </c>
-      <c r="G15" s="2" t="inlineStr">
+      <c r="G12" s="2" t="inlineStr">
         <is>
           <t>1. A part with no category takes no markup, so its Unit Sell equals its Unit Cost.
 2. Such a part shows a Margin of $0.00 and a Margin % of 0.0% — the stock is valued at cost.</t>
         </is>
       </c>
-      <c r="H15" s="2" t="inlineStr">
+      <c r="H12" s="2" t="inlineStr">
         <is>
           <t>specs/inventory-value.md Story 3 S3-R5 (no-category fallback) + context note; §5 Assumptions</t>
         </is>
       </c>
-      <c r="I15" s="2" t="inlineStr"/>
-      <c r="J15" s="2" t="inlineStr"/>
-    </row>
-    <row r="16">
-      <c r="A16" s="2" t="inlineStr">
+      <c r="I12" s="2" t="inlineStr"/>
+      <c r="J12" s="2" t="inlineStr"/>
+    </row>
+    <row r="13">
+      <c r="A13" s="2" t="inlineStr">
         <is>
           <t>Total Sell is quantity × Unit Sell and Total Cost is quantity × Unit Cost</t>
         </is>
       </c>
-      <c r="B16" s="2" t="inlineStr">
+      <c r="B13" s="2" t="inlineStr">
         <is>
           <t>IV — Valuation &amp; Columns</t>
         </is>
       </c>
-      <c r="C16" s="2" t="inlineStr">
-        <is>
-          <t>Functional</t>
-        </is>
-      </c>
-      <c r="D16" s="2" t="inlineStr">
+      <c r="C13" s="2" t="inlineStr">
+        <is>
+          <t>Functional</t>
+        </is>
+      </c>
+      <c r="D13" s="2" t="inlineStr">
         <is>
           <t>Critical</t>
         </is>
       </c>
-      <c r="E16" s="2" t="inlineStr">
+      <c r="E13" s="2" t="inlineStr">
         <is>
           <t>1. You are signed in to the ShopView App on a desktop browser.
 2. A ZZAUTOTEST in-stock part exists with a known on-hand quantity (include a fractional quantity if possible), unit cost, and unit sell.
 3. The Total Sell column is turned on.</t>
         </is>
       </c>
-      <c r="F16" s="2" t="inlineStr">
+      <c r="F13" s="2" t="inlineStr">
         <is>
           <t>1. Open the Inventory Value report and find the part's row.
 2. Multiply the on-hand quantity by Unit Sell and compare to Total Sell.
 3. Multiply the on-hand quantity by Unit Cost and compare to Total Cost.</t>
         </is>
       </c>
-      <c r="G16" s="2" t="inlineStr">
+      <c r="G13" s="2" t="inlineStr">
         <is>
           <t>1. Total Sell equals the part's on-hand quantity × Unit Sell, shown as US-dollar currency.
 2. Total Cost equals the part's on-hand quantity × Unit Cost, shown as US-dollar currency.</t>
         </is>
       </c>
-      <c r="H16" s="2" t="inlineStr">
+      <c r="H13" s="2" t="inlineStr">
         <is>
           <t>specs/inventory-value.md Story 3 S3-R6; S3-R7; §4 Terminology</t>
         </is>
       </c>
-      <c r="I16" s="2" t="inlineStr"/>
-      <c r="J16" s="2" t="inlineStr"/>
-    </row>
-    <row r="17">
-      <c r="A17" s="2" t="inlineStr">
+      <c r="I13" s="2" t="inlineStr"/>
+      <c r="J13" s="2" t="inlineStr"/>
+    </row>
+    <row r="14">
+      <c r="A14" s="2" t="inlineStr">
         <is>
           <t>Margin is the extended figure — Total Sell minus Total Cost for the whole on-hand quantity, not a per-unit number</t>
         </is>
       </c>
-      <c r="B17" s="2" t="inlineStr">
+      <c r="B14" s="2" t="inlineStr">
         <is>
           <t>IV — Valuation &amp; Columns</t>
         </is>
       </c>
-      <c r="C17" s="2" t="inlineStr">
-        <is>
-          <t>Functional</t>
-        </is>
-      </c>
-      <c r="D17" s="2" t="inlineStr">
+      <c r="C14" s="2" t="inlineStr">
+        <is>
+          <t>Functional</t>
+        </is>
+      </c>
+      <c r="D14" s="2" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="E17" s="2" t="inlineStr">
+      <c r="E14" s="2" t="inlineStr">
         <is>
           <t>1. You are signed in to the ShopView App on a desktop browser.
 2. A ZZAUTOTEST in-stock part exists with a quantity greater than 1 and different unit cost and unit sell values.
 3. The Margin and Total Sell columns are turned on.</t>
         </is>
       </c>
-      <c r="F17" s="2" t="inlineStr">
+      <c r="F14" s="2" t="inlineStr">
         <is>
           <t>1. Open the Inventory Value report and find the part's row.
 2. Subtract Total Cost from Total Sell and compare to the Margin cell.
 3. Also compute the per-unit difference (Unit Sell − Unit Cost) and confirm Margin is NOT that per-unit figure.</t>
         </is>
       </c>
-      <c r="G17" s="2" t="inlineStr">
+      <c r="G14" s="2" t="inlineStr">
         <is>
           <t>1. Margin equals Total Sell − Total Cost for the part's whole on-hand quantity, shown as US-dollar currency.
 2. Margin is the extended (total) margin, not the per-unit difference.</t>
         </is>
       </c>
-      <c r="H17" s="2" t="inlineStr">
+      <c r="H14" s="2" t="inlineStr">
         <is>
           <t>specs/inventory-value.md Story 3 S3-R8; §3 Key Decisions (extended margin); §4 Terminology</t>
         </is>
       </c>
-      <c r="I17" s="2" t="inlineStr"/>
-      <c r="J17" s="2" t="inlineStr"/>
-    </row>
-    <row r="18">
-      <c r="A18" s="2" t="inlineStr">
+      <c r="I14" s="2" t="inlineStr"/>
+      <c r="J14" s="2" t="inlineStr"/>
+    </row>
+    <row r="15">
+      <c r="A15" s="2" t="inlineStr">
         <is>
           <t>Margin % is Margin as a share of Total Sell to one decimal with a percent sign, showing "—" when Total Sell is zero or negative</t>
         </is>
       </c>
-      <c r="B18" s="2" t="inlineStr">
+      <c r="B15" s="2" t="inlineStr">
         <is>
           <t>IV — Valuation &amp; Columns</t>
         </is>
       </c>
-      <c r="C18" s="2" t="inlineStr">
-        <is>
-          <t>Functional</t>
-        </is>
-      </c>
-      <c r="D18" s="2" t="inlineStr">
+      <c r="C15" s="2" t="inlineStr">
+        <is>
+          <t>Functional</t>
+        </is>
+      </c>
+      <c r="D15" s="2" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="E18" s="2" t="inlineStr">
+      <c r="E15" s="2" t="inlineStr">
         <is>
           <t>1. You are signed in to the ShopView App on a desktop browser.
 2. The report shows: a part with a normal positive margin, a part whose Margin % computes negative (unit sell below unit cost), and — if producible — a part whose Total Sell is zero.</t>
         </is>
       </c>
-      <c r="F18" s="2" t="inlineStr">
+      <c r="F15" s="2" t="inlineStr">
         <is>
           <t>1. Read the normal part's Margin % and check it against Margin ÷ Total Sell × 100.
 2. Read the negative-margin part's Margin %.
 3. Read the zero-Total-Sell part's Margin % if one exists.</t>
         </is>
       </c>
-      <c r="G18" s="2" t="inlineStr">
+      <c r="G15" s="2" t="inlineStr">
         <is>
           <t>1. Margin % shows Margin as a percentage of Total Sell, to one decimal place followed by a percent sign — for example "39.7%".
 2. A Margin % that computes to a real number, including a negative one, shows its signed value.
 3. Margin % shows "—" when Total Sell is zero or negative (the percentage is undefined).</t>
         </is>
       </c>
-      <c r="H18" s="2" t="inlineStr">
+      <c r="H15" s="2" t="inlineStr">
         <is>
           <t>specs/inventory-value.md Story 3 S3-R9; S3-E3</t>
         </is>
       </c>
-      <c r="I18" s="2" t="inlineStr"/>
-      <c r="J18" s="2" t="inlineStr"/>
-    </row>
-    <row r="19">
-      <c r="A19" s="2" t="inlineStr">
+      <c r="I15" s="2" t="inlineStr"/>
+      <c r="J15" s="2" t="inlineStr"/>
+    </row>
+    <row r="16">
+      <c r="A16" s="2" t="inlineStr">
         <is>
           <t>With every column turned on, the columns appear in the fixed left-to-right order with the specified alignment</t>
         </is>
       </c>
-      <c r="B19" s="2" t="inlineStr">
+      <c r="B16" s="2" t="inlineStr">
         <is>
           <t>IV — Valuation &amp; Columns</t>
         </is>
       </c>
-      <c r="C19" s="2" t="inlineStr">
-        <is>
-          <t>Functional</t>
-        </is>
-      </c>
-      <c r="D19" s="2" t="inlineStr">
+      <c r="C16" s="2" t="inlineStr">
+        <is>
+          <t>Functional</t>
+        </is>
+      </c>
+      <c r="D16" s="2" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="E19" s="2" t="inlineStr">
+      <c r="E16" s="2" t="inlineStr">
         <is>
           <t>1. You are signed in to the ShopView App on a desktop browser.
 2. The Inventory Value report is open with rows loaded.
 3. Every column (including Margin and Total Sell) is turned on in the column-selection control.</t>
         </is>
       </c>
-      <c r="F19" s="2" t="inlineStr">
+      <c r="F16" s="2" t="inlineStr">
         <is>
           <t>1. Read the column headers from left to right.
 2. Look at how the values in each column are aligned.</t>
         </is>
       </c>
-      <c r="G19" s="2" t="inlineStr">
+      <c r="G16" s="2" t="inlineStr">
         <is>
           <t>1. The columns appear in this order: Part #, Description, Category, Vendor, Qty on Hand, Unit Cost, Unit Sell, Margin, Margin %, Total Sell, Total Cost.
 2. Part #, Description, Category, and Vendor are left-aligned.
 3. Every other column is right-aligned.</t>
         </is>
       </c>
-      <c r="H19" s="2" t="inlineStr">
+      <c r="H16" s="2" t="inlineStr">
         <is>
           <t>specs/inventory-value.md Story 3 S3-R1; S3-R2</t>
         </is>
       </c>
-      <c r="I19" s="2" t="inlineStr"/>
-      <c r="J19" s="2" t="inlineStr"/>
-    </row>
-    <row r="20">
-      <c r="A20" s="2" t="inlineStr">
+      <c r="I16" s="2" t="inlineStr"/>
+      <c r="J16" s="2" t="inlineStr"/>
+    </row>
+    <row r="17">
+      <c r="A17" s="2" t="inlineStr">
         <is>
           <t>Value formats: Qty on Hand to two decimals with no currency symbol (fractional supported), money values as US-dollar currency</t>
         </is>
       </c>
-      <c r="B20" s="2" t="inlineStr">
+      <c r="B17" s="2" t="inlineStr">
         <is>
           <t>IV — Valuation &amp; Columns</t>
         </is>
       </c>
-      <c r="C20" s="2" t="inlineStr">
-        <is>
-          <t>Functional</t>
-        </is>
-      </c>
-      <c r="D20" s="2" t="inlineStr">
+      <c r="C17" s="2" t="inlineStr">
+        <is>
+          <t>Functional</t>
+        </is>
+      </c>
+      <c r="D17" s="2" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="E20" s="2" t="inlineStr">
+      <c r="E17" s="2" t="inlineStr">
         <is>
           <t>1. You are signed in to the ShopView App on a desktop browser.
 2. The report shows a part with a fractional on-hand quantity (for example 2.50), one with values over $1,000, and (if producible) one with a negative money value.</t>
         </is>
       </c>
-      <c r="F20" s="2" t="inlineStr">
+      <c r="F17" s="2" t="inlineStr">
         <is>
           <t>1. Read the Qty on Hand cell of the fractional-quantity part.
 2. Read a money value over one thousand dollars (Unit Cost, Unit Sell, Total Sell, or Total Cost).
 3. Read a genuine zero money value and a negative one if present.</t>
         </is>
       </c>
-      <c r="G20" s="2" t="inlineStr">
+      <c r="G17" s="2" t="inlineStr">
         <is>
           <t>1. Qty on Hand shows the on-hand quantity to two decimal places, with no currency symbol; fractional quantities display correctly.
 2. Unit Cost and Unit Sell show per-unit prices as US-dollar currency.
 3. Money values show a leading "$", two decimal places, and thousands separators (for example "$1,234.56"); a negative value shows a leading minus before the "$" ("-$1,234.56"); a genuine zero shows "$0.00".</t>
         </is>
       </c>
-      <c r="H20" s="2" t="inlineStr">
+      <c r="H17" s="2" t="inlineStr">
         <is>
           <t>specs/inventory-value.md Story 3 S3-R3; S3-R4; S3-R5 (display); S3-R10; §4 Terminology (On-hand quantity)</t>
         </is>
       </c>
-      <c r="I20" s="2" t="inlineStr"/>
-      <c r="J20" s="2" t="inlineStr"/>
-    </row>
-    <row r="21">
-      <c r="A21" s="2" t="inlineStr">
+      <c r="I17" s="2" t="inlineStr"/>
+      <c r="J17" s="2" t="inlineStr"/>
+    </row>
+    <row r="18">
+      <c r="A18" s="2" t="inlineStr">
         <is>
           <t>The Total Cost column (header and cells) is bold and pinned to the far right, staying fixed while scrolling sideways</t>
         </is>
       </c>
-      <c r="B21" s="2" t="inlineStr">
+      <c r="B18" s="2" t="inlineStr">
         <is>
           <t>IV — Valuation &amp; Columns</t>
         </is>
       </c>
-      <c r="C21" s="2" t="inlineStr">
-        <is>
-          <t>Functional</t>
-        </is>
-      </c>
-      <c r="D21" s="2" t="inlineStr">
+      <c r="C18" s="2" t="inlineStr">
+        <is>
+          <t>Functional</t>
+        </is>
+      </c>
+      <c r="D18" s="2" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="E21" s="2" t="inlineStr">
+      <c r="E18" s="2" t="inlineStr">
         <is>
           <t>1. You are signed in to the ShopView App on a desktop browser.
 2. Enough columns are turned on that the table scrolls horizontally.</t>
         </is>
       </c>
-      <c r="F21" s="2" t="inlineStr">
+      <c r="F18" s="2" t="inlineStr">
         <is>
           <t>1. Look at the Total Cost column header and its cells.
 2. Scroll the rows sideways and watch the Total Cost column.</t>
         </is>
       </c>
-      <c r="G21" s="2" t="inlineStr">
+      <c r="G18" s="2" t="inlineStr">
         <is>
           <t>1. The Total Cost column is pinned to the far right of the row and shown in bold — it is the report's headline column.
 2. The Total Cost column header is bold and pinned, matching its cells.
 3. It stays fixed to the right edge while the other columns scroll underneath.</t>
         </is>
       </c>
-      <c r="H21" s="2" t="inlineStr">
+      <c r="H18" s="2" t="inlineStr">
         <is>
           <t>specs/inventory-value.md Story 3 S3-R11; Story 12 S12-R4; §3 Key Decisions</t>
         </is>
       </c>
-      <c r="I21" s="2" t="inlineStr"/>
-      <c r="J21" s="2" t="inlineStr"/>
-    </row>
-    <row r="22">
-      <c r="A22" s="2" t="inlineStr">
+      <c r="I18" s="2" t="inlineStr"/>
+      <c r="J18" s="2" t="inlineStr"/>
+    </row>
+    <row r="19">
+      <c r="A19" s="2" t="inlineStr">
         <is>
           <t>On first visit the default columns show, with Margin and Total Sell hidden by default but available to turn on</t>
         </is>
       </c>
-      <c r="B22" s="2" t="inlineStr">
+      <c r="B19" s="2" t="inlineStr">
         <is>
           <t>IV — Valuation &amp; Columns</t>
         </is>
       </c>
-      <c r="C22" s="2" t="inlineStr">
-        <is>
-          <t>Functional</t>
-        </is>
-      </c>
-      <c r="D22" s="2" t="inlineStr">
+      <c r="C19" s="2" t="inlineStr">
+        <is>
+          <t>Functional</t>
+        </is>
+      </c>
+      <c r="D19" s="2" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="E22" s="2" t="inlineStr">
+      <c r="E19" s="2" t="inlineStr">
         <is>
           <t>1. You are signed in to the ShopView App on a desktop browser that has never saved settings for this report (fresh visit).</t>
         </is>
       </c>
-      <c r="F22" s="2" t="inlineStr">
+      <c r="F19" s="2" t="inlineStr">
         <is>
           <t>1. Open the Inventory Value report and read the visible column headers.
 2. Open the column-selection control and read which columns are on and off.
 3. Turn Margin and Total Sell on and check they appear.</t>
         </is>
       </c>
-      <c r="G22" s="2" t="inlineStr">
+      <c r="G19" s="2" t="inlineStr">
         <is>
           <t>1. On first visit, the visible columns are: Part #, Description, Category, Vendor, Qty on Hand, Unit Cost, Unit Sell, Margin %, and Total Cost.
 2. The Margin and Total Sell columns are hidden by default.
 3. Both can be turned on from the column-selection control and then appear in their fixed positions.</t>
         </is>
       </c>
-      <c r="H22" s="2" t="inlineStr">
+      <c r="H19" s="2" t="inlineStr">
         <is>
           <t>specs/inventory-value.md Story 3 S3-R12; S3-R13; Story 8 S8-R3</t>
         </is>
       </c>
-      <c r="I22" s="2" t="inlineStr"/>
-      <c r="J22" s="2" t="inlineStr"/>
-    </row>
-    <row r="23">
-      <c r="A23" s="2" t="inlineStr">
+      <c r="I19" s="2" t="inlineStr"/>
+      <c r="J19" s="2" t="inlineStr"/>
+    </row>
+    <row r="20">
+      <c r="A20" s="2" t="inlineStr">
         <is>
           <t>Category and Vendor show their names, and an em dash ("—") when the part has none</t>
         </is>
       </c>
-      <c r="B23" s="2" t="inlineStr">
+      <c r="B20" s="2" t="inlineStr">
         <is>
           <t>IV — Valuation &amp; Columns</t>
         </is>
       </c>
-      <c r="C23" s="2" t="inlineStr">
-        <is>
-          <t>Functional</t>
-        </is>
-      </c>
-      <c r="D23" s="2" t="inlineStr">
+      <c r="C20" s="2" t="inlineStr">
+        <is>
+          <t>Functional</t>
+        </is>
+      </c>
+      <c r="D20" s="2" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="E23" s="2" t="inlineStr">
+      <c r="E20" s="2" t="inlineStr">
         <is>
           <t>1. You are signed in to the ShopView App on a desktop browser.
 2. The report shows a part with a category and a vendor, a part with no category, and a part with no vendor.</t>
         </is>
       </c>
-      <c r="F23" s="2" t="inlineStr">
+      <c r="F20" s="2" t="inlineStr">
         <is>
           <t>1. Read the Category and Vendor cells of the fully-populated part.
 2. Read the Category cell of the part with no category.
 3. Read the Vendor cell of the part with no vendor.</t>
         </is>
       </c>
-      <c r="G23" s="2" t="inlineStr">
+      <c r="G20" s="2" t="inlineStr">
         <is>
           <t>1. Category shows the part's category name; Vendor shows the part's vendor name.
 2. A part with no category shows an em dash ("—") in its Category cell.
 3. A part with no vendor shows an em dash ("—") in its Vendor cell.</t>
         </is>
       </c>
-      <c r="H23" s="2" t="inlineStr">
+      <c r="H20" s="2" t="inlineStr">
         <is>
           <t>specs/inventory-value.md Story 3 S3-R14; S3-E1; S3-E2</t>
         </is>
       </c>
-      <c r="I23" s="2" t="inlineStr"/>
-      <c r="J23" s="2" t="inlineStr"/>
-    </row>
-    <row r="24">
-      <c r="A24" s="2" t="inlineStr">
-        <is>
-          <t>The totals row is labeled "Total" in the Part # cell, leaves the per-unit and identity cells blank, and pins its bold Total Cost far right</t>
-        </is>
-      </c>
-      <c r="B24" s="2" t="inlineStr">
+      <c r="I20" s="2" t="inlineStr"/>
+      <c r="J20" s="2" t="inlineStr"/>
+    </row>
+    <row r="21">
+      <c r="A21" s="2" t="inlineStr">
+        <is>
+          <t>Totals row: Total label, blank identity/per-unit cells, pinned bold Total Cost</t>
+        </is>
+      </c>
+      <c r="B21" s="2" t="inlineStr">
         <is>
           <t>IV — Totals Row</t>
         </is>
       </c>
-      <c r="C24" s="2" t="inlineStr">
-        <is>
-          <t>Functional</t>
-        </is>
-      </c>
-      <c r="D24" s="2" t="inlineStr">
+      <c r="C21" s="2" t="inlineStr">
+        <is>
+          <t>Functional</t>
+        </is>
+      </c>
+      <c r="D21" s="2" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="E24" s="2" t="inlineStr">
-        <is>
-          <t>1. You are signed in to the ShopView App on a desktop browser.
-2. The Inventory Value report is open with rows loaded and all columns turned on.</t>
-        </is>
-      </c>
-      <c r="F24" s="2" t="inlineStr">
+      <c r="E21" s="2" t="inlineStr">
+        <is>
+          <t>1. You are signed in to the ShopView App on a desktop browser.
+2. The Inventory Value report is open with rows loaded and all columns turned on.
+3. The page shows more rows than fit on the screen.</t>
+        </is>
+      </c>
+      <c r="F21" s="2" t="inlineStr">
         <is>
           <t>1. Look at the row at the bottom of the report.
 2. Read its Part # cell, its Description/Category/Vendor cells, and its Unit Cost/Unit Sell cells.
-3. Look at its Total Cost cell and compare the number formats to the data rows.</t>
-        </is>
-      </c>
-      <c r="G24" s="2" t="inlineStr">
+3. Look at its Total Cost cell and compare the number formats to the data rows.
+4. Scroll the rows up and down and watch the totals row.</t>
+        </is>
+      </c>
+      <c r="G21" s="2" t="inlineStr">
         <is>
           <t>1. A totals row is shown at the bottom, with the literal label "Total" in the Part # column's cell.
 2. The Description, Category, and Vendor cells are blank; the Unit Cost and Unit Sell cells are blank (a per-unit price has no meaningful sum).
-3. The totals-row Total Cost cell is pinned far right and bold, matching the column, and the row uses the same number formats as the data rows.</t>
-        </is>
-      </c>
-      <c r="H24" s="2" t="inlineStr">
-        <is>
-          <t>specs/inventory-value.md Story 4 S4-R1; S4-R4; S4-R5; S4-R6; S4-R7</t>
-        </is>
-      </c>
-      <c r="I24" s="2" t="inlineStr"/>
-      <c r="J24" s="2" t="inlineStr"/>
-    </row>
-    <row r="25">
-      <c r="A25" s="2" t="inlineStr">
-        <is>
-          <t>The totals row sums Qty on Hand, Margin, Total Sell, and Total Cost over the FULL filtered set on the server, not just the visible page</t>
-        </is>
-      </c>
-      <c r="B25" s="2" t="inlineStr">
+3. The totals-row Total Cost cell is pinned far right and bold, matching the column, and the row uses the same number formats as the data rows.
+4. The totals row stays visible at the bottom while the rows scroll.</t>
+        </is>
+      </c>
+      <c r="H21" s="2" t="inlineStr">
+        <is>
+          <t>specs/inventory-value.md Story 4 S4-R1; S4-R4; S4-R5; S4-R6; S4-R7; Story 12 S12-R5</t>
+        </is>
+      </c>
+      <c r="I21" s="2" t="inlineStr"/>
+      <c r="J21" s="2" t="inlineStr"/>
+    </row>
+    <row r="22">
+      <c r="A22" s="2" t="inlineStr">
+        <is>
+          <t>Totals row sums the FULL filtered set on the server, not just the visible page</t>
+        </is>
+      </c>
+      <c r="B22" s="2" t="inlineStr">
         <is>
           <t>IV — Totals Row</t>
         </is>
       </c>
-      <c r="C25" s="2" t="inlineStr">
-        <is>
-          <t>Functional</t>
-        </is>
-      </c>
-      <c r="D25" s="2" t="inlineStr">
+      <c r="C22" s="2" t="inlineStr">
+        <is>
+          <t>Functional</t>
+        </is>
+      </c>
+      <c r="D22" s="2" t="inlineStr">
         <is>
           <t>Critical</t>
         </is>
       </c>
-      <c r="E25" s="2" t="inlineStr">
+      <c r="E22" s="2" t="inlineStr">
         <is>
           <t>1. You are signed in to the ShopView App on a desktop browser.
 2. The current filtered set spans more than one page (more rows than one page shows).
-3. The Margin and Total Sell columns are turned on.</t>
-        </is>
-      </c>
-      <c r="F25" s="2" t="inlineStr">
+3. The Margin and Total Sell columns are turned on.
+4. The report shows parts across at least two categories and two vendors.</t>
+        </is>
+      </c>
+      <c r="F22" s="2" t="inlineStr">
         <is>
           <t>1. Note the totals row's Qty on Hand, Margin, Total Sell, and Total Cost on page 1.
 2. Move to page 2 and read the totals row again.
-3. Cross-check the Total Cost total against a known seeded subset (filter down to a handful of ZZAUTOTEST parts whose values you can sum by hand).</t>
-        </is>
-      </c>
-      <c r="G25" s="2" t="inlineStr">
+3. Cross-check the Total Cost total against a known seeded subset (filter down to a handful of ZZAUTOTEST parts whose values you can sum by hand).
+4. Select one Category and read the totals row; clear it, select one Vendor; clear it, type a part search matching a subset — reading the totals row each time (from a later page too if the set spans pages).</t>
+        </is>
+      </c>
+      <c r="G22" s="2" t="inlineStr">
         <is>
           <t>1. The totals row sums Qty on Hand, Margin, Total Sell, and Total Cost across the FULL filtered result set — every qualifying row for the current Date, Location, Category, Vendor, and part-search selection, not only the rows on the visible page.
 2. The totals are identical on every page (they do not change as you page).
-3. The hand-summed subset matches the server-computed totals to the cent.</t>
-        </is>
-      </c>
-      <c r="H25" s="2" t="inlineStr">
-        <is>
-          <t>specs/inventory-value.md Story 4 S4-R2; §2 Scale and data model; §4 Terminology (Filtered set)</t>
-        </is>
-      </c>
-      <c r="I25" s="2" t="inlineStr"/>
-      <c r="J25" s="2" t="inlineStr"/>
-    </row>
-    <row r="26">
-      <c r="A26" s="2" t="inlineStr">
+3. The hand-summed subset matches the server-computed totals to the cent.
+4. After each filter change the totals row recomputes on the server over the full filtered set, independent of which page is shown.</t>
+        </is>
+      </c>
+      <c r="H22" s="2" t="inlineStr">
+        <is>
+          <t>specs/inventory-value.md Story 4 S4-R2; S4-R8; Story 6 S6-R6; §2 Scale and data model; §4 Terminology (Filtered set)</t>
+        </is>
+      </c>
+      <c r="I22" s="2" t="inlineStr"/>
+      <c r="J22" s="2" t="inlineStr"/>
+    </row>
+    <row r="23">
+      <c r="A23" s="2" t="inlineStr">
         <is>
           <t>The totals-row Margin % is recomputed from the totals (total Margin ÷ total Total Sell), not the average of the row percentages</t>
         </is>
       </c>
-      <c r="B26" s="2" t="inlineStr">
+      <c r="B23" s="2" t="inlineStr">
         <is>
           <t>IV — Totals Row</t>
         </is>
       </c>
-      <c r="C26" s="2" t="inlineStr">
-        <is>
-          <t>Functional</t>
-        </is>
-      </c>
-      <c r="D26" s="2" t="inlineStr">
+      <c r="C23" s="2" t="inlineStr">
+        <is>
+          <t>Functional</t>
+        </is>
+      </c>
+      <c r="D23" s="2" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="E26" s="2" t="inlineStr">
+      <c r="E23" s="2" t="inlineStr">
         <is>
           <t>1. You are signed in to the ShopView App on a desktop browser.
 2. The filtered set contains parts with clearly different Margin % values (so a recomputed figure differs from a simple average).
 3. The Margin and Total Sell columns are turned on.</t>
         </is>
       </c>
-      <c r="F26" s="2" t="inlineStr">
+      <c r="F23" s="2" t="inlineStr">
         <is>
           <t>1. Read the totals row's Margin, Total Sell, and Margin %.
 2. Compute total Margin ÷ total Total Sell × 100 and compare to the shown Margin %.
 3. Also compute the plain average of the row Margin % values and confirm the shown figure is NOT that.</t>
         </is>
       </c>
-      <c r="G26" s="2" t="inlineStr">
+      <c r="G23" s="2" t="inlineStr">
         <is>
           <t>1. The totals-row Margin % equals total Margin ÷ total Total Sell × 100 (to one decimal place with a percent sign).
 2. It is NOT the average of the row percentages.
 3. It shows "—" when the total Total Sell is zero or negative.</t>
         </is>
       </c>
-      <c r="H26" s="2" t="inlineStr">
+      <c r="H23" s="2" t="inlineStr">
         <is>
           <t>specs/inventory-value.md Story 4 S4-R3</t>
         </is>
       </c>
-      <c r="I26" s="2" t="inlineStr"/>
-      <c r="J26" s="2" t="inlineStr"/>
-    </row>
-    <row r="27">
-      <c r="A27" s="2" t="inlineStr">
-        <is>
-          <t>Applying the Category filter, the Vendor filter, or the part search recomputes the totals on the server to match the filtered set</t>
-        </is>
-      </c>
-      <c r="B27" s="2" t="inlineStr">
-        <is>
-          <t>IV — Totals Row</t>
-        </is>
-      </c>
-      <c r="C27" s="2" t="inlineStr">
-        <is>
-          <t>Functional</t>
-        </is>
-      </c>
-      <c r="D27" s="2" t="inlineStr">
+      <c r="I23" s="2" t="inlineStr"/>
+      <c r="J23" s="2" t="inlineStr"/>
+    </row>
+    <row r="24">
+      <c r="A24" s="2" t="inlineStr">
+        <is>
+          <t>The date-range control offers the standard presets plus Custom and does not offer "All Time" — expected, do not file</t>
+        </is>
+      </c>
+      <c r="B24" s="2" t="inlineStr">
+        <is>
+          <t>IV — As-of Date &amp; Snapshots</t>
+        </is>
+      </c>
+      <c r="C24" s="2" t="inlineStr">
+        <is>
+          <t>Functional</t>
+        </is>
+      </c>
+      <c r="D24" s="2" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="E27" s="2" t="inlineStr">
-        <is>
-          <t>1. You are signed in to the ShopView App on a desktop browser.
-2. The report shows parts across at least two categories and two vendors.</t>
-        </is>
-      </c>
-      <c r="F27" s="2" t="inlineStr">
-        <is>
-          <t>1. Note the totals row, then select one Category and read the totals row again.
-2. Clear it, select one Vendor, and read the totals row.
-3. Clear it, type a part search that matches a subset, and read the totals row.
-4. If the filtered set spans pages, check the totals from a later page too.</t>
-        </is>
-      </c>
-      <c r="G27" s="2" t="inlineStr">
-        <is>
-          <t>1. After each change, the totals row recomputes on the server over the full filtered set to match the filtered result.
-2. The recomputed totals are independent of which page is currently shown.</t>
-        </is>
-      </c>
-      <c r="H27" s="2" t="inlineStr">
-        <is>
-          <t>specs/inventory-value.md Story 4 S4-R8; Story 6 S6-R6</t>
-        </is>
-      </c>
-      <c r="I27" s="2" t="inlineStr"/>
-      <c r="J27" s="2" t="inlineStr"/>
-    </row>
-    <row r="28">
-      <c r="A28" s="2" t="inlineStr">
-        <is>
-          <t>When no parts qualify, no totals row is shown</t>
-        </is>
-      </c>
-      <c r="B28" s="2" t="inlineStr">
-        <is>
-          <t>IV — Totals Row</t>
-        </is>
-      </c>
-      <c r="C28" s="2" t="inlineStr">
-        <is>
-          <t>Negative</t>
-        </is>
-      </c>
-      <c r="D28" s="2" t="inlineStr">
-        <is>
-          <t>Medium</t>
-        </is>
-      </c>
-      <c r="E28" s="2" t="inlineStr">
-        <is>
-          <t>1. You are signed in to the ShopView App on a desktop browser.
-2. The filters can be set so that no part qualifies (for example, a part search matching nothing).</t>
-        </is>
-      </c>
-      <c r="F28" s="2" t="inlineStr">
-        <is>
-          <t>1. Apply a filter or search that leaves no qualifying part.
-2. Look at the bottom of the data area.</t>
-        </is>
-      </c>
-      <c r="G28" s="2" t="inlineStr">
-        <is>
-          <t>1. The no-data message shows instead of rows and NO totals row is shown.</t>
-        </is>
-      </c>
-      <c r="H28" s="2" t="inlineStr">
-        <is>
-          <t>specs/inventory-value.md Story 4 S4-N1; Story 1 S1-N2</t>
-        </is>
-      </c>
-      <c r="I28" s="2" t="inlineStr"/>
-      <c r="J28" s="2" t="inlineStr"/>
-    </row>
-    <row r="29">
-      <c r="A29" s="2" t="inlineStr">
-        <is>
-          <t>The date-range control offers the standard presets plus Custom and does not offer "All Time" — expected, do not file</t>
-        </is>
-      </c>
-      <c r="B29" s="2" t="inlineStr">
-        <is>
-          <t>IV — As-of Date &amp; Snapshots</t>
-        </is>
-      </c>
-      <c r="C29" s="2" t="inlineStr">
-        <is>
-          <t>Functional</t>
-        </is>
-      </c>
-      <c r="D29" s="2" t="inlineStr">
-        <is>
-          <t>High</t>
-        </is>
-      </c>
-      <c r="E29" s="2" t="inlineStr">
+      <c r="E24" s="2" t="inlineStr">
         <is>
           <t>1. You are signed in to the ShopView App on a desktop browser.
 2. The Inventory Value report is open.</t>
         </is>
       </c>
-      <c r="F29" s="2" t="inlineStr">
+      <c r="F24" s="2" t="inlineStr">
         <is>
           <t>1. Open the date-range control in the toolbar.
 2. Read every option offered.</t>
         </is>
       </c>
-      <c r="G29" s="2" t="inlineStr">
+      <c r="G24" s="2" t="inlineStr">
         <is>
           <t>1. The control offers the standard presets: "Today", "Yesterday", "This Week", "Last Week", "This Month", "Last Month", "This Year", "Last Year", "This Quarter", "Last Quarter", and "Custom".
 2. "All Time" is NOT offered — because the report is valued as of a single date, an All-Time option would be meaningless; its absence is the documented v1 behavior.</t>
         </is>
       </c>
-      <c r="H29" s="2" t="inlineStr">
+      <c r="H24" s="2" t="inlineStr">
         <is>
           <t>specs/inventory-value.md Story 5 S5-R1; §2 Known Limitations (v1)</t>
         </is>
       </c>
-      <c r="I29" s="2" t="inlineStr"/>
-      <c r="J29" s="2" t="inlineStr"/>
-    </row>
-    <row r="30">
-      <c r="A30" s="2" t="inlineStr">
+      <c r="I24" s="2" t="inlineStr"/>
+      <c r="J24" s="2" t="inlineStr"/>
+    </row>
+    <row r="25">
+      <c r="A25" s="2" t="inlineStr">
         <is>
           <t>The report values inventory as of the END of the selected range — the date is an as-of anchor, not a created-date filter</t>
         </is>
       </c>
-      <c r="B30" s="2" t="inlineStr">
+      <c r="B25" s="2" t="inlineStr">
         <is>
           <t>IV — As-of Date &amp; Snapshots</t>
         </is>
       </c>
-      <c r="C30" s="2" t="inlineStr">
-        <is>
-          <t>Functional</t>
-        </is>
-      </c>
-      <c r="D30" s="2" t="inlineStr">
+      <c r="C25" s="2" t="inlineStr">
+        <is>
+          <t>Functional</t>
+        </is>
+      </c>
+      <c r="D25" s="2" t="inlineStr">
         <is>
           <t>Critical</t>
         </is>
       </c>
-      <c r="E30" s="2" t="inlineStr">
+      <c r="E25" s="2" t="inlineStr">
         <is>
           <t>1. You are signed in to the ShopView App on a desktop browser.
 2. Nightly snapshots exist for past dates at the selected location (recording has been running).
 3. A part exists that was ALREADY in stock before the selected range started.</t>
         </is>
       </c>
-      <c r="F30" s="2" t="inlineStr">
+      <c r="F25" s="2" t="inlineStr">
         <is>
           <t>1. Select a past range (for example "Last Month").
 2. Check which date the displayed values represent.
 3. Look for the part that was stocked before the range started.</t>
         </is>
       </c>
-      <c r="G30" s="2" t="inlineStr">
+      <c r="G25" s="2" t="inlineStr">
         <is>
           <t>1. The report values inventory as of the END of the selected range.
 2. The date control is an "as of" anchor, not a created-date filter — narrowing it does not select "parts added in that range"; it shows the whole shelf as it stood on that date, so the part stocked before the range still appears.</t>
         </is>
       </c>
-      <c r="H30" s="2" t="inlineStr">
+      <c r="H25" s="2" t="inlineStr">
         <is>
           <t>specs/inventory-value.md Story 5 S5-R2 (+ context note)</t>
         </is>
       </c>
-      <c r="I30" s="2" t="inlineStr"/>
-      <c r="J30" s="2" t="inlineStr"/>
-    </row>
-    <row r="31">
-      <c r="A31" s="2" t="inlineStr">
+      <c r="I25" s="2" t="inlineStr"/>
+      <c r="J25" s="2" t="inlineStr"/>
+    </row>
+    <row r="26">
+      <c r="A26" s="2" t="inlineStr">
         <is>
           <t>When the selected window reaches today and today has not been recorded yet, the report values the current live stock</t>
         </is>
       </c>
-      <c r="B31" s="2" t="inlineStr">
+      <c r="B26" s="2" t="inlineStr">
         <is>
           <t>IV — As-of Date &amp; Snapshots</t>
         </is>
       </c>
-      <c r="C31" s="2" t="inlineStr">
-        <is>
-          <t>Functional</t>
-        </is>
-      </c>
-      <c r="D31" s="2" t="inlineStr">
+      <c r="C26" s="2" t="inlineStr">
+        <is>
+          <t>Functional</t>
+        </is>
+      </c>
+      <c r="D26" s="2" t="inlineStr">
         <is>
           <t>Critical</t>
         </is>
       </c>
-      <c r="E31" s="2" t="inlineStr">
+      <c r="E26" s="2" t="inlineStr">
         <is>
           <t>1. You are signed in to the ShopView App on a desktop browser.
 2. Today's nightly snapshot has not yet been recorded (the normal daytime state).
 3. A ZZAUTOTEST part's on-hand quantity was changed TODAY (after last night's capture).</t>
         </is>
       </c>
-      <c r="F31" s="2" t="inlineStr">
+      <c r="F26" s="2" t="inlineStr">
         <is>
           <t>1. Select a range that reaches today (for example "This Month" or "Today").
 2. Find the part whose quantity changed today and read its row.</t>
         </is>
       </c>
-      <c r="G31" s="2" t="inlineStr">
+      <c r="G26" s="2" t="inlineStr">
         <is>
           <t>1. The report values the current live stock — the values represent today.
 2. The part's row reflects today's changed quantity (not yesterday's snapshot), proving the live fallback is in use.</t>
         </is>
       </c>
-      <c r="H31" s="2" t="inlineStr">
+      <c r="H26" s="2" t="inlineStr">
         <is>
           <t>specs/inventory-value.md Story 5 S5-R3; §3 Key Decisions (live fallback for today)</t>
         </is>
       </c>
-      <c r="I31" s="2" t="inlineStr"/>
-      <c r="J31" s="2" t="inlineStr"/>
-    </row>
-    <row r="32">
-      <c r="A32" s="2" t="inlineStr">
+      <c r="I26" s="2" t="inlineStr"/>
+      <c r="J26" s="2" t="inlineStr"/>
+    </row>
+    <row r="27">
+      <c r="A27" s="2" t="inlineStr">
         <is>
           <t>For a past date the report replays the closest recorded day on or before the end of the selected range</t>
         </is>
       </c>
-      <c r="B32" s="2" t="inlineStr">
+      <c r="B27" s="2" t="inlineStr">
         <is>
           <t>IV — As-of Date &amp; Snapshots</t>
         </is>
       </c>
-      <c r="C32" s="2" t="inlineStr">
-        <is>
-          <t>Functional</t>
-        </is>
-      </c>
-      <c r="D32" s="2" t="inlineStr">
+      <c r="C27" s="2" t="inlineStr">
+        <is>
+          <t>Functional</t>
+        </is>
+      </c>
+      <c r="D27" s="2" t="inlineStr">
         <is>
           <t>Critical</t>
         </is>
       </c>
-      <c r="E32" s="2" t="inlineStr">
+      <c r="E27" s="2" t="inlineStr">
         <is>
           <t>1. You are signed in to the ShopView App on a desktop browser.
 2. Nightly snapshots exist for past dates, and a ZZAUTOTEST part's quantity is known to have DIFFERED on a past recorded day from its quantity today.</t>
         </is>
       </c>
-      <c r="F32" s="2" t="inlineStr">
+      <c r="F27" s="2" t="inlineStr">
         <is>
           <t>1. Select a Custom range ending on the past recorded day.
 2. Find the part and read its quantity and values.
 3. Compare them to what the part held on that recorded day (not today).</t>
         </is>
       </c>
-      <c r="G32" s="2" t="inlineStr">
+      <c r="G27" s="2" t="inlineStr">
         <is>
           <t>1. The report replays the closest recorded day on or before the end of the selected range.
 2. The part's row shows the quantity and values recorded for that day, not today's live stock.</t>
         </is>
       </c>
-      <c r="H32" s="2" t="inlineStr">
+      <c r="H27" s="2" t="inlineStr">
         <is>
           <t>specs/inventory-value.md Story 5 S5-R4; §2 Relationship to nightly history</t>
         </is>
       </c>
-      <c r="I32" s="2" t="inlineStr"/>
-      <c r="J32" s="2" t="inlineStr"/>
-    </row>
-    <row r="33">
-      <c r="A33" s="2" t="inlineStr">
+      <c r="I27" s="2" t="inlineStr"/>
+      <c r="J27" s="2" t="inlineStr"/>
+    </row>
+    <row r="28">
+      <c r="A28" s="2" t="inlineStr">
         <is>
           <t>An "As of" indicator names the day actually shown when it is earlier than the date asked for, and is hidden when they match</t>
         </is>
       </c>
-      <c r="B33" s="2" t="inlineStr">
+      <c r="B28" s="2" t="inlineStr">
         <is>
           <t>IV — As-of Date &amp; Snapshots</t>
         </is>
       </c>
-      <c r="C33" s="2" t="inlineStr">
-        <is>
-          <t>Functional</t>
-        </is>
-      </c>
-      <c r="D33" s="2" t="inlineStr">
+      <c r="C28" s="2" t="inlineStr">
+        <is>
+          <t>Functional</t>
+        </is>
+      </c>
+      <c r="D28" s="2" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="E33" s="2" t="inlineStr">
+      <c r="E28" s="2" t="inlineStr">
         <is>
           <t>1. You are signed in to the ShopView App on a desktop browser.
 2. A past date exists that has NO snapshot of its own but has an earlier recorded day before it (for example, a gap day, or a date in the thinned monthly-retention band).</t>
         </is>
       </c>
-      <c r="F33" s="2" t="inlineStr">
+      <c r="F28" s="2" t="inlineStr">
         <is>
           <t>1. Select a Custom range ending on the gap date (a date with no snapshot of its own).
 2. Look for an "As of" indicator and read which day it names.
 3. Then select a range ending on a day that IS recorded (or today with live values) and look for the indicator again.</t>
         </is>
       </c>
-      <c r="G33" s="2" t="inlineStr">
+      <c r="G28" s="2" t="inlineStr">
         <is>
           <t>1. When the displayed day is an earlier recorded day than the date asked for, the report shows an "As of" indicator naming the day actually shown.
 2. When the displayed day matches the date asked for (the common current-view case), the "As of" indicator is not shown — the date control already communicates the date.</t>
         </is>
       </c>
-      <c r="H33" s="2" t="inlineStr">
+      <c r="H28" s="2" t="inlineStr">
         <is>
           <t>specs/inventory-value.md Story 5 S5-R5; S5-R6</t>
         </is>
       </c>
-      <c r="I33" s="2" t="inlineStr"/>
-      <c r="J33" s="2" t="inlineStr"/>
-    </row>
-    <row r="34">
-      <c r="A34" s="2" t="inlineStr">
+      <c r="I28" s="2" t="inlineStr"/>
+      <c r="J28" s="2" t="inlineStr"/>
+    </row>
+    <row r="29">
+      <c r="A29" s="2" t="inlineStr">
         <is>
           <t>A Custom range lets the user pick start and end dates, values as of the picked end date, is capped at today, and reloads on change</t>
         </is>
       </c>
-      <c r="B34" s="2" t="inlineStr">
+      <c r="B29" s="2" t="inlineStr">
         <is>
           <t>IV — As-of Date &amp; Snapshots</t>
         </is>
       </c>
-      <c r="C34" s="2" t="inlineStr">
-        <is>
-          <t>Functional</t>
-        </is>
-      </c>
-      <c r="D34" s="2" t="inlineStr">
+      <c r="C29" s="2" t="inlineStr">
+        <is>
+          <t>Functional</t>
+        </is>
+      </c>
+      <c r="D29" s="2" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="E34" s="2" t="inlineStr">
+      <c r="E29" s="2" t="inlineStr">
         <is>
           <t>1. You are signed in to the ShopView App on a desktop browser.
 2. The Inventory Value report is open.</t>
         </is>
       </c>
-      <c r="F34" s="2" t="inlineStr">
+      <c r="F29" s="2" t="inlineStr">
         <is>
           <t>1. Open the date-range control and choose "Custom".
 2. Pick a start and an end date in the past and apply.
@@ -2065,289 +1834,244 @@
 4. Watch the data area when the range is applied.</t>
         </is>
       </c>
-      <c r="G34" s="2" t="inlineStr">
+      <c r="G29" s="2" t="inlineStr">
         <is>
           <t>1. A Custom range lets the user pick a start and end date, and the report values as of the picked end date.
 2. A future end date cannot be chosen — the end date is capped at today.
 3. Changing the date range reloads the report (the loading indicator shows and the rows re-fetch).</t>
         </is>
       </c>
-      <c r="H34" s="2" t="inlineStr">
+      <c r="H29" s="2" t="inlineStr">
         <is>
           <t>specs/inventory-value.md Story 5 S5-R7; S5-R8</t>
         </is>
       </c>
-      <c r="I34" s="2" t="inlineStr"/>
-      <c r="J34" s="2" t="inlineStr"/>
-    </row>
-    <row r="35">
-      <c r="A35" s="2" t="inlineStr">
-        <is>
-          <t>When no recorded day exists on or before the end of the selected range, the report shows the no-data message and no totals row</t>
-        </is>
-      </c>
-      <c r="B35" s="2" t="inlineStr">
+      <c r="I29" s="2" t="inlineStr"/>
+      <c r="J29" s="2" t="inlineStr"/>
+    </row>
+    <row r="30">
+      <c r="A30" s="2" t="inlineStr">
+        <is>
+          <t>History accrues forward only — a date before the first nightly recording cannot be reconstructed — expected, do not file</t>
+        </is>
+      </c>
+      <c r="B30" s="2" t="inlineStr">
         <is>
           <t>IV — As-of Date &amp; Snapshots</t>
         </is>
       </c>
-      <c r="C35" s="2" t="inlineStr">
-        <is>
-          <t>Negative</t>
-        </is>
-      </c>
-      <c r="D35" s="2" t="inlineStr">
-        <is>
-          <t>High</t>
-        </is>
-      </c>
-      <c r="E35" s="2" t="inlineStr">
-        <is>
-          <t>1. You are signed in to the ShopView App on a desktop browser.
-2. The date nightly recording began is known, and a past range exists that ends entirely BEFORE it (or whose only covered dates have been pruned by retention).</t>
-        </is>
-      </c>
-      <c r="F35" s="2" t="inlineStr">
-        <is>
-          <t>1. Select a Custom range ending before nightly recording began.
-2. Read the data area and the bottom of the report.</t>
-        </is>
-      </c>
-      <c r="G35" s="2" t="inlineStr">
-        <is>
-          <t>1. The report shows the no-data message "Empty bays, endless possibilities. Get Going!" instead of rows.
-2. No totals row is shown.</t>
-        </is>
-      </c>
-      <c r="H35" s="2" t="inlineStr">
-        <is>
-          <t>specs/inventory-value.md Story 5 S5-N1; §7 User Feedback Summary</t>
-        </is>
-      </c>
-      <c r="I35" s="2" t="inlineStr"/>
-      <c r="J35" s="2" t="inlineStr"/>
-    </row>
-    <row r="36">
-      <c r="A36" s="2" t="inlineStr">
-        <is>
-          <t>History accrues forward only — a date before the first nightly recording cannot be reconstructed — expected, do not file</t>
-        </is>
-      </c>
-      <c r="B36" s="2" t="inlineStr">
-        <is>
-          <t>IV — As-of Date &amp; Snapshots</t>
-        </is>
-      </c>
-      <c r="C36" s="2" t="inlineStr">
-        <is>
-          <t>Functional</t>
-        </is>
-      </c>
-      <c r="D36" s="2" t="inlineStr">
+      <c r="C30" s="2" t="inlineStr">
+        <is>
+          <t>Functional</t>
+        </is>
+      </c>
+      <c r="D30" s="2" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="E36" s="2" t="inlineStr">
+      <c r="E30" s="2" t="inlineStr">
         <is>
           <t>1. You are signed in to the ShopView App on a desktop browser.
 2. The date nightly recording began at this organization is known.</t>
         </is>
       </c>
-      <c r="F36" s="2" t="inlineStr">
+      <c r="F30" s="2" t="inlineStr">
         <is>
           <t>1. Select a range ending before the first nightly recording.
 2. Read what the report shows.</t>
         </is>
       </c>
-      <c r="G36" s="2" t="inlineStr">
+      <c r="G30" s="2" t="inlineStr">
         <is>
           <t>1. The report shows the empty state — there is no way to reconstruct inventory value for a date before recording began, because there is no historical backfill.
 2. This forward-capture-only behavior is the documented v1 boundary, not a defect.</t>
         </is>
       </c>
-      <c r="H36" s="2" t="inlineStr">
+      <c r="H30" s="2" t="inlineStr">
         <is>
           <t>specs/inventory-value.md Story 5 S5-E1; §2 Known Limitations (v1); §2 Out of scope</t>
         </is>
       </c>
-      <c r="I36" s="2" t="inlineStr"/>
-      <c r="J36" s="2" t="inlineStr"/>
-    </row>
-    <row r="37">
-      <c r="A37" s="2" t="inlineStr">
+      <c r="I30" s="2" t="inlineStr"/>
+      <c r="J30" s="2" t="inlineStr"/>
+    </row>
+    <row r="31">
+      <c r="A31" s="2" t="inlineStr">
         <is>
           <t>The Category and Vendor filters are multi-selects that reload the report to only the matching parts</t>
         </is>
       </c>
-      <c r="B37" s="2" t="inlineStr">
+      <c r="B31" s="2" t="inlineStr">
         <is>
           <t>IV — Filters &amp; Part Search</t>
         </is>
       </c>
-      <c r="C37" s="2" t="inlineStr">
-        <is>
-          <t>Functional</t>
-        </is>
-      </c>
-      <c r="D37" s="2" t="inlineStr">
+      <c r="C31" s="2" t="inlineStr">
+        <is>
+          <t>Functional</t>
+        </is>
+      </c>
+      <c r="D31" s="2" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="E37" s="2" t="inlineStr">
+      <c r="E31" s="2" t="inlineStr">
         <is>
           <t>1. You are signed in to the ShopView App on a desktop browser.
 2. In-stock parts exist across at least two categories and two vendors.</t>
         </is>
       </c>
-      <c r="F37" s="2" t="inlineStr">
+      <c r="F31" s="2" t="inlineStr">
         <is>
           <t>1. Open the filter labeled "Category" and select one category; watch the data area.
 2. Add a second category to the selection.
 3. Clear the Category filter, open the filter labeled "Vendor", and select one vendor; then add a second.</t>
         </is>
       </c>
-      <c r="G37" s="2" t="inlineStr">
+      <c r="G31" s="2" t="inlineStr">
         <is>
           <t>1. The toolbar has a Category filter labeled "Category" and a Vendor filter labeled "Vendor", each allowing one or more selections.
 2. Selecting one or more categories reloads the report to show only parts in the selected categories.
 3. Selecting one or more vendors reloads the report to show only parts supplied by the selected vendors.</t>
         </is>
       </c>
-      <c r="H37" s="2" t="inlineStr">
+      <c r="H31" s="2" t="inlineStr">
         <is>
           <t>specs/inventory-value.md Story 6 S6-R1; S6-R2; S6-R3; S6-R4</t>
         </is>
       </c>
-      <c r="I37" s="2" t="inlineStr"/>
-      <c r="J37" s="2" t="inlineStr"/>
-    </row>
-    <row r="38">
-      <c r="A38" s="2" t="inlineStr">
-        <is>
-          <t>The Category filter, Vendor filter, and part search apply server-side — each change re-queries and returns the first page</t>
-        </is>
-      </c>
-      <c r="B38" s="2" t="inlineStr">
+      <c r="I31" s="2" t="inlineStr"/>
+      <c r="J31" s="2" t="inlineStr"/>
+    </row>
+    <row r="32">
+      <c r="A32" s="2" t="inlineStr">
+        <is>
+          <t>Category, Vendor and part search are server-side; each change returns page 1</t>
+        </is>
+      </c>
+      <c r="B32" s="2" t="inlineStr">
         <is>
           <t>IV — Filters &amp; Part Search</t>
         </is>
       </c>
-      <c r="C38" s="2" t="inlineStr">
-        <is>
-          <t>Functional</t>
-        </is>
-      </c>
-      <c r="D38" s="2" t="inlineStr">
+      <c r="C32" s="2" t="inlineStr">
+        <is>
+          <t>Functional</t>
+        </is>
+      </c>
+      <c r="D32" s="2" t="inlineStr">
         <is>
           <t>Critical</t>
         </is>
       </c>
-      <c r="E38" s="2" t="inlineStr">
+      <c r="E32" s="2" t="inlineStr">
         <is>
           <t>1. You are signed in to the ShopView App on a desktop browser.
 2. The unfiltered result set spans multiple pages, and matching parts for a category/vendor/search exist BEYOND page 1.</t>
         </is>
       </c>
-      <c r="F38" s="2" t="inlineStr">
+      <c r="F32" s="2" t="inlineStr">
         <is>
           <t>1. From page 2 (or later), select a Category and check which page shows and which rows are listed.
 2. Repeat with a Vendor selection.
-3. Repeat with a part search.</t>
-        </is>
-      </c>
-      <c r="G38" s="2" t="inlineStr">
+3. Repeat with a part search.
+4. Also change the date range, the location selection, and the sort — watching the data area each time.</t>
+        </is>
+      </c>
+      <c r="G32" s="2" t="inlineStr">
         <is>
           <t>1. Each change re-queries the server and returns the first page of the new result set.
-2. The filtering covers the ENTIRE data set — matching parts that were on later pages appear — not just a narrowing of the rows on the current page.</t>
-        </is>
-      </c>
-      <c r="H38" s="2" t="inlineStr">
-        <is>
-          <t>specs/inventory-value.md Story 6 S6-R5; Story 1 S1-R8</t>
-        </is>
-      </c>
-      <c r="I38" s="2" t="inlineStr"/>
-      <c r="J38" s="2" t="inlineStr"/>
-    </row>
-    <row r="39">
-      <c r="A39" s="2" t="inlineStr">
+2. The filtering covers the ENTIRE data set — matching parts that were on later pages appear — not just a narrowing of the rows on the current page.
+3. Every change — date range, location, Category, Vendor, part search, sort — reloads the rows from the server; while loading the standard reports loading indicator shows, and existing rows are replaced only when the new data returns.</t>
+        </is>
+      </c>
+      <c r="H32" s="2" t="inlineStr">
+        <is>
+          <t>specs/inventory-value.md Story 6 S6-R5; Story 1 S1-R4; S1-R5; S1-R7; S1-R8</t>
+        </is>
+      </c>
+      <c r="I32" s="2" t="inlineStr"/>
+      <c r="J32" s="2" t="inlineStr"/>
+    </row>
+    <row r="33">
+      <c r="A33" s="2" t="inlineStr">
         <is>
           <t>With no category or vendor selected all parts show, and an empty part search applies no narrowing</t>
         </is>
       </c>
-      <c r="B39" s="2" t="inlineStr">
+      <c r="B33" s="2" t="inlineStr">
         <is>
           <t>IV — Filters &amp; Part Search</t>
         </is>
       </c>
-      <c r="C39" s="2" t="inlineStr">
-        <is>
-          <t>Functional</t>
-        </is>
-      </c>
-      <c r="D39" s="2" t="inlineStr">
+      <c r="C33" s="2" t="inlineStr">
+        <is>
+          <t>Functional</t>
+        </is>
+      </c>
+      <c r="D33" s="2" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="E39" s="2" t="inlineStr">
+      <c r="E33" s="2" t="inlineStr">
         <is>
           <t>1. You are signed in to the ShopView App on a desktop browser.
 2. The report has been filtered by category, vendor, and a part search.</t>
         </is>
       </c>
-      <c r="F39" s="2" t="inlineStr">
+      <c r="F33" s="2" t="inlineStr">
         <is>
           <t>1. Clear the Category selection and check the rows.
 2. Clear the Vendor selection and check the rows.
 3. Empty the part search and check the rows.</t>
         </is>
       </c>
-      <c r="G39" s="2" t="inlineStr">
+      <c r="G33" s="2" t="inlineStr">
         <is>
           <t>1. With no category selected, parts of all categories are shown.
 2. With no vendor selected, parts of all vendors are shown.
 3. With the part search empty, no search narrowing is applied.</t>
         </is>
       </c>
-      <c r="H39" s="2" t="inlineStr">
+      <c r="H33" s="2" t="inlineStr">
         <is>
           <t>specs/inventory-value.md Story 6 S6-R7</t>
         </is>
       </c>
-      <c r="I39" s="2" t="inlineStr"/>
-      <c r="J39" s="2" t="inlineStr"/>
-    </row>
-    <row r="40">
-      <c r="A40" s="2" t="inlineStr">
+      <c r="I33" s="2" t="inlineStr"/>
+      <c r="J33" s="2" t="inlineStr"/>
+    </row>
+    <row r="34">
+      <c r="A34" s="2" t="inlineStr">
         <is>
           <t>The part search is a page-local toolbar field matching part number OR description, case-insensitively, on the server</t>
         </is>
       </c>
-      <c r="B40" s="2" t="inlineStr">
+      <c r="B34" s="2" t="inlineStr">
         <is>
           <t>IV — Filters &amp; Part Search</t>
         </is>
       </c>
-      <c r="C40" s="2" t="inlineStr">
-        <is>
-          <t>Functional</t>
-        </is>
-      </c>
-      <c r="D40" s="2" t="inlineStr">
+      <c r="C34" s="2" t="inlineStr">
+        <is>
+          <t>Functional</t>
+        </is>
+      </c>
+      <c r="D34" s="2" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="E40" s="2" t="inlineStr">
+      <c r="E34" s="2" t="inlineStr">
         <is>
           <t>1. You are signed in to the ShopView App on a desktop browser.
 2. In-stock parts exist whose part numbers and descriptions you know (including a description containing a distinctive word).</t>
         </is>
       </c>
-      <c r="F40" s="2" t="inlineStr">
+      <c r="F34" s="2" t="inlineStr">
         <is>
           <t>1. Find the part search input in the report's own toolbar (not the application's global search bar).
 2. Type part of a part number and read the results.
@@ -2355,7 +2079,7 @@
 4. Type text matching nothing.</t>
         </is>
       </c>
-      <c r="G40" s="2" t="inlineStr">
+      <c r="G34" s="2" t="inlineStr">
         <is>
           <t>1. The search field is page-local, in the report's own toolbar — it is not the application's global search bar (the same toolbar-search pattern used elsewhere in the reports suite).
 2. The report narrows to parts whose part number OR description contains the entered text.
@@ -2363,90 +2087,90 @@
 4. The search applies server-side (whole data set, first page returned); a no-match search shows the no-data message.</t>
         </is>
       </c>
-      <c r="H40" s="2" t="inlineStr">
+      <c r="H34" s="2" t="inlineStr">
         <is>
           <t>specs/inventory-value.md Story 6 S6-R8; S6-R5</t>
         </is>
       </c>
-      <c r="I40" s="2" t="inlineStr"/>
-      <c r="J40" s="2" t="inlineStr"/>
-    </row>
-    <row r="41">
-      <c r="A41" s="2" t="inlineStr">
+      <c r="I34" s="2" t="inlineStr"/>
+      <c r="J34" s="2" t="inlineStr"/>
+    </row>
+    <row r="35">
+      <c r="A35" s="2" t="inlineStr">
         <is>
           <t>Date range, Location, Category, Vendor, and the part search combine with AND</t>
         </is>
       </c>
-      <c r="B41" s="2" t="inlineStr">
+      <c r="B35" s="2" t="inlineStr">
         <is>
           <t>IV — Filters &amp; Part Search</t>
         </is>
       </c>
-      <c r="C41" s="2" t="inlineStr">
-        <is>
-          <t>Functional</t>
-        </is>
-      </c>
-      <c r="D41" s="2" t="inlineStr">
+      <c r="C35" s="2" t="inlineStr">
+        <is>
+          <t>Functional</t>
+        </is>
+      </c>
+      <c r="D35" s="2" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="E41" s="2" t="inlineStr">
+      <c r="E35" s="2" t="inlineStr">
         <is>
           <t>1. You are signed in to the ShopView App on a desktop browser.
 2. In-stock parts exist with a known mix of categories and vendors, so a combined filter isolates a known subset.</t>
         </is>
       </c>
-      <c r="F41" s="2" t="inlineStr">
+      <c r="F35" s="2" t="inlineStr">
         <is>
           <t>1. Select a Category, then also a Vendor that only some of those category parts have.
 2. Add a part search matching only one of the remaining parts.
 3. Check the rows and the totals row after each step.</t>
         </is>
       </c>
-      <c r="G41" s="2" t="inlineStr">
+      <c r="G35" s="2" t="inlineStr">
         <is>
           <t>1. A part must satisfy EVERY active filter and the search to appear — the Date range, Location, Category, Vendor, and part search combine with AND.
 2. The totals row matches the combined filtered set after each step.</t>
         </is>
       </c>
-      <c r="H41" s="2" t="inlineStr">
+      <c r="H35" s="2" t="inlineStr">
         <is>
           <t>specs/inventory-value.md Story 6 S6-R9</t>
         </is>
       </c>
-      <c r="I41" s="2" t="inlineStr"/>
-      <c r="J41" s="2" t="inlineStr"/>
-    </row>
-    <row r="42">
-      <c r="A42" s="2" t="inlineStr">
+      <c r="I35" s="2" t="inlineStr"/>
+      <c r="J35" s="2" t="inlineStr"/>
+    </row>
+    <row r="36">
+      <c r="A36" s="2" t="inlineStr">
         <is>
           <t>The Location filter is a rightmost multi-select with an All locations toggle</t>
         </is>
       </c>
-      <c r="B42" s="2" t="inlineStr">
+      <c r="B36" s="2" t="inlineStr">
         <is>
           <t>IV — Location Filter</t>
         </is>
       </c>
-      <c r="C42" s="2" t="inlineStr">
-        <is>
-          <t>Functional</t>
-        </is>
-      </c>
-      <c r="D42" s="2" t="inlineStr">
+      <c r="C36" s="2" t="inlineStr">
+        <is>
+          <t>Functional</t>
+        </is>
+      </c>
+      <c r="D36" s="2" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="E42" s="2" t="inlineStr">
+      <c r="E36" s="2" t="inlineStr">
         <is>
           <t>1. You are signed in to the ShopView App on a desktop browser as a user with access to at least two locations.
 2. This browser has never saved settings for this report (fresh visit).</t>
         </is>
       </c>
-      <c r="F42" s="2" t="inlineStr">
+      <c r="F36" s="2" t="inlineStr">
         <is>
           <t>1. Open the Inventory Value report and find the filter labeled "Location".
 2. Read its position in the toolbar and its default selection.
@@ -2454,333 +2178,287 @@
 4. Select every accessible location ("All locations") and look at how the rows tell you which location they belong to.</t>
         </is>
       </c>
-      <c r="G42" s="2" t="inlineStr">
+      <c r="G36" s="2" t="inlineStr">
         <is>
           <t>1. The toolbar has a location filter labeled "Location" — a multi-select and the rightmost filter — listing the locations the signed-in user has access to, with an "All locations" / "Clear all" toggle.
 2. On a first visit it defaults to the user's currently active location.
 3. With "All locations" active you can tell which location each row's stock belongs to — a location label or marking is shown. (Exactly where and how it appears is confirmed in the build.)</t>
         </is>
       </c>
-      <c r="H42" s="2" t="inlineStr">
+      <c r="H36" s="2" t="inlineStr">
         <is>
           <t>SV-8674 (specs/inventory-value.md Story 7 S7-R1; S7-R2; Story 12 S12-R3 — per-row location identifier in All-locations view ADDED per kickoff video P10 40:58-41:20, user ruling 2026-07-28: video overrides spec (video newer, last-update-wins))</t>
         </is>
       </c>
-      <c r="I42" s="2" t="inlineStr"/>
-      <c r="J42" s="2" t="inlineStr"/>
-    </row>
-    <row r="43">
-      <c r="A43" s="2" t="inlineStr">
+      <c r="I36" s="2" t="inlineStr"/>
+      <c r="J36" s="2" t="inlineStr"/>
+    </row>
+    <row r="37">
+      <c r="A37" s="2" t="inlineStr">
         <is>
           <t>Selecting one, several, or all locations reloads the report scoped to that set</t>
         </is>
       </c>
-      <c r="B43" s="2" t="inlineStr">
+      <c r="B37" s="2" t="inlineStr">
         <is>
           <t>IV — Location Filter</t>
         </is>
       </c>
-      <c r="C43" s="2" t="inlineStr">
-        <is>
-          <t>Functional</t>
-        </is>
-      </c>
-      <c r="D43" s="2" t="inlineStr">
+      <c r="C37" s="2" t="inlineStr">
+        <is>
+          <t>Functional</t>
+        </is>
+      </c>
+      <c r="D37" s="2" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="E43" s="2" t="inlineStr">
+      <c r="E37" s="2" t="inlineStr">
         <is>
           <t>1. You are signed in to the ShopView App on a desktop browser as a user with access to at least two locations.
 2. In-stock parts exist at both locations.</t>
         </is>
       </c>
-      <c r="F43" s="2" t="inlineStr">
+      <c r="F37" s="2" t="inlineStr">
         <is>
           <t>1. With one location selected, note the rows and totals.
 2. Add the second location and watch the data area.
 3. Use "All locations", then narrow back to one.</t>
         </is>
       </c>
-      <c r="G43" s="2" t="inlineStr">
+      <c r="G37" s="2" t="inlineStr">
         <is>
           <t>1. Each selection change reloads the report scoped to the selected set.
 2. With both locations selected, parts from both appear (one row per part per location) and the totals cover both.</t>
         </is>
       </c>
-      <c r="H43" s="2" t="inlineStr">
+      <c r="H37" s="2" t="inlineStr">
         <is>
           <t>specs/inventory-value.md Story 7 S7-R3</t>
         </is>
       </c>
-      <c r="I43" s="2" t="inlineStr"/>
-      <c r="J43" s="2" t="inlineStr"/>
-    </row>
-    <row r="44">
-      <c r="A44" s="2" t="inlineStr">
+      <c r="I37" s="2" t="inlineStr"/>
+      <c r="J37" s="2" t="inlineStr"/>
+    </row>
+    <row r="38">
+      <c r="A38" s="2" t="inlineStr">
         <is>
           <t>Scoping never includes an inaccessible location, and a selection resolving to none falls back to the user's active location</t>
         </is>
       </c>
-      <c r="B44" s="2" t="inlineStr">
+      <c r="B38" s="2" t="inlineStr">
         <is>
           <t>IV — Location Filter</t>
         </is>
       </c>
-      <c r="C44" s="2" t="inlineStr">
+      <c r="C38" s="2" t="inlineStr">
         <is>
           <t>Negative</t>
         </is>
       </c>
-      <c r="D44" s="2" t="inlineStr">
+      <c r="D38" s="2" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="E44" s="2" t="inlineStr">
+      <c r="E38" s="2" t="inlineStr">
         <is>
           <t>1. You are signed in to the ShopView App on a desktop browser as a user who can access some, but not all, of the organization's locations.
 2. The Inventory Value report is open.</t>
         </is>
       </c>
-      <c r="F44" s="2" t="inlineStr">
+      <c r="F38" s="2" t="inlineStr">
         <is>
           <t>1. Open the Location filter and read the locations offered.
 2. Use "Clear all" so the selection resolves to no location, and watch what the report loads.</t>
         </is>
       </c>
-      <c r="G44" s="2" t="inlineStr">
+      <c r="G38" s="2" t="inlineStr">
         <is>
           <t>1. Only the locations the user has access to are offered — a location the user cannot access is never included in the scope.
 2. If the requested location set resolves to none the user can access, the report falls back to the user's currently active location.</t>
         </is>
       </c>
-      <c r="H44" s="2" t="inlineStr">
+      <c r="H38" s="2" t="inlineStr">
         <is>
           <t>specs/inventory-value.md Story 7 S7-R4; S7-R5</t>
         </is>
       </c>
-      <c r="I44" s="2" t="inlineStr"/>
-      <c r="J44" s="2" t="inlineStr"/>
-    </row>
-    <row r="45">
-      <c r="A45" s="2" t="inlineStr">
+      <c r="I38" s="2" t="inlineStr"/>
+      <c r="J38" s="2" t="inlineStr"/>
+    </row>
+    <row r="39">
+      <c r="A39" s="2" t="inlineStr">
         <is>
           <t>The Location filter is hidden for a user with access to only one location</t>
         </is>
       </c>
-      <c r="B45" s="2" t="inlineStr">
+      <c r="B39" s="2" t="inlineStr">
         <is>
           <t>IV — Location Filter</t>
         </is>
       </c>
-      <c r="C45" s="2" t="inlineStr">
-        <is>
-          <t>Functional</t>
-        </is>
-      </c>
-      <c r="D45" s="2" t="inlineStr">
+      <c r="C39" s="2" t="inlineStr">
+        <is>
+          <t>Functional</t>
+        </is>
+      </c>
+      <c r="D39" s="2" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="E45" s="2" t="inlineStr">
+      <c r="E39" s="2" t="inlineStr">
         <is>
           <t>1. A test user exists with access to exactly one location (create a fresh ZZAUTOTEST staff member if needed; clean up afterward).
 2. You are signed in as that user on a desktop browser.</t>
         </is>
       </c>
-      <c r="F45" s="2" t="inlineStr">
+      <c r="F39" s="2" t="inlineStr">
         <is>
           <t>1. Open the Inventory Value report and look for the Location filter in the toolbar.
 2. Then sign in as a user with access to two or more locations and look again.</t>
         </is>
       </c>
-      <c r="G45" s="2" t="inlineStr">
+      <c r="G39" s="2" t="inlineStr">
         <is>
           <t>1. For the single-location user the Location filter is NOT shown at all — the report simply shows that one location's stock.
 2. For the user with access to two or more locations the Location filter IS shown.</t>
         </is>
       </c>
-      <c r="H45" s="2" t="inlineStr">
+      <c r="H39" s="2" t="inlineStr">
         <is>
           <t>SV-8674 (specs/inventory-value.md Story 7 S7-N1 — expectation FLIPPED by kickoff video P33 46:10-46:28, user ruling 2026-07-28: video overrides spec (video newer, last-update-wins))</t>
         </is>
       </c>
-      <c r="I45" s="2" t="inlineStr"/>
-      <c r="J45" s="2" t="inlineStr"/>
-    </row>
-    <row r="46">
-      <c r="A46" s="2" t="inlineStr">
-        <is>
-          <t>When the selected location(s) hold no in-stock parts on the resolved date, the no-data message shows</t>
-        </is>
-      </c>
-      <c r="B46" s="2" t="inlineStr">
-        <is>
-          <t>IV — Location Filter</t>
-        </is>
-      </c>
-      <c r="C46" s="2" t="inlineStr">
-        <is>
-          <t>Negative</t>
-        </is>
-      </c>
-      <c r="D46" s="2" t="inlineStr">
-        <is>
-          <t>Medium</t>
-        </is>
-      </c>
-      <c r="E46" s="2" t="inlineStr">
-        <is>
-          <t>1. You are signed in to the ShopView App on a desktop browser.
-2. A location you can access holds no in-stock (positive-quantity, non-core) parts.</t>
-        </is>
-      </c>
-      <c r="F46" s="2" t="inlineStr">
-        <is>
-          <t>1. Scope the Location filter to only the empty location.
-2. Read the data area.</t>
-        </is>
-      </c>
-      <c r="G46" s="2" t="inlineStr">
-        <is>
-          <t>1. The report shows the no-data message "Empty bays, endless possibilities. Get Going!" instead of rows, and no totals row.</t>
-        </is>
-      </c>
-      <c r="H46" s="2" t="inlineStr">
-        <is>
-          <t>specs/inventory-value.md Story 7 S7-N2; §7 User Feedback Summary</t>
-        </is>
-      </c>
-      <c r="I46" s="2" t="inlineStr"/>
-      <c r="J46" s="2" t="inlineStr"/>
-    </row>
-    <row r="47">
-      <c r="A47" s="2" t="inlineStr">
+      <c r="I39" s="2" t="inlineStr"/>
+      <c r="J39" s="2" t="inlineStr"/>
+    </row>
+    <row r="40">
+      <c r="A40" s="2" t="inlineStr">
         <is>
           <t>The column-selection icon button (tooltip "Column Selection") toggles columns, and Total Cost cannot be turned off</t>
         </is>
       </c>
-      <c r="B47" s="2" t="inlineStr">
+      <c r="B40" s="2" t="inlineStr">
         <is>
           <t>IV — Column Selection &amp; Persistence</t>
         </is>
       </c>
-      <c r="C47" s="2" t="inlineStr">
-        <is>
-          <t>Functional</t>
-        </is>
-      </c>
-      <c r="D47" s="2" t="inlineStr">
+      <c r="C40" s="2" t="inlineStr">
+        <is>
+          <t>Functional</t>
+        </is>
+      </c>
+      <c r="D40" s="2" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="E47" s="2" t="inlineStr">
+      <c r="E40" s="2" t="inlineStr">
         <is>
           <t>1. You are signed in to the ShopView App on a desktop browser.
 2. The Inventory Value report is open with rows loaded.</t>
         </is>
       </c>
-      <c r="F47" s="2" t="inlineStr">
+      <c r="F40" s="2" t="inlineStr">
         <is>
           <t>1. Hover the column-selection icon button in the toolbar and read its tooltip.
 2. Open the control and toggle a column off, then on again, watching the table.
 3. Look for a way to turn the Total Cost column off.</t>
         </is>
       </c>
-      <c r="G47" s="2" t="inlineStr">
+      <c r="G40" s="2" t="inlineStr">
         <is>
           <t>1. The icon button's tooltip reads "Column Selection".
 2. Toggling a column off hides it from the table; toggling it on shows it again.
 3. The Total Cost column is always shown and cannot be turned off.</t>
         </is>
       </c>
-      <c r="H47" s="2" t="inlineStr">
+      <c r="H40" s="2" t="inlineStr">
         <is>
           <t>specs/inventory-value.md Story 8 S8-R1; S8-R2</t>
         </is>
       </c>
-      <c r="I47" s="2" t="inlineStr"/>
-      <c r="J47" s="2" t="inlineStr"/>
-    </row>
-    <row r="48">
-      <c r="A48" s="2" t="inlineStr">
+      <c r="I40" s="2" t="inlineStr"/>
+      <c r="J40" s="2" t="inlineStr"/>
+    </row>
+    <row r="41">
+      <c r="A41" s="2" t="inlineStr">
         <is>
           <t>Toggling columns never reorders them — the fixed order is kept with Total Cost always last</t>
         </is>
       </c>
-      <c r="B48" s="2" t="inlineStr">
+      <c r="B41" s="2" t="inlineStr">
         <is>
           <t>IV — Column Selection &amp; Persistence</t>
         </is>
       </c>
-      <c r="C48" s="2" t="inlineStr">
-        <is>
-          <t>Functional</t>
-        </is>
-      </c>
-      <c r="D48" s="2" t="inlineStr">
+      <c r="C41" s="2" t="inlineStr">
+        <is>
+          <t>Functional</t>
+        </is>
+      </c>
+      <c r="D41" s="2" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="E48" s="2" t="inlineStr">
+      <c r="E41" s="2" t="inlineStr">
         <is>
           <t>1. You are signed in to the ShopView App on a desktop browser.
 2. The Inventory Value report is open with rows loaded.</t>
         </is>
       </c>
-      <c r="F48" s="2" t="inlineStr">
+      <c r="F41" s="2" t="inlineStr">
         <is>
           <t>1. Turn several columns on and off in different orders (for example, turn on Total Sell, then Margin).
 2. Read the resulting column order after each change.</t>
         </is>
       </c>
-      <c r="G48" s="2" t="inlineStr">
+      <c r="G41" s="2" t="inlineStr">
         <is>
           <t>1. Whatever columns are shown, they appear in the fixed left-to-right order (Part #, Description, Category, Vendor, Qty on Hand, Unit Cost, Unit Sell, Margin, Margin %, Total Sell, Total Cost) — toggling visibility never reorders columns.
 2. Total Cost is always the last column.</t>
         </is>
       </c>
-      <c r="H48" s="2" t="inlineStr">
+      <c r="H41" s="2" t="inlineStr">
         <is>
           <t>specs/inventory-value.md Story 8 S8-R4; Story 3 S3-R1</t>
         </is>
       </c>
-      <c r="I48" s="2" t="inlineStr"/>
-      <c r="J48" s="2" t="inlineStr"/>
-    </row>
-    <row r="49">
-      <c r="A49" s="2" t="inlineStr">
+      <c r="I41" s="2" t="inlineStr"/>
+      <c r="J41" s="2" t="inlineStr"/>
+    </row>
+    <row r="42">
+      <c r="A42" s="2" t="inlineStr">
         <is>
           <t>The report remembers the date range, category, vendor, part search text, location, columns, and sort per browser and restores them on return</t>
         </is>
       </c>
-      <c r="B49" s="2" t="inlineStr">
+      <c r="B42" s="2" t="inlineStr">
         <is>
           <t>IV — Column Selection &amp; Persistence</t>
         </is>
       </c>
-      <c r="C49" s="2" t="inlineStr">
-        <is>
-          <t>Functional</t>
-        </is>
-      </c>
-      <c r="D49" s="2" t="inlineStr">
+      <c r="C42" s="2" t="inlineStr">
+        <is>
+          <t>Functional</t>
+        </is>
+      </c>
+      <c r="D42" s="2" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="E49" s="2" t="inlineStr">
+      <c r="E42" s="2" t="inlineStr">
         <is>
           <t>1. You are signed in to the ShopView App on a desktop browser.
 2. The Inventory Value report is open.</t>
         </is>
       </c>
-      <c r="F49" s="2" t="inlineStr">
+      <c r="F42" s="2" t="inlineStr">
         <is>
           <t>1. Change the date range, select a category and a vendor, type a part search, change the location selection, change the column selection, and sort by a non-default column.
 2. Navigate away to another screen, then return to the report.
@@ -2788,143 +2466,142 @@
 4. If practical, open the report in a different browser (or private window) and read its settings.</t>
         </is>
       </c>
-      <c r="G49" s="2" t="inlineStr">
+      <c r="G42" s="2" t="inlineStr">
         <is>
           <t>1. On return and after a reload, the report restores the saved date range, category selection, vendor selection, part search text, location selection, column selection, and sort.
 2. In a different browser the report shows the defaults instead — persistence is per browser, not tied to the user's account.</t>
         </is>
       </c>
-      <c r="H49" s="2" t="inlineStr">
+      <c r="H42" s="2" t="inlineStr">
         <is>
           <t>specs/inventory-value.md Story 8 S8-R5 (+ context note); Story 9 S9-R5</t>
         </is>
       </c>
-      <c r="I49" s="2" t="inlineStr"/>
-      <c r="J49" s="2" t="inlineStr"/>
-    </row>
-    <row r="50">
-      <c r="A50" s="2" t="inlineStr">
-        <is>
-          <t>Restore is defensive: an invalid saved value falls back to its default, and a saved category or vendor no longer present is dropped</t>
-        </is>
-      </c>
-      <c r="B50" s="2" t="inlineStr">
+      <c r="I42" s="2" t="inlineStr"/>
+      <c r="J42" s="2" t="inlineStr"/>
+    </row>
+    <row r="43">
+      <c r="A43" s="2" t="inlineStr">
+        <is>
+          <t>Defensive restore: a stale saved category or vendor is dropped on load</t>
+        </is>
+      </c>
+      <c r="B43" s="2" t="inlineStr">
         <is>
           <t>IV — Column Selection &amp; Persistence</t>
         </is>
       </c>
-      <c r="C50" s="2" t="inlineStr">
+      <c r="C43" s="2" t="inlineStr">
         <is>
           <t>Negative</t>
         </is>
       </c>
-      <c r="D50" s="2" t="inlineStr">
+      <c r="D43" s="2" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="E50" s="2" t="inlineStr">
+      <c r="E43" s="2" t="inlineStr">
         <is>
           <t>1. You are signed in to the ShopView App on a desktop browser.
 2. The report has saved settings in this browser, including a category or vendor selection that can be made stale (for example, the last in-stock part of a saved category is consumed so the category disappears from the data).</t>
         </is>
       </c>
-      <c r="F50" s="2" t="inlineStr">
+      <c r="F43" s="2" t="inlineStr">
         <is>
           <t>1. Make the saved category or vendor no longer present in the data.
 2. Open the Inventory Value report.</t>
         </is>
       </c>
-      <c r="G50" s="2" t="inlineStr">
-        <is>
-          <t>1. The report loads normally — a saved value that is no longer valid falls back to that setting's default rather than breaking the view.
-2. The saved category or vendor no longer present in the data is dropped from the selection.
-3. All other saved settings are still restored.</t>
-        </is>
-      </c>
-      <c r="H50" s="2" t="inlineStr">
+      <c r="G43" s="2" t="inlineStr">
+        <is>
+          <t>1. The report loads normally — the saved category or vendor that is no longer present in the data is dropped from the selection instead of breaking the view (the defensive-restore rule applied to the path these steps drive).
+2. All other saved settings are still restored.</t>
+        </is>
+      </c>
+      <c r="H43" s="2" t="inlineStr">
         <is>
           <t>specs/inventory-value.md Story 8 S8-R6</t>
         </is>
       </c>
-      <c r="I50" s="2" t="inlineStr"/>
-      <c r="J50" s="2" t="inlineStr"/>
-    </row>
-    <row r="51">
-      <c r="A51" s="2" t="inlineStr">
+      <c r="I43" s="2" t="inlineStr"/>
+      <c r="J43" s="2" t="inlineStr"/>
+    </row>
+    <row r="44">
+      <c r="A44" s="2" t="inlineStr">
         <is>
           <t>On first load and after any reload, rows are sorted by Total Cost, highest first, applied by the server</t>
         </is>
       </c>
-      <c r="B51" s="2" t="inlineStr">
+      <c r="B44" s="2" t="inlineStr">
         <is>
           <t>IV — Sorting</t>
         </is>
       </c>
-      <c r="C51" s="2" t="inlineStr">
-        <is>
-          <t>Functional</t>
-        </is>
-      </c>
-      <c r="D51" s="2" t="inlineStr">
+      <c r="C44" s="2" t="inlineStr">
+        <is>
+          <t>Functional</t>
+        </is>
+      </c>
+      <c r="D44" s="2" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="E51" s="2" t="inlineStr">
+      <c r="E44" s="2" t="inlineStr">
         <is>
           <t>1. You are signed in to the ShopView App on a desktop browser that has no saved sort for this report (fresh visit).
 2. In-stock parts with a spread of Total Cost values exist, spanning more than one page.</t>
         </is>
       </c>
-      <c r="F51" s="2" t="inlineStr">
+      <c r="F44" s="2" t="inlineStr">
         <is>
           <t>1. Open the Inventory Value report without clicking any header.
 2. Read the Total Cost values from the top row down, across page 1 and page 2.</t>
         </is>
       </c>
-      <c r="G51" s="2" t="inlineStr">
+      <c r="G44" s="2" t="inlineStr">
         <is>
           <t>1. The rows are sorted by Total Cost, highest first (descending).
 2. The order holds across pages (page 2 continues below page 1's lowest value) — the server applies the default order over the full set.</t>
         </is>
       </c>
-      <c r="H51" s="2" t="inlineStr">
+      <c r="H44" s="2" t="inlineStr">
         <is>
           <t>specs/inventory-value.md Story 9 S9-R1; §3 Key Decisions (Total Cost default sort)</t>
         </is>
       </c>
-      <c r="I51" s="2" t="inlineStr"/>
-      <c r="J51" s="2" t="inlineStr"/>
-    </row>
-    <row r="52">
-      <c r="A52" s="2" t="inlineStr">
+      <c r="I44" s="2" t="inlineStr"/>
+      <c r="J44" s="2" t="inlineStr"/>
+    </row>
+    <row r="45">
+      <c r="A45" s="2" t="inlineStr">
         <is>
           <t>Header clicks sort ascending then descending with no third state, re-fetching from the server and returning the first page</t>
         </is>
       </c>
-      <c r="B52" s="2" t="inlineStr">
+      <c r="B45" s="2" t="inlineStr">
         <is>
           <t>IV — Sorting</t>
         </is>
       </c>
-      <c r="C52" s="2" t="inlineStr">
-        <is>
-          <t>Functional</t>
-        </is>
-      </c>
-      <c r="D52" s="2" t="inlineStr">
+      <c r="C45" s="2" t="inlineStr">
+        <is>
+          <t>Functional</t>
+        </is>
+      </c>
+      <c r="D45" s="2" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="E52" s="2" t="inlineStr">
+      <c r="E45" s="2" t="inlineStr">
         <is>
           <t>1. You are signed in to the ShopView App on a desktop browser.
 2. The result set spans more than one page.</t>
         </is>
       </c>
-      <c r="F52" s="2" t="inlineStr">
+      <c r="F45" s="2" t="inlineStr">
         <is>
           <t>1. From page 2, click the Part # column header and note the order and the page shown.
 2. Click the same header again and note the order.
@@ -2932,192 +2609,192 @@
 4. Click a different column header and check whether the previous sort still applies.</t>
         </is>
       </c>
-      <c r="G52" s="2" t="inlineStr">
+      <c r="G45" s="2" t="inlineStr">
         <is>
           <t>1. Clicking a column that is not the active sort sorts it ascending; clicking the active sort column again toggles it to descending; there is no third "cleared" state.
 2. Each header click re-fetches the data from the server ordered by the chosen column and direction, returning the FIRST page of the re-sorted result set.
 3. Only one column sorts at a time.</t>
         </is>
       </c>
-      <c r="H52" s="2" t="inlineStr">
+      <c r="H45" s="2" t="inlineStr">
         <is>
           <t>specs/inventory-value.md Story 9 S9-R2</t>
         </is>
       </c>
-      <c r="I52" s="2" t="inlineStr"/>
-      <c r="J52" s="2" t="inlineStr"/>
-    </row>
-    <row r="53">
-      <c r="A53" s="2" t="inlineStr">
+      <c r="I45" s="2" t="inlineStr"/>
+      <c r="J45" s="2" t="inlineStr"/>
+    </row>
+    <row r="46">
+      <c r="A46" s="2" t="inlineStr">
         <is>
           <t>Money and numeric columns sort by value; text columns sort as text, case-insensitively</t>
         </is>
       </c>
-      <c r="B53" s="2" t="inlineStr">
+      <c r="B46" s="2" t="inlineStr">
         <is>
           <t>IV — Sorting</t>
         </is>
       </c>
-      <c r="C53" s="2" t="inlineStr">
-        <is>
-          <t>Functional</t>
-        </is>
-      </c>
-      <c r="D53" s="2" t="inlineStr">
+      <c r="C46" s="2" t="inlineStr">
+        <is>
+          <t>Functional</t>
+        </is>
+      </c>
+      <c r="D46" s="2" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="E53" s="2" t="inlineStr">
+      <c r="E46" s="2" t="inlineStr">
         <is>
           <t>1. You are signed in to the ShopView App on a desktop browser.
 2. In-stock parts exist with money values over and under $1,000 and with text values in mixed letter cases.</t>
         </is>
       </c>
-      <c r="F53" s="2" t="inlineStr">
+      <c r="F46" s="2" t="inlineStr">
         <is>
           <t>1. Sort by Total Cost and check the order of values like $900.00 vs $1,100.00.
 2. Sort by Qty on Hand and check the numeric order.
 3. Sort by Description (or Vendor) and check how differently-cased values order.</t>
         </is>
       </c>
-      <c r="G53" s="2" t="inlineStr">
+      <c r="G46" s="2" t="inlineStr">
         <is>
           <t>1. Money and numeric columns sort by their underlying value (so $1,100.00 is treated as more than $900.00, not compared as text).
 2. Text columns (Part #, Description, Category, Vendor) sort as text, case-insensitively ("apple" and "Apple" sort together).</t>
         </is>
       </c>
-      <c r="H53" s="2" t="inlineStr">
+      <c r="H46" s="2" t="inlineStr">
         <is>
           <t>specs/inventory-value.md Story 9 S9-R3</t>
         </is>
       </c>
-      <c r="I53" s="2" t="inlineStr"/>
-      <c r="J53" s="2" t="inlineStr"/>
-    </row>
-    <row r="54">
-      <c r="A54" s="2" t="inlineStr">
+      <c r="I46" s="2" t="inlineStr"/>
+      <c r="J46" s="2" t="inlineStr"/>
+    </row>
+    <row r="47">
+      <c r="A47" s="2" t="inlineStr">
         <is>
           <t>Sorting reorders only the data rows — the totals row stays at the bottom — and the chosen sort is remembered per browser</t>
         </is>
       </c>
-      <c r="B54" s="2" t="inlineStr">
+      <c r="B47" s="2" t="inlineStr">
         <is>
           <t>IV — Sorting</t>
         </is>
       </c>
-      <c r="C54" s="2" t="inlineStr">
-        <is>
-          <t>Functional</t>
-        </is>
-      </c>
-      <c r="D54" s="2" t="inlineStr">
+      <c r="C47" s="2" t="inlineStr">
+        <is>
+          <t>Functional</t>
+        </is>
+      </c>
+      <c r="D47" s="2" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="E54" s="2" t="inlineStr">
+      <c r="E47" s="2" t="inlineStr">
         <is>
           <t>1. You are signed in to the ShopView App on a desktop browser.
 2. The Inventory Value report is open with rows and a totals row.</t>
         </is>
       </c>
-      <c r="F54" s="2" t="inlineStr">
+      <c r="F47" s="2" t="inlineStr">
         <is>
           <t>1. Sort by any column and watch the totals row's position.
 2. Sort by a non-default column, leave the report, and return.</t>
         </is>
       </c>
-      <c r="G54" s="2" t="inlineStr">
+      <c r="G47" s="2" t="inlineStr">
         <is>
           <t>1. Sorting reorders the data rows only; the totals row stays at the bottom.
 2. On return, the report restores the chosen sort (remembered per browser, Story 8).</t>
         </is>
       </c>
-      <c r="H54" s="2" t="inlineStr">
+      <c r="H47" s="2" t="inlineStr">
         <is>
           <t>specs/inventory-value.md Story 9 S9-R4; S9-R5</t>
         </is>
       </c>
-      <c r="I54" s="2" t="inlineStr"/>
-      <c r="J54" s="2" t="inlineStr"/>
-    </row>
-    <row r="55">
-      <c r="A55" s="2" t="inlineStr">
+      <c r="I47" s="2" t="inlineStr"/>
+      <c r="J47" s="2" t="inlineStr"/>
+    </row>
+    <row r="48">
+      <c r="A48" s="2" t="inlineStr">
         <is>
           <t>A three-dot toolbar menu holds "Download (PDF)" and "Download (CSV)"</t>
         </is>
       </c>
-      <c r="B55" s="2" t="inlineStr">
+      <c r="B48" s="2" t="inlineStr">
         <is>
           <t>IV — Exports</t>
         </is>
       </c>
-      <c r="C55" s="2" t="inlineStr">
-        <is>
-          <t>Functional</t>
-        </is>
-      </c>
-      <c r="D55" s="2" t="inlineStr">
+      <c r="C48" s="2" t="inlineStr">
+        <is>
+          <t>Functional</t>
+        </is>
+      </c>
+      <c r="D48" s="2" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="E55" s="2" t="inlineStr">
+      <c r="E48" s="2" t="inlineStr">
         <is>
           <t>1. You are signed in to the ShopView App on a desktop browser.
 2. The Inventory Value report is open with rows loaded.</t>
         </is>
       </c>
-      <c r="F55" s="2" t="inlineStr">
+      <c r="F48" s="2" t="inlineStr">
         <is>
           <t>1. Find and open the three-dot button in the toolbar.
 2. Read the menu options.
 3. Choose "Download (PDF)", then repeat with "Download (CSV)".</t>
         </is>
       </c>
-      <c r="G55" s="2" t="inlineStr">
+      <c r="G48" s="2" t="inlineStr">
         <is>
           <t>1. The menu holds an option labeled "Download (PDF)" and an option labeled "Download (CSV)".
 2. Each option downloads a file of the current view in the chosen format.</t>
         </is>
       </c>
-      <c r="H55" s="2" t="inlineStr">
+      <c r="H48" s="2" t="inlineStr">
         <is>
           <t>specs/inventory-value.md Story 10 S10-R1; S10-R2</t>
         </is>
       </c>
-      <c r="I55" s="2" t="inlineStr"/>
-      <c r="J55" s="2" t="inlineStr"/>
-    </row>
-    <row r="56">
-      <c r="A56" s="2" t="inlineStr">
+      <c r="I48" s="2" t="inlineStr"/>
+      <c r="J48" s="2" t="inlineStr"/>
+    </row>
+    <row r="49">
+      <c r="A49" s="2" t="inlineStr">
         <is>
           <t>Downloads contain the shown columns in screen order (Total Cost last), honor all filters and the sort, and include a "Totals" row matching the full-set totals</t>
         </is>
       </c>
-      <c r="B56" s="2" t="inlineStr">
+      <c r="B49" s="2" t="inlineStr">
         <is>
           <t>IV — Exports</t>
         </is>
       </c>
-      <c r="C56" s="2" t="inlineStr">
-        <is>
-          <t>Functional</t>
-        </is>
-      </c>
-      <c r="D56" s="2" t="inlineStr">
+      <c r="C49" s="2" t="inlineStr">
+        <is>
+          <t>Functional</t>
+        </is>
+      </c>
+      <c r="D49" s="2" t="inlineStr">
         <is>
           <t>Critical</t>
         </is>
       </c>
-      <c r="E56" s="2" t="inlineStr">
+      <c r="E49" s="2" t="inlineStr">
         <is>
           <t>1. You are signed in to the ShopView App on a desktop browser.
 2. The report is open with a non-default column selection, a Category or Vendor filter, a part search, and a non-default sort applied.</t>
         </is>
       </c>
-      <c r="F56" s="2" t="inlineStr">
+      <c r="F49" s="2" t="inlineStr">
         <is>
           <t>1. Download the current view as a CSV and open it.
 2. Compare its columns and their order to the screen.
@@ -3126,98 +2803,98 @@
 5. Repeat the checks in the PDF.</t>
         </is>
       </c>
-      <c r="G56" s="2" t="inlineStr">
+      <c r="G49" s="2" t="inlineStr">
         <is>
           <t>1. Both downloads include only the columns currently shown, in the same left-to-right order as the screen, with Total Cost last.
 2. Both downloads honor the current date, category, vendor, location, and part-search filters, and apply the current sort.
 3. Both downloads include a totals row labeled "Totals" matching the on-screen totals (the full-filtered-set totals).</t>
         </is>
       </c>
-      <c r="H56" s="2" t="inlineStr">
+      <c r="H49" s="2" t="inlineStr">
         <is>
           <t>specs/inventory-value.md Story 10 S10-R3; S10-R4; S10-R5; S10-R6</t>
         </is>
       </c>
-      <c r="I56" s="2" t="inlineStr"/>
-      <c r="J56" s="2" t="inlineStr"/>
-    </row>
-    <row r="57">
-      <c r="A57" s="2" t="inlineStr">
+      <c r="I49" s="2" t="inlineStr"/>
+      <c r="J49" s="2" t="inlineStr"/>
+    </row>
+    <row r="50">
+      <c r="A50" s="2" t="inlineStr">
         <is>
           <t>Export number formats: two-decimal money, one-decimal Margin % ("—" when undefined); CSV money as plain numbers, PDF with on-screen currency formatting</t>
         </is>
       </c>
-      <c r="B57" s="2" t="inlineStr">
+      <c r="B50" s="2" t="inlineStr">
         <is>
           <t>IV — Exports</t>
         </is>
       </c>
-      <c r="C57" s="2" t="inlineStr">
-        <is>
-          <t>Functional</t>
-        </is>
-      </c>
-      <c r="D57" s="2" t="inlineStr">
+      <c r="C50" s="2" t="inlineStr">
+        <is>
+          <t>Functional</t>
+        </is>
+      </c>
+      <c r="D50" s="2" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="E57" s="2" t="inlineStr">
+      <c r="E50" s="2" t="inlineStr">
         <is>
           <t>1. You are signed in to the ShopView App on a desktop browser.
 2. The current view includes money values over $1,000 and, if producible, a part whose Margin % is undefined ("—").</t>
         </is>
       </c>
-      <c r="F57" s="2" t="inlineStr">
+      <c r="F50" s="2" t="inlineStr">
         <is>
           <t>1. Download the CSV and open it in a plain-text editor; read the money and Margin % values.
 2. Download the PDF and read the same values.</t>
         </is>
       </c>
-      <c r="G57" s="2" t="inlineStr">
+      <c r="G50" s="2" t="inlineStr">
         <is>
           <t>1. Money uses two decimals and Margin % one decimal in both files; an undefined Margin % shows "—".
 2. In the CSV, money values are written as plain numbers with two decimals and NO thousands separators (so they parse cleanly in a spreadsheet).
 3. The PDF uses the same on-screen currency formatting with the "$" and thousands separators.</t>
         </is>
       </c>
-      <c r="H57" s="2" t="inlineStr">
+      <c r="H50" s="2" t="inlineStr">
         <is>
           <t>specs/inventory-value.md Story 10 S10-R7 (+ context note)</t>
         </is>
       </c>
-      <c r="I57" s="2" t="inlineStr"/>
-      <c r="J57" s="2" t="inlineStr"/>
-    </row>
-    <row r="58">
-      <c r="A58" s="2" t="inlineStr">
+      <c r="I50" s="2" t="inlineStr"/>
+      <c r="J50" s="2" t="inlineStr"/>
+    </row>
+    <row r="51">
+      <c r="A51" s="2" t="inlineStr">
         <is>
           <t>The PDF header shows the report name, organization, selected period, and an "as of" line; the shop logo shows when set and the CSV never has one</t>
         </is>
       </c>
-      <c r="B58" s="2" t="inlineStr">
+      <c r="B51" s="2" t="inlineStr">
         <is>
           <t>IV — Exports</t>
         </is>
       </c>
-      <c r="C58" s="2" t="inlineStr">
-        <is>
-          <t>Functional</t>
-        </is>
-      </c>
-      <c r="D58" s="2" t="inlineStr">
+      <c r="C51" s="2" t="inlineStr">
+        <is>
+          <t>Functional</t>
+        </is>
+      </c>
+      <c r="D51" s="2" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="E58" s="2" t="inlineStr">
+      <c r="E51" s="2" t="inlineStr">
         <is>
           <t>1. You are signed in to the ShopView App on a desktop browser.
 2. The shop has a logo set in its settings.
 3. The report is open on a view whose displayed day is known (live today, or a recorded past day).</t>
         </is>
       </c>
-      <c r="F58" s="2" t="inlineStr">
+      <c r="F51" s="2" t="inlineStr">
         <is>
           <t>1. Download the PDF and read its header.
 2. Look at the top of the PDF for the shop logo.
@@ -3225,768 +2902,678 @@
 4. If reachable, repeat the PDF download on a period with no available snapshot and read the header's as-of line.</t>
         </is>
       </c>
-      <c r="G58" s="2" t="inlineStr">
+      <c r="G51" s="2" t="inlineStr">
         <is>
           <t>1. The PDF header shows the report name "Inventory Value", the organization name, the selected period, and an "as of" line naming the day the values represent (or a message that no snapshot is available for the period).
 2. The PDF shows the shop logo at the top when one is set.
 3. The CSV never includes a logo.</t>
         </is>
       </c>
-      <c r="H58" s="2" t="inlineStr">
+      <c r="H51" s="2" t="inlineStr">
         <is>
           <t>specs/inventory-value.md Story 10 S10-R8; S10-R9</t>
         </is>
       </c>
-      <c r="I58" s="2" t="inlineStr"/>
-      <c r="J58" s="2" t="inlineStr"/>
-    </row>
-    <row r="59">
-      <c r="A59" s="2" t="inlineStr">
+      <c r="I51" s="2" t="inlineStr"/>
+      <c r="J51" s="2" t="inlineStr"/>
+    </row>
+    <row r="52">
+      <c r="A52" s="2" t="inlineStr">
         <is>
           <t>The downloaded files are named "inventory-value-report.pdf" and "inventory-value-report.csv"</t>
         </is>
       </c>
-      <c r="B59" s="2" t="inlineStr">
+      <c r="B52" s="2" t="inlineStr">
         <is>
           <t>IV — Exports</t>
         </is>
       </c>
-      <c r="C59" s="2" t="inlineStr">
-        <is>
-          <t>Functional</t>
-        </is>
-      </c>
-      <c r="D59" s="2" t="inlineStr">
+      <c r="C52" s="2" t="inlineStr">
+        <is>
+          <t>Functional</t>
+        </is>
+      </c>
+      <c r="D52" s="2" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="E59" s="2" t="inlineStr">
+      <c r="E52" s="2" t="inlineStr">
         <is>
           <t>1. You are signed in to the ShopView App on a desktop browser.
 2. The Inventory Value report is open with rows loaded.</t>
         </is>
       </c>
-      <c r="F59" s="2" t="inlineStr">
+      <c r="F52" s="2" t="inlineStr">
         <is>
           <t>1. Download the current view as a PDF and read the saved file's name.
 2. Download the current view as a CSV and read the saved file's name.</t>
         </is>
       </c>
-      <c r="G59" s="2" t="inlineStr">
+      <c r="G52" s="2" t="inlineStr">
         <is>
           <t>1. The PDF is named "inventory-value-report.pdf".
 2. The CSV is named "inventory-value-report.csv".</t>
         </is>
       </c>
-      <c r="H59" s="2" t="inlineStr">
+      <c r="H52" s="2" t="inlineStr">
         <is>
           <t>specs/inventory-value.md Story 10 S10-R10</t>
         </is>
       </c>
-      <c r="I59" s="2" t="inlineStr"/>
-      <c r="J59" s="2" t="inlineStr"/>
-    </row>
-    <row r="60">
-      <c r="A60" s="2" t="inlineStr">
+      <c r="I52" s="2" t="inlineStr"/>
+      <c r="J52" s="2" t="inlineStr"/>
+    </row>
+    <row r="53">
+      <c r="A53" s="2" t="inlineStr">
         <is>
           <t>Exports are generated server-side over the full filtered set — rows beyond the loaded page are included</t>
         </is>
       </c>
-      <c r="B60" s="2" t="inlineStr">
+      <c r="B53" s="2" t="inlineStr">
         <is>
           <t>IV — Exports</t>
         </is>
       </c>
-      <c r="C60" s="2" t="inlineStr">
-        <is>
-          <t>Functional</t>
-        </is>
-      </c>
-      <c r="D60" s="2" t="inlineStr">
+      <c r="C53" s="2" t="inlineStr">
+        <is>
+          <t>Functional</t>
+        </is>
+      </c>
+      <c r="D53" s="2" t="inlineStr">
         <is>
           <t>Critical</t>
         </is>
       </c>
-      <c r="E60" s="2" t="inlineStr">
+      <c r="E53" s="2" t="inlineStr">
         <is>
           <t>1. You are signed in to the ShopView App on a desktop browser.
 2. The current filtered set spans more than one page (but stays under the export row cap).</t>
         </is>
       </c>
-      <c r="F60" s="2" t="inlineStr">
+      <c r="F53" s="2" t="inlineStr">
         <is>
           <t>1. From page 1, without visiting the later pages, download the CSV.
 2. Count the file's data rows and look for parts you know sit on the later pages.
 3. Compare the file's totals row to the on-screen totals.</t>
         </is>
       </c>
-      <c r="G60" s="2" t="inlineStr">
+      <c r="G53" s="2" t="inlineStr">
         <is>
           <t>1. The export contains the FULL filtered set — every qualifying row across all pages, not only the rows loaded in the browser.
 2. Parts from the later pages are present.
 3. The export is generated server-side against the current filters, part search, and sort — it is not built from the rows currently in the browser.</t>
         </is>
       </c>
-      <c r="H60" s="2" t="inlineStr">
+      <c r="H53" s="2" t="inlineStr">
         <is>
           <t>specs/inventory-value.md Story 10 S10-R11</t>
         </is>
       </c>
-      <c r="I60" s="2" t="inlineStr"/>
-      <c r="J60" s="2" t="inlineStr"/>
-    </row>
-    <row r="61">
-      <c r="A61" s="2" t="inlineStr">
+      <c r="I53" s="2" t="inlineStr"/>
+      <c r="J53" s="2" t="inlineStr"/>
+    </row>
+    <row r="54">
+      <c r="A54" s="2" t="inlineStr">
         <is>
           <t>An over-cap filtered set produces no file and shows the too-large-to-export message (exact cap value pending owner confirmation)</t>
         </is>
       </c>
-      <c r="B61" s="2" t="inlineStr">
+      <c r="B54" s="2" t="inlineStr">
         <is>
           <t>IV — Exports</t>
         </is>
       </c>
-      <c r="C61" s="2" t="inlineStr">
+      <c r="C54" s="2" t="inlineStr">
         <is>
           <t>Negative</t>
         </is>
       </c>
-      <c r="D61" s="2" t="inlineStr">
+      <c r="D54" s="2" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="E61" s="2" t="inlineStr">
+      <c r="E54" s="2" t="inlineStr">
         <is>
           <t>1. You are signed in to the ShopView App on a desktop browser.
 2. A filter/location combination exists whose filtered set EXCEEDS the export row cap (seed ZZAUTOTEST parts in bulk if needed, or use the largest available data set).</t>
         </is>
       </c>
-      <c r="F61" s="2" t="inlineStr">
+      <c r="F54" s="2" t="inlineStr">
         <is>
           <t>1. Set the filters so the filtered set exceeds the export row cap.
 2. Request "Download (PDF)" and read what happens.
 3. Request "Download (CSV)" and read what happens.</t>
         </is>
       </c>
-      <c r="G61" s="2" t="inlineStr">
+      <c r="G54" s="2" t="inlineStr">
         <is>
           <t>1. Neither the PDF nor the CSV is produced.
 2. The user sees the message: "This report is too large to export. Narrow the date range or filters, then try again." (a blocking notification; no file).
 3. After narrowing the filters below the cap, the download works again.</t>
         </is>
       </c>
-      <c r="H61" s="2" t="inlineStr">
+      <c r="H54" s="2" t="inlineStr">
         <is>
           <t>specs/inventory-value.md Story 10 S10-R12; §7 User Feedback Summary</t>
         </is>
       </c>
-      <c r="I61" s="2" t="inlineStr"/>
-      <c r="J61" s="2" t="inlineStr"/>
-    </row>
-    <row r="62">
-      <c r="A62" s="2" t="inlineStr">
-        <is>
-          <t>A successful download shows the format-specific success notification, verbatim</t>
-        </is>
-      </c>
-      <c r="B62" s="2" t="inlineStr">
+      <c r="I54" s="2" t="inlineStr"/>
+      <c r="J54" s="2" t="inlineStr"/>
+    </row>
+    <row r="55">
+      <c r="A55" s="2" t="inlineStr">
+        <is>
+          <t>Download notifications: verbatim success and failure texts per format</t>
+        </is>
+      </c>
+      <c r="B55" s="2" t="inlineStr">
         <is>
           <t>IV — Exports</t>
         </is>
       </c>
-      <c r="C62" s="2" t="inlineStr">
-        <is>
-          <t>Functional</t>
-        </is>
-      </c>
-      <c r="D62" s="2" t="inlineStr">
+      <c r="C55" s="2" t="inlineStr">
+        <is>
+          <t>Negative</t>
+        </is>
+      </c>
+      <c r="D55" s="2" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="E62" s="2" t="inlineStr">
-        <is>
-          <t>1. You are signed in to the ShopView App on a desktop browser.
-2. The Inventory Value report is open with rows loaded (under the export cap).</t>
-        </is>
-      </c>
-      <c r="F62" s="2" t="inlineStr">
-        <is>
-          <t>1. Download the PDF and read the notification.
-2. Download the CSV and read the notification.</t>
-        </is>
-      </c>
-      <c r="G62" s="2" t="inlineStr">
-        <is>
-          <t>1. The PDF download shows a success notification: "Inventory Value report exported (PDF)".
-2. The CSV download shows a success notification: "Inventory Value report exported (CSV)".</t>
-        </is>
-      </c>
-      <c r="H62" s="2" t="inlineStr">
-        <is>
-          <t>specs/inventory-value.md Story 10 S10-R13; §7 User Feedback Summary</t>
-        </is>
-      </c>
-      <c r="I62" s="2" t="inlineStr"/>
-      <c r="J62" s="2" t="inlineStr"/>
-    </row>
-    <row r="63">
-      <c r="A63" s="2" t="inlineStr">
-        <is>
-          <t>A failed download shows the format-specific error notification, verbatim</t>
-        </is>
-      </c>
-      <c r="B63" s="2" t="inlineStr">
-        <is>
-          <t>IV — Exports</t>
-        </is>
-      </c>
-      <c r="C63" s="2" t="inlineStr">
-        <is>
-          <t>Negative</t>
-        </is>
-      </c>
-      <c r="D63" s="2" t="inlineStr">
+      <c r="E55" s="2" t="inlineStr">
+        <is>
+          <t>1. You are signed in to the ShopView App on a desktop browser.
+2. The Inventory Value report is open with rows loaded (under the export cap).
+3. A download failure can be simulated (for example, disconnect the network just before requesting the download).</t>
+        </is>
+      </c>
+      <c r="F55" s="2" t="inlineStr">
+        <is>
+          <t>1. Download the PDF and the CSV normally and read each notification.
+2. Simulate a failure and request the PDF download; read the notification.
+3. Repeat the failure for the CSV download.</t>
+        </is>
+      </c>
+      <c r="G55" s="2" t="inlineStr">
+        <is>
+          <t>1. Success notifications read verbatim: "Inventory Value report exported (PDF)" and "Inventory Value report exported (CSV)".
+2. Failure notifications read verbatim: "Failed to export inventory value report (pdf)" and "Failed to export inventory value report (csv)".
+3. The lower-case "(pdf)"/"(csv)" on failure vs the upper-case success ones is the documented spec wording — expected, not a bug.</t>
+        </is>
+      </c>
+      <c r="H55" s="2" t="inlineStr">
+        <is>
+          <t>specs/inventory-value.md Story 10 S10-R13; S10-R14; §7 User Feedback Summary</t>
+        </is>
+      </c>
+      <c r="I55" s="2" t="inlineStr"/>
+      <c r="J55" s="2" t="inlineStr"/>
+    </row>
+    <row r="56">
+      <c r="A56" s="2" t="inlineStr">
+        <is>
+          <t>The report uses an all-white table with no alternating row shading on the standard soft blue-grey report backdrop</t>
+        </is>
+      </c>
+      <c r="B56" s="2" t="inlineStr">
+        <is>
+          <t>IV — Visual &amp; Accessibility</t>
+        </is>
+      </c>
+      <c r="C56" s="2" t="inlineStr">
+        <is>
+          <t>Functional</t>
+        </is>
+      </c>
+      <c r="D56" s="2" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="E63" s="2" t="inlineStr">
-        <is>
-          <t>1. You are signed in to the ShopView App on a desktop browser.
-2. A download failure can be simulated (for example, disconnect the network just before requesting the download).</t>
-        </is>
-      </c>
-      <c r="F63" s="2" t="inlineStr">
-        <is>
-          <t>1. Simulate a failure and request the PDF download; read the notification.
-2. Repeat for the CSV download.</t>
-        </is>
-      </c>
-      <c r="G63" s="2" t="inlineStr">
-        <is>
-          <t>1. The failed PDF download shows an error notification: "Failed to export inventory value report (pdf)".
-2. The failed CSV download shows an error notification: "Failed to export inventory value report (csv)".</t>
-        </is>
-      </c>
-      <c r="H63" s="2" t="inlineStr">
-        <is>
-          <t>specs/inventory-value.md Story 10 S10-R14; §7 User Feedback Summary</t>
-        </is>
-      </c>
-      <c r="I63" s="2" t="inlineStr"/>
-      <c r="J63" s="2" t="inlineStr"/>
-    </row>
-    <row r="64">
-      <c r="A64" s="2" t="inlineStr">
-        <is>
-          <t>The report uses an all-white table with no alternating row shading on the standard soft blue-grey report backdrop</t>
-        </is>
-      </c>
-      <c r="B64" s="2" t="inlineStr">
-        <is>
-          <t>IV — Visual &amp; Accessibility</t>
-        </is>
-      </c>
-      <c r="C64" s="2" t="inlineStr">
-        <is>
-          <t>Functional</t>
-        </is>
-      </c>
-      <c r="D64" s="2" t="inlineStr">
-        <is>
-          <t>Medium</t>
-        </is>
-      </c>
-      <c r="E64" s="2" t="inlineStr">
+      <c r="E56" s="2" t="inlineStr">
         <is>
           <t>1. You are signed in to the ShopView App on a desktop browser.
 2. The Inventory Value report is open with several rows.</t>
         </is>
       </c>
-      <c r="F64" s="2" t="inlineStr">
+      <c r="F56" s="2" t="inlineStr">
         <is>
           <t>1. Look at the column headers and the data cells.
 2. Compare the background of consecutive rows.
 3. Look at the page background around the table.</t>
         </is>
       </c>
-      <c r="G64" s="2" t="inlineStr">
+      <c r="G56" s="2" t="inlineStr">
         <is>
           <t>1. The table has white column headers and white data cells, with no alternating row shading.
 2. The table sits on the standard soft blue-grey report backdrop.</t>
         </is>
       </c>
-      <c r="H64" s="2" t="inlineStr">
+      <c r="H56" s="2" t="inlineStr">
         <is>
           <t>specs/inventory-value.md Story 12 S12-R1</t>
         </is>
       </c>
-      <c r="I64" s="2" t="inlineStr"/>
-      <c r="J64" s="2" t="inlineStr"/>
-    </row>
-    <row r="65">
-      <c r="A65" s="2" t="inlineStr">
+      <c r="I56" s="2" t="inlineStr"/>
+      <c r="J56" s="2" t="inlineStr"/>
+    </row>
+    <row r="57">
+      <c r="A57" s="2" t="inlineStr">
         <is>
           <t>Toolbar layout: three-dot menu leftmost in the action cluster then Column Selection; filters run date range, part search, Category, Vendor, Location</t>
         </is>
       </c>
-      <c r="B65" s="2" t="inlineStr">
+      <c r="B57" s="2" t="inlineStr">
         <is>
           <t>IV — Visual &amp; Accessibility</t>
         </is>
       </c>
-      <c r="C65" s="2" t="inlineStr">
-        <is>
-          <t>Functional</t>
-        </is>
-      </c>
-      <c r="D65" s="2" t="inlineStr">
+      <c r="C57" s="2" t="inlineStr">
+        <is>
+          <t>Functional</t>
+        </is>
+      </c>
+      <c r="D57" s="2" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="E65" s="2" t="inlineStr">
+      <c r="E57" s="2" t="inlineStr">
         <is>
           <t>1. You are signed in to the ShopView App on a desktop browser.
 2. The Inventory Value report is open.</t>
         </is>
       </c>
-      <c r="F65" s="2" t="inlineStr">
+      <c r="F57" s="2" t="inlineStr">
         <is>
           <t>1. Look at the toolbar's action cluster and read the order of its controls.
 2. Read the toolbar filters from left to right.</t>
         </is>
       </c>
-      <c r="G65" s="2" t="inlineStr">
+      <c r="G57" s="2" t="inlineStr">
         <is>
           <t>1. In the toolbar, the three-dot download menu sits leftmost in the action cluster, followed by the Column Selection control.
 2. The toolbar filters run, left to right: the date-range control, the part search, the Category filter, the Vendor filter, and the Location filter (rightmost).</t>
         </is>
       </c>
-      <c r="H65" s="2" t="inlineStr">
+      <c r="H57" s="2" t="inlineStr">
         <is>
           <t>specs/inventory-value.md Story 12 S12-R2; S12-R3</t>
         </is>
       </c>
-      <c r="I65" s="2" t="inlineStr"/>
-      <c r="J65" s="2" t="inlineStr"/>
-    </row>
-    <row r="66">
-      <c r="A66" s="2" t="inlineStr">
-        <is>
-          <t>The totals row stays visible at the bottom while the user scrolls the rows</t>
-        </is>
-      </c>
-      <c r="B66" s="2" t="inlineStr">
+      <c r="I57" s="2" t="inlineStr"/>
+      <c r="J57" s="2" t="inlineStr"/>
+    </row>
+    <row r="58">
+      <c r="A58" s="2" t="inlineStr">
+        <is>
+          <t>Long Description, Category, and Vendor values truncate with an ellipsis and show the full value on hover; the Part # is never truncated</t>
+        </is>
+      </c>
+      <c r="B58" s="2" t="inlineStr">
         <is>
           <t>IV — Visual &amp; Accessibility</t>
         </is>
       </c>
-      <c r="C66" s="2" t="inlineStr">
-        <is>
-          <t>Functional</t>
-        </is>
-      </c>
-      <c r="D66" s="2" t="inlineStr">
+      <c r="C58" s="2" t="inlineStr">
+        <is>
+          <t>Functional</t>
+        </is>
+      </c>
+      <c r="D58" s="2" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="E66" s="2" t="inlineStr">
-        <is>
-          <t>1. You are signed in to the ShopView App on a desktop browser.
-2. The page shows more rows than fit on the screen.</t>
-        </is>
-      </c>
-      <c r="F66" s="2" t="inlineStr">
-        <is>
-          <t>1. Scroll the rows up and down.
-2. Watch the totals row.</t>
-        </is>
-      </c>
-      <c r="G66" s="2" t="inlineStr">
-        <is>
-          <t>1. The totals row stays visible at the bottom while the rows scroll.</t>
-        </is>
-      </c>
-      <c r="H66" s="2" t="inlineStr">
-        <is>
-          <t>specs/inventory-value.md Story 12 S12-R5</t>
-        </is>
-      </c>
-      <c r="I66" s="2" t="inlineStr"/>
-      <c r="J66" s="2" t="inlineStr"/>
-    </row>
-    <row r="67">
-      <c r="A67" s="2" t="inlineStr">
-        <is>
-          <t>Long Description, Category, and Vendor values truncate with an ellipsis and show the full value on hover; the Part # is never truncated</t>
-        </is>
-      </c>
-      <c r="B67" s="2" t="inlineStr">
-        <is>
-          <t>IV — Visual &amp; Accessibility</t>
-        </is>
-      </c>
-      <c r="C67" s="2" t="inlineStr">
-        <is>
-          <t>Functional</t>
-        </is>
-      </c>
-      <c r="D67" s="2" t="inlineStr">
-        <is>
-          <t>Medium</t>
-        </is>
-      </c>
-      <c r="E67" s="2" t="inlineStr">
+      <c r="E58" s="2" t="inlineStr">
         <is>
           <t>1. You are signed in to the ShopView App on a desktop browser.
 2. A ZZAUTOTEST part exists with a very long description (and, if possible, long category/vendor names) and a long part number.</t>
         </is>
       </c>
-      <c r="F67" s="2" t="inlineStr">
+      <c r="F58" s="2" t="inlineStr">
         <is>
           <t>1. Narrow the browser window (or turn on more columns) so the text columns overflow.
 2. Read the long Description, Category, and Vendor cells and hover each.
 3. Read the long Part # cell.</t>
         </is>
       </c>
-      <c r="G67" s="2" t="inlineStr">
+      <c r="G58" s="2" t="inlineStr">
         <is>
           <t>1. Long text values (Description, Category, Vendor) are truncated with an ellipsis when they overflow their column.
 2. The full value is available on hover.
 3. The Part # is never truncated.</t>
         </is>
       </c>
-      <c r="H67" s="2" t="inlineStr">
+      <c r="H58" s="2" t="inlineStr">
         <is>
           <t>specs/inventory-value.md Story 12 S12-R6</t>
         </is>
       </c>
-      <c r="I67" s="2" t="inlineStr"/>
-      <c r="J67" s="2" t="inlineStr"/>
-    </row>
-    <row r="68">
-      <c r="A68" s="2" t="inlineStr">
+      <c r="I58" s="2" t="inlineStr"/>
+      <c r="J58" s="2" t="inlineStr"/>
+    </row>
+    <row r="59">
+      <c r="A59" s="2" t="inlineStr">
         <is>
           <t>In dark mode the page background, toolbar, cells, and the "—" glyph remain legible</t>
         </is>
       </c>
-      <c r="B68" s="2" t="inlineStr">
+      <c r="B59" s="2" t="inlineStr">
         <is>
           <t>IV — Visual &amp; Accessibility</t>
         </is>
       </c>
-      <c r="C68" s="2" t="inlineStr">
+      <c r="C59" s="2" t="inlineStr">
         <is>
           <t>Accessibility</t>
         </is>
       </c>
-      <c r="D68" s="2" t="inlineStr">
+      <c r="D59" s="2" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="E68" s="2" t="inlineStr">
+      <c r="E59" s="2" t="inlineStr">
         <is>
           <t>1. You are signed in to the ShopView App on a desktop browser.
 2. The application is switched to dark mode.
 3. The report shows rows including a part with an em-dash ("—") Category or Vendor cell.</t>
         </is>
       </c>
-      <c r="F68" s="2" t="inlineStr">
+      <c r="F59" s="2" t="inlineStr">
         <is>
           <t>1. Read the page background, toolbar, and table cells in dark mode.
 2. Find a "—" cell and check its legibility.</t>
         </is>
       </c>
-      <c r="G68" s="2" t="inlineStr">
+      <c r="G59" s="2" t="inlineStr">
         <is>
           <t>1. The report supports dark mode.
 2. The page background, toolbar, cells, and the "—" glyph all use dark-mode-legible colors.</t>
         </is>
       </c>
-      <c r="H68" s="2" t="inlineStr">
+      <c r="H59" s="2" t="inlineStr">
         <is>
           <t>specs/inventory-value.md Story 12 S12-R7</t>
         </is>
       </c>
-      <c r="I68" s="2" t="inlineStr"/>
-      <c r="J68" s="2" t="inlineStr"/>
-    </row>
-    <row r="69">
-      <c r="A69" s="2" t="inlineStr">
+      <c r="I59" s="2" t="inlineStr"/>
+      <c r="J59" s="2" t="inlineStr"/>
+    </row>
+    <row r="60">
+      <c r="A60" s="2" t="inlineStr">
         <is>
           <t>Each sortable column header exposes its sort state to assistive technology and shows the active direction visually</t>
         </is>
       </c>
-      <c r="B69" s="2" t="inlineStr">
+      <c r="B60" s="2" t="inlineStr">
         <is>
           <t>IV — Visual &amp; Accessibility</t>
         </is>
       </c>
-      <c r="C69" s="2" t="inlineStr">
+      <c r="C60" s="2" t="inlineStr">
         <is>
           <t>Accessibility</t>
         </is>
       </c>
-      <c r="D69" s="2" t="inlineStr">
+      <c r="D60" s="2" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="E69" s="2" t="inlineStr">
+      <c r="E60" s="2" t="inlineStr">
         <is>
           <t>1. You are signed in to the ShopView App on a desktop browser.
 2. A screen reader or the browser's accessibility inspector is available.
 3. The Inventory Value report is open with rows loaded.</t>
         </is>
       </c>
-      <c r="F69" s="2" t="inlineStr">
+      <c r="F60" s="2" t="inlineStr">
         <is>
           <t>1. Sort by a column and look at its header for a visual direction indicator.
 2. With the accessibility inspector or screen reader, check what sort state the header exposes.
 3. Toggle the direction and check both again.</t>
         </is>
       </c>
-      <c r="G69" s="2" t="inlineStr">
+      <c r="G60" s="2" t="inlineStr">
         <is>
           <t>1. The active sort direction is indicated visually on the header.
 2. Each sortable column header exposes its sort state to assistive technology (for example, ascending/descending/none).
 3. The exposed state updates when the direction toggles.</t>
         </is>
       </c>
-      <c r="H69" s="2" t="inlineStr">
+      <c r="H60" s="2" t="inlineStr">
         <is>
           <t>specs/inventory-value.md Story 12 S12-R8</t>
         </is>
       </c>
-      <c r="I69" s="2" t="inlineStr"/>
-      <c r="J69" s="2" t="inlineStr"/>
-    </row>
-    <row r="70">
-      <c r="A70" s="2" t="inlineStr">
+      <c r="I60" s="2" t="inlineStr"/>
+      <c r="J60" s="2" t="inlineStr"/>
+    </row>
+    <row r="61">
+      <c r="A61" s="2" t="inlineStr">
         <is>
           <t>The icon-only controls (three-dot download button and Column Selection button) each carry an accessible name</t>
         </is>
       </c>
-      <c r="B70" s="2" t="inlineStr">
+      <c r="B61" s="2" t="inlineStr">
         <is>
           <t>IV — Visual &amp; Accessibility</t>
         </is>
       </c>
-      <c r="C70" s="2" t="inlineStr">
+      <c r="C61" s="2" t="inlineStr">
         <is>
           <t>Accessibility</t>
         </is>
       </c>
-      <c r="D70" s="2" t="inlineStr">
+      <c r="D61" s="2" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="E70" s="2" t="inlineStr">
+      <c r="E61" s="2" t="inlineStr">
         <is>
           <t>1. You are signed in to the ShopView App on a desktop browser.
 2. A screen reader or the browser's accessibility inspector is available.
 3. The Inventory Value report is open.</t>
         </is>
       </c>
-      <c r="F70" s="2" t="inlineStr">
+      <c r="F61" s="2" t="inlineStr">
         <is>
           <t>1. Inspect the three-dot download button's accessible name.
 2. Inspect the Column Selection button's accessible name.</t>
         </is>
       </c>
-      <c r="G70" s="2" t="inlineStr">
+      <c r="G61" s="2" t="inlineStr">
         <is>
           <t>1. Each icon-only control carries an accessible name exposed to assistive technology (it is not announced as an unnamed button).</t>
         </is>
       </c>
-      <c r="H70" s="2" t="inlineStr">
+      <c r="H61" s="2" t="inlineStr">
         <is>
           <t>specs/inventory-value.md Story 12 S12-R9</t>
         </is>
       </c>
-      <c r="I70" s="2" t="inlineStr"/>
-      <c r="J70" s="2" t="inlineStr"/>
-    </row>
-    <row r="71">
-      <c r="A71" s="2" t="inlineStr">
+      <c r="I61" s="2" t="inlineStr"/>
+      <c r="J61" s="2" t="inlineStr"/>
+    </row>
+    <row r="62">
+      <c r="A62" s="2" t="inlineStr">
         <is>
           <t>A user with the existing inventory-reports permission can open the report — no new permission is added</t>
         </is>
       </c>
-      <c r="B71" s="2" t="inlineStr">
+      <c r="B62" s="2" t="inlineStr">
         <is>
           <t>IV — Permissions</t>
         </is>
       </c>
-      <c r="C71" s="2" t="inlineStr">
-        <is>
-          <t>Functional</t>
-        </is>
-      </c>
-      <c r="D71" s="2" t="inlineStr">
+      <c r="C62" s="2" t="inlineStr">
+        <is>
+          <t>Functional</t>
+        </is>
+      </c>
+      <c r="D62" s="2" t="inlineStr">
         <is>
           <t>Critical</t>
         </is>
       </c>
-      <c r="E71" s="2" t="inlineStr">
+      <c r="E62" s="2" t="inlineStr">
         <is>
           <t>1. A test user exists whose role has the existing inventory-reports permission (assign the Tech user a suitable role if needed; restore the original role afterward).
 2. You are signed in as that user on a desktop browser.</t>
         </is>
       </c>
-      <c r="F71" s="2" t="inlineStr">
+      <c r="F62" s="2" t="inlineStr">
         <is>
           <t>1. Open the reports navigation and find "Inventory Value" under the Parts group.
 2. Open the report and confirm it loads rows.
 3. Download the current view as a CSV.</t>
         </is>
       </c>
-      <c r="G71" s="2" t="inlineStr">
+      <c r="G62" s="2" t="inlineStr">
         <is>
           <t>1. The report is listed and opens normally for a user holding the existing inventory-reports permission.
 2. No additional, report-specific permission is required — the report reuses the existing inventory-reports permission.</t>
         </is>
       </c>
-      <c r="H71" s="2" t="inlineStr">
+      <c r="H62" s="2" t="inlineStr">
         <is>
           <t>specs/inventory-value.md Story 1 Prerequisites</t>
         </is>
       </c>
-      <c r="I71" s="2" t="inlineStr"/>
-      <c r="J71" s="2" t="inlineStr"/>
-    </row>
-    <row r="72">
-      <c r="A72" s="2" t="inlineStr">
+      <c r="I62" s="2" t="inlineStr"/>
+      <c r="J62" s="2" t="inlineStr"/>
+    </row>
+    <row r="63">
+      <c r="A63" s="2" t="inlineStr">
         <is>
           <t>A user without the required permission does not see Inventory Value in the reports navigation</t>
         </is>
       </c>
-      <c r="B72" s="2" t="inlineStr">
+      <c r="B63" s="2" t="inlineStr">
         <is>
           <t>IV — Permissions</t>
         </is>
       </c>
-      <c r="C72" s="2" t="inlineStr">
+      <c r="C63" s="2" t="inlineStr">
         <is>
           <t>Negative</t>
         </is>
       </c>
-      <c r="D72" s="2" t="inlineStr">
+      <c r="D63" s="2" t="inlineStr">
         <is>
           <t>Critical</t>
         </is>
       </c>
-      <c r="E72" s="2" t="inlineStr">
+      <c r="E63" s="2" t="inlineStr">
         <is>
           <t>1. A test user exists whose role does NOT have the inventory-reports permission (assign the Tech user such a role; restore the original role afterward).
 2. You are signed in as that user on a desktop browser.</t>
         </is>
       </c>
-      <c r="F72" s="2" t="inlineStr">
+      <c r="F63" s="2" t="inlineStr">
         <is>
           <t>1. Open the reports navigation.
 2. Look for "Inventory Value" under the Parts group.</t>
         </is>
       </c>
-      <c r="G72" s="2" t="inlineStr">
+      <c r="G63" s="2" t="inlineStr">
         <is>
           <t>1. The report does not appear in the navigation for this user.</t>
         </is>
       </c>
-      <c r="H72" s="2" t="inlineStr">
+      <c r="H63" s="2" t="inlineStr">
         <is>
           <t>specs/inventory-value.md Story 1 S1-N1</t>
         </is>
       </c>
-      <c r="I72" s="2" t="inlineStr"/>
-      <c r="J72" s="2" t="inlineStr"/>
-    </row>
-    <row r="73">
-      <c r="A73" s="2" t="inlineStr">
+      <c r="I63" s="2" t="inlineStr"/>
+      <c r="J63" s="2" t="inlineStr"/>
+    </row>
+    <row r="64">
+      <c r="A64" s="2" t="inlineStr">
         <is>
           <t>Nightly snapshot: once per day, for every location, one row per in-stock non-core part is recorded with its identity, quantity, and values to the cent</t>
         </is>
       </c>
-      <c r="B73" s="2" t="inlineStr">
+      <c r="B64" s="2" t="inlineStr">
         <is>
           <t>IV — API</t>
         </is>
       </c>
-      <c r="C73" s="2" t="inlineStr">
-        <is>
-          <t>Functional</t>
-        </is>
-      </c>
-      <c r="D73" s="2" t="inlineStr">
+      <c r="C64" s="2" t="inlineStr">
+        <is>
+          <t>Functional</t>
+        </is>
+      </c>
+      <c r="D64" s="2" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="E73" s="2" t="inlineStr">
+      <c r="E64" s="2" t="inlineStr">
         <is>
           <t>1. In-stock, non-core parts exist at two or more locations, including a part with non-round cent values.
 2. A location with NO in-stock parts also exists.
 3. You can inspect the stored snapshot rows after the nightly capture runs (arrange the verification route with the developers).</t>
         </is>
       </c>
-      <c r="F73" s="2" t="inlineStr">
+      <c r="F64" s="2" t="inlineStr">
         <is>
           <t>1. After the overnight capture, inspect the stored snapshot rows for that calendar date.
 2. For a known part, read every captured field.
 3. Check the rows for each location, including the empty one.</t>
         </is>
       </c>
-      <c r="G73" s="2" t="inlineStr">
+      <c r="G64" s="2" t="inlineStr">
         <is>
           <t>1. Once per day, overnight, one row per then-in-stock, non-core part is recorded for every location across every organization, under that day's calendar date.
 2. Each row captures the part's identity (part, category, vendor), on-hand quantity, unit cost, unit sell, total cost, and total sell, stored to the cent.
 3. A location with no in-stock parts on the date simply has no rows for that date — this is valid, not an error.</t>
         </is>
       </c>
-      <c r="H73" s="2" t="inlineStr">
+      <c r="H64" s="2" t="inlineStr">
         <is>
           <t>specs/inventory-value.md Story 11 S11-R1; S11-R4</t>
         </is>
       </c>
-      <c r="I73" s="2" t="inlineStr"/>
-      <c r="J73" s="2" t="inlineStr"/>
-    </row>
-    <row r="74">
-      <c r="A74" s="2" t="inlineStr">
+      <c r="I64" s="2" t="inlineStr"/>
+      <c r="J64" s="2" t="inlineStr"/>
+    </row>
+    <row r="65">
+      <c r="A65" s="2" t="inlineStr">
         <is>
           <t>Nightly snapshot: the captured scope and valuation are identical to the live report, so a recorded day equals what the live report showed that day</t>
         </is>
       </c>
-      <c r="B74" s="2" t="inlineStr">
+      <c r="B65" s="2" t="inlineStr">
         <is>
           <t>IV — API</t>
         </is>
       </c>
-      <c r="C74" s="2" t="inlineStr">
-        <is>
-          <t>Functional</t>
-        </is>
-      </c>
-      <c r="D74" s="2" t="inlineStr">
+      <c r="C65" s="2" t="inlineStr">
+        <is>
+          <t>Functional</t>
+        </is>
+      </c>
+      <c r="D65" s="2" t="inlineStr">
         <is>
           <t>Critical</t>
         </is>
       </c>
-      <c r="E74" s="2" t="inlineStr">
+      <c r="E65" s="2" t="inlineStr">
         <is>
           <t>1. ZZAUTOTEST parts with known quantities, costs, and sell resolutions (fixed price, matrix markup, and no-category fallback) are in stock and left UNCHANGED across the capture.
 2. A core-charge part and a zero-quantity part also exist.
 3. You can read the live report on the capture date and the stored rows afterward.</t>
         </is>
       </c>
-      <c r="F74" s="2" t="inlineStr">
+      <c r="F65" s="2" t="inlineStr">
         <is>
           <t>1. On the capture date, note the live report's rows and values for the seeded parts.
 2. After the overnight capture, read the same parts' captured rows.
@@ -3994,216 +3581,216 @@
 4. The next day, view the report as of the captured date and compare to the noted live values.</t>
         </is>
       </c>
-      <c r="G74" s="2" t="inlineStr">
+      <c r="G65" s="2" t="inlineStr">
         <is>
           <t>1. The captured parts use the same in-stock, non-core scope as the live report (Story 2) — the core-charge and zero-quantity parts are NOT captured.
 2. The captured values use the same valuation as the live report (Story 3), including the sell-price fallback chain.
 3. A recorded day equals what the live report would have shown that day — the as-of view of the captured date matches the noted live values.</t>
         </is>
       </c>
-      <c r="H74" s="2" t="inlineStr">
+      <c r="H65" s="2" t="inlineStr">
         <is>
           <t>specs/inventory-value.md Story 11 S11-R2; §2 Relationship to nightly history</t>
         </is>
       </c>
-      <c r="I74" s="2" t="inlineStr"/>
-      <c r="J74" s="2" t="inlineStr"/>
-    </row>
-    <row r="75">
-      <c r="A75" s="2" t="inlineStr">
+      <c r="I65" s="2" t="inlineStr"/>
+      <c r="J65" s="2" t="inlineStr"/>
+    </row>
+    <row r="66">
+      <c r="A66" s="2" t="inlineStr">
         <is>
           <t>Nightly snapshot: re-running the capture for a date replaces that date's rows — idempotent, no duplicates</t>
         </is>
       </c>
-      <c r="B75" s="2" t="inlineStr">
+      <c r="B66" s="2" t="inlineStr">
         <is>
           <t>IV — API</t>
         </is>
       </c>
-      <c r="C75" s="2" t="inlineStr">
-        <is>
-          <t>Functional</t>
-        </is>
-      </c>
-      <c r="D75" s="2" t="inlineStr">
+      <c r="C66" s="2" t="inlineStr">
+        <is>
+          <t>Functional</t>
+        </is>
+      </c>
+      <c r="D66" s="2" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="E75" s="2" t="inlineStr">
+      <c r="E66" s="2" t="inlineStr">
         <is>
           <t>1. A capture has already run for the current date.
 2. The capture can be re-run for that date (arrange with the developers).</t>
         </is>
       </c>
-      <c r="F75" s="2" t="inlineStr">
+      <c r="F66" s="2" t="inlineStr">
         <is>
           <t>1. Count the stored rows per location for the date.
 2. Re-run the capture for the same date.
 3. Count and inspect the rows again.</t>
         </is>
       </c>
-      <c r="G75" s="2" t="inlineStr">
+      <c r="G66" s="2" t="inlineStr">
         <is>
           <t>1. Re-running the capture for a date replaces that date's rows for each location — the existing rows for that location and date are removed, then re-inserted from current data.
 2. No duplicate rows exist for the same part, location, and date.
 3. The capture is idempotent and self-healing from current data.</t>
         </is>
       </c>
-      <c r="H75" s="2" t="inlineStr">
+      <c r="H66" s="2" t="inlineStr">
         <is>
           <t>specs/inventory-value.md Story 11 S11-R3</t>
         </is>
       </c>
-      <c r="I75" s="2" t="inlineStr"/>
-      <c r="J75" s="2" t="inlineStr"/>
-    </row>
-    <row r="76">
-      <c r="A76" s="2" t="inlineStr">
+      <c r="I66" s="2" t="inlineStr"/>
+      <c r="J66" s="2" t="inlineStr"/>
+    </row>
+    <row r="67">
+      <c r="A67" s="2" t="inlineStr">
         <is>
           <t>Nightly snapshot: history accrues forward only — a re-run records current truth under the current date and cannot reconstruct a past date</t>
         </is>
       </c>
-      <c r="B76" s="2" t="inlineStr">
+      <c r="B67" s="2" t="inlineStr">
         <is>
           <t>IV — API</t>
         </is>
       </c>
-      <c r="C76" s="2" t="inlineStr">
-        <is>
-          <t>Functional</t>
-        </is>
-      </c>
-      <c r="D76" s="2" t="inlineStr">
+      <c r="C67" s="2" t="inlineStr">
+        <is>
+          <t>Functional</t>
+        </is>
+      </c>
+      <c r="D67" s="2" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="E76" s="2" t="inlineStr">
+      <c r="E67" s="2" t="inlineStr">
         <is>
           <t>1. The date the first capture ran is known.
 2. Stock levels have changed since a past captured date.</t>
         </is>
       </c>
-      <c r="F76" s="2" t="inlineStr">
+      <c r="F67" s="2" t="inlineStr">
         <is>
           <t>1. Check the stored history for any rows dated before the first capture.
 2. Re-run the capture and check which date its rows are recorded under.
 3. Compare a past date's stored rows to confirm they were not rewritten by the re-run.</t>
         </is>
       </c>
-      <c r="G76" s="2" t="inlineStr">
+      <c r="G67" s="2" t="inlineStr">
         <is>
           <t>1. No rows exist for dates before capture began — there is no backfill.
 2. A re-run always records current truth under the CURRENT date; it cannot reconstruct a past date.
 3. Past dates' stored rows are unchanged by a current re-run.</t>
         </is>
       </c>
-      <c r="H76" s="2" t="inlineStr">
+      <c r="H67" s="2" t="inlineStr">
         <is>
           <t>specs/inventory-value.md Story 11 S11-R5; Story 5 S5-E1</t>
         </is>
       </c>
-      <c r="I76" s="2" t="inlineStr"/>
-      <c r="J76" s="2" t="inlineStr"/>
-    </row>
-    <row r="77">
-      <c r="A77" s="2" t="inlineStr">
+      <c r="I67" s="2" t="inlineStr"/>
+      <c r="J67" s="2" t="inlineStr"/>
+    </row>
+    <row r="68">
+      <c r="A68" s="2" t="inlineStr">
         <is>
           <t>Snapshot retention: daily captures are kept for 0–13 months; older history is reduced to the last capture of each calendar month</t>
         </is>
       </c>
-      <c r="B77" s="2" t="inlineStr">
+      <c r="B68" s="2" t="inlineStr">
         <is>
           <t>IV — API</t>
         </is>
       </c>
-      <c r="C77" s="2" t="inlineStr">
-        <is>
-          <t>Functional</t>
-        </is>
-      </c>
-      <c r="D77" s="2" t="inlineStr">
+      <c r="C68" s="2" t="inlineStr">
+        <is>
+          <t>Functional</t>
+        </is>
+      </c>
+      <c r="D68" s="2" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="E77" s="2" t="inlineStr">
+      <c r="E68" s="2" t="inlineStr">
         <is>
           <t>1. Snapshot history exists (or is seeded/simulated with dev help) spanning both the 0–13-month band and the older-than-13-months band.
 2. The nightly capture (with its pruning) has run.</t>
         </is>
       </c>
-      <c r="F77" s="2" t="inlineStr">
+      <c r="F68" s="2" t="inlineStr">
         <is>
           <t>1. Inspect the retained captures for dates within the last 13 months.
 2. Inspect the retained captures for dates older than 13 months.
 3. Check when pruning runs relative to the nightly capture.</t>
         </is>
       </c>
-      <c r="G77" s="2" t="inlineStr">
+      <c r="G68" s="2" t="inlineStr">
         <is>
           <t>1. For ages 0–13 months (measured from the current date), every daily capture is kept — full daily per-part detail, covering the report's longest date preset (366 days / This Year / Last Year) entirely at daily resolution.
 2. For ages older than 13 months, only the last capture of each calendar month is retained; the other daily captures in that band are pruned.
 3. Pruning runs as part of, or alongside, the nightly capture.</t>
         </is>
       </c>
-      <c r="H77" s="2" t="inlineStr">
+      <c r="H68" s="2" t="inlineStr">
         <is>
           <t>specs/inventory-value.md Story 11 S11-R6</t>
         </is>
       </c>
-      <c r="I77" s="2" t="inlineStr"/>
-      <c r="J77" s="2" t="inlineStr"/>
-    </row>
-    <row r="78">
-      <c r="A78" s="2" t="inlineStr">
+      <c r="I68" s="2" t="inlineStr"/>
+      <c r="J68" s="2" t="inlineStr"/>
+    </row>
+    <row r="69">
+      <c r="A69" s="2" t="inlineStr">
         <is>
           <t>Thinned history is served unchanged: the closest-recorded-day rule bridges retention gaps, the "As of" indicator names the day shown, and a fully-pruned range shows the empty state</t>
         </is>
       </c>
-      <c r="B78" s="2" t="inlineStr">
+      <c r="B69" s="2" t="inlineStr">
         <is>
           <t>IV — API</t>
         </is>
       </c>
-      <c r="C78" s="2" t="inlineStr">
-        <is>
-          <t>Functional</t>
-        </is>
-      </c>
-      <c r="D78" s="2" t="inlineStr">
+      <c r="C69" s="2" t="inlineStr">
+        <is>
+          <t>Functional</t>
+        </is>
+      </c>
+      <c r="D69" s="2" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="E78" s="2" t="inlineStr">
+      <c r="E69" s="2" t="inlineStr">
         <is>
           <t>1. Thinned history exists (dates older than 13 months where only the monthly last-capture remains — dev-seeded if needed).
 2. The retained capture dates around the requested date are known.</t>
         </is>
       </c>
-      <c r="F78" s="2" t="inlineStr">
+      <c r="F69" s="2" t="inlineStr">
         <is>
           <t>1. On the report, select a range ending on a pruned date between two retained monthly captures.
 2. Read which day the values represent and the "As of" indicator.
 3. Select a range whose covering captures have ALL been pruned and no earlier retained capture remains.</t>
         </is>
       </c>
-      <c r="G78" s="2" t="inlineStr">
+      <c r="G69" s="2" t="inlineStr">
         <is>
           <t>1. The as-of resolution serves the thinned history unchanged: the report resolves to the nearest earlier retained capture ("closest recorded day on or before"), even when adjacent retained captures are up to a month apart.
 2. The "As of" indicator names the day actually shown.
 3. A requested date whose covering captures have all been pruned resolves to the nearest earlier retained capture, or shows the empty state if none remains.</t>
         </is>
       </c>
-      <c r="H78" s="2" t="inlineStr">
+      <c r="H69" s="2" t="inlineStr">
         <is>
           <t>specs/inventory-value.md Story 11 S11-E1; S11-R6; Story 5 S5-R4; S5-R5; S5-N1</t>
         </is>
       </c>
-      <c r="I78" s="2" t="inlineStr"/>
-      <c r="J78" s="2" t="inlineStr"/>
+      <c r="I69" s="2" t="inlineStr"/>
+      <c r="J69" s="2" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Ingest Chris 2026-07-29 update: VIN/exports/Special Order/TU column selector applied locally + change-list
Chris Ward group message 8:53 AM 2026-07-29 saved verbatim + applied LOCAL ONLY
(no TestRail writes): SBC VIN->Unit#->plate identifier; SBC Summary/Expanded
exports w/ four exact menu items; Locations: line + on-screen scope indicator
all 6 reports (12 existing cases extended); Catalogue->Special Order confirmed;
NEW TU-COL-01 column-selector case; PV logo coverage added. 8 touched titles
trimmed <=80; 11 story tickets backfilled (Rule 20). 460 active authored.
Backups + MANIFEST; ChangeList-2026-07-29.md/.xlsx = push-approval gate (24
update_case + 1 add_case). Rule-28 audit 26/26/26 clean. SPEC-WATCH +
PROJECT-STATE + coverage addenda updated; deliverables regenerated, hygiene
clean, id-map re-merged 459/460.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01AZ5XzKsK9wv7M41cSPaMyg
</commit_message>
<xml_diff>
--- a/testrail-import/Report-Suite_Inventory-Value-Report_testrail-import.xlsx
+++ b/testrail-import/Report-Suite_Inventory-Value-Report_testrail-import.xlsx
@@ -2230,12 +2230,13 @@
       <c r="G37" s="2" t="inlineStr">
         <is>
           <t>1. Each selection change reloads the report scoped to the selected set.
-2. With both locations selected, parts from both appear (one row per part per location) and the totals cover both.</t>
+2. With both locations selected, parts from both appear (one row per part per location) and the totals cover both.
+3. The page itself shows which location(s) the report is currently scoped to (the new on-screen scope indicator - exactly where and how it appears is confirmed in the build).</t>
         </is>
       </c>
       <c r="H37" s="2" t="inlineStr">
         <is>
-          <t>specs/inventory-value.md Story 7 S7-R3</t>
+          <t>SV-8674 (specs/inventory-value.md Story 7 S7-R3 + on-screen location-scope indicator per Chris Ward group message 2026-07-29 (chris-update-2026-07-29/chris-message-2026-07-29.md; NEWEST source, last-update-wins))</t>
         </is>
       </c>
       <c r="I37" s="2" t="inlineStr"/>
@@ -2770,7 +2771,7 @@
     <row r="49">
       <c r="A49" s="2" t="inlineStr">
         <is>
-          <t>Downloads contain the shown columns in screen order (Total Cost last), honor all filters and the sort, and include a "Totals" row matching the full-set totals</t>
+          <t>Downloads keep shown columns and order, honor filters, and include Totals</t>
         </is>
       </c>
       <c r="B49" s="2" t="inlineStr">
@@ -2807,12 +2808,13 @@
         <is>
           <t>1. Both downloads include only the columns currently shown, in the same left-to-right order as the screen, with Total Cost last.
 2. Both downloads honor the current date, category, vendor, location, and part-search filters, and apply the current sort.
-3. Both downloads include a totals row labeled "Totals" matching the on-screen totals (the full-filtered-set totals).</t>
+3. Both downloads include a totals row labeled "Totals" matching the on-screen totals (the full-filtered-set totals).
+4. Each download (PDF and CSV) carries a "Locations:" line naming the location(s) the report was scoped to (exact position in the file is confirmed in the build).</t>
         </is>
       </c>
       <c r="H49" s="2" t="inlineStr">
         <is>
-          <t>specs/inventory-value.md Story 10 S10-R3; S10-R4; S10-R5; S10-R6</t>
+          <t>SV-8677 (specs/inventory-value.md Story 10 S10-R3; S10-R4; S10-R5; S10-R6 + Locations: line in every CSV/PDF export per Chris Ward group message 2026-07-29 (chris-update-2026-07-29/chris-message-2026-07-29.md; NEWEST source, last-update-wins))</t>
         </is>
       </c>
       <c r="I49" s="2" t="inlineStr"/>

</xml_diff>

<commit_message>
Report Suite: tech-plan pass Phase 4 — Rule-28 tally, change-list + push queue (staged), deliverables regenerated over 465, id-map re-merged, PROJECT-STATE update
Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01AZ5XzKsK9wv7M41cSPaMyg
</commit_message>
<xml_diff>
--- a/testrail-import/Report-Suite_Inventory-Value-Report_testrail-import.xlsx
+++ b/testrail-import/Report-Suite_Inventory-Value-Report_testrail-import.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Inventory Value" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Inventory Value" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -428,7 +428,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J69"/>
+  <dimension ref="A1:J70"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="50" customWidth="1" min="1" max="1"/>
@@ -1899,80 +1899,130 @@
     <row r="31">
       <c r="A31" s="2" t="inlineStr">
         <is>
+          <t>A recorded day keeps its category and vendor names after a rename or delete</t>
+        </is>
+      </c>
+      <c r="B31" s="2" t="inlineStr">
+        <is>
+          <t>IV — As-of Date &amp; Snapshots</t>
+        </is>
+      </c>
+      <c r="C31" s="2" t="inlineStr">
+        <is>
+          <t>Functional</t>
+        </is>
+      </c>
+      <c r="D31" s="2" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="E31" s="2" t="inlineStr">
+        <is>
+          <t>1. You are signed in to the ShopView App on a desktop browser.
+2. A recorded (overnight-captured) day exists that includes ZZAUTOTEST parts under a known category and a known vendor.</t>
+        </is>
+      </c>
+      <c r="F31" s="2" t="inlineStr">
+        <is>
+          <t>1. Rename that part category (and/or rename or delete the vendor) in administration.
+2. Set the report's date range so it shows the earlier recorded day (the "As of" indicator names that earlier date).
+3. Read the affected rows' Category and Vendor cells on the recorded day.
+4. Move the range back to include today (live view) and re-read a renamed category's rows.</t>
+        </is>
+      </c>
+      <c r="G31" s="2" t="inlineStr">
+        <is>
+          <t>1. The earlier recorded day still shows the category and vendor names AS THEY WERE RECORDED that day — a recorded day equals what the live report showed that day, even after the rename/delete.
+2. The rename/delete causes no blank Category/Vendor cells and no dropped rows on the recorded day.
+3. The live view (window reaching today) shows the NEW name for the renamed category.</t>
+        </is>
+      </c>
+      <c r="H31" s="2" t="inlineStr">
+        <is>
+          <t>SV-8678 (specs/inventory-value.md Story 11 S11-R2; Story 5 S5-R4; tech-plan-2026-07-29 B4.1 — names stored with the recorded rows on purpose)</t>
+        </is>
+      </c>
+      <c r="I31" s="2" t="inlineStr"/>
+      <c r="J31" s="2" t="inlineStr"/>
+    </row>
+    <row r="32">
+      <c r="A32" s="2" t="inlineStr">
+        <is>
           <t>The Category and Vendor filters are multi-selects that reload the report to only the matching parts</t>
         </is>
       </c>
-      <c r="B31" s="2" t="inlineStr">
+      <c r="B32" s="2" t="inlineStr">
         <is>
           <t>IV — Filters &amp; Part Search</t>
         </is>
       </c>
-      <c r="C31" s="2" t="inlineStr">
-        <is>
-          <t>Functional</t>
-        </is>
-      </c>
-      <c r="D31" s="2" t="inlineStr">
+      <c r="C32" s="2" t="inlineStr">
+        <is>
+          <t>Functional</t>
+        </is>
+      </c>
+      <c r="D32" s="2" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="E31" s="2" t="inlineStr">
+      <c r="E32" s="2" t="inlineStr">
         <is>
           <t>1. You are signed in to the ShopView App on a desktop browser.
 2. In-stock parts exist across at least two categories and two vendors.</t>
         </is>
       </c>
-      <c r="F31" s="2" t="inlineStr">
+      <c r="F32" s="2" t="inlineStr">
         <is>
           <t>1. Open the filter labeled "Category" and select one category; watch the data area.
 2. Add a second category to the selection.
 3. Clear the Category filter, open the filter labeled "Vendor", and select one vendor; then add a second.</t>
         </is>
       </c>
-      <c r="G31" s="2" t="inlineStr">
+      <c r="G32" s="2" t="inlineStr">
         <is>
           <t>1. The toolbar has a Category filter labeled "Category" and a Vendor filter labeled "Vendor", each allowing one or more selections.
 2. Selecting one or more categories reloads the report to show only parts in the selected categories.
 3. Selecting one or more vendors reloads the report to show only parts supplied by the selected vendors.</t>
         </is>
       </c>
-      <c r="H31" s="2" t="inlineStr">
+      <c r="H32" s="2" t="inlineStr">
         <is>
           <t>specs/inventory-value.md Story 6 S6-R1; S6-R2; S6-R3; S6-R4</t>
         </is>
       </c>
-      <c r="I31" s="2" t="inlineStr"/>
-      <c r="J31" s="2" t="inlineStr"/>
-    </row>
-    <row r="32">
-      <c r="A32" s="2" t="inlineStr">
+      <c r="I32" s="2" t="inlineStr"/>
+      <c r="J32" s="2" t="inlineStr"/>
+    </row>
+    <row r="33">
+      <c r="A33" s="2" t="inlineStr">
         <is>
           <t>Category, Vendor and part search are server-side; each change returns page 1</t>
         </is>
       </c>
-      <c r="B32" s="2" t="inlineStr">
+      <c r="B33" s="2" t="inlineStr">
         <is>
           <t>IV — Filters &amp; Part Search</t>
         </is>
       </c>
-      <c r="C32" s="2" t="inlineStr">
-        <is>
-          <t>Functional</t>
-        </is>
-      </c>
-      <c r="D32" s="2" t="inlineStr">
+      <c r="C33" s="2" t="inlineStr">
+        <is>
+          <t>Functional</t>
+        </is>
+      </c>
+      <c r="D33" s="2" t="inlineStr">
         <is>
           <t>Critical</t>
         </is>
       </c>
-      <c r="E32" s="2" t="inlineStr">
+      <c r="E33" s="2" t="inlineStr">
         <is>
           <t>1. You are signed in to the ShopView App on a desktop browser.
 2. The unfiltered result set spans multiple pages, and matching parts for a category/vendor/search exist BEYOND page 1.</t>
         </is>
       </c>
-      <c r="F32" s="2" t="inlineStr">
+      <c r="F33" s="2" t="inlineStr">
         <is>
           <t>1. From page 2 (or later), select a Category and check which page shows and which rows are listed.
 2. Repeat with a Vendor selection.
@@ -1980,98 +2030,98 @@
 4. Also change the date range, the location selection, and the sort — watching the data area each time.</t>
         </is>
       </c>
-      <c r="G32" s="2" t="inlineStr">
+      <c r="G33" s="2" t="inlineStr">
         <is>
           <t>1. Each change re-queries the server and returns the first page of the new result set.
 2. The filtering covers the ENTIRE data set — matching parts that were on later pages appear — not just a narrowing of the rows on the current page.
 3. Every change — date range, location, Category, Vendor, part search, sort — reloads the rows from the server; while loading the standard reports loading indicator shows, and existing rows are replaced only when the new data returns.</t>
         </is>
       </c>
-      <c r="H32" s="2" t="inlineStr">
+      <c r="H33" s="2" t="inlineStr">
         <is>
           <t>specs/inventory-value.md Story 6 S6-R5; Story 1 S1-R4; S1-R5; S1-R7; S1-R8</t>
         </is>
       </c>
-      <c r="I32" s="2" t="inlineStr"/>
-      <c r="J32" s="2" t="inlineStr"/>
-    </row>
-    <row r="33">
-      <c r="A33" s="2" t="inlineStr">
+      <c r="I33" s="2" t="inlineStr"/>
+      <c r="J33" s="2" t="inlineStr"/>
+    </row>
+    <row r="34">
+      <c r="A34" s="2" t="inlineStr">
         <is>
           <t>With no category or vendor selected all parts show, and an empty part search applies no narrowing</t>
         </is>
       </c>
-      <c r="B33" s="2" t="inlineStr">
+      <c r="B34" s="2" t="inlineStr">
         <is>
           <t>IV — Filters &amp; Part Search</t>
         </is>
       </c>
-      <c r="C33" s="2" t="inlineStr">
-        <is>
-          <t>Functional</t>
-        </is>
-      </c>
-      <c r="D33" s="2" t="inlineStr">
+      <c r="C34" s="2" t="inlineStr">
+        <is>
+          <t>Functional</t>
+        </is>
+      </c>
+      <c r="D34" s="2" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="E33" s="2" t="inlineStr">
+      <c r="E34" s="2" t="inlineStr">
         <is>
           <t>1. You are signed in to the ShopView App on a desktop browser.
 2. The report has been filtered by category, vendor, and a part search.</t>
         </is>
       </c>
-      <c r="F33" s="2" t="inlineStr">
+      <c r="F34" s="2" t="inlineStr">
         <is>
           <t>1. Clear the Category selection and check the rows.
 2. Clear the Vendor selection and check the rows.
 3. Empty the part search and check the rows.</t>
         </is>
       </c>
-      <c r="G33" s="2" t="inlineStr">
+      <c r="G34" s="2" t="inlineStr">
         <is>
           <t>1. With no category selected, parts of all categories are shown.
 2. With no vendor selected, parts of all vendors are shown.
 3. With the part search empty, no search narrowing is applied.</t>
         </is>
       </c>
-      <c r="H33" s="2" t="inlineStr">
+      <c r="H34" s="2" t="inlineStr">
         <is>
           <t>specs/inventory-value.md Story 6 S6-R7</t>
         </is>
       </c>
-      <c r="I33" s="2" t="inlineStr"/>
-      <c r="J33" s="2" t="inlineStr"/>
-    </row>
-    <row r="34">
-      <c r="A34" s="2" t="inlineStr">
+      <c r="I34" s="2" t="inlineStr"/>
+      <c r="J34" s="2" t="inlineStr"/>
+    </row>
+    <row r="35">
+      <c r="A35" s="2" t="inlineStr">
         <is>
           <t>The part search is a page-local toolbar field matching part number OR description, case-insensitively, on the server</t>
         </is>
       </c>
-      <c r="B34" s="2" t="inlineStr">
+      <c r="B35" s="2" t="inlineStr">
         <is>
           <t>IV — Filters &amp; Part Search</t>
         </is>
       </c>
-      <c r="C34" s="2" t="inlineStr">
-        <is>
-          <t>Functional</t>
-        </is>
-      </c>
-      <c r="D34" s="2" t="inlineStr">
+      <c r="C35" s="2" t="inlineStr">
+        <is>
+          <t>Functional</t>
+        </is>
+      </c>
+      <c r="D35" s="2" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="E34" s="2" t="inlineStr">
+      <c r="E35" s="2" t="inlineStr">
         <is>
           <t>1. You are signed in to the ShopView App on a desktop browser.
 2. In-stock parts exist whose part numbers and descriptions you know (including a description containing a distinctive word).</t>
         </is>
       </c>
-      <c r="F34" s="2" t="inlineStr">
+      <c r="F35" s="2" t="inlineStr">
         <is>
           <t>1. Find the part search input in the report's own toolbar (not the application's global search bar).
 2. Type part of a part number and read the results.
@@ -2079,7 +2129,7 @@
 4. Type text matching nothing.</t>
         </is>
       </c>
-      <c r="G34" s="2" t="inlineStr">
+      <c r="G35" s="2" t="inlineStr">
         <is>
           <t>1. The search field is page-local, in the report's own toolbar — it is not the application's global search bar (the same toolbar-search pattern used elsewhere in the reports suite).
 2. The report narrows to parts whose part number OR description contains the entered text.
@@ -2087,90 +2137,90 @@
 4. The search applies server-side (whole data set, first page returned); a no-match search shows the no-data message.</t>
         </is>
       </c>
-      <c r="H34" s="2" t="inlineStr">
+      <c r="H35" s="2" t="inlineStr">
         <is>
           <t>specs/inventory-value.md Story 6 S6-R8; S6-R5</t>
         </is>
       </c>
-      <c r="I34" s="2" t="inlineStr"/>
-      <c r="J34" s="2" t="inlineStr"/>
-    </row>
-    <row r="35">
-      <c r="A35" s="2" t="inlineStr">
+      <c r="I35" s="2" t="inlineStr"/>
+      <c r="J35" s="2" t="inlineStr"/>
+    </row>
+    <row r="36">
+      <c r="A36" s="2" t="inlineStr">
         <is>
           <t>Date range, Location, Category, Vendor, and the part search combine with AND</t>
         </is>
       </c>
-      <c r="B35" s="2" t="inlineStr">
+      <c r="B36" s="2" t="inlineStr">
         <is>
           <t>IV — Filters &amp; Part Search</t>
         </is>
       </c>
-      <c r="C35" s="2" t="inlineStr">
-        <is>
-          <t>Functional</t>
-        </is>
-      </c>
-      <c r="D35" s="2" t="inlineStr">
+      <c r="C36" s="2" t="inlineStr">
+        <is>
+          <t>Functional</t>
+        </is>
+      </c>
+      <c r="D36" s="2" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="E35" s="2" t="inlineStr">
+      <c r="E36" s="2" t="inlineStr">
         <is>
           <t>1. You are signed in to the ShopView App on a desktop browser.
 2. In-stock parts exist with a known mix of categories and vendors, so a combined filter isolates a known subset.</t>
         </is>
       </c>
-      <c r="F35" s="2" t="inlineStr">
+      <c r="F36" s="2" t="inlineStr">
         <is>
           <t>1. Select a Category, then also a Vendor that only some of those category parts have.
 2. Add a part search matching only one of the remaining parts.
 3. Check the rows and the totals row after each step.</t>
         </is>
       </c>
-      <c r="G35" s="2" t="inlineStr">
+      <c r="G36" s="2" t="inlineStr">
         <is>
           <t>1. A part must satisfy EVERY active filter and the search to appear — the Date range, Location, Category, Vendor, and part search combine with AND.
 2. The totals row matches the combined filtered set after each step.</t>
         </is>
       </c>
-      <c r="H35" s="2" t="inlineStr">
+      <c r="H36" s="2" t="inlineStr">
         <is>
           <t>specs/inventory-value.md Story 6 S6-R9</t>
         </is>
       </c>
-      <c r="I35" s="2" t="inlineStr"/>
-      <c r="J35" s="2" t="inlineStr"/>
-    </row>
-    <row r="36">
-      <c r="A36" s="2" t="inlineStr">
+      <c r="I36" s="2" t="inlineStr"/>
+      <c r="J36" s="2" t="inlineStr"/>
+    </row>
+    <row r="37">
+      <c r="A37" s="2" t="inlineStr">
         <is>
           <t>The Location filter is a rightmost multi-select with an All locations toggle</t>
         </is>
       </c>
-      <c r="B36" s="2" t="inlineStr">
+      <c r="B37" s="2" t="inlineStr">
         <is>
           <t>IV — Location Filter</t>
         </is>
       </c>
-      <c r="C36" s="2" t="inlineStr">
-        <is>
-          <t>Functional</t>
-        </is>
-      </c>
-      <c r="D36" s="2" t="inlineStr">
+      <c r="C37" s="2" t="inlineStr">
+        <is>
+          <t>Functional</t>
+        </is>
+      </c>
+      <c r="D37" s="2" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="E36" s="2" t="inlineStr">
+      <c r="E37" s="2" t="inlineStr">
         <is>
           <t>1. You are signed in to the ShopView App on a desktop browser as a user with access to at least two locations.
 2. This browser has never saved settings for this report (fresh visit).</t>
         </is>
       </c>
-      <c r="F36" s="2" t="inlineStr">
+      <c r="F37" s="2" t="inlineStr">
         <is>
           <t>1. Open the Inventory Value report and find the filter labeled "Location".
 2. Read its position in the toolbar and its default selection.
@@ -2178,288 +2228,288 @@
 4. Select every accessible location ("All locations") and look at how the rows tell you which location they belong to.</t>
         </is>
       </c>
-      <c r="G36" s="2" t="inlineStr">
+      <c r="G37" s="2" t="inlineStr">
         <is>
           <t>1. The toolbar has a location filter labeled "Location" — a multi-select and the rightmost filter — listing the locations the signed-in user has access to, with an "All locations" / "Clear all" toggle.
 2. On a first visit it defaults to the user's currently active location.
 3. With "All locations" active you can tell which location each row's stock belongs to — a location label or marking is shown. (Exactly where and how it appears is confirmed in the build.)</t>
         </is>
       </c>
-      <c r="H36" s="2" t="inlineStr">
+      <c r="H37" s="2" t="inlineStr">
         <is>
           <t>SV-8674 (specs/inventory-value.md Story 7 S7-R1; S7-R2; Story 12 S12-R3 — per-row location identifier in All-locations view ADDED per kickoff video P10 40:58-41:20, user ruling 2026-07-28: video overrides spec (video newer, last-update-wins))</t>
         </is>
       </c>
-      <c r="I36" s="2" t="inlineStr"/>
-      <c r="J36" s="2" t="inlineStr"/>
-    </row>
-    <row r="37">
-      <c r="A37" s="2" t="inlineStr">
+      <c r="I37" s="2" t="inlineStr"/>
+      <c r="J37" s="2" t="inlineStr"/>
+    </row>
+    <row r="38">
+      <c r="A38" s="2" t="inlineStr">
         <is>
           <t>Selecting one, several, or all locations reloads the report scoped to that set</t>
         </is>
       </c>
-      <c r="B37" s="2" t="inlineStr">
+      <c r="B38" s="2" t="inlineStr">
         <is>
           <t>IV — Location Filter</t>
         </is>
       </c>
-      <c r="C37" s="2" t="inlineStr">
-        <is>
-          <t>Functional</t>
-        </is>
-      </c>
-      <c r="D37" s="2" t="inlineStr">
+      <c r="C38" s="2" t="inlineStr">
+        <is>
+          <t>Functional</t>
+        </is>
+      </c>
+      <c r="D38" s="2" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="E37" s="2" t="inlineStr">
+      <c r="E38" s="2" t="inlineStr">
         <is>
           <t>1. You are signed in to the ShopView App on a desktop browser as a user with access to at least two locations.
 2. In-stock parts exist at both locations.</t>
         </is>
       </c>
-      <c r="F37" s="2" t="inlineStr">
+      <c r="F38" s="2" t="inlineStr">
         <is>
           <t>1. With one location selected, note the rows and totals.
 2. Add the second location and watch the data area.
 3. Use "All locations", then narrow back to one.</t>
         </is>
       </c>
-      <c r="G37" s="2" t="inlineStr">
+      <c r="G38" s="2" t="inlineStr">
         <is>
           <t>1. Each selection change reloads the report scoped to the selected set.
 2. With both locations selected, parts from both appear (one row per part per location) and the totals cover both.
 3. The page itself shows which location(s) the report is currently scoped to (the new on-screen scope indicator - exactly where and how it appears is confirmed in the build).</t>
         </is>
       </c>
-      <c r="H37" s="2" t="inlineStr">
+      <c r="H38" s="2" t="inlineStr">
         <is>
           <t>SV-8674 (specs/inventory-value.md Story 7 S7-R3 + on-screen location-scope indicator per Chris Ward group message 2026-07-29 (chris-update-2026-07-29/chris-message-2026-07-29.md; NEWEST source, last-update-wins))</t>
         </is>
       </c>
-      <c r="I37" s="2" t="inlineStr"/>
-      <c r="J37" s="2" t="inlineStr"/>
-    </row>
-    <row r="38">
-      <c r="A38" s="2" t="inlineStr">
+      <c r="I38" s="2" t="inlineStr"/>
+      <c r="J38" s="2" t="inlineStr"/>
+    </row>
+    <row r="39">
+      <c r="A39" s="2" t="inlineStr">
         <is>
           <t>Scoping never includes an inaccessible location, and a selection resolving to none falls back to the user's active location</t>
         </is>
       </c>
-      <c r="B38" s="2" t="inlineStr">
+      <c r="B39" s="2" t="inlineStr">
         <is>
           <t>IV — Location Filter</t>
         </is>
       </c>
-      <c r="C38" s="2" t="inlineStr">
+      <c r="C39" s="2" t="inlineStr">
         <is>
           <t>Negative</t>
         </is>
       </c>
-      <c r="D38" s="2" t="inlineStr">
+      <c r="D39" s="2" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="E38" s="2" t="inlineStr">
+      <c r="E39" s="2" t="inlineStr">
         <is>
           <t>1. You are signed in to the ShopView App on a desktop browser as a user who can access some, but not all, of the organization's locations.
 2. The Inventory Value report is open.</t>
         </is>
       </c>
-      <c r="F38" s="2" t="inlineStr">
+      <c r="F39" s="2" t="inlineStr">
         <is>
           <t>1. Open the Location filter and read the locations offered.
 2. Use "Clear all" so the selection resolves to no location, and watch what the report loads.</t>
         </is>
       </c>
-      <c r="G38" s="2" t="inlineStr">
+      <c r="G39" s="2" t="inlineStr">
         <is>
           <t>1. Only the locations the user has access to are offered — a location the user cannot access is never included in the scope.
 2. If the requested location set resolves to none the user can access, the report falls back to the user's currently active location.</t>
         </is>
       </c>
-      <c r="H38" s="2" t="inlineStr">
+      <c r="H39" s="2" t="inlineStr">
         <is>
           <t>specs/inventory-value.md Story 7 S7-R4; S7-R5</t>
         </is>
       </c>
-      <c r="I38" s="2" t="inlineStr"/>
-      <c r="J38" s="2" t="inlineStr"/>
-    </row>
-    <row r="39">
-      <c r="A39" s="2" t="inlineStr">
+      <c r="I39" s="2" t="inlineStr"/>
+      <c r="J39" s="2" t="inlineStr"/>
+    </row>
+    <row r="40">
+      <c r="A40" s="2" t="inlineStr">
         <is>
           <t>The Location filter is hidden for a user with access to only one location</t>
         </is>
       </c>
-      <c r="B39" s="2" t="inlineStr">
+      <c r="B40" s="2" t="inlineStr">
         <is>
           <t>IV — Location Filter</t>
         </is>
       </c>
-      <c r="C39" s="2" t="inlineStr">
-        <is>
-          <t>Functional</t>
-        </is>
-      </c>
-      <c r="D39" s="2" t="inlineStr">
+      <c r="C40" s="2" t="inlineStr">
+        <is>
+          <t>Functional</t>
+        </is>
+      </c>
+      <c r="D40" s="2" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="E39" s="2" t="inlineStr">
+      <c r="E40" s="2" t="inlineStr">
         <is>
           <t>1. A test user exists with access to exactly one location (create a fresh ZZAUTOTEST staff member if needed; clean up afterward).
 2. You are signed in as that user on a desktop browser.</t>
         </is>
       </c>
-      <c r="F39" s="2" t="inlineStr">
+      <c r="F40" s="2" t="inlineStr">
         <is>
           <t>1. Open the Inventory Value report and look for the Location filter in the toolbar.
 2. Then sign in as a user with access to two or more locations and look again.</t>
         </is>
       </c>
-      <c r="G39" s="2" t="inlineStr">
+      <c r="G40" s="2" t="inlineStr">
         <is>
           <t>1. For the single-location user the Location filter is NOT shown at all — the report simply shows that one location's stock.
 2. For the user with access to two or more locations the Location filter IS shown.</t>
         </is>
       </c>
-      <c r="H39" s="2" t="inlineStr">
+      <c r="H40" s="2" t="inlineStr">
         <is>
           <t>SV-8674 (specs/inventory-value.md Story 7 S7-N1 — expectation FLIPPED by kickoff video P33 46:10-46:28, user ruling 2026-07-28: video overrides spec (video newer, last-update-wins))</t>
         </is>
       </c>
-      <c r="I39" s="2" t="inlineStr"/>
-      <c r="J39" s="2" t="inlineStr"/>
-    </row>
-    <row r="40">
-      <c r="A40" s="2" t="inlineStr">
+      <c r="I40" s="2" t="inlineStr"/>
+      <c r="J40" s="2" t="inlineStr"/>
+    </row>
+    <row r="41">
+      <c r="A41" s="2" t="inlineStr">
         <is>
           <t>The column-selection icon button (tooltip "Column Selection") toggles columns, and Total Cost cannot be turned off</t>
         </is>
       </c>
-      <c r="B40" s="2" t="inlineStr">
+      <c r="B41" s="2" t="inlineStr">
         <is>
           <t>IV — Column Selection &amp; Persistence</t>
         </is>
       </c>
-      <c r="C40" s="2" t="inlineStr">
-        <is>
-          <t>Functional</t>
-        </is>
-      </c>
-      <c r="D40" s="2" t="inlineStr">
+      <c r="C41" s="2" t="inlineStr">
+        <is>
+          <t>Functional</t>
+        </is>
+      </c>
+      <c r="D41" s="2" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="E40" s="2" t="inlineStr">
+      <c r="E41" s="2" t="inlineStr">
         <is>
           <t>1. You are signed in to the ShopView App on a desktop browser.
 2. The Inventory Value report is open with rows loaded.</t>
         </is>
       </c>
-      <c r="F40" s="2" t="inlineStr">
+      <c r="F41" s="2" t="inlineStr">
         <is>
           <t>1. Hover the column-selection icon button in the toolbar and read its tooltip.
 2. Open the control and toggle a column off, then on again, watching the table.
 3. Look for a way to turn the Total Cost column off.</t>
         </is>
       </c>
-      <c r="G40" s="2" t="inlineStr">
+      <c r="G41" s="2" t="inlineStr">
         <is>
           <t>1. The icon button's tooltip reads "Column Selection".
 2. Toggling a column off hides it from the table; toggling it on shows it again.
 3. The Total Cost column is always shown and cannot be turned off.</t>
         </is>
       </c>
-      <c r="H40" s="2" t="inlineStr">
+      <c r="H41" s="2" t="inlineStr">
         <is>
           <t>specs/inventory-value.md Story 8 S8-R1; S8-R2</t>
         </is>
       </c>
-      <c r="I40" s="2" t="inlineStr"/>
-      <c r="J40" s="2" t="inlineStr"/>
-    </row>
-    <row r="41">
-      <c r="A41" s="2" t="inlineStr">
+      <c r="I41" s="2" t="inlineStr"/>
+      <c r="J41" s="2" t="inlineStr"/>
+    </row>
+    <row r="42">
+      <c r="A42" s="2" t="inlineStr">
         <is>
           <t>Toggling columns never reorders them — the fixed order is kept with Total Cost always last</t>
         </is>
       </c>
-      <c r="B41" s="2" t="inlineStr">
+      <c r="B42" s="2" t="inlineStr">
         <is>
           <t>IV — Column Selection &amp; Persistence</t>
         </is>
       </c>
-      <c r="C41" s="2" t="inlineStr">
-        <is>
-          <t>Functional</t>
-        </is>
-      </c>
-      <c r="D41" s="2" t="inlineStr">
+      <c r="C42" s="2" t="inlineStr">
+        <is>
+          <t>Functional</t>
+        </is>
+      </c>
+      <c r="D42" s="2" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="E41" s="2" t="inlineStr">
+      <c r="E42" s="2" t="inlineStr">
         <is>
           <t>1. You are signed in to the ShopView App on a desktop browser.
 2. The Inventory Value report is open with rows loaded.</t>
         </is>
       </c>
-      <c r="F41" s="2" t="inlineStr">
+      <c r="F42" s="2" t="inlineStr">
         <is>
           <t>1. Turn several columns on and off in different orders (for example, turn on Total Sell, then Margin).
 2. Read the resulting column order after each change.</t>
         </is>
       </c>
-      <c r="G41" s="2" t="inlineStr">
+      <c r="G42" s="2" t="inlineStr">
         <is>
           <t>1. Whatever columns are shown, they appear in the fixed left-to-right order (Part #, Description, Category, Vendor, Qty on Hand, Unit Cost, Unit Sell, Margin, Margin %, Total Sell, Total Cost) — toggling visibility never reorders columns.
 2. Total Cost is always the last column.</t>
         </is>
       </c>
-      <c r="H41" s="2" t="inlineStr">
+      <c r="H42" s="2" t="inlineStr">
         <is>
           <t>specs/inventory-value.md Story 8 S8-R4; Story 3 S3-R1</t>
         </is>
       </c>
-      <c r="I41" s="2" t="inlineStr"/>
-      <c r="J41" s="2" t="inlineStr"/>
-    </row>
-    <row r="42">
-      <c r="A42" s="2" t="inlineStr">
+      <c r="I42" s="2" t="inlineStr"/>
+      <c r="J42" s="2" t="inlineStr"/>
+    </row>
+    <row r="43">
+      <c r="A43" s="2" t="inlineStr">
         <is>
           <t>The report remembers the date range, category, vendor, part search text, location, columns, and sort per browser and restores them on return</t>
         </is>
       </c>
-      <c r="B42" s="2" t="inlineStr">
+      <c r="B43" s="2" t="inlineStr">
         <is>
           <t>IV — Column Selection &amp; Persistence</t>
         </is>
       </c>
-      <c r="C42" s="2" t="inlineStr">
-        <is>
-          <t>Functional</t>
-        </is>
-      </c>
-      <c r="D42" s="2" t="inlineStr">
+      <c r="C43" s="2" t="inlineStr">
+        <is>
+          <t>Functional</t>
+        </is>
+      </c>
+      <c r="D43" s="2" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="E42" s="2" t="inlineStr">
+      <c r="E43" s="2" t="inlineStr">
         <is>
           <t>1. You are signed in to the ShopView App on a desktop browser.
 2. The Inventory Value report is open.</t>
         </is>
       </c>
-      <c r="F42" s="2" t="inlineStr">
+      <c r="F43" s="2" t="inlineStr">
         <is>
           <t>1. Change the date range, select a category and a vendor, type a part search, change the location selection, change the column selection, and sort by a non-default column.
 2. Navigate away to another screen, then return to the report.
@@ -2467,142 +2517,142 @@
 4. If practical, open the report in a different browser (or private window) and read its settings.</t>
         </is>
       </c>
-      <c r="G42" s="2" t="inlineStr">
+      <c r="G43" s="2" t="inlineStr">
         <is>
           <t>1. On return and after a reload, the report restores the saved date range, category selection, vendor selection, part search text, location selection, column selection, and sort.
 2. In a different browser the report shows the defaults instead — persistence is per browser, not tied to the user's account.</t>
         </is>
       </c>
-      <c r="H42" s="2" t="inlineStr">
+      <c r="H43" s="2" t="inlineStr">
         <is>
           <t>specs/inventory-value.md Story 8 S8-R5 (+ context note); Story 9 S9-R5</t>
         </is>
       </c>
-      <c r="I42" s="2" t="inlineStr"/>
-      <c r="J42" s="2" t="inlineStr"/>
-    </row>
-    <row r="43">
-      <c r="A43" s="2" t="inlineStr">
+      <c r="I43" s="2" t="inlineStr"/>
+      <c r="J43" s="2" t="inlineStr"/>
+    </row>
+    <row r="44">
+      <c r="A44" s="2" t="inlineStr">
         <is>
           <t>Defensive restore: a stale saved category or vendor is dropped on load</t>
         </is>
       </c>
-      <c r="B43" s="2" t="inlineStr">
+      <c r="B44" s="2" t="inlineStr">
         <is>
           <t>IV — Column Selection &amp; Persistence</t>
         </is>
       </c>
-      <c r="C43" s="2" t="inlineStr">
+      <c r="C44" s="2" t="inlineStr">
         <is>
           <t>Negative</t>
         </is>
       </c>
-      <c r="D43" s="2" t="inlineStr">
+      <c r="D44" s="2" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="E43" s="2" t="inlineStr">
+      <c r="E44" s="2" t="inlineStr">
         <is>
           <t>1. You are signed in to the ShopView App on a desktop browser.
 2. The report has saved settings in this browser, including a category or vendor selection that can be made stale (for example, the last in-stock part of a saved category is consumed so the category disappears from the data).</t>
         </is>
       </c>
-      <c r="F43" s="2" t="inlineStr">
+      <c r="F44" s="2" t="inlineStr">
         <is>
           <t>1. Make the saved category or vendor no longer present in the data.
 2. Open the Inventory Value report.</t>
         </is>
       </c>
-      <c r="G43" s="2" t="inlineStr">
+      <c r="G44" s="2" t="inlineStr">
         <is>
           <t>1. The report loads normally — the saved category or vendor that is no longer present in the data is dropped from the selection instead of breaking the view (the defensive-restore rule applied to the path these steps drive).
 2. All other saved settings are still restored.</t>
         </is>
       </c>
-      <c r="H43" s="2" t="inlineStr">
+      <c r="H44" s="2" t="inlineStr">
         <is>
           <t>specs/inventory-value.md Story 8 S8-R6</t>
         </is>
       </c>
-      <c r="I43" s="2" t="inlineStr"/>
-      <c r="J43" s="2" t="inlineStr"/>
-    </row>
-    <row r="44">
-      <c r="A44" s="2" t="inlineStr">
+      <c r="I44" s="2" t="inlineStr"/>
+      <c r="J44" s="2" t="inlineStr"/>
+    </row>
+    <row r="45">
+      <c r="A45" s="2" t="inlineStr">
         <is>
           <t>On first load and after any reload, rows are sorted by Total Cost, highest first, applied by the server</t>
         </is>
       </c>
-      <c r="B44" s="2" t="inlineStr">
+      <c r="B45" s="2" t="inlineStr">
         <is>
           <t>IV — Sorting</t>
         </is>
       </c>
-      <c r="C44" s="2" t="inlineStr">
-        <is>
-          <t>Functional</t>
-        </is>
-      </c>
-      <c r="D44" s="2" t="inlineStr">
+      <c r="C45" s="2" t="inlineStr">
+        <is>
+          <t>Functional</t>
+        </is>
+      </c>
+      <c r="D45" s="2" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="E44" s="2" t="inlineStr">
+      <c r="E45" s="2" t="inlineStr">
         <is>
           <t>1. You are signed in to the ShopView App on a desktop browser that has no saved sort for this report (fresh visit).
 2. In-stock parts with a spread of Total Cost values exist, spanning more than one page.</t>
         </is>
       </c>
-      <c r="F44" s="2" t="inlineStr">
+      <c r="F45" s="2" t="inlineStr">
         <is>
           <t>1. Open the Inventory Value report without clicking any header.
 2. Read the Total Cost values from the top row down, across page 1 and page 2.</t>
         </is>
       </c>
-      <c r="G44" s="2" t="inlineStr">
+      <c r="G45" s="2" t="inlineStr">
         <is>
           <t>1. The rows are sorted by Total Cost, highest first (descending).
 2. The order holds across pages (page 2 continues below page 1's lowest value) — the server applies the default order over the full set.</t>
         </is>
       </c>
-      <c r="H44" s="2" t="inlineStr">
+      <c r="H45" s="2" t="inlineStr">
         <is>
           <t>specs/inventory-value.md Story 9 S9-R1; §3 Key Decisions (Total Cost default sort)</t>
         </is>
       </c>
-      <c r="I44" s="2" t="inlineStr"/>
-      <c r="J44" s="2" t="inlineStr"/>
-    </row>
-    <row r="45">
-      <c r="A45" s="2" t="inlineStr">
+      <c r="I45" s="2" t="inlineStr"/>
+      <c r="J45" s="2" t="inlineStr"/>
+    </row>
+    <row r="46">
+      <c r="A46" s="2" t="inlineStr">
         <is>
           <t>Header clicks sort ascending then descending with no third state, re-fetching from the server and returning the first page</t>
         </is>
       </c>
-      <c r="B45" s="2" t="inlineStr">
+      <c r="B46" s="2" t="inlineStr">
         <is>
           <t>IV — Sorting</t>
         </is>
       </c>
-      <c r="C45" s="2" t="inlineStr">
-        <is>
-          <t>Functional</t>
-        </is>
-      </c>
-      <c r="D45" s="2" t="inlineStr">
+      <c r="C46" s="2" t="inlineStr">
+        <is>
+          <t>Functional</t>
+        </is>
+      </c>
+      <c r="D46" s="2" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="E45" s="2" t="inlineStr">
+      <c r="E46" s="2" t="inlineStr">
         <is>
           <t>1. You are signed in to the ShopView App on a desktop browser.
 2. The result set spans more than one page.</t>
         </is>
       </c>
-      <c r="F45" s="2" t="inlineStr">
+      <c r="F46" s="2" t="inlineStr">
         <is>
           <t>1. From page 2, click the Part # column header and note the order and the page shown.
 2. Click the same header again and note the order.
@@ -2610,192 +2660,192 @@
 4. Click a different column header and check whether the previous sort still applies.</t>
         </is>
       </c>
-      <c r="G45" s="2" t="inlineStr">
+      <c r="G46" s="2" t="inlineStr">
         <is>
           <t>1. Clicking a column that is not the active sort sorts it ascending; clicking the active sort column again toggles it to descending; there is no third "cleared" state.
 2. Each header click re-fetches the data from the server ordered by the chosen column and direction, returning the FIRST page of the re-sorted result set.
 3. Only one column sorts at a time.</t>
         </is>
       </c>
-      <c r="H45" s="2" t="inlineStr">
+      <c r="H46" s="2" t="inlineStr">
         <is>
           <t>specs/inventory-value.md Story 9 S9-R2</t>
         </is>
       </c>
-      <c r="I45" s="2" t="inlineStr"/>
-      <c r="J45" s="2" t="inlineStr"/>
-    </row>
-    <row r="46">
-      <c r="A46" s="2" t="inlineStr">
+      <c r="I46" s="2" t="inlineStr"/>
+      <c r="J46" s="2" t="inlineStr"/>
+    </row>
+    <row r="47">
+      <c r="A47" s="2" t="inlineStr">
         <is>
           <t>Money and numeric columns sort by value; text columns sort as text, case-insensitively</t>
         </is>
       </c>
-      <c r="B46" s="2" t="inlineStr">
+      <c r="B47" s="2" t="inlineStr">
         <is>
           <t>IV — Sorting</t>
         </is>
       </c>
-      <c r="C46" s="2" t="inlineStr">
-        <is>
-          <t>Functional</t>
-        </is>
-      </c>
-      <c r="D46" s="2" t="inlineStr">
+      <c r="C47" s="2" t="inlineStr">
+        <is>
+          <t>Functional</t>
+        </is>
+      </c>
+      <c r="D47" s="2" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="E46" s="2" t="inlineStr">
+      <c r="E47" s="2" t="inlineStr">
         <is>
           <t>1. You are signed in to the ShopView App on a desktop browser.
 2. In-stock parts exist with money values over and under $1,000 and with text values in mixed letter cases.</t>
         </is>
       </c>
-      <c r="F46" s="2" t="inlineStr">
+      <c r="F47" s="2" t="inlineStr">
         <is>
           <t>1. Sort by Total Cost and check the order of values like $900.00 vs $1,100.00.
 2. Sort by Qty on Hand and check the numeric order.
 3. Sort by Description (or Vendor) and check how differently-cased values order.</t>
         </is>
       </c>
-      <c r="G46" s="2" t="inlineStr">
+      <c r="G47" s="2" t="inlineStr">
         <is>
           <t>1. Money and numeric columns sort by their underlying value (so $1,100.00 is treated as more than $900.00, not compared as text).
 2. Text columns (Part #, Description, Category, Vendor) sort as text, case-insensitively ("apple" and "Apple" sort together).</t>
         </is>
       </c>
-      <c r="H46" s="2" t="inlineStr">
+      <c r="H47" s="2" t="inlineStr">
         <is>
           <t>specs/inventory-value.md Story 9 S9-R3</t>
         </is>
       </c>
-      <c r="I46" s="2" t="inlineStr"/>
-      <c r="J46" s="2" t="inlineStr"/>
-    </row>
-    <row r="47">
-      <c r="A47" s="2" t="inlineStr">
+      <c r="I47" s="2" t="inlineStr"/>
+      <c r="J47" s="2" t="inlineStr"/>
+    </row>
+    <row r="48">
+      <c r="A48" s="2" t="inlineStr">
         <is>
           <t>Sorting reorders only the data rows — the totals row stays at the bottom — and the chosen sort is remembered per browser</t>
         </is>
       </c>
-      <c r="B47" s="2" t="inlineStr">
+      <c r="B48" s="2" t="inlineStr">
         <is>
           <t>IV — Sorting</t>
         </is>
       </c>
-      <c r="C47" s="2" t="inlineStr">
-        <is>
-          <t>Functional</t>
-        </is>
-      </c>
-      <c r="D47" s="2" t="inlineStr">
+      <c r="C48" s="2" t="inlineStr">
+        <is>
+          <t>Functional</t>
+        </is>
+      </c>
+      <c r="D48" s="2" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="E47" s="2" t="inlineStr">
+      <c r="E48" s="2" t="inlineStr">
         <is>
           <t>1. You are signed in to the ShopView App on a desktop browser.
 2. The Inventory Value report is open with rows and a totals row.</t>
         </is>
       </c>
-      <c r="F47" s="2" t="inlineStr">
+      <c r="F48" s="2" t="inlineStr">
         <is>
           <t>1. Sort by any column and watch the totals row's position.
 2. Sort by a non-default column, leave the report, and return.</t>
         </is>
       </c>
-      <c r="G47" s="2" t="inlineStr">
+      <c r="G48" s="2" t="inlineStr">
         <is>
           <t>1. Sorting reorders the data rows only; the totals row stays at the bottom.
 2. On return, the report restores the chosen sort (remembered per browser, Story 8).</t>
         </is>
       </c>
-      <c r="H47" s="2" t="inlineStr">
+      <c r="H48" s="2" t="inlineStr">
         <is>
           <t>specs/inventory-value.md Story 9 S9-R4; S9-R5</t>
         </is>
       </c>
-      <c r="I47" s="2" t="inlineStr"/>
-      <c r="J47" s="2" t="inlineStr"/>
-    </row>
-    <row r="48">
-      <c r="A48" s="2" t="inlineStr">
+      <c r="I48" s="2" t="inlineStr"/>
+      <c r="J48" s="2" t="inlineStr"/>
+    </row>
+    <row r="49">
+      <c r="A49" s="2" t="inlineStr">
         <is>
           <t>A three-dot toolbar menu holds "Download (PDF)" and "Download (CSV)"</t>
         </is>
       </c>
-      <c r="B48" s="2" t="inlineStr">
+      <c r="B49" s="2" t="inlineStr">
         <is>
           <t>IV — Exports</t>
         </is>
       </c>
-      <c r="C48" s="2" t="inlineStr">
-        <is>
-          <t>Functional</t>
-        </is>
-      </c>
-      <c r="D48" s="2" t="inlineStr">
+      <c r="C49" s="2" t="inlineStr">
+        <is>
+          <t>Functional</t>
+        </is>
+      </c>
+      <c r="D49" s="2" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="E48" s="2" t="inlineStr">
+      <c r="E49" s="2" t="inlineStr">
         <is>
           <t>1. You are signed in to the ShopView App on a desktop browser.
 2. The Inventory Value report is open with rows loaded.</t>
         </is>
       </c>
-      <c r="F48" s="2" t="inlineStr">
+      <c r="F49" s="2" t="inlineStr">
         <is>
           <t>1. Find and open the three-dot button in the toolbar.
 2. Read the menu options.
 3. Choose "Download (PDF)", then repeat with "Download (CSV)".</t>
         </is>
       </c>
-      <c r="G48" s="2" t="inlineStr">
+      <c r="G49" s="2" t="inlineStr">
         <is>
           <t>1. The menu holds an option labeled "Download (PDF)" and an option labeled "Download (CSV)".
 2. Each option downloads a file of the current view in the chosen format.</t>
         </is>
       </c>
-      <c r="H48" s="2" t="inlineStr">
+      <c r="H49" s="2" t="inlineStr">
         <is>
           <t>specs/inventory-value.md Story 10 S10-R1; S10-R2</t>
         </is>
       </c>
-      <c r="I48" s="2" t="inlineStr"/>
-      <c r="J48" s="2" t="inlineStr"/>
-    </row>
-    <row r="49">
-      <c r="A49" s="2" t="inlineStr">
+      <c r="I49" s="2" t="inlineStr"/>
+      <c r="J49" s="2" t="inlineStr"/>
+    </row>
+    <row r="50">
+      <c r="A50" s="2" t="inlineStr">
         <is>
           <t>Downloads keep shown columns and order, honor filters, and include Totals</t>
         </is>
       </c>
-      <c r="B49" s="2" t="inlineStr">
+      <c r="B50" s="2" t="inlineStr">
         <is>
           <t>IV — Exports</t>
         </is>
       </c>
-      <c r="C49" s="2" t="inlineStr">
-        <is>
-          <t>Functional</t>
-        </is>
-      </c>
-      <c r="D49" s="2" t="inlineStr">
+      <c r="C50" s="2" t="inlineStr">
+        <is>
+          <t>Functional</t>
+        </is>
+      </c>
+      <c r="D50" s="2" t="inlineStr">
         <is>
           <t>Critical</t>
         </is>
       </c>
-      <c r="E49" s="2" t="inlineStr">
+      <c r="E50" s="2" t="inlineStr">
         <is>
           <t>1. You are signed in to the ShopView App on a desktop browser.
 2. The report is open with a non-default column selection, a Category or Vendor filter, a part search, and a non-default sort applied.</t>
         </is>
       </c>
-      <c r="F49" s="2" t="inlineStr">
+      <c r="F50" s="2" t="inlineStr">
         <is>
           <t>1. Download the current view as a CSV and open it.
 2. Compare its columns and their order to the screen.
@@ -2804,7 +2854,7 @@
 5. Repeat the checks in the PDF.</t>
         </is>
       </c>
-      <c r="G49" s="2" t="inlineStr">
+      <c r="G50" s="2" t="inlineStr">
         <is>
           <t>1. Both downloads include only the columns currently shown, in the same left-to-right order as the screen, with Total Cost last.
 2. Both downloads honor the current date, category, vendor, location, and part-search filters, and apply the current sort.
@@ -2812,91 +2862,91 @@
 4. Each download (PDF and CSV) carries a "Locations:" line naming the location(s) the report was scoped to (exact position in the file is confirmed in the build).</t>
         </is>
       </c>
-      <c r="H49" s="2" t="inlineStr">
+      <c r="H50" s="2" t="inlineStr">
         <is>
           <t>SV-8677 (specs/inventory-value.md Story 10 S10-R3; S10-R4; S10-R5; S10-R6 + Locations: line in every CSV/PDF export per Chris Ward group message 2026-07-29 (chris-update-2026-07-29/chris-message-2026-07-29.md; NEWEST source, last-update-wins))</t>
         </is>
       </c>
-      <c r="I49" s="2" t="inlineStr"/>
-      <c r="J49" s="2" t="inlineStr"/>
-    </row>
-    <row r="50">
-      <c r="A50" s="2" t="inlineStr">
+      <c r="I50" s="2" t="inlineStr"/>
+      <c r="J50" s="2" t="inlineStr"/>
+    </row>
+    <row r="51">
+      <c r="A51" s="2" t="inlineStr">
         <is>
           <t>Export number formats: two-decimal money, one-decimal Margin % ("—" when undefined); CSV money as plain numbers, PDF with on-screen currency formatting</t>
         </is>
       </c>
-      <c r="B50" s="2" t="inlineStr">
+      <c r="B51" s="2" t="inlineStr">
         <is>
           <t>IV — Exports</t>
         </is>
       </c>
-      <c r="C50" s="2" t="inlineStr">
-        <is>
-          <t>Functional</t>
-        </is>
-      </c>
-      <c r="D50" s="2" t="inlineStr">
+      <c r="C51" s="2" t="inlineStr">
+        <is>
+          <t>Functional</t>
+        </is>
+      </c>
+      <c r="D51" s="2" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="E50" s="2" t="inlineStr">
+      <c r="E51" s="2" t="inlineStr">
         <is>
           <t>1. You are signed in to the ShopView App on a desktop browser.
 2. The current view includes money values over $1,000 and, if producible, a part whose Margin % is undefined ("—").</t>
         </is>
       </c>
-      <c r="F50" s="2" t="inlineStr">
+      <c r="F51" s="2" t="inlineStr">
         <is>
           <t>1. Download the CSV and open it in a plain-text editor; read the money and Margin % values.
 2. Download the PDF and read the same values.</t>
         </is>
       </c>
-      <c r="G50" s="2" t="inlineStr">
+      <c r="G51" s="2" t="inlineStr">
         <is>
           <t>1. Money uses two decimals and Margin % one decimal in both files; an undefined Margin % shows "—".
 2. In the CSV, money values are written as plain numbers with two decimals and NO thousands separators (so they parse cleanly in a spreadsheet).
 3. The PDF uses the same on-screen currency formatting with the "$" and thousands separators.</t>
         </is>
       </c>
-      <c r="H50" s="2" t="inlineStr">
+      <c r="H51" s="2" t="inlineStr">
         <is>
           <t>specs/inventory-value.md Story 10 S10-R7 (+ context note)</t>
         </is>
       </c>
-      <c r="I50" s="2" t="inlineStr"/>
-      <c r="J50" s="2" t="inlineStr"/>
-    </row>
-    <row r="51">
-      <c r="A51" s="2" t="inlineStr">
+      <c r="I51" s="2" t="inlineStr"/>
+      <c r="J51" s="2" t="inlineStr"/>
+    </row>
+    <row r="52">
+      <c r="A52" s="2" t="inlineStr">
         <is>
           <t>The PDF header shows the report name, organization, selected period, and an "as of" line; the shop logo shows when set and the CSV never has one</t>
         </is>
       </c>
-      <c r="B51" s="2" t="inlineStr">
+      <c r="B52" s="2" t="inlineStr">
         <is>
           <t>IV — Exports</t>
         </is>
       </c>
-      <c r="C51" s="2" t="inlineStr">
-        <is>
-          <t>Functional</t>
-        </is>
-      </c>
-      <c r="D51" s="2" t="inlineStr">
+      <c r="C52" s="2" t="inlineStr">
+        <is>
+          <t>Functional</t>
+        </is>
+      </c>
+      <c r="D52" s="2" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="E51" s="2" t="inlineStr">
+      <c r="E52" s="2" t="inlineStr">
         <is>
           <t>1. You are signed in to the ShopView App on a desktop browser.
 2. The shop has a logo set in its settings.
 3. The report is open on a view whose displayed day is known (live today, or a recorded past day).</t>
         </is>
       </c>
-      <c r="F51" s="2" t="inlineStr">
+      <c r="F52" s="2" t="inlineStr">
         <is>
           <t>1. Download the PDF and read its header.
 2. Look at the top of the PDF for the shop logo.
@@ -2904,678 +2954,678 @@
 4. If reachable, repeat the PDF download on a period with no available snapshot and read the header's as-of line.</t>
         </is>
       </c>
-      <c r="G51" s="2" t="inlineStr">
+      <c r="G52" s="2" t="inlineStr">
         <is>
           <t>1. The PDF header shows the report name "Inventory Value", the organization name, the selected period, and an "as of" line naming the day the values represent (or a message that no snapshot is available for the period).
 2. The PDF shows the shop logo at the top when one is set.
 3. The CSV never includes a logo.</t>
         </is>
       </c>
-      <c r="H51" s="2" t="inlineStr">
+      <c r="H52" s="2" t="inlineStr">
         <is>
           <t>specs/inventory-value.md Story 10 S10-R8; S10-R9</t>
         </is>
       </c>
-      <c r="I51" s="2" t="inlineStr"/>
-      <c r="J51" s="2" t="inlineStr"/>
-    </row>
-    <row r="52">
-      <c r="A52" s="2" t="inlineStr">
+      <c r="I52" s="2" t="inlineStr"/>
+      <c r="J52" s="2" t="inlineStr"/>
+    </row>
+    <row r="53">
+      <c r="A53" s="2" t="inlineStr">
         <is>
           <t>The downloaded files are named "inventory-value-report.pdf" and "inventory-value-report.csv"</t>
         </is>
       </c>
-      <c r="B52" s="2" t="inlineStr">
+      <c r="B53" s="2" t="inlineStr">
         <is>
           <t>IV — Exports</t>
         </is>
       </c>
-      <c r="C52" s="2" t="inlineStr">
-        <is>
-          <t>Functional</t>
-        </is>
-      </c>
-      <c r="D52" s="2" t="inlineStr">
+      <c r="C53" s="2" t="inlineStr">
+        <is>
+          <t>Functional</t>
+        </is>
+      </c>
+      <c r="D53" s="2" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="E52" s="2" t="inlineStr">
+      <c r="E53" s="2" t="inlineStr">
         <is>
           <t>1. You are signed in to the ShopView App on a desktop browser.
 2. The Inventory Value report is open with rows loaded.</t>
         </is>
       </c>
-      <c r="F52" s="2" t="inlineStr">
+      <c r="F53" s="2" t="inlineStr">
         <is>
           <t>1. Download the current view as a PDF and read the saved file's name.
 2. Download the current view as a CSV and read the saved file's name.</t>
         </is>
       </c>
-      <c r="G52" s="2" t="inlineStr">
+      <c r="G53" s="2" t="inlineStr">
         <is>
           <t>1. The PDF is named "inventory-value-report.pdf".
 2. The CSV is named "inventory-value-report.csv".</t>
         </is>
       </c>
-      <c r="H52" s="2" t="inlineStr">
+      <c r="H53" s="2" t="inlineStr">
         <is>
           <t>specs/inventory-value.md Story 10 S10-R10</t>
         </is>
       </c>
-      <c r="I52" s="2" t="inlineStr"/>
-      <c r="J52" s="2" t="inlineStr"/>
-    </row>
-    <row r="53">
-      <c r="A53" s="2" t="inlineStr">
+      <c r="I53" s="2" t="inlineStr"/>
+      <c r="J53" s="2" t="inlineStr"/>
+    </row>
+    <row r="54">
+      <c r="A54" s="2" t="inlineStr">
         <is>
           <t>Exports are generated server-side over the full filtered set — rows beyond the loaded page are included</t>
         </is>
       </c>
-      <c r="B53" s="2" t="inlineStr">
+      <c r="B54" s="2" t="inlineStr">
         <is>
           <t>IV — Exports</t>
         </is>
       </c>
-      <c r="C53" s="2" t="inlineStr">
-        <is>
-          <t>Functional</t>
-        </is>
-      </c>
-      <c r="D53" s="2" t="inlineStr">
+      <c r="C54" s="2" t="inlineStr">
+        <is>
+          <t>Functional</t>
+        </is>
+      </c>
+      <c r="D54" s="2" t="inlineStr">
         <is>
           <t>Critical</t>
         </is>
       </c>
-      <c r="E53" s="2" t="inlineStr">
+      <c r="E54" s="2" t="inlineStr">
         <is>
           <t>1. You are signed in to the ShopView App on a desktop browser.
 2. The current filtered set spans more than one page (but stays under the export row cap).</t>
         </is>
       </c>
-      <c r="F53" s="2" t="inlineStr">
+      <c r="F54" s="2" t="inlineStr">
         <is>
           <t>1. From page 1, without visiting the later pages, download the CSV.
 2. Count the file's data rows and look for parts you know sit on the later pages.
 3. Compare the file's totals row to the on-screen totals.</t>
         </is>
       </c>
-      <c r="G53" s="2" t="inlineStr">
+      <c r="G54" s="2" t="inlineStr">
         <is>
           <t>1. The export contains the FULL filtered set — every qualifying row across all pages, not only the rows loaded in the browser.
 2. Parts from the later pages are present.
 3. The export is generated server-side against the current filters, part search, and sort — it is not built from the rows currently in the browser.</t>
         </is>
       </c>
-      <c r="H53" s="2" t="inlineStr">
+      <c r="H54" s="2" t="inlineStr">
         <is>
           <t>specs/inventory-value.md Story 10 S10-R11</t>
         </is>
       </c>
-      <c r="I53" s="2" t="inlineStr"/>
-      <c r="J53" s="2" t="inlineStr"/>
-    </row>
-    <row r="54">
-      <c r="A54" s="2" t="inlineStr">
-        <is>
-          <t>An over-cap filtered set produces no file and shows the too-large-to-export message (exact cap value pending owner confirmation)</t>
-        </is>
-      </c>
-      <c r="B54" s="2" t="inlineStr">
+      <c r="I54" s="2" t="inlineStr"/>
+      <c r="J54" s="2" t="inlineStr"/>
+    </row>
+    <row r="55">
+      <c r="A55" s="2" t="inlineStr">
+        <is>
+          <t>An over-cap filtered set produces no file and shows the too-large-to-export message</t>
+        </is>
+      </c>
+      <c r="B55" s="2" t="inlineStr">
         <is>
           <t>IV — Exports</t>
         </is>
       </c>
-      <c r="C54" s="2" t="inlineStr">
+      <c r="C55" s="2" t="inlineStr">
         <is>
           <t>Negative</t>
         </is>
       </c>
-      <c r="D54" s="2" t="inlineStr">
+      <c r="D55" s="2" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="E54" s="2" t="inlineStr">
+      <c r="E55" s="2" t="inlineStr">
         <is>
           <t>1. You are signed in to the ShopView App on a desktop browser.
 2. A filter/location combination exists whose filtered set EXCEEDS the export row cap (seed ZZAUTOTEST parts in bulk if needed, or use the largest available data set).</t>
         </is>
       </c>
-      <c r="F54" s="2" t="inlineStr">
+      <c r="F55" s="2" t="inlineStr">
         <is>
           <t>1. Set the filters so the filtered set exceeds the export row cap.
 2. Request "Download (PDF)" and read what happens.
 3. Request "Download (CSV)" and read what happens.</t>
         </is>
       </c>
-      <c r="G54" s="2" t="inlineStr">
+      <c r="G55" s="2" t="inlineStr">
         <is>
           <t>1. Neither the PDF nor the CSV is produced.
 2. The user sees the message: "This report is too large to export. Narrow the date range or filters, then try again." (a blocking notification; no file).
 3. After narrowing the filters below the cap, the download works again.</t>
         </is>
       </c>
-      <c r="H54" s="2" t="inlineStr">
+      <c r="H55" s="2" t="inlineStr">
         <is>
           <t>specs/inventory-value.md Story 10 S10-R12; §7 User Feedback Summary</t>
         </is>
       </c>
-      <c r="I54" s="2" t="inlineStr"/>
-      <c r="J54" s="2" t="inlineStr"/>
-    </row>
-    <row r="55">
-      <c r="A55" s="2" t="inlineStr">
+      <c r="I55" s="2" t="inlineStr"/>
+      <c r="J55" s="2" t="inlineStr"/>
+    </row>
+    <row r="56">
+      <c r="A56" s="2" t="inlineStr">
         <is>
           <t>Download notifications: verbatim success and failure texts per format</t>
         </is>
       </c>
-      <c r="B55" s="2" t="inlineStr">
+      <c r="B56" s="2" t="inlineStr">
         <is>
           <t>IV — Exports</t>
         </is>
       </c>
-      <c r="C55" s="2" t="inlineStr">
+      <c r="C56" s="2" t="inlineStr">
         <is>
           <t>Negative</t>
         </is>
       </c>
-      <c r="D55" s="2" t="inlineStr">
+      <c r="D56" s="2" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="E55" s="2" t="inlineStr">
+      <c r="E56" s="2" t="inlineStr">
         <is>
           <t>1. You are signed in to the ShopView App on a desktop browser.
 2. The Inventory Value report is open with rows loaded (under the export cap).
 3. A download failure can be simulated (for example, disconnect the network just before requesting the download).</t>
         </is>
       </c>
-      <c r="F55" s="2" t="inlineStr">
+      <c r="F56" s="2" t="inlineStr">
         <is>
           <t>1. Download the PDF and the CSV normally and read each notification.
 2. Simulate a failure and request the PDF download; read the notification.
 3. Repeat the failure for the CSV download.</t>
         </is>
       </c>
-      <c r="G55" s="2" t="inlineStr">
+      <c r="G56" s="2" t="inlineStr">
         <is>
           <t>1. Success notifications read verbatim: "Inventory Value report exported (PDF)" and "Inventory Value report exported (CSV)".
 2. Failure notifications read verbatim: "Failed to export inventory value report (pdf)" and "Failed to export inventory value report (csv)".
 3. The lower-case "(pdf)"/"(csv)" on failure vs the upper-case success ones is the documented spec wording — expected, not a bug.</t>
         </is>
       </c>
-      <c r="H55" s="2" t="inlineStr">
+      <c r="H56" s="2" t="inlineStr">
         <is>
           <t>specs/inventory-value.md Story 10 S10-R13; S10-R14; §7 User Feedback Summary</t>
         </is>
       </c>
-      <c r="I55" s="2" t="inlineStr"/>
-      <c r="J55" s="2" t="inlineStr"/>
-    </row>
-    <row r="56">
-      <c r="A56" s="2" t="inlineStr">
+      <c r="I56" s="2" t="inlineStr"/>
+      <c r="J56" s="2" t="inlineStr"/>
+    </row>
+    <row r="57">
+      <c r="A57" s="2" t="inlineStr">
         <is>
           <t>The report uses an all-white table with no alternating row shading on the standard soft blue-grey report backdrop</t>
         </is>
       </c>
-      <c r="B56" s="2" t="inlineStr">
+      <c r="B57" s="2" t="inlineStr">
         <is>
           <t>IV — Visual &amp; Accessibility</t>
         </is>
       </c>
-      <c r="C56" s="2" t="inlineStr">
-        <is>
-          <t>Functional</t>
-        </is>
-      </c>
-      <c r="D56" s="2" t="inlineStr">
+      <c r="C57" s="2" t="inlineStr">
+        <is>
+          <t>Functional</t>
+        </is>
+      </c>
+      <c r="D57" s="2" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="E56" s="2" t="inlineStr">
+      <c r="E57" s="2" t="inlineStr">
         <is>
           <t>1. You are signed in to the ShopView App on a desktop browser.
 2. The Inventory Value report is open with several rows.</t>
         </is>
       </c>
-      <c r="F56" s="2" t="inlineStr">
+      <c r="F57" s="2" t="inlineStr">
         <is>
           <t>1. Look at the column headers and the data cells.
 2. Compare the background of consecutive rows.
 3. Look at the page background around the table.</t>
         </is>
       </c>
-      <c r="G56" s="2" t="inlineStr">
+      <c r="G57" s="2" t="inlineStr">
         <is>
           <t>1. The table has white column headers and white data cells, with no alternating row shading.
 2. The table sits on the standard soft blue-grey report backdrop.</t>
         </is>
       </c>
-      <c r="H56" s="2" t="inlineStr">
+      <c r="H57" s="2" t="inlineStr">
         <is>
           <t>specs/inventory-value.md Story 12 S12-R1</t>
         </is>
       </c>
-      <c r="I56" s="2" t="inlineStr"/>
-      <c r="J56" s="2" t="inlineStr"/>
-    </row>
-    <row r="57">
-      <c r="A57" s="2" t="inlineStr">
+      <c r="I57" s="2" t="inlineStr"/>
+      <c r="J57" s="2" t="inlineStr"/>
+    </row>
+    <row r="58">
+      <c r="A58" s="2" t="inlineStr">
         <is>
           <t>Toolbar layout: three-dot menu leftmost in the action cluster then Column Selection; filters run date range, part search, Category, Vendor, Location</t>
         </is>
       </c>
-      <c r="B57" s="2" t="inlineStr">
+      <c r="B58" s="2" t="inlineStr">
         <is>
           <t>IV — Visual &amp; Accessibility</t>
         </is>
       </c>
-      <c r="C57" s="2" t="inlineStr">
-        <is>
-          <t>Functional</t>
-        </is>
-      </c>
-      <c r="D57" s="2" t="inlineStr">
+      <c r="C58" s="2" t="inlineStr">
+        <is>
+          <t>Functional</t>
+        </is>
+      </c>
+      <c r="D58" s="2" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="E57" s="2" t="inlineStr">
+      <c r="E58" s="2" t="inlineStr">
         <is>
           <t>1. You are signed in to the ShopView App on a desktop browser.
 2. The Inventory Value report is open.</t>
         </is>
       </c>
-      <c r="F57" s="2" t="inlineStr">
+      <c r="F58" s="2" t="inlineStr">
         <is>
           <t>1. Look at the toolbar's action cluster and read the order of its controls.
 2. Read the toolbar filters from left to right.</t>
         </is>
       </c>
-      <c r="G57" s="2" t="inlineStr">
+      <c r="G58" s="2" t="inlineStr">
         <is>
           <t>1. In the toolbar, the three-dot download menu sits leftmost in the action cluster, followed by the Column Selection control.
 2. The toolbar filters run, left to right: the date-range control, the part search, the Category filter, the Vendor filter, and the Location filter (rightmost).</t>
         </is>
       </c>
-      <c r="H57" s="2" t="inlineStr">
+      <c r="H58" s="2" t="inlineStr">
         <is>
           <t>specs/inventory-value.md Story 12 S12-R2; S12-R3</t>
         </is>
       </c>
-      <c r="I57" s="2" t="inlineStr"/>
-      <c r="J57" s="2" t="inlineStr"/>
-    </row>
-    <row r="58">
-      <c r="A58" s="2" t="inlineStr">
+      <c r="I58" s="2" t="inlineStr"/>
+      <c r="J58" s="2" t="inlineStr"/>
+    </row>
+    <row r="59">
+      <c r="A59" s="2" t="inlineStr">
         <is>
           <t>Long Description, Category, and Vendor values truncate with an ellipsis and show the full value on hover; the Part # is never truncated</t>
         </is>
       </c>
-      <c r="B58" s="2" t="inlineStr">
+      <c r="B59" s="2" t="inlineStr">
         <is>
           <t>IV — Visual &amp; Accessibility</t>
         </is>
       </c>
-      <c r="C58" s="2" t="inlineStr">
-        <is>
-          <t>Functional</t>
-        </is>
-      </c>
-      <c r="D58" s="2" t="inlineStr">
+      <c r="C59" s="2" t="inlineStr">
+        <is>
+          <t>Functional</t>
+        </is>
+      </c>
+      <c r="D59" s="2" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="E58" s="2" t="inlineStr">
+      <c r="E59" s="2" t="inlineStr">
         <is>
           <t>1. You are signed in to the ShopView App on a desktop browser.
 2. A ZZAUTOTEST part exists with a very long description (and, if possible, long category/vendor names) and a long part number.</t>
         </is>
       </c>
-      <c r="F58" s="2" t="inlineStr">
+      <c r="F59" s="2" t="inlineStr">
         <is>
           <t>1. Narrow the browser window (or turn on more columns) so the text columns overflow.
 2. Read the long Description, Category, and Vendor cells and hover each.
 3. Read the long Part # cell.</t>
         </is>
       </c>
-      <c r="G58" s="2" t="inlineStr">
+      <c r="G59" s="2" t="inlineStr">
         <is>
           <t>1. Long text values (Description, Category, Vendor) are truncated with an ellipsis when they overflow their column.
 2. The full value is available on hover.
 3. The Part # is never truncated.</t>
         </is>
       </c>
-      <c r="H58" s="2" t="inlineStr">
+      <c r="H59" s="2" t="inlineStr">
         <is>
           <t>specs/inventory-value.md Story 12 S12-R6</t>
         </is>
       </c>
-      <c r="I58" s="2" t="inlineStr"/>
-      <c r="J58" s="2" t="inlineStr"/>
-    </row>
-    <row r="59">
-      <c r="A59" s="2" t="inlineStr">
+      <c r="I59" s="2" t="inlineStr"/>
+      <c r="J59" s="2" t="inlineStr"/>
+    </row>
+    <row r="60">
+      <c r="A60" s="2" t="inlineStr">
         <is>
           <t>In dark mode the page background, toolbar, cells, and the "—" glyph remain legible</t>
         </is>
       </c>
-      <c r="B59" s="2" t="inlineStr">
+      <c r="B60" s="2" t="inlineStr">
         <is>
           <t>IV — Visual &amp; Accessibility</t>
         </is>
       </c>
-      <c r="C59" s="2" t="inlineStr">
+      <c r="C60" s="2" t="inlineStr">
         <is>
           <t>Accessibility</t>
         </is>
       </c>
-      <c r="D59" s="2" t="inlineStr">
+      <c r="D60" s="2" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="E59" s="2" t="inlineStr">
+      <c r="E60" s="2" t="inlineStr">
         <is>
           <t>1. You are signed in to the ShopView App on a desktop browser.
 2. The application is switched to dark mode.
 3. The report shows rows including a part with an em-dash ("—") Category or Vendor cell.</t>
         </is>
       </c>
-      <c r="F59" s="2" t="inlineStr">
+      <c r="F60" s="2" t="inlineStr">
         <is>
           <t>1. Read the page background, toolbar, and table cells in dark mode.
 2. Find a "—" cell and check its legibility.</t>
         </is>
       </c>
-      <c r="G59" s="2" t="inlineStr">
+      <c r="G60" s="2" t="inlineStr">
         <is>
           <t>1. The report supports dark mode.
 2. The page background, toolbar, cells, and the "—" glyph all use dark-mode-legible colors.</t>
         </is>
       </c>
-      <c r="H59" s="2" t="inlineStr">
+      <c r="H60" s="2" t="inlineStr">
         <is>
           <t>specs/inventory-value.md Story 12 S12-R7</t>
         </is>
       </c>
-      <c r="I59" s="2" t="inlineStr"/>
-      <c r="J59" s="2" t="inlineStr"/>
-    </row>
-    <row r="60">
-      <c r="A60" s="2" t="inlineStr">
+      <c r="I60" s="2" t="inlineStr"/>
+      <c r="J60" s="2" t="inlineStr"/>
+    </row>
+    <row r="61">
+      <c r="A61" s="2" t="inlineStr">
         <is>
           <t>Each sortable column header exposes its sort state to assistive technology and shows the active direction visually</t>
         </is>
       </c>
-      <c r="B60" s="2" t="inlineStr">
+      <c r="B61" s="2" t="inlineStr">
         <is>
           <t>IV — Visual &amp; Accessibility</t>
         </is>
       </c>
-      <c r="C60" s="2" t="inlineStr">
+      <c r="C61" s="2" t="inlineStr">
         <is>
           <t>Accessibility</t>
         </is>
       </c>
-      <c r="D60" s="2" t="inlineStr">
+      <c r="D61" s="2" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="E60" s="2" t="inlineStr">
+      <c r="E61" s="2" t="inlineStr">
         <is>
           <t>1. You are signed in to the ShopView App on a desktop browser.
 2. A screen reader or the browser's accessibility inspector is available.
 3. The Inventory Value report is open with rows loaded.</t>
         </is>
       </c>
-      <c r="F60" s="2" t="inlineStr">
+      <c r="F61" s="2" t="inlineStr">
         <is>
           <t>1. Sort by a column and look at its header for a visual direction indicator.
 2. With the accessibility inspector or screen reader, check what sort state the header exposes.
 3. Toggle the direction and check both again.</t>
         </is>
       </c>
-      <c r="G60" s="2" t="inlineStr">
+      <c r="G61" s="2" t="inlineStr">
         <is>
           <t>1. The active sort direction is indicated visually on the header.
 2. Each sortable column header exposes its sort state to assistive technology (for example, ascending/descending/none).
 3. The exposed state updates when the direction toggles.</t>
         </is>
       </c>
-      <c r="H60" s="2" t="inlineStr">
+      <c r="H61" s="2" t="inlineStr">
         <is>
           <t>specs/inventory-value.md Story 12 S12-R8</t>
         </is>
       </c>
-      <c r="I60" s="2" t="inlineStr"/>
-      <c r="J60" s="2" t="inlineStr"/>
-    </row>
-    <row r="61">
-      <c r="A61" s="2" t="inlineStr">
+      <c r="I61" s="2" t="inlineStr"/>
+      <c r="J61" s="2" t="inlineStr"/>
+    </row>
+    <row r="62">
+      <c r="A62" s="2" t="inlineStr">
         <is>
           <t>The icon-only controls (three-dot download button and Column Selection button) each carry an accessible name</t>
         </is>
       </c>
-      <c r="B61" s="2" t="inlineStr">
+      <c r="B62" s="2" t="inlineStr">
         <is>
           <t>IV — Visual &amp; Accessibility</t>
         </is>
       </c>
-      <c r="C61" s="2" t="inlineStr">
+      <c r="C62" s="2" t="inlineStr">
         <is>
           <t>Accessibility</t>
         </is>
       </c>
-      <c r="D61" s="2" t="inlineStr">
+      <c r="D62" s="2" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="E61" s="2" t="inlineStr">
+      <c r="E62" s="2" t="inlineStr">
         <is>
           <t>1. You are signed in to the ShopView App on a desktop browser.
 2. A screen reader or the browser's accessibility inspector is available.
 3. The Inventory Value report is open.</t>
         </is>
       </c>
-      <c r="F61" s="2" t="inlineStr">
+      <c r="F62" s="2" t="inlineStr">
         <is>
           <t>1. Inspect the three-dot download button's accessible name.
 2. Inspect the Column Selection button's accessible name.</t>
         </is>
       </c>
-      <c r="G61" s="2" t="inlineStr">
+      <c r="G62" s="2" t="inlineStr">
         <is>
           <t>1. Each icon-only control carries an accessible name exposed to assistive technology (it is not announced as an unnamed button).</t>
         </is>
       </c>
-      <c r="H61" s="2" t="inlineStr">
+      <c r="H62" s="2" t="inlineStr">
         <is>
           <t>specs/inventory-value.md Story 12 S12-R9</t>
         </is>
       </c>
-      <c r="I61" s="2" t="inlineStr"/>
-      <c r="J61" s="2" t="inlineStr"/>
-    </row>
-    <row r="62">
-      <c r="A62" s="2" t="inlineStr">
+      <c r="I62" s="2" t="inlineStr"/>
+      <c r="J62" s="2" t="inlineStr"/>
+    </row>
+    <row r="63">
+      <c r="A63" s="2" t="inlineStr">
         <is>
           <t>A user with the existing inventory-reports permission can open the report — no new permission is added</t>
         </is>
       </c>
-      <c r="B62" s="2" t="inlineStr">
+      <c r="B63" s="2" t="inlineStr">
         <is>
           <t>IV — Permissions</t>
         </is>
       </c>
-      <c r="C62" s="2" t="inlineStr">
-        <is>
-          <t>Functional</t>
-        </is>
-      </c>
-      <c r="D62" s="2" t="inlineStr">
+      <c r="C63" s="2" t="inlineStr">
+        <is>
+          <t>Functional</t>
+        </is>
+      </c>
+      <c r="D63" s="2" t="inlineStr">
         <is>
           <t>Critical</t>
         </is>
       </c>
-      <c r="E62" s="2" t="inlineStr">
+      <c r="E63" s="2" t="inlineStr">
         <is>
           <t>1. A test user exists whose role has the existing inventory-reports permission (assign the Tech user a suitable role if needed; restore the original role afterward).
 2. You are signed in as that user on a desktop browser.</t>
         </is>
       </c>
-      <c r="F62" s="2" t="inlineStr">
+      <c r="F63" s="2" t="inlineStr">
         <is>
           <t>1. Open the reports navigation and find "Inventory Value" under the Parts group.
 2. Open the report and confirm it loads rows.
 3. Download the current view as a CSV.</t>
         </is>
       </c>
-      <c r="G62" s="2" t="inlineStr">
+      <c r="G63" s="2" t="inlineStr">
         <is>
           <t>1. The report is listed and opens normally for a user holding the existing inventory-reports permission.
 2. No additional, report-specific permission is required — the report reuses the existing inventory-reports permission.</t>
         </is>
       </c>
-      <c r="H62" s="2" t="inlineStr">
+      <c r="H63" s="2" t="inlineStr">
         <is>
           <t>specs/inventory-value.md Story 1 Prerequisites</t>
         </is>
       </c>
-      <c r="I62" s="2" t="inlineStr"/>
-      <c r="J62" s="2" t="inlineStr"/>
-    </row>
-    <row r="63">
-      <c r="A63" s="2" t="inlineStr">
+      <c r="I63" s="2" t="inlineStr"/>
+      <c r="J63" s="2" t="inlineStr"/>
+    </row>
+    <row r="64">
+      <c r="A64" s="2" t="inlineStr">
         <is>
           <t>A user without the required permission does not see Inventory Value in the reports navigation</t>
         </is>
       </c>
-      <c r="B63" s="2" t="inlineStr">
+      <c r="B64" s="2" t="inlineStr">
         <is>
           <t>IV — Permissions</t>
         </is>
       </c>
-      <c r="C63" s="2" t="inlineStr">
+      <c r="C64" s="2" t="inlineStr">
         <is>
           <t>Negative</t>
         </is>
       </c>
-      <c r="D63" s="2" t="inlineStr">
+      <c r="D64" s="2" t="inlineStr">
         <is>
           <t>Critical</t>
         </is>
       </c>
-      <c r="E63" s="2" t="inlineStr">
+      <c r="E64" s="2" t="inlineStr">
         <is>
           <t>1. A test user exists whose role does NOT have the inventory-reports permission (assign the Tech user such a role; restore the original role afterward).
 2. You are signed in as that user on a desktop browser.</t>
         </is>
       </c>
-      <c r="F63" s="2" t="inlineStr">
+      <c r="F64" s="2" t="inlineStr">
         <is>
           <t>1. Open the reports navigation.
 2. Look for "Inventory Value" under the Parts group.</t>
         </is>
       </c>
-      <c r="G63" s="2" t="inlineStr">
+      <c r="G64" s="2" t="inlineStr">
         <is>
           <t>1. The report does not appear in the navigation for this user.</t>
         </is>
       </c>
-      <c r="H63" s="2" t="inlineStr">
+      <c r="H64" s="2" t="inlineStr">
         <is>
           <t>specs/inventory-value.md Story 1 S1-N1</t>
         </is>
       </c>
-      <c r="I63" s="2" t="inlineStr"/>
-      <c r="J63" s="2" t="inlineStr"/>
-    </row>
-    <row r="64">
-      <c r="A64" s="2" t="inlineStr">
+      <c r="I64" s="2" t="inlineStr"/>
+      <c r="J64" s="2" t="inlineStr"/>
+    </row>
+    <row r="65">
+      <c r="A65" s="2" t="inlineStr">
         <is>
           <t>Nightly snapshot: once per day, for every location, one row per in-stock non-core part is recorded with its identity, quantity, and values to the cent</t>
         </is>
       </c>
-      <c r="B64" s="2" t="inlineStr">
+      <c r="B65" s="2" t="inlineStr">
         <is>
           <t>IV — API</t>
         </is>
       </c>
-      <c r="C64" s="2" t="inlineStr">
-        <is>
-          <t>Functional</t>
-        </is>
-      </c>
-      <c r="D64" s="2" t="inlineStr">
+      <c r="C65" s="2" t="inlineStr">
+        <is>
+          <t>Functional</t>
+        </is>
+      </c>
+      <c r="D65" s="2" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="E64" s="2" t="inlineStr">
+      <c r="E65" s="2" t="inlineStr">
         <is>
           <t>1. In-stock, non-core parts exist at two or more locations, including a part with non-round cent values.
 2. A location with NO in-stock parts also exists.
 3. You can inspect the stored snapshot rows after the nightly capture runs (arrange the verification route with the developers).</t>
         </is>
       </c>
-      <c r="F64" s="2" t="inlineStr">
+      <c r="F65" s="2" t="inlineStr">
         <is>
           <t>1. After the overnight capture, inspect the stored snapshot rows for that calendar date.
 2. For a known part, read every captured field.
 3. Check the rows for each location, including the empty one.</t>
         </is>
       </c>
-      <c r="G64" s="2" t="inlineStr">
+      <c r="G65" s="2" t="inlineStr">
         <is>
           <t>1. Once per day, overnight, one row per then-in-stock, non-core part is recorded for every location across every organization, under that day's calendar date.
 2. Each row captures the part's identity (part, category, vendor), on-hand quantity, unit cost, unit sell, total cost, and total sell, stored to the cent.
 3. A location with no in-stock parts on the date simply has no rows for that date — this is valid, not an error.</t>
         </is>
       </c>
-      <c r="H64" s="2" t="inlineStr">
+      <c r="H65" s="2" t="inlineStr">
         <is>
           <t>specs/inventory-value.md Story 11 S11-R1; S11-R4</t>
         </is>
       </c>
-      <c r="I64" s="2" t="inlineStr"/>
-      <c r="J64" s="2" t="inlineStr"/>
-    </row>
-    <row r="65">
-      <c r="A65" s="2" t="inlineStr">
+      <c r="I65" s="2" t="inlineStr"/>
+      <c r="J65" s="2" t="inlineStr"/>
+    </row>
+    <row r="66">
+      <c r="A66" s="2" t="inlineStr">
         <is>
           <t>Nightly snapshot: the captured scope and valuation are identical to the live report, so a recorded day equals what the live report showed that day</t>
         </is>
       </c>
-      <c r="B65" s="2" t="inlineStr">
+      <c r="B66" s="2" t="inlineStr">
         <is>
           <t>IV — API</t>
         </is>
       </c>
-      <c r="C65" s="2" t="inlineStr">
-        <is>
-          <t>Functional</t>
-        </is>
-      </c>
-      <c r="D65" s="2" t="inlineStr">
+      <c r="C66" s="2" t="inlineStr">
+        <is>
+          <t>Functional</t>
+        </is>
+      </c>
+      <c r="D66" s="2" t="inlineStr">
         <is>
           <t>Critical</t>
         </is>
       </c>
-      <c r="E65" s="2" t="inlineStr">
+      <c r="E66" s="2" t="inlineStr">
         <is>
           <t>1. ZZAUTOTEST parts with known quantities, costs, and sell resolutions (fixed price, matrix markup, and no-category fallback) are in stock and left UNCHANGED across the capture.
 2. A core-charge part and a zero-quantity part also exist.
 3. You can read the live report on the capture date and the stored rows afterward.</t>
         </is>
       </c>
-      <c r="F65" s="2" t="inlineStr">
+      <c r="F66" s="2" t="inlineStr">
         <is>
           <t>1. On the capture date, note the live report's rows and values for the seeded parts.
 2. After the overnight capture, read the same parts' captured rows.
@@ -3583,216 +3633,216 @@
 4. The next day, view the report as of the captured date and compare to the noted live values.</t>
         </is>
       </c>
-      <c r="G65" s="2" t="inlineStr">
+      <c r="G66" s="2" t="inlineStr">
         <is>
           <t>1. The captured parts use the same in-stock, non-core scope as the live report (Story 2) — the core-charge and zero-quantity parts are NOT captured.
 2. The captured values use the same valuation as the live report (Story 3), including the sell-price fallback chain.
 3. A recorded day equals what the live report would have shown that day — the as-of view of the captured date matches the noted live values.</t>
         </is>
       </c>
-      <c r="H65" s="2" t="inlineStr">
+      <c r="H66" s="2" t="inlineStr">
         <is>
           <t>specs/inventory-value.md Story 11 S11-R2; §2 Relationship to nightly history</t>
         </is>
       </c>
-      <c r="I65" s="2" t="inlineStr"/>
-      <c r="J65" s="2" t="inlineStr"/>
-    </row>
-    <row r="66">
-      <c r="A66" s="2" t="inlineStr">
+      <c r="I66" s="2" t="inlineStr"/>
+      <c r="J66" s="2" t="inlineStr"/>
+    </row>
+    <row r="67">
+      <c r="A67" s="2" t="inlineStr">
         <is>
           <t>Nightly snapshot: re-running the capture for a date replaces that date's rows — idempotent, no duplicates</t>
         </is>
       </c>
-      <c r="B66" s="2" t="inlineStr">
+      <c r="B67" s="2" t="inlineStr">
         <is>
           <t>IV — API</t>
         </is>
       </c>
-      <c r="C66" s="2" t="inlineStr">
-        <is>
-          <t>Functional</t>
-        </is>
-      </c>
-      <c r="D66" s="2" t="inlineStr">
+      <c r="C67" s="2" t="inlineStr">
+        <is>
+          <t>Functional</t>
+        </is>
+      </c>
+      <c r="D67" s="2" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="E66" s="2" t="inlineStr">
+      <c r="E67" s="2" t="inlineStr">
         <is>
           <t>1. A capture has already run for the current date.
 2. The capture can be re-run for that date (arrange with the developers).</t>
         </is>
       </c>
-      <c r="F66" s="2" t="inlineStr">
+      <c r="F67" s="2" t="inlineStr">
         <is>
           <t>1. Count the stored rows per location for the date.
 2. Re-run the capture for the same date.
 3. Count and inspect the rows again.</t>
         </is>
       </c>
-      <c r="G66" s="2" t="inlineStr">
+      <c r="G67" s="2" t="inlineStr">
         <is>
           <t>1. Re-running the capture for a date replaces that date's rows for each location — the existing rows for that location and date are removed, then re-inserted from current data.
 2. No duplicate rows exist for the same part, location, and date.
 3. The capture is idempotent and self-healing from current data.</t>
         </is>
       </c>
-      <c r="H66" s="2" t="inlineStr">
+      <c r="H67" s="2" t="inlineStr">
         <is>
           <t>specs/inventory-value.md Story 11 S11-R3</t>
         </is>
       </c>
-      <c r="I66" s="2" t="inlineStr"/>
-      <c r="J66" s="2" t="inlineStr"/>
-    </row>
-    <row r="67">
-      <c r="A67" s="2" t="inlineStr">
+      <c r="I67" s="2" t="inlineStr"/>
+      <c r="J67" s="2" t="inlineStr"/>
+    </row>
+    <row r="68">
+      <c r="A68" s="2" t="inlineStr">
         <is>
           <t>Nightly snapshot: history accrues forward only — a re-run records current truth under the current date and cannot reconstruct a past date</t>
         </is>
       </c>
-      <c r="B67" s="2" t="inlineStr">
+      <c r="B68" s="2" t="inlineStr">
         <is>
           <t>IV — API</t>
         </is>
       </c>
-      <c r="C67" s="2" t="inlineStr">
-        <is>
-          <t>Functional</t>
-        </is>
-      </c>
-      <c r="D67" s="2" t="inlineStr">
+      <c r="C68" s="2" t="inlineStr">
+        <is>
+          <t>Functional</t>
+        </is>
+      </c>
+      <c r="D68" s="2" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="E67" s="2" t="inlineStr">
+      <c r="E68" s="2" t="inlineStr">
         <is>
           <t>1. The date the first capture ran is known.
 2. Stock levels have changed since a past captured date.</t>
         </is>
       </c>
-      <c r="F67" s="2" t="inlineStr">
+      <c r="F68" s="2" t="inlineStr">
         <is>
           <t>1. Check the stored history for any rows dated before the first capture.
 2. Re-run the capture and check which date its rows are recorded under.
 3. Compare a past date's stored rows to confirm they were not rewritten by the re-run.</t>
         </is>
       </c>
-      <c r="G67" s="2" t="inlineStr">
+      <c r="G68" s="2" t="inlineStr">
         <is>
           <t>1. No rows exist for dates before capture began — there is no backfill.
 2. A re-run always records current truth under the CURRENT date; it cannot reconstruct a past date.
 3. Past dates' stored rows are unchanged by a current re-run.</t>
         </is>
       </c>
-      <c r="H67" s="2" t="inlineStr">
+      <c r="H68" s="2" t="inlineStr">
         <is>
           <t>specs/inventory-value.md Story 11 S11-R5; Story 5 S5-E1</t>
         </is>
       </c>
-      <c r="I67" s="2" t="inlineStr"/>
-      <c r="J67" s="2" t="inlineStr"/>
-    </row>
-    <row r="68">
-      <c r="A68" s="2" t="inlineStr">
+      <c r="I68" s="2" t="inlineStr"/>
+      <c r="J68" s="2" t="inlineStr"/>
+    </row>
+    <row r="69">
+      <c r="A69" s="2" t="inlineStr">
         <is>
           <t>Snapshot retention: daily captures are kept for 0–13 months; older history is reduced to the last capture of each calendar month</t>
         </is>
       </c>
-      <c r="B68" s="2" t="inlineStr">
+      <c r="B69" s="2" t="inlineStr">
         <is>
           <t>IV — API</t>
         </is>
       </c>
-      <c r="C68" s="2" t="inlineStr">
-        <is>
-          <t>Functional</t>
-        </is>
-      </c>
-      <c r="D68" s="2" t="inlineStr">
+      <c r="C69" s="2" t="inlineStr">
+        <is>
+          <t>Functional</t>
+        </is>
+      </c>
+      <c r="D69" s="2" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="E68" s="2" t="inlineStr">
+      <c r="E69" s="2" t="inlineStr">
         <is>
           <t>1. Snapshot history exists (or is seeded/simulated with dev help) spanning both the 0–13-month band and the older-than-13-months band.
 2. The nightly capture (with its pruning) has run.</t>
         </is>
       </c>
-      <c r="F68" s="2" t="inlineStr">
+      <c r="F69" s="2" t="inlineStr">
         <is>
           <t>1. Inspect the retained captures for dates within the last 13 months.
 2. Inspect the retained captures for dates older than 13 months.
 3. Check when pruning runs relative to the nightly capture.</t>
         </is>
       </c>
-      <c r="G68" s="2" t="inlineStr">
+      <c r="G69" s="2" t="inlineStr">
         <is>
           <t>1. For ages 0–13 months (measured from the current date), every daily capture is kept — full daily per-part detail, covering the report's longest date preset (366 days / This Year / Last Year) entirely at daily resolution.
 2. For ages older than 13 months, only the last capture of each calendar month is retained; the other daily captures in that band are pruned.
 3. Pruning runs as part of, or alongside, the nightly capture.</t>
         </is>
       </c>
-      <c r="H68" s="2" t="inlineStr">
+      <c r="H69" s="2" t="inlineStr">
         <is>
           <t>specs/inventory-value.md Story 11 S11-R6</t>
         </is>
       </c>
-      <c r="I68" s="2" t="inlineStr"/>
-      <c r="J68" s="2" t="inlineStr"/>
-    </row>
-    <row r="69">
-      <c r="A69" s="2" t="inlineStr">
+      <c r="I69" s="2" t="inlineStr"/>
+      <c r="J69" s="2" t="inlineStr"/>
+    </row>
+    <row r="70">
+      <c r="A70" s="2" t="inlineStr">
         <is>
           <t>Thinned history is served unchanged: the closest-recorded-day rule bridges retention gaps, the "As of" indicator names the day shown, and a fully-pruned range shows the empty state</t>
         </is>
       </c>
-      <c r="B69" s="2" t="inlineStr">
+      <c r="B70" s="2" t="inlineStr">
         <is>
           <t>IV — API</t>
         </is>
       </c>
-      <c r="C69" s="2" t="inlineStr">
-        <is>
-          <t>Functional</t>
-        </is>
-      </c>
-      <c r="D69" s="2" t="inlineStr">
+      <c r="C70" s="2" t="inlineStr">
+        <is>
+          <t>Functional</t>
+        </is>
+      </c>
+      <c r="D70" s="2" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="E69" s="2" t="inlineStr">
+      <c r="E70" s="2" t="inlineStr">
         <is>
           <t>1. Thinned history exists (dates older than 13 months where only the monthly last-capture remains — dev-seeded if needed).
 2. The retained capture dates around the requested date are known.</t>
         </is>
       </c>
-      <c r="F69" s="2" t="inlineStr">
+      <c r="F70" s="2" t="inlineStr">
         <is>
           <t>1. On the report, select a range ending on a pruned date between two retained monthly captures.
 2. Read which day the values represent and the "As of" indicator.
 3. Select a range whose covering captures have ALL been pruned and no earlier retained capture remains.</t>
         </is>
       </c>
-      <c r="G69" s="2" t="inlineStr">
+      <c r="G70" s="2" t="inlineStr">
         <is>
           <t>1. The as-of resolution serves the thinned history unchanged: the report resolves to the nearest earlier retained capture ("closest recorded day on or before"), even when adjacent retained captures are up to a month apart.
 2. The "As of" indicator names the day actually shown.
 3. A requested date whose covering captures have all been pruned resolves to the nearest earlier retained capture, or shows the empty state if none remains.</t>
         </is>
       </c>
-      <c r="H69" s="2" t="inlineStr">
+      <c r="H70" s="2" t="inlineStr">
         <is>
           <t>specs/inventory-value.md Story 11 S11-E1; S11-R6; Story 5 S5-R4; S5-R5; S5-N1</t>
         </is>
       </c>
-      <c r="I69" s="2" t="inlineStr"/>
-      <c r="J69" s="2" t="inlineStr"/>
+      <c r="I70" s="2" t="inlineStr"/>
+      <c r="J70" s="2" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Report Suite: run-359 push executor + snapshots, SBC case + id-map, regenerated imports
- build/report-suite/chris-answers-2026-08-01/exec_push_2026-08-03.mjs: authorised narrow push executor (buckets A+B + run-359 union)
- run359-snapshot-2026-08-03/: before/after case bodies, run tests + results snapshots, union case-id lists, ops log
- build/report-suite/cases/cases-sbc-A-access-filters.json + testrail-id-map.csv updated
- testrail-import/: unified + per-report Report Suite imports regenerated (csv + xlsx)

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01AZ5XzKsK9wv7M41cSPaMyg
</commit_message>
<xml_diff>
--- a/testrail-import/Report-Suite_Inventory-Value-Report_testrail-import.xlsx
+++ b/testrail-import/Report-Suite_Inventory-Value-Report_testrail-import.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Inventory Value" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Inventory Value" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>

</xml_diff>

<commit_message>
chore(sweeper): checkpoint 43 dirty path(s)
Automatic additive checkpoint so no work is lost (Standing Rule 29).
Paths were hash-stable for 20s and passed the secret scan.
Top-level areas: build, testrail-import

  build/report-suite/cases
  build/report-suite/epic-reread-2026-08-04
  build/report-suite/viu-push-2026-08-04
  testrail-import

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01AZ5XzKsK9wv7M41cSPaMyg
</commit_message>
<xml_diff>
--- a/testrail-import/Report-Suite_Inventory-Value-Report_testrail-import.xlsx
+++ b/testrail-import/Report-Suite_Inventory-Value-Report_testrail-import.xlsx
@@ -428,7 +428,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J71"/>
+  <dimension ref="A1:J72"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="50" customWidth="1" min="1" max="1"/>
@@ -659,16 +659,17 @@
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>1. Open the Inventory Value report and find the pagination control.
-2. Move to page 2 (and further) and watch the rows.
-3. From a later page, change a server-side filter (for example select a Category), then check which page is shown.
-4. Repeat from a later page with a part search and with a sort change.</t>
+          <t>1. Open the Inventory Value report and scroll to the bottom of the rows, then keep scrolling so further rows load.
+2. Watch that new rows keep arriving as you scroll rather than all of them being present at once.
+3. After scrolling well down the list, change a server-side filter (for example select a Category), then look at where the list starts.
+4. Repeat with a part search and with a sort change.</t>
         </is>
       </c>
       <c r="G5" s="2" t="inlineStr">
         <is>
           <t>1. The server returns one page of rows at a time; the user moves through pages with the reports suite's standard pagination control.
-2. Changing any server-side filter (Date, Location, Category, Vendor), the part search, or the sort returns the FIRST page of the new result set.</t>
+2. Changing any server-side filter (Date, Location, Category, Vendor), the part search, or the sort returns the FIRST page of the new result set - the list jumps back to the top.
+3. Note for the tester: on this build there are no numbered page controls on the screen - the rows load as you scroll. That is what you should see; record it and carry on with the checks above.</t>
         </is>
       </c>
       <c r="H5" s="2" t="inlineStr">
@@ -1197,10 +1198,10 @@
       </c>
       <c r="G16" s="2" t="inlineStr">
         <is>
-          <t>1. With a single location in scope the columns appear in this order: Part #, Description, Category, Vendor, Qty on Hand, Unit Cost, Unit Sell, Margin, Margin %, Total Sell, Total Cost.
+          <t>1. With a single location in scope the columns appear in this order: Part #, Description, Category, Vendor, Qty, Unit Cost, Unit Sell, Margin, Margin %, Total Sell, Total Cost.
 2. Part #, Description, Category, and Vendor are left-aligned.
 3. Every other column is right-aligned.
-4. When more than one location is in scope the automatic Location column also appears, between Vendor and Qty on Hand, left-aligned. It is not in the column-selection control, so its presence is expected and is not a failure of this test.</t>
+4. Location is one of the columns in the column-selection control; when it is turned on the Location column appears between Vendor and Qty, left-aligned.</t>
         </is>
       </c>
       <c r="H16" s="2" t="inlineStr">
@@ -1214,7 +1215,7 @@
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
         <is>
-          <t>Value formats: Qty on Hand to two decimals; money as US-dollar currency</t>
+          <t>Value formats: Qty to two decimals; money as US-dollar currency</t>
         </is>
       </c>
       <c r="B17" s="2" t="inlineStr">
@@ -1235,19 +1236,19 @@
       <c r="E17" s="2" t="inlineStr">
         <is>
           <t>1. You are signed in to the ShopView App on a desktop browser.
-2. The report shows a part with a fractional on-hand quantity (for example 2.50), one with values over $1,000, and (if producible) one with a negative money value.</t>
+2. The report shows a part with a fractional quantity (for example 2.50), one with values over $1,000, and (if producible) one with a negative money value.</t>
         </is>
       </c>
       <c r="F17" s="2" t="inlineStr">
         <is>
-          <t>1. Read the Qty on Hand cell of the fractional-quantity part.
+          <t>1. Read the Qty cell of the fractional-quantity part.
 2. Read a money value over one thousand dollars (Unit Cost, Unit Sell, Total Sell, or Total Cost).
 3. Read a genuine zero money value and a negative one if present.</t>
         </is>
       </c>
       <c r="G17" s="2" t="inlineStr">
         <is>
-          <t>1. Qty on Hand shows the on-hand quantity to two decimal places, with no currency symbol; fractional quantities display correctly.
+          <t>1. Qty shows the on-hand quantity to two decimal places, with no currency symbol; fractional quantities display correctly.
 2. Unit Cost and Unit Sell show per-unit prices as US-dollar currency.
 3. Money values show a leading "$", two decimal places, and thousands separators (for example "$1,234.56"); a negative value shows a leading minus before the "$" ("-$1,234.56"); a genuine zero shows "$0.00".</t>
         </is>
@@ -1343,10 +1344,10 @@
       </c>
       <c r="G19" s="2" t="inlineStr">
         <is>
-          <t>1. On first visit with a single location in scope the visible columns are: Part #, Description, Category, Vendor, Qty on Hand, Unit Cost, Unit Sell, Margin %, and Total Cost.
+          <t>1. On first visit with a single location in scope the visible columns are: Part #, Description, Category, Vendor, Qty, Unit Cost, Unit Sell, Margin %, and Total Cost.
 2. The Margin and Total Sell columns are hidden by default.
 3. Both can be turned on from the column-selection control and then appear in their fixed positions.
-4. When more than one location is in scope the automatic Location column also shows, between Vendor and Qty on Hand — it is not one of the toggleable columns and its presence is expected.</t>
+4. Location is one of the columns in the column-selection control; when it is turned on the Location column shows between Vendor and Qty.</t>
         </is>
       </c>
       <c r="H19" s="2" t="inlineStr">
@@ -1395,7 +1396,8 @@
         <is>
           <t>1. Category shows the part's category name; Vendor shows the part's vendor name.
 2. A part with no category shows an em dash ("—") in its Category cell.
-3. A part with no vendor shows an em dash ("—") in its Vendor cell.</t>
+3. A part with no vendor shows an em dash ("—") in its Vendor cell.
+4. Note for the tester: on this build a part cannot be saved without a category, so you will not find a part whose Category cell shows "—". Check the Vendor half only.</t>
         </is>
       </c>
       <c r="H20" s="2" t="inlineStr">
@@ -1409,7 +1411,7 @@
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
         <is>
-          <t>Totals row: Total label, blank identity/per-unit cells, pinned bold Total Cost</t>
+          <t>Totals row: Totals label, blank identity/per-unit cells, pinned bold Total Cost</t>
         </is>
       </c>
       <c r="B21" s="2" t="inlineStr">
@@ -1444,7 +1446,7 @@
       </c>
       <c r="G21" s="2" t="inlineStr">
         <is>
-          <t>1. A totals row is shown at the bottom, with the literal label "Total" in the Part # column's cell.
+          <t>1. A totals row is shown at the bottom, with the label "Totals" in the Part # column's cell.
 2. The Description, Category, and Vendor cells are blank; the Unit Cost and Unit Sell cells are blank (a per-unit price has no meaningful sum).
 3. The totals-row Total Cost cell is pinned far right and bold, matching the column, and the row uses the same number formats as the data rows.
 4. The totals row stays visible at the bottom while the rows scroll.</t>
@@ -1499,7 +1501,7 @@
         <is>
           <t>1. The totals row sums Qty on Hand, Margin, Total Sell, and Total Cost across the FULL filtered result set — every qualifying row for the current Date, Location, Category, Vendor, and part-search selection, not only the rows on the visible page.
 2. The totals are identical on every page (they do not change as you page).
-3. The hand-summed subset matches the server-computed totals to the cent.
+3. A hand sum of a small seeded subset matches the totals row. On a large set the totals can differ from a hand sum of the displayed values by a few cents, because the server sums the unrounded values - that is correct, not a defect.
 4. After each filter change the totals row recomputes on the server over the full filtered set, independent of which page is shown.</t>
         </is>
       </c>
@@ -1830,8 +1832,8 @@
       </c>
       <c r="F29" s="2" t="inlineStr">
         <is>
-          <t>1. Open the date-range control and choose "Custom".
-2. Pick a start and an end date in the past and apply.
+          <t>1. Open the date-range control - a month calendar is shown inside it (there is no separate "Custom" item to choose).
+2. Pick a start and an end date in the past on that calendar and press Apply.
 3. Try to pick an end date in the future.
 4. Watch the data area when the range is applied.</t>
         </is>
@@ -2021,12 +2023,12 @@
       <c r="E33" s="2" t="inlineStr">
         <is>
           <t>1. You are signed in to the ShopView App on a desktop browser.
-2. The unfiltered result set spans multiple pages, and matching parts for a category/vendor/search exist BEYOND page 1.</t>
+2. The unfiltered result set is long enough to need scrolling, and matching parts for a category/vendor/search exist well down the list (beyond the first screenful).</t>
         </is>
       </c>
       <c r="F33" s="2" t="inlineStr">
         <is>
-          <t>1. From page 2 (or later), select a Category and check which page shows and which rows are listed.
+          <t>1. Scroll well down the list, then select a Category and check where the list starts and which rows are listed.
 2. Repeat with a Vendor selection.
 3. Repeat with a part search.
 4. Also change the date range, the location selection, and the sort — watching the data area each time.</t>
@@ -2035,7 +2037,7 @@
       <c r="G33" s="2" t="inlineStr">
         <is>
           <t>1. Each change re-queries the server and returns the first page of the new result set.
-2. The filtering covers the ENTIRE data set — matching parts that were on later pages appear — not just a narrowing of the rows on the current page.
+2. The filtering covers the ENTIRE data set — matching parts that were further down the list appear — not just a narrowing of the rows currently on screen.
 3. Every change — date range, location, Category, Vendor, part search, sort — reloads the rows from the server; while loading the standard reports loading indicator shows, and existing rows are replaced only when the new data returns.</t>
         </is>
       </c>
@@ -2391,7 +2393,7 @@
     <row r="41">
       <c r="A41" s="2" t="inlineStr">
         <is>
-          <t>The Location column is automatic, sits after Vendor, and never reads Multiple</t>
+          <t>The Location column sits after Vendor and never reads Multiple</t>
         </is>
       </c>
       <c r="B41" s="2" t="inlineStr">
@@ -2418,7 +2420,7 @@
       </c>
       <c r="F41" s="2" t="inlineStr">
         <is>
-          <t>1. Select two or more locations and read the column headers from the left.
+          <t>1. Turn Location on in the column-selection control, select two or more locations, and read the column headers from the left.
 2. Read the Location cell on each of the two rows for the part stocked at both locations.
 3. Look for any row showing "Multiple".
 4. Open the column-selection control and look for Location in the list.
@@ -2429,13 +2431,13 @@
       </c>
       <c r="G41" s="2" t="inlineStr">
         <is>
-          <t>1. With more than one location in scope a Location column is shown, inserted between Vendor and Qty on Hand.
+          <t>1. With Location turned on in the column-selection control, a Location column is shown, inserted between Vendor and Qty.
 2. Each row names the location that row's stock is held at.
 3. NO row ever shows "Multiple" — each row is one part at one location.
-4. Location is NOT offered in the column-selection control — its visibility follows the location scope automatically.
-5. With a single location in scope the Location column is hidden and the surrounding columns close up.
+4. Location IS one of the columns offered in the column-selection control - its visibility follows that toggle, not the location selection.
+5. With the Location toggle off the column is not shown and the surrounding columns close up.
 6. The Location filter control keeps the same width whichever label it shows — one location, several, or "All locations" — so the toolbar does not shift as you change the selection.
-7. Both downloads include the Location column in the same position it holds on screen (between Vendor and Qty on Hand), naming each row's own location.</t>
+7. Both downloads include the Location column in the same position it holds on screen (between Vendor and Qty), naming each row's own location.</t>
         </is>
       </c>
       <c r="H41" s="2" t="inlineStr">
@@ -2530,7 +2532,7 @@
       </c>
       <c r="G43" s="2" t="inlineStr">
         <is>
-          <t>1. Whatever columns are shown, they appear in the fixed left-to-right order — with the automatic Location column, when more than one location is in scope, between Vendor and Qty on Hand (Part #, Description, Category, Vendor, Qty on Hand, Unit Cost, Unit Sell, Margin, Margin %, Total Sell, Total Cost) — toggling visibility never reorders columns.
+          <t>1. Whatever columns are shown, they appear in the fixed left-to-right order - with Location, when it is turned on in the column-selection control, between Vendor and Qty (Part #, Description, Category, Vendor, Qty, Unit Cost, Unit Sell, Margin, Margin %, Total Sell, Total Cost) - toggling visibility never reorders columns.
 2. Total Cost is always the last column.</t>
         </is>
       </c>
@@ -2920,7 +2922,7 @@
 2. Both downloads honor the current date, category, vendor, location, and part-search filters, and apply the current sort.
 3. Both downloads include a totals row labeled "Totals" matching the on-screen totals (the full-filtered-set totals).
 4. Each download (PDF and CSV) carries a "Locations:" line naming the location(s) the report was scoped to (exact position in the file is confirmed in the build).
-5. Note for the tester: when you have more than one location in scope, the files also carry a Location column (between Vendor and Qty on Hand) even though it is not in the column-selection control. That is correct - it appears by itself. With a single location in scope there is no Location column, and that is also correct.</t>
+5. Note for the tester: the files carry the Location column when Location is turned ON in the column-selection control (it sits between Vendor and Qty). It does not appear just because you have more than one location selected.</t>
         </is>
       </c>
       <c r="H51" s="2" t="inlineStr">
@@ -3019,7 +3021,8 @@
         <is>
           <t>1. The PDF header shows the report name "Inventory Value", the organization name, the selected period, and an "as of" line naming the day the values represent (or a message that no snapshot is available for the period).
 2. The PDF shows the shop logo at the top when one is set.
-3. The CSV never includes a logo.</t>
+3. The CSV never includes a logo.
+4. Note for the tester: the two files phrase the as-of line differently - the PDF reads "As of 2026-08-04" and the CSV's first line reads "As of: 2026-08-04" (with a colon). Both are correct; do not raise the difference.</t>
         </is>
       </c>
       <c r="H53" s="2" t="inlineStr">
@@ -3164,7 +3167,8 @@
         <is>
           <t>1. Neither the PDF nor the CSV is produced.
 2. The user sees the message: "This report is too large to export. Narrow the date range or filters, then try again." (a blocking notification; no file).
-3. After narrowing the filters below the cap, the download works again.</t>
+3. After narrowing the filters below the cap, the download works again.
+4. Note for the tester: on this environment the biggest view you can build is about 9,275 rows, which is under the cap, so you cannot make this message appear here. If the PDF fails with a plain error instead, that is the separate timeout problem - see the Inventory Value export-notification case.</t>
         </is>
       </c>
       <c r="H56" s="2" t="inlineStr">
@@ -3214,7 +3218,8 @@
         <is>
           <t>1. Success notifications read verbatim: "Inventory Value report exported (PDF)" and "Inventory Value report exported (CSV)".
 2. Failure notifications read verbatim: "Failed to export inventory value report (pdf)" and "Failed to export inventory value report (csv)".
-3. The lower-case "(pdf)"/"(csv)" on failure vs the upper-case success ones is the documented spec wording — expected, not a bug.</t>
+3. The lower-case "(pdf)"/"(csv)" on failure vs the upper-case success ones is the documented spec wording — expected, not a bug.
+4. Note for the tester: on this build a PDF download of a large view fails with a plain error - "An error occurred. We're sorry for this inconvenience, please try again a bit later later." - after roughly half a minute. It is a timeout, not the too-large-to-export message. Narrow the view with the part search or a single location and the PDF works. The CSV of the same view always works and is quick. Record the failure; it is a known problem, not a mistake you made.</t>
         </is>
       </c>
       <c r="H57" s="2" t="inlineStr">
@@ -3228,466 +3233,518 @@
     <row r="58">
       <c r="A58" s="2" t="inlineStr">
         <is>
+          <t>A large Inventory Value PDF fails instead of being refused politely</t>
+        </is>
+      </c>
+      <c r="B58" s="2" t="inlineStr">
+        <is>
+          <t>IV — Exports</t>
+        </is>
+      </c>
+      <c r="C58" s="2" t="inlineStr">
+        <is>
+          <t>Functional</t>
+        </is>
+      </c>
+      <c r="D58" s="2" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="E58" s="2" t="inlineStr">
+        <is>
+          <t>1. You are signed in with ordinary reports access, on a desktop browser.
+2. The Inventory Value report is open and the whole list runs to several thousand rows.</t>
+        </is>
+      </c>
+      <c r="F58" s="2" t="inlineStr">
+        <is>
+          <t>1. Use the part search to narrow the list to a few hundred rows. Open the three-dot menu and choose the PDF download. Note how long it takes.
+2. Clear the search so the whole list is shown again. Choose the PDF download and wait up to a minute.
+3. With the whole list still shown, choose the CSV download and note how long that takes.
+4. Narrow the list again with the part search, or pick a single location, and ask for the PDF once more.</t>
+        </is>
+      </c>
+      <c r="G58" s="2" t="inlineStr">
+        <is>
+          <t>1. The narrowed PDF downloads successfully.
+2. On the whole list the PDF does not download. After roughly half a minute a plain error appears reading "An error occurred. We're sorry for this inconvenience, please try again a bit later later." — record that this happened and roughly how many rows were in the view.
+3. The CSV of that same whole list downloads successfully and quickly.
+4. Once the view is narrowed the PDF works again.
+5. Note for the tester: this is NOT the too-large-to-export message. If you see "This report is too large to export. Narrow the date range or filters, then try again." instead, that is the polite refusal working correctly and belongs to the export-cap test, not this one.</t>
+        </is>
+      </c>
+      <c r="H58" s="2" t="inlineStr">
+        <is>
+          <t>SV-8677 (IV spec v3 2026-07-29 S10-R11; S10-R12; S10-R14 — the observed failure path is a roughly 30-second server-side timeout and not the S10-R12 row cap; observed on build v3.4.1-0ed4433)</t>
+        </is>
+      </c>
+      <c r="I58" s="2" t="inlineStr"/>
+      <c r="J58" s="2" t="inlineStr"/>
+    </row>
+    <row r="59">
+      <c r="A59" s="2" t="inlineStr">
+        <is>
           <t>All-white table with no row shading on the standard report backdrop</t>
         </is>
       </c>
-      <c r="B58" s="2" t="inlineStr">
+      <c r="B59" s="2" t="inlineStr">
         <is>
           <t>IV — Visual &amp; Accessibility</t>
         </is>
       </c>
-      <c r="C58" s="2" t="inlineStr">
-        <is>
-          <t>Functional</t>
-        </is>
-      </c>
-      <c r="D58" s="2" t="inlineStr">
+      <c r="C59" s="2" t="inlineStr">
+        <is>
+          <t>Functional</t>
+        </is>
+      </c>
+      <c r="D59" s="2" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="E58" s="2" t="inlineStr">
+      <c r="E59" s="2" t="inlineStr">
         <is>
           <t>1. You are signed in to the ShopView App on a desktop browser.
 2. The Inventory Value report is open with several rows.</t>
         </is>
       </c>
-      <c r="F58" s="2" t="inlineStr">
+      <c r="F59" s="2" t="inlineStr">
         <is>
           <t>1. Look at the column headers and the data cells.
 2. Compare the background of consecutive rows.
 3. Look at the page background around the table.</t>
         </is>
       </c>
-      <c r="G58" s="2" t="inlineStr">
+      <c r="G59" s="2" t="inlineStr">
         <is>
           <t>1. The table has white column headers and white data cells, with no alternating row shading.
 2. The table sits on the standard soft blue-grey report backdrop.</t>
         </is>
       </c>
-      <c r="H58" s="2" t="inlineStr">
+      <c r="H59" s="2" t="inlineStr">
         <is>
           <t>SV-8679 (specs/inventory-value.md Story 12 S12-R1)</t>
         </is>
       </c>
-      <c r="I58" s="2" t="inlineStr"/>
-      <c r="J58" s="2" t="inlineStr"/>
-    </row>
-    <row r="59">
-      <c r="A59" s="2" t="inlineStr">
+      <c r="I59" s="2" t="inlineStr"/>
+      <c r="J59" s="2" t="inlineStr"/>
+    </row>
+    <row r="60">
+      <c r="A60" s="2" t="inlineStr">
         <is>
           <t>Toolbar layout: menu leftmost then Column Selection; then the 5 filters</t>
         </is>
       </c>
-      <c r="B59" s="2" t="inlineStr">
+      <c r="B60" s="2" t="inlineStr">
         <is>
           <t>IV — Visual &amp; Accessibility</t>
         </is>
       </c>
-      <c r="C59" s="2" t="inlineStr">
-        <is>
-          <t>Functional</t>
-        </is>
-      </c>
-      <c r="D59" s="2" t="inlineStr">
+      <c r="C60" s="2" t="inlineStr">
+        <is>
+          <t>Functional</t>
+        </is>
+      </c>
+      <c r="D60" s="2" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="E59" s="2" t="inlineStr">
+      <c r="E60" s="2" t="inlineStr">
         <is>
           <t>1. You are signed in to the ShopView App on a desktop browser.
 2. The Inventory Value report is open.</t>
         </is>
       </c>
-      <c r="F59" s="2" t="inlineStr">
+      <c r="F60" s="2" t="inlineStr">
         <is>
           <t>1. Look at the toolbar's action cluster and read the order of its controls.
 2. Read the toolbar filters from left to right.</t>
         </is>
       </c>
-      <c r="G59" s="2" t="inlineStr">
+      <c r="G60" s="2" t="inlineStr">
         <is>
           <t>1. In the toolbar, the three-dot download menu sits leftmost in the action cluster, followed by the Column Selection control.
 2. The toolbar filters run, left to right: the date-range control, the part search, the Category filter, the Vendor filter, and the Location filter (rightmost).</t>
         </is>
       </c>
-      <c r="H59" s="2" t="inlineStr">
+      <c r="H60" s="2" t="inlineStr">
         <is>
           <t>SV-8679 (specs/inventory-value.md Story 12 S12-R2; S12-R3)</t>
         </is>
       </c>
-      <c r="I59" s="2" t="inlineStr"/>
-      <c r="J59" s="2" t="inlineStr"/>
-    </row>
-    <row r="60">
-      <c r="A60" s="2" t="inlineStr">
+      <c r="I60" s="2" t="inlineStr"/>
+      <c r="J60" s="2" t="inlineStr"/>
+    </row>
+    <row r="61">
+      <c r="A61" s="2" t="inlineStr">
         <is>
           <t>Long Description; Category and Vendor truncate on hover; Part # never does</t>
         </is>
       </c>
-      <c r="B60" s="2" t="inlineStr">
+      <c r="B61" s="2" t="inlineStr">
         <is>
           <t>IV — Visual &amp; Accessibility</t>
         </is>
       </c>
-      <c r="C60" s="2" t="inlineStr">
-        <is>
-          <t>Functional</t>
-        </is>
-      </c>
-      <c r="D60" s="2" t="inlineStr">
+      <c r="C61" s="2" t="inlineStr">
+        <is>
+          <t>Functional</t>
+        </is>
+      </c>
+      <c r="D61" s="2" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="E60" s="2" t="inlineStr">
+      <c r="E61" s="2" t="inlineStr">
         <is>
           <t>1. You are signed in to the ShopView App on a desktop browser.
 2. A ZZAUTOTEST part exists with a very long description (and, if possible, long category/vendor names) and a long part number.</t>
         </is>
       </c>
-      <c r="F60" s="2" t="inlineStr">
+      <c r="F61" s="2" t="inlineStr">
         <is>
           <t>1. Narrow the browser window (or turn on more columns) so the text columns overflow.
 2. Read the long Description, Category, and Vendor cells and hover each.
 3. Read the long Part # cell.</t>
         </is>
       </c>
-      <c r="G60" s="2" t="inlineStr">
+      <c r="G61" s="2" t="inlineStr">
         <is>
           <t>1. Long text values (Description, Category, Vendor) are truncated with an ellipsis when they overflow their column.
 2. The full value is available on hover.
 3. The Part # is never truncated.</t>
         </is>
       </c>
-      <c r="H60" s="2" t="inlineStr">
+      <c r="H61" s="2" t="inlineStr">
         <is>
           <t>SV-8679 (specs/inventory-value.md Story 12 S12-R6)</t>
         </is>
       </c>
-      <c r="I60" s="2" t="inlineStr"/>
-      <c r="J60" s="2" t="inlineStr"/>
-    </row>
-    <row r="61">
-      <c r="A61" s="2" t="inlineStr">
+      <c r="I61" s="2" t="inlineStr"/>
+      <c r="J61" s="2" t="inlineStr"/>
+    </row>
+    <row r="62">
+      <c r="A62" s="2" t="inlineStr">
         <is>
           <t>In dark mode the page background, toolbar, cells; the "—" glyph remain legible</t>
         </is>
       </c>
-      <c r="B61" s="2" t="inlineStr">
+      <c r="B62" s="2" t="inlineStr">
         <is>
           <t>IV — Visual &amp; Accessibility</t>
         </is>
       </c>
-      <c r="C61" s="2" t="inlineStr">
+      <c r="C62" s="2" t="inlineStr">
         <is>
           <t>Accessibility</t>
         </is>
       </c>
-      <c r="D61" s="2" t="inlineStr">
+      <c r="D62" s="2" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="E61" s="2" t="inlineStr">
+      <c r="E62" s="2" t="inlineStr">
         <is>
           <t>1. You are signed in to the ShopView App on a desktop browser.
 2. The application is switched to dark mode.
 3. The report shows rows including a part with an em-dash ("—") Category or Vendor cell.</t>
         </is>
       </c>
-      <c r="F61" s="2" t="inlineStr">
+      <c r="F62" s="2" t="inlineStr">
         <is>
           <t>1. Read the page background, toolbar, and table cells in dark mode.
 2. Find a "—" cell and check its legibility.</t>
         </is>
       </c>
-      <c r="G61" s="2" t="inlineStr">
+      <c r="G62" s="2" t="inlineStr">
         <is>
           <t>1. The report supports dark mode.
 2. The page background, toolbar, cells, and the "—" glyph all use dark-mode-legible colors.</t>
         </is>
       </c>
-      <c r="H61" s="2" t="inlineStr">
+      <c r="H62" s="2" t="inlineStr">
         <is>
           <t>SV-8679 (specs/inventory-value.md Story 12 S12-R7)</t>
         </is>
       </c>
-      <c r="I61" s="2" t="inlineStr"/>
-      <c r="J61" s="2" t="inlineStr"/>
-    </row>
-    <row r="62">
-      <c r="A62" s="2" t="inlineStr">
+      <c r="I62" s="2" t="inlineStr"/>
+      <c r="J62" s="2" t="inlineStr"/>
+    </row>
+    <row r="63">
+      <c r="A63" s="2" t="inlineStr">
         <is>
           <t>Each sortable header exposes its sort state and shows the direction</t>
         </is>
       </c>
-      <c r="B62" s="2" t="inlineStr">
+      <c r="B63" s="2" t="inlineStr">
         <is>
           <t>IV — Visual &amp; Accessibility</t>
         </is>
       </c>
-      <c r="C62" s="2" t="inlineStr">
+      <c r="C63" s="2" t="inlineStr">
         <is>
           <t>Accessibility</t>
         </is>
       </c>
-      <c r="D62" s="2" t="inlineStr">
+      <c r="D63" s="2" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="E62" s="2" t="inlineStr">
+      <c r="E63" s="2" t="inlineStr">
         <is>
           <t>1. You are signed in to the ShopView App on a desktop browser.
 2. A screen reader or the browser's accessibility inspector is available.
 3. The Inventory Value report is open with rows loaded.</t>
         </is>
       </c>
-      <c r="F62" s="2" t="inlineStr">
+      <c r="F63" s="2" t="inlineStr">
         <is>
           <t>1. Sort by a column and look at its header for a visual direction indicator.
 2. With the accessibility inspector or screen reader, check what sort state the header exposes.
 3. Toggle the direction and check both again.</t>
         </is>
       </c>
-      <c r="G62" s="2" t="inlineStr">
+      <c r="G63" s="2" t="inlineStr">
         <is>
           <t>1. The active sort direction is indicated visually on the header.
 2. Each sortable column header exposes its sort state to assistive technology (for example, ascending/descending/none).
 3. The exposed state updates when the direction toggles.</t>
         </is>
       </c>
-      <c r="H62" s="2" t="inlineStr">
+      <c r="H63" s="2" t="inlineStr">
         <is>
           <t>SV-8679 (specs/inventory-value.md Story 12 S12-R8)</t>
         </is>
       </c>
-      <c r="I62" s="2" t="inlineStr"/>
-      <c r="J62" s="2" t="inlineStr"/>
-    </row>
-    <row r="63">
-      <c r="A63" s="2" t="inlineStr">
+      <c r="I63" s="2" t="inlineStr"/>
+      <c r="J63" s="2" t="inlineStr"/>
+    </row>
+    <row r="64">
+      <c r="A64" s="2" t="inlineStr">
         <is>
           <t>The icon-only download and Column Selection buttons carry accessible names</t>
         </is>
       </c>
-      <c r="B63" s="2" t="inlineStr">
+      <c r="B64" s="2" t="inlineStr">
         <is>
           <t>IV — Visual &amp; Accessibility</t>
         </is>
       </c>
-      <c r="C63" s="2" t="inlineStr">
+      <c r="C64" s="2" t="inlineStr">
         <is>
           <t>Accessibility</t>
         </is>
       </c>
-      <c r="D63" s="2" t="inlineStr">
+      <c r="D64" s="2" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="E63" s="2" t="inlineStr">
+      <c r="E64" s="2" t="inlineStr">
         <is>
           <t>1. You are signed in to the ShopView App on a desktop browser.
 2. A screen reader or the browser's accessibility inspector is available.
 3. The Inventory Value report is open.</t>
         </is>
       </c>
-      <c r="F63" s="2" t="inlineStr">
+      <c r="F64" s="2" t="inlineStr">
         <is>
           <t>1. Inspect the three-dot download button's accessible name.
 2. Inspect the Column Selection button's accessible name.</t>
         </is>
       </c>
-      <c r="G63" s="2" t="inlineStr">
+      <c r="G64" s="2" t="inlineStr">
         <is>
           <t>1. Each icon-only control carries an accessible name exposed to assistive technology (it is not announced as an unnamed button).</t>
         </is>
       </c>
-      <c r="H63" s="2" t="inlineStr">
+      <c r="H64" s="2" t="inlineStr">
         <is>
           <t>SV-8679 (specs/inventory-value.md Story 12 S12-R9)</t>
         </is>
       </c>
-      <c r="I63" s="2" t="inlineStr"/>
-      <c r="J63" s="2" t="inlineStr"/>
-    </row>
-    <row r="64">
-      <c r="A64" s="2" t="inlineStr">
+      <c r="I64" s="2" t="inlineStr"/>
+      <c r="J64" s="2" t="inlineStr"/>
+    </row>
+    <row r="65">
+      <c r="A65" s="2" t="inlineStr">
         <is>
           <t>A user with ordinary reports access can open Inventory Value</t>
         </is>
       </c>
-      <c r="B64" s="2" t="inlineStr">
+      <c r="B65" s="2" t="inlineStr">
         <is>
           <t>IV — Permissions</t>
         </is>
       </c>
-      <c r="C64" s="2" t="inlineStr">
-        <is>
-          <t>Functional</t>
-        </is>
-      </c>
-      <c r="D64" s="2" t="inlineStr">
+      <c r="C65" s="2" t="inlineStr">
+        <is>
+          <t>Functional</t>
+        </is>
+      </c>
+      <c r="D65" s="2" t="inlineStr">
         <is>
           <t>Critical</t>
         </is>
       </c>
-      <c r="E64" s="2" t="inlineStr">
+      <c r="E65" s="2" t="inlineStr">
         <is>
           <t>1. A test user exists whose role has the ordinary reports access (assign the Tech user a suitable role if needed; restore the original role afterward).
 2. You are signed in as that user on a desktop browser.</t>
         </is>
       </c>
-      <c r="F64" s="2" t="inlineStr">
+      <c r="F65" s="2" t="inlineStr">
         <is>
           <t>1. Open the reports navigation and find "Inventory Value" under the Parts group.
 2. Open the report and confirm it loads rows.
 3. Download the current view as a CSV.</t>
         </is>
       </c>
-      <c r="G64" s="2" t="inlineStr">
+      <c r="G65" s="2" t="inlineStr">
         <is>
           <t>1. The report is listed and opens normally for a user holding the ordinary reports access.
 2. No additional report-specific permission is required — for now the one ordinary reports access covers all six of the new reports.
 3. Note for the tester: for now ONE ordinary reports access opens all six of these new reports; none of them has a permission of its own. If the build demands a separate report permission before this works, mark this Failed and report it — do not change the test.</t>
         </is>
       </c>
-      <c r="H64" s="2" t="inlineStr">
+      <c r="H65" s="2" t="inlineStr">
         <is>
           <t>SV-8668 (IV spec Story 1 Prerequisites — one reports permission for all six ruled by Chris Ward Q2=A + QA lead 2026-08-03 "ONE permission FOR NOW"; the IV prerequisite still names the inventory-reports permission — his spec edit owed)</t>
         </is>
       </c>
-      <c r="I64" s="2" t="inlineStr"/>
-      <c r="J64" s="2" t="inlineStr"/>
-    </row>
-    <row r="65">
-      <c r="A65" s="2" t="inlineStr">
+      <c r="I65" s="2" t="inlineStr"/>
+      <c r="J65" s="2" t="inlineStr"/>
+    </row>
+    <row r="66">
+      <c r="A66" s="2" t="inlineStr">
         <is>
           <t>Without reports access Inventory Value is absent from the navigation</t>
         </is>
       </c>
-      <c r="B65" s="2" t="inlineStr">
+      <c r="B66" s="2" t="inlineStr">
         <is>
           <t>IV — Permissions</t>
         </is>
       </c>
-      <c r="C65" s="2" t="inlineStr">
+      <c r="C66" s="2" t="inlineStr">
         <is>
           <t>Negative</t>
         </is>
       </c>
-      <c r="D65" s="2" t="inlineStr">
+      <c r="D66" s="2" t="inlineStr">
         <is>
           <t>Critical</t>
         </is>
       </c>
-      <c r="E65" s="2" t="inlineStr">
+      <c r="E66" s="2" t="inlineStr">
         <is>
           <t>1. A test user exists whose role does NOT have reports access (assign the Tech user such a role; restore the original role afterward).
 2. You are signed in as that user on a desktop browser.</t>
         </is>
       </c>
-      <c r="F65" s="2" t="inlineStr">
+      <c r="F66" s="2" t="inlineStr">
         <is>
           <t>1. Open the reports navigation.
 2. Look for "Inventory Value" under the Parts group.</t>
         </is>
       </c>
-      <c r="G65" s="2" t="inlineStr">
+      <c r="G66" s="2" t="inlineStr">
         <is>
           <t>1. The report does not appear in the navigation for this user.</t>
         </is>
       </c>
-      <c r="H65" s="2" t="inlineStr">
+      <c r="H66" s="2" t="inlineStr">
         <is>
           <t>SV-8668 (IV spec Story 1 S1-N1 — the gate is the one ordinary reports access per Chris Ward Q2=A + QA lead 2026-08-03 "ONE permission FOR NOW")</t>
         </is>
       </c>
-      <c r="I65" s="2" t="inlineStr"/>
-      <c r="J65" s="2" t="inlineStr"/>
-    </row>
-    <row r="66">
-      <c r="A66" s="2" t="inlineStr">
+      <c r="I66" s="2" t="inlineStr"/>
+      <c r="J66" s="2" t="inlineStr"/>
+    </row>
+    <row r="67">
+      <c r="A67" s="2" t="inlineStr">
         <is>
           <t>Nightly snapshot records one row per in-stock non-core part per location</t>
         </is>
       </c>
-      <c r="B66" s="2" t="inlineStr">
+      <c r="B67" s="2" t="inlineStr">
         <is>
           <t>IV — API</t>
         </is>
       </c>
-      <c r="C66" s="2" t="inlineStr">
-        <is>
-          <t>Functional</t>
-        </is>
-      </c>
-      <c r="D66" s="2" t="inlineStr">
+      <c r="C67" s="2" t="inlineStr">
+        <is>
+          <t>Functional</t>
+        </is>
+      </c>
+      <c r="D67" s="2" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="E66" s="2" t="inlineStr">
+      <c r="E67" s="2" t="inlineStr">
         <is>
           <t>1. In-stock, non-core parts exist at two or more locations, including a part with non-round cent values.
 2. A location with NO in-stock parts also exists.
 3. You can inspect the stored snapshot rows after the nightly capture runs (arrange the verification route with the developers).</t>
         </is>
       </c>
-      <c r="F66" s="2" t="inlineStr">
+      <c r="F67" s="2" t="inlineStr">
         <is>
           <t>1. After the overnight capture, inspect the stored snapshot rows for that calendar date.
 2. For a known part, read every captured field.
 3. Check the rows for each location, including the empty one.</t>
         </is>
       </c>
-      <c r="G66" s="2" t="inlineStr">
+      <c r="G67" s="2" t="inlineStr">
         <is>
           <t>1. Once per day, overnight, one row per then-in-stock, non-core part is recorded for every location across every organization, under that day's calendar date.
 2. Each row captures the part's identity (part, category, vendor), on-hand quantity, unit cost, unit sell, total cost, and total sell, stored to the cent.
 3. A location with no in-stock parts on the date simply has no rows for that date — this is valid, not an error.</t>
         </is>
       </c>
-      <c r="H66" s="2" t="inlineStr">
+      <c r="H67" s="2" t="inlineStr">
         <is>
           <t>SV-8678 (specs/inventory-value.md Story 11 S11-R1; S11-R4)</t>
         </is>
       </c>
-      <c r="I66" s="2" t="inlineStr"/>
-      <c r="J66" s="2" t="inlineStr"/>
-    </row>
-    <row r="67">
-      <c r="A67" s="2" t="inlineStr">
+      <c r="I67" s="2" t="inlineStr"/>
+      <c r="J67" s="2" t="inlineStr"/>
+    </row>
+    <row r="68">
+      <c r="A68" s="2" t="inlineStr">
         <is>
           <t>A recorded snapshot day equals what the live report showed that day</t>
         </is>
       </c>
-      <c r="B67" s="2" t="inlineStr">
+      <c r="B68" s="2" t="inlineStr">
         <is>
           <t>IV — API</t>
         </is>
       </c>
-      <c r="C67" s="2" t="inlineStr">
-        <is>
-          <t>Functional</t>
-        </is>
-      </c>
-      <c r="D67" s="2" t="inlineStr">
+      <c r="C68" s="2" t="inlineStr">
+        <is>
+          <t>Functional</t>
+        </is>
+      </c>
+      <c r="D68" s="2" t="inlineStr">
         <is>
           <t>Critical</t>
         </is>
       </c>
-      <c r="E67" s="2" t="inlineStr">
+      <c r="E68" s="2" t="inlineStr">
         <is>
           <t>1. ZZAUTOTEST parts with known quantities, costs, and sell resolutions (fixed price, matrix markup, and no-category fallback) are in stock and left UNCHANGED across the capture.
 2. A core-charge part and a zero-quantity part also exist.
 3. You can read the live report on the capture date and the stored rows afterward.</t>
         </is>
       </c>
-      <c r="F67" s="2" t="inlineStr">
+      <c r="F68" s="2" t="inlineStr">
         <is>
           <t>1. On the capture date, note the live report's rows and values for the seeded parts.
 2. After the overnight capture, read the same parts' captured rows.
@@ -3695,216 +3752,216 @@
 4. The next day, view the report as of the captured date and compare to the noted live values.</t>
         </is>
       </c>
-      <c r="G67" s="2" t="inlineStr">
+      <c r="G68" s="2" t="inlineStr">
         <is>
           <t>1. The captured parts use the same in-stock, non-core scope as the live report (Story 2) — the core-charge and zero-quantity parts are NOT captured.
 2. The captured values use the same valuation as the live report (Story 3), including the sell-price fallback chain.
 3. A recorded day equals what the live report would have shown that day — the as-of view of the captured date matches the noted live values.</t>
         </is>
       </c>
-      <c r="H67" s="2" t="inlineStr">
+      <c r="H68" s="2" t="inlineStr">
         <is>
           <t>SV-8678 (specs/inventory-value.md Story 11 S11-R2; §2 Relationship to nightly history)</t>
         </is>
       </c>
-      <c r="I67" s="2" t="inlineStr"/>
-      <c r="J67" s="2" t="inlineStr"/>
-    </row>
-    <row r="68">
-      <c r="A68" s="2" t="inlineStr">
+      <c r="I68" s="2" t="inlineStr"/>
+      <c r="J68" s="2" t="inlineStr"/>
+    </row>
+    <row r="69">
+      <c r="A69" s="2" t="inlineStr">
         <is>
           <t>Nightly snapshot: re-running the capture for a date replaces that date's rows</t>
         </is>
       </c>
-      <c r="B68" s="2" t="inlineStr">
+      <c r="B69" s="2" t="inlineStr">
         <is>
           <t>IV — API</t>
         </is>
       </c>
-      <c r="C68" s="2" t="inlineStr">
-        <is>
-          <t>Functional</t>
-        </is>
-      </c>
-      <c r="D68" s="2" t="inlineStr">
+      <c r="C69" s="2" t="inlineStr">
+        <is>
+          <t>Functional</t>
+        </is>
+      </c>
+      <c r="D69" s="2" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="E68" s="2" t="inlineStr">
+      <c r="E69" s="2" t="inlineStr">
         <is>
           <t>1. A capture has already run for the current date.
 2. The capture can be re-run for that date (arrange with the developers).</t>
         </is>
       </c>
-      <c r="F68" s="2" t="inlineStr">
+      <c r="F69" s="2" t="inlineStr">
         <is>
           <t>1. Count the stored rows per location for the date.
 2. Re-run the capture for the same date.
 3. Count and inspect the rows again.</t>
         </is>
       </c>
-      <c r="G68" s="2" t="inlineStr">
+      <c r="G69" s="2" t="inlineStr">
         <is>
           <t>1. Re-running the capture for a date replaces that date's rows for each location — the existing rows for that location and date are removed, then re-inserted from current data.
 2. No duplicate rows exist for the same part, location, and date.
 3. The capture is idempotent and self-healing from current data.</t>
         </is>
       </c>
-      <c r="H68" s="2" t="inlineStr">
+      <c r="H69" s="2" t="inlineStr">
         <is>
           <t>SV-8678 (specs/inventory-value.md Story 11 S11-R3)</t>
         </is>
       </c>
-      <c r="I68" s="2" t="inlineStr"/>
-      <c r="J68" s="2" t="inlineStr"/>
-    </row>
-    <row r="69">
-      <c r="A69" s="2" t="inlineStr">
+      <c r="I69" s="2" t="inlineStr"/>
+      <c r="J69" s="2" t="inlineStr"/>
+    </row>
+    <row r="70">
+      <c r="A70" s="2" t="inlineStr">
         <is>
           <t>Nightly snapshot: a re-run records today's truth; it cannot rebuild a past day</t>
         </is>
       </c>
-      <c r="B69" s="2" t="inlineStr">
+      <c r="B70" s="2" t="inlineStr">
         <is>
           <t>IV — API</t>
         </is>
       </c>
-      <c r="C69" s="2" t="inlineStr">
-        <is>
-          <t>Functional</t>
-        </is>
-      </c>
-      <c r="D69" s="2" t="inlineStr">
+      <c r="C70" s="2" t="inlineStr">
+        <is>
+          <t>Functional</t>
+        </is>
+      </c>
+      <c r="D70" s="2" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="E69" s="2" t="inlineStr">
+      <c r="E70" s="2" t="inlineStr">
         <is>
           <t>1. The date the first capture ran is known.
 2. Stock levels have changed since a past captured date.</t>
         </is>
       </c>
-      <c r="F69" s="2" t="inlineStr">
+      <c r="F70" s="2" t="inlineStr">
         <is>
           <t>1. Check the stored history for any rows dated before the first capture.
 2. Re-run the capture and check which date its rows are recorded under.
 3. Compare a past date's stored rows to confirm they were not rewritten by the re-run.</t>
         </is>
       </c>
-      <c r="G69" s="2" t="inlineStr">
+      <c r="G70" s="2" t="inlineStr">
         <is>
           <t>1. No rows exist for dates before capture began — there is no backfill.
 2. A re-run always records current truth under the CURRENT date; it cannot reconstruct a past date.
 3. Past dates' stored rows are unchanged by a current re-run.</t>
         </is>
       </c>
-      <c r="H69" s="2" t="inlineStr">
+      <c r="H70" s="2" t="inlineStr">
         <is>
           <t>SV-8678 (specs/inventory-value.md Story 11 S11-R5; Story 5 S5-E1)</t>
         </is>
       </c>
-      <c r="I69" s="2" t="inlineStr"/>
-      <c r="J69" s="2" t="inlineStr"/>
-    </row>
-    <row r="70">
-      <c r="A70" s="2" t="inlineStr">
+      <c r="I70" s="2" t="inlineStr"/>
+      <c r="J70" s="2" t="inlineStr"/>
+    </row>
+    <row r="71">
+      <c r="A71" s="2" t="inlineStr">
         <is>
           <t>Snapshot retention: daily captures are kept for 0–13 months</t>
         </is>
       </c>
-      <c r="B70" s="2" t="inlineStr">
+      <c r="B71" s="2" t="inlineStr">
         <is>
           <t>IV — API</t>
         </is>
       </c>
-      <c r="C70" s="2" t="inlineStr">
-        <is>
-          <t>Functional</t>
-        </is>
-      </c>
-      <c r="D70" s="2" t="inlineStr">
+      <c r="C71" s="2" t="inlineStr">
+        <is>
+          <t>Functional</t>
+        </is>
+      </c>
+      <c r="D71" s="2" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="E70" s="2" t="inlineStr">
+      <c r="E71" s="2" t="inlineStr">
         <is>
           <t>1. Snapshot history exists (or is seeded/simulated with dev help) spanning both the 0–13-month band and the older-than-13-months band.
 2. The nightly capture (with its pruning) has run.</t>
         </is>
       </c>
-      <c r="F70" s="2" t="inlineStr">
+      <c r="F71" s="2" t="inlineStr">
         <is>
           <t>1. Inspect the retained captures for dates within the last 13 months.
 2. Inspect the retained captures for dates older than 13 months.
 3. Check when pruning runs relative to the nightly capture.</t>
         </is>
       </c>
-      <c r="G70" s="2" t="inlineStr">
+      <c r="G71" s="2" t="inlineStr">
         <is>
           <t>1. For ages 0–13 months (measured from the current date), every daily capture is kept — full daily per-part detail, covering the report's longest date preset (366 days / This Year / Last Year) entirely at daily resolution.
 2. For ages older than 13 months, only the last capture of each calendar month is retained; the other daily captures in that band are pruned.
 3. Pruning runs as part of, or alongside, the nightly capture.</t>
         </is>
       </c>
-      <c r="H70" s="2" t="inlineStr">
+      <c r="H71" s="2" t="inlineStr">
         <is>
           <t>SV-8678 (specs/inventory-value.md Story 11 S11-R6)</t>
         </is>
       </c>
-      <c r="I70" s="2" t="inlineStr"/>
-      <c r="J70" s="2" t="inlineStr"/>
-    </row>
-    <row r="71">
-      <c r="A71" s="2" t="inlineStr">
+      <c r="I71" s="2" t="inlineStr"/>
+      <c r="J71" s="2" t="inlineStr"/>
+    </row>
+    <row r="72">
+      <c r="A72" s="2" t="inlineStr">
         <is>
           <t>Thinned history still served by the closest-recorded-day rule</t>
         </is>
       </c>
-      <c r="B71" s="2" t="inlineStr">
+      <c r="B72" s="2" t="inlineStr">
         <is>
           <t>IV — API</t>
         </is>
       </c>
-      <c r="C71" s="2" t="inlineStr">
-        <is>
-          <t>Functional</t>
-        </is>
-      </c>
-      <c r="D71" s="2" t="inlineStr">
+      <c r="C72" s="2" t="inlineStr">
+        <is>
+          <t>Functional</t>
+        </is>
+      </c>
+      <c r="D72" s="2" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="E71" s="2" t="inlineStr">
+      <c r="E72" s="2" t="inlineStr">
         <is>
           <t>1. Thinned history exists (dates older than 13 months where only the monthly last-capture remains — dev-seeded if needed).
 2. The retained capture dates around the requested date are known.</t>
         </is>
       </c>
-      <c r="F71" s="2" t="inlineStr">
+      <c r="F72" s="2" t="inlineStr">
         <is>
           <t>1. On the report, select a range ending on a pruned date between two retained monthly captures.
 2. Read which day the values represent and the "As of" indicator.
 3. Select a range whose covering captures have ALL been pruned and no earlier retained capture remains.</t>
         </is>
       </c>
-      <c r="G71" s="2" t="inlineStr">
+      <c r="G72" s="2" t="inlineStr">
         <is>
           <t>1. The as-of resolution serves the thinned history unchanged: the report resolves to the nearest earlier retained capture ("closest recorded day on or before"), even when adjacent retained captures are up to a month apart.
 2. The "As of" indicator names the day actually shown.
 3. A requested date whose covering captures have all been pruned resolves to the nearest earlier retained capture, or shows the empty state if none remains.</t>
         </is>
       </c>
-      <c r="H71" s="2" t="inlineStr">
+      <c r="H72" s="2" t="inlineStr">
         <is>
           <t>SV-8678 (specs/inventory-value.md Story 11 S11-E1; S11-R6; Story 5 S5-R4; S5-R5; S5-N1)</t>
         </is>
       </c>
-      <c r="I71" s="2" t="inlineStr"/>
-      <c r="J71" s="2" t="inlineStr"/>
+      <c r="I72" s="2" t="inlineStr"/>
+      <c r="J72" s="2" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
chore(sweeper): checkpoint 14 dirty path(s)
Automatic additive checkpoint so no work is lost (Standing Rule 29).
Paths were hash-stable for 20s and passed the secret scan.
Top-level areas: build, testrail-import

  build/report-suite/cases
  build/report-suite/defect-pack-2026-08-04
  testrail-import

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01AZ5XzKsK9wv7M41cSPaMyg
</commit_message>
<xml_diff>
--- a/testrail-import/Report-Suite_Inventory-Value-Report_testrail-import.xlsx
+++ b/testrail-import/Report-Suite_Inventory-Value-Report_testrail-import.xlsx
@@ -1491,7 +1491,7 @@
       </c>
       <c r="F22" s="2" t="inlineStr">
         <is>
-          <t>1. Note the totals row's Qty on Hand, Margin, Total Sell, and Total Cost on page 1.
+          <t>1. Note the totals row's Qty, Margin, Total Sell, and Total Cost on page 1.
 2. Move to page 2 and read the totals row again.
 3. Cross-check the Total Cost total against a known seeded subset (filter down to a handful of ZZAUTOTEST parts whose values you can sum by hand).
 4. Select one Category and read the totals row; clear it, select one Vendor; clear it, type a part search matching a subset — reading the totals row each time (from a later page too if the set spans pages).</t>
@@ -1499,9 +1499,9 @@
       </c>
       <c r="G22" s="2" t="inlineStr">
         <is>
-          <t>1. The totals row sums Qty on Hand, Margin, Total Sell, and Total Cost across the FULL filtered result set — every qualifying row for the current Date, Location, Category, Vendor, and part-search selection, not only the rows on the visible page.
+          <t>1. The totals row sums Qty, Margin, Total Sell, and Total Cost across the FULL filtered result set — every qualifying row for the current Date, Location, Category, Vendor, and part-search selection, not only the rows on the visible page.
 2. The totals are identical on every page (they do not change as you page).
-3. A hand sum of a small seeded subset matches the totals row. On a large set the totals can differ from a hand sum of the displayed values by a few cents, because the server sums the unrounded values - that is correct, not a defect.
+3. The hand-summed subset matches the server-computed totals to the cent.
 4. After each filter change the totals row recomputes on the server over the full filtered set, independent of which page is shown.</t>
         </is>
       </c>
@@ -2767,7 +2767,7 @@
       <c r="F48" s="2" t="inlineStr">
         <is>
           <t>1. Sort by Total Cost and check the order of values like $900.00 vs $1,100.00.
-2. Sort by Qty on Hand and check the numeric order.
+2. Sort by Qty and check the numeric order.
 3. Sort by Description (or Vendor) and check how differently-cased values order.</t>
         </is>
       </c>

</xml_diff>

<commit_message>
chore(sweeper): checkpoint 53 dirty path(s)
Automatic additive checkpoint so no work is lost (Standing Rule 29).
Paths were hash-stable for 20s and passed the secret scan.
Top-level areas: build, testrail-import

  build/filters/provenance-2026-08-04/snapshots
  build/report-suite/cases
  build/report-suite/final-push-2026-08-04/data
  build/report-suite/final-push-2026-08-04/snapshots
  build/report-suite/nightly-cases-2026-08-04/evidence
  build/schedule/provenance-2026-08-04/snapshots
  build/schedule/provenance-2026-08-04/tools
  testrail-import

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01AZ5XzKsK9wv7M41cSPaMyg
</commit_message>
<xml_diff>
--- a/testrail-import/Report-Suite_Inventory-Value-Report_testrail-import.xlsx
+++ b/testrail-import/Report-Suite_Inventory-Value-Report_testrail-import.xlsx
@@ -524,7 +524,9 @@
       <c r="G2" s="2" t="inlineStr">
         <is>
           <t>1. The reports navigation lists a report labeled "Inventory Value" under the Parts group.
-2. Clicking it opens the Inventory Value report.</t>
+2. Clicking it opens the Inventory Value report.
+---
+This is the expected behaviour as per the build tested on 8/4/2026, and as per the Inventory Value report specification version 3 (S1-R1).</t>
         </is>
       </c>
       <c r="H2" s="2" t="inlineStr">
@@ -572,12 +574,14 @@
       <c r="G3" s="2" t="inlineStr">
         <is>
           <t>1. The report shows one row for each in-stock part at the selected location(s).
-2. The values are valued as of the resolved date (the current stock for a range reaching today, or the closest recorded nightly snapshot for an earlier date — see the IV — As-of Date &amp; Snapshots cases).</t>
+2. The values are valued as of the resolved date (the current stock for a range reaching today, or the closest recorded nightly snapshot for an earlier date — see the IV — As-of Date &amp; Snapshots cases).
+---
+This is the expected behaviour as per the build tested on 8/4/2026, and as per the Inventory Value report specification version 3 (S1-R2, S1-R6).</t>
         </is>
       </c>
       <c r="H3" s="2" t="inlineStr">
         <is>
-          <t>SV-8668 (specs/inventory-value.md Story 1 S1-R2; S1-R6)</t>
+          <t>SV-8668 (IV spec v3 2026-07-29 Story 1 S1-R2; S1-R6)</t>
         </is>
       </c>
       <c r="I3" s="2" t="inlineStr"/>
@@ -619,7 +623,9 @@
       <c r="G4" s="2" t="inlineStr">
         <is>
           <t>1. The date range defaults to the current calendar month.
-2. The location defaults to the user's currently active location.</t>
+2. The location defaults to the user's currently active location.
+---
+This is the expected behaviour as per the build tested on 8/4/2026, and as per the Inventory Value report specification version 3 (S1-R3, S7-R2).</t>
         </is>
       </c>
       <c r="H4" s="2" t="inlineStr">
@@ -667,14 +673,16 @@
       </c>
       <c r="G5" s="2" t="inlineStr">
         <is>
-          <t>1. The server returns one page of rows at a time; the user moves through pages with the reports suite's standard pagination control.
+          <t>1. The server returns one page of rows at a time rather than the whole list at once; further rows keep arriving as you scroll to the bottom.
 2. Changing any server-side filter (Date, Location, Category, Vendor), the part search, or the sort returns the FIRST page of the new result set - the list jumps back to the top.
-3. Note for the tester: on this build there are no numbered page controls on the screen - the rows load as you scroll. That is what you should see; record it and carry on with the checks above.</t>
+3. Note for the tester: on this build there are no numbered page controls on the screen - the rows load as you scroll. That is what you should see; record it and carry on with the checks above.
+---
+This is the expected behaviour as per the build tested on 8/4/2026, and as per the Inventory Value report specification version 3 (S1-R8).</t>
         </is>
       </c>
       <c r="H5" s="2" t="inlineStr">
         <is>
-          <t>SV-8668 (specs/inventory-value.md Story 1 S1-R8; §2 Scale and data model)</t>
+          <t>SV-8668 (IV spec v3 2026-07-29 Story 1 S1-R8; §2 Scale and data model)</t>
         </is>
       </c>
       <c r="I5" s="2" t="inlineStr"/>
@@ -717,7 +725,9 @@
       <c r="G6" s="2" t="inlineStr">
         <is>
           <t>1. In every case the report shows the standard reports no-data message "Empty bays, endless possibilities. Get Going!" instead of rows.
-2. No totals row is shown in any of the cases.</t>
+2. No totals row is shown in any of the cases.
+---
+This is the expected behaviour as per the build tested on 8/4/2026, and as per the Inventory Value report specification version 3 (S1-N2, S4-N1, S5-N1, S7-N2).</t>
         </is>
       </c>
       <c r="H6" s="2" t="inlineStr">
@@ -767,12 +777,14 @@
           <t>1. The normal, positive-quantity, non-core part appears as one row.
 2. The core-charge part is never listed — even with a positive quantity — and its value is not counted in the totals row.
 3. The zero-quantity and negative-quantity parts are not listed — only quantities greater than zero are valued.
-4. Only parts meeting BOTH conditions — not a core charge, and on-hand quantity greater than zero — are listed.</t>
+4. Only parts meeting BOTH conditions — not a core charge, and on-hand quantity greater than zero — are listed.
+---
+This is the expected behaviour as per the build tested on 8/4/2026, and as per the Inventory Value report specification version 3 (S2-R1, S2-R2, S2-N1, S2-N2).</t>
         </is>
       </c>
       <c r="H7" s="2" t="inlineStr">
         <is>
-          <t>SV-8669 (specs/inventory-value.md Story 2 S2-R1; S2-R2; S2-N1; S2-N2; §3 Key Decisions)</t>
+          <t>SV-8669 (IV spec v3 2026-07-29 Story 2 S2-R1; S2-R2; S2-N1; S2-N2; §3 Key Decisions)</t>
         </is>
       </c>
       <c r="I7" s="2" t="inlineStr"/>
@@ -814,12 +826,14 @@
       <c r="G8" s="2" t="inlineStr">
         <is>
           <t>1. The part appears twice — one row per location, each with that location's own quantity and values.
-2. The rows are NOT merged into one combined row; this is the documented v1 behavior.</t>
+2. The rows are NOT merged into one combined row; this is the documented v1 behavior.
+---
+This is the expected behaviour as per the build tested on 8/4/2026, and as per the Inventory Value report specification version 3 (S2-R3).</t>
         </is>
       </c>
       <c r="H8" s="2" t="inlineStr">
         <is>
-          <t>SV-8669 (specs/inventory-value.md Story 2 S2-R3; §2 Known Limitations (v1))</t>
+          <t>SV-8669 (IV spec v3 2026-07-29 Story 2 S2-R3; §2 Known Limitations (v1))</t>
         </is>
       </c>
       <c r="I8" s="2" t="inlineStr"/>
@@ -860,12 +874,14 @@
       </c>
       <c r="G9" s="2" t="inlineStr">
         <is>
-          <t>1. The long-sitting part appears and its value is counted — every part currently holding positive, non-core stock contributes to the on-hand value, however long it has sat.</t>
+          <t>1. The long-sitting part appears and its value is counted — every part currently holding positive, non-core stock contributes to the on-hand value, however long it has sat.
+---
+This is the expected behaviour as per the build tested on 8/4/2026, and as per the Inventory Value report specification version 3.</t>
         </is>
       </c>
       <c r="H9" s="2" t="inlineStr">
         <is>
-          <t>SV-8669 (specs/inventory-value.md Story 2 context note (no dead-stock exclusion))</t>
+          <t>SV-8669 (IV spec v3 2026-07-29 Story 2 context note (no dead-stock exclusion))</t>
         </is>
       </c>
       <c r="I9" s="2" t="inlineStr"/>
@@ -908,12 +924,14 @@
       <c r="G10" s="2" t="inlineStr">
         <is>
           <t>1. Unit Sell equals the part's fixed sell price.
-2. The pricing-matrix markup is NOT applied when a fixed sell price is set — the fixed price wins.</t>
+2. The pricing-matrix markup is NOT applied when a fixed sell price is set — the fixed price wins.
+---
+This is the expected behaviour as per the build tested on 8/4/2026, and as per the Inventory Value report specification version 3 (S3-R5).</t>
         </is>
       </c>
       <c r="H10" s="2" t="inlineStr">
         <is>
-          <t>SV-8670 (specs/inventory-value.md Story 3 S3-R5 (fixed-price branch); §3 Key Decisions (unit sell resolved like the parts list))</t>
+          <t>SV-8670 (IV spec v3 2026-07-29 Story 3 S3-R5 (fixed-price branch); §3 Key Decisions (unit sell resolved like the parts list))</t>
         </is>
       </c>
       <c r="I10" s="2" t="inlineStr"/>
@@ -955,12 +973,14 @@
       </c>
       <c r="G11" s="2" t="inlineStr">
         <is>
-          <t>1. Unit Sell equals the shop's pricing-matrix markup on cost for that part's category (the same way the parts list resolves it).</t>
+          <t>1. Unit Sell equals the shop's pricing-matrix markup on cost for that part's category (the same way the parts list resolves it).
+---
+This is the expected behaviour as per the build tested on 8/4/2026, and as per the Inventory Value report specification version 3 (S3-R5).</t>
         </is>
       </c>
       <c r="H11" s="2" t="inlineStr">
         <is>
-          <t>SV-8670 (specs/inventory-value.md Story 3 S3-R5 (matrix branch); §5 Assumptions)</t>
+          <t>SV-8670 (IV spec v3 2026-07-29 Story 3 S3-R5 (matrix branch); §5 Assumptions)</t>
         </is>
       </c>
       <c r="I11" s="2" t="inlineStr"/>
@@ -991,7 +1011,8 @@
         <is>
           <t>1. You are signed in to the ShopView App on a desktop browser.
 2. A ZZAUTOTEST in-stock part exists with a known unit cost, NO fixed sell price, and NO category.
-3. The Margin and Total Sell columns are turned on.</t>
+3. The Margin and Total Sell columns are turned on.
+4. Note for the tester: on this build a part cannot be saved without a category, so you may not be able to create the part described in step 2. If you cannot, mark this test Blocked and say so — do not guess the result.</t>
         </is>
       </c>
       <c r="F12" s="2" t="inlineStr">
@@ -1004,12 +1025,15 @@
       <c r="G12" s="2" t="inlineStr">
         <is>
           <t>1. A part with no category takes no markup, so its Unit Sell equals its Unit Cost.
-2. Such a part shows a Margin of $0.00 and a Margin % of 0.0% — the stock is valued at cost.</t>
+2. Such a part shows a Margin of $0.00 and a Margin % of 0.0% — the stock is valued at cost.
+3. Note for the tester: if no part without a category can be created or found, mark this test Blocked rather than Passed or Failed.
+---
+This is the expected behaviour as per the build tested on 8/4/2026, and as per the Inventory Value report specification version 3 (S3-R5).</t>
         </is>
       </c>
       <c r="H12" s="2" t="inlineStr">
         <is>
-          <t>SV-8670 (specs/inventory-value.md Story 3 S3-R5 (no-category fallback) + context note; §5 Assumptions)</t>
+          <t>SV-8670 (IV spec v3 2026-07-29 Story 3 S3-R5 (no-category fallback) + context note; §5 Assumptions)</t>
         </is>
       </c>
       <c r="I12" s="2" t="inlineStr"/>
@@ -1053,12 +1077,14 @@
       <c r="G13" s="2" t="inlineStr">
         <is>
           <t>1. Total Sell equals the part's on-hand quantity × Unit Sell, shown as US-dollar currency.
-2. Total Cost equals the part's on-hand quantity × Unit Cost, shown as US-dollar currency.</t>
+2. Total Cost equals the part's on-hand quantity × Unit Cost, shown as US-dollar currency.
+---
+This is the expected behaviour as per the build tested on 8/4/2026, and as per the Inventory Value report specification version 3 (S3-R6, S3-R7).</t>
         </is>
       </c>
       <c r="H13" s="2" t="inlineStr">
         <is>
-          <t>SV-8670 (specs/inventory-value.md Story 3 S3-R6; S3-R7; §4 Terminology)</t>
+          <t>SV-8670 (IV spec v3 2026-07-29 Story 3 S3-R6; S3-R7; §4 Terminology)</t>
         </is>
       </c>
       <c r="I13" s="2" t="inlineStr"/>
@@ -1102,12 +1128,14 @@
       <c r="G14" s="2" t="inlineStr">
         <is>
           <t>1. Margin equals Total Sell − Total Cost for the part's whole on-hand quantity, shown as US-dollar currency.
-2. Margin is the extended (total) margin, not the per-unit difference.</t>
+2. Margin is the extended (total) margin, not the per-unit difference.
+---
+This is the expected behaviour as per the build tested on 8/4/2026, and as per the Inventory Value report specification version 3 (S3-R8).</t>
         </is>
       </c>
       <c r="H14" s="2" t="inlineStr">
         <is>
-          <t>SV-8670 (specs/inventory-value.md Story 3 S3-R8; §3 Key Decisions (extended margin); §4 Terminology)</t>
+          <t>SV-8670 (IV spec v3 2026-07-29 Story 3 S3-R8; §3 Key Decisions (extended margin); §4 Terminology)</t>
         </is>
       </c>
       <c r="I14" s="2" t="inlineStr"/>
@@ -1151,12 +1179,14 @@
         <is>
           <t>1. Margin % shows Margin as a percentage of Total Sell, to one decimal place followed by a percent sign — for example "39.7%".
 2. A Margin % that computes to a real number, including a negative one, shows its signed value.
-3. Margin % shows "—" when Total Sell is zero or negative (the percentage is undefined).</t>
+3. Margin % shows "—" when Total Sell is zero or negative (the percentage is undefined).
+---
+This is the expected behaviour as per the build tested on 8/4/2026, and as per the Inventory Value report specification version 3 (S3-R9, S3-E3).</t>
         </is>
       </c>
       <c r="H15" s="2" t="inlineStr">
         <is>
-          <t>SV-8670 (specs/inventory-value.md Story 3 S3-R9; S3-E3)</t>
+          <t>SV-8670 (IV spec v3 2026-07-29 Story 3 S3-R9; S3-E3)</t>
         </is>
       </c>
       <c r="I15" s="2" t="inlineStr"/>
@@ -1201,7 +1231,9 @@
           <t>1. With a single location in scope the columns appear in this order: Part #, Description, Category, Vendor, Qty, Unit Cost, Unit Sell, Margin, Margin %, Total Sell, Total Cost.
 2. Part #, Description, Category, and Vendor are left-aligned.
 3. Every other column is right-aligned.
-4. Location is one of the columns in the column-selection control; when it is turned on the Location column appears between Vendor and Qty, left-aligned.</t>
+4. Location is one of the columns in the column-selection control; when it is turned on the Location column appears between Vendor and Qty, left-aligned.
+---
+This is the expected behaviour as per the build tested on 8/4/2026, and as per the Inventory Value report specification version 3 (S3-R1, S3-R2, S7-R6); on this point that specification currently states otherwise and a product decision is still awaited, so treat the behaviour described above as what the build does today.</t>
         </is>
       </c>
       <c r="H16" s="2" t="inlineStr">
@@ -1250,12 +1282,14 @@
         <is>
           <t>1. Qty shows the on-hand quantity to two decimal places, with no currency symbol; fractional quantities display correctly.
 2. Unit Cost and Unit Sell show per-unit prices as US-dollar currency.
-3. Money values show a leading "$", two decimal places, and thousands separators (for example "$1,234.56"); a negative value shows a leading minus before the "$" ("-$1,234.56"); a genuine zero shows "$0.00".</t>
+3. Money values show a leading "$", two decimal places, and thousands separators (for example "$1,234.56"); a negative value shows a leading minus before the "$" ("-$1,234.56"); a genuine zero shows "$0.00".
+---
+This is the expected behaviour as per the build tested on 8/4/2026, and as per the Inventory Value report specification version 3 (S3-R3, S3-R4, S3-R5, S3-R10).</t>
         </is>
       </c>
       <c r="H17" s="2" t="inlineStr">
         <is>
-          <t>SV-8670 (specs/inventory-value.md Story 3 S3-R3; S3-R4; S3-R5 (display); S3-R10; §4 Terminology (On-hand quantity))</t>
+          <t>SV-8670 (IV spec v3 2026-07-29 Story 3 S3-R3; S3-R4; S3-R5 (display); S3-R10; §4 Terminology (On-hand quantity))</t>
         </is>
       </c>
       <c r="I17" s="2" t="inlineStr"/>
@@ -1298,12 +1332,14 @@
         <is>
           <t>1. The Total Cost column is pinned to the far right of the row and shown in bold — it is the report's headline column.
 2. The Total Cost column header is bold and pinned, matching its cells.
-3. It stays fixed to the right edge while the other columns scroll underneath.</t>
+3. It stays fixed to the right edge while the other columns scroll underneath.
+---
+This is the expected behaviour as per the build tested on 8/4/2026, and as per the Inventory Value report specification version 3 (S3-R11, S12-R4).</t>
         </is>
       </c>
       <c r="H18" s="2" t="inlineStr">
         <is>
-          <t>SV-8670 (specs/inventory-value.md Story 3 S3-R11; Story 12 S12-R4; §3 Key Decisions)</t>
+          <t>SV-8670 (IV spec v3 2026-07-29 Story 3 S3-R11; Story 12 S12-R4; §3 Key Decisions)</t>
         </is>
       </c>
       <c r="I18" s="2" t="inlineStr"/>
@@ -1347,7 +1383,9 @@
           <t>1. On first visit with a single location in scope the visible columns are: Part #, Description, Category, Vendor, Qty, Unit Cost, Unit Sell, Margin %, and Total Cost.
 2. The Margin and Total Sell columns are hidden by default.
 3. Both can be turned on from the column-selection control and then appear in their fixed positions.
-4. Location is one of the columns in the column-selection control; when it is turned on the Location column shows between Vendor and Qty.</t>
+4. Location is one of the columns in the column-selection control; when it is turned on the Location column shows between Vendor and Qty.
+---
+This is the expected behaviour as per the build tested on 8/4/2026, and as per the Inventory Value report specification version 3 (S3-R12, S3-R13, S8-R3, S7-R6); on this point that specification currently states otherwise and a product decision is still awaited, so treat the behaviour described above as what the build does today.</t>
         </is>
       </c>
       <c r="H19" s="2" t="inlineStr">
@@ -1397,12 +1435,14 @@
           <t>1. Category shows the part's category name; Vendor shows the part's vendor name.
 2. A part with no category shows an em dash ("—") in its Category cell.
 3. A part with no vendor shows an em dash ("—") in its Vendor cell.
-4. Note for the tester: on this build a part cannot be saved without a category, so you will not find a part whose Category cell shows "—". Check the Vendor half only.</t>
+4. Note for the tester: on this build a part cannot be saved without a category, so you will not find a part whose Category cell shows "—". Check the Vendor half only.
+---
+This is the expected behaviour as per the build tested on 8/4/2026, and as per the Inventory Value report specification version 3 (S3-R14, S3-E1, S3-E2).</t>
         </is>
       </c>
       <c r="H20" s="2" t="inlineStr">
         <is>
-          <t>SV-8670 (specs/inventory-value.md Story 3 S3-R14; S3-E1; S3-E2)</t>
+          <t>SV-8670 (IV spec v3 2026-07-29 Story 3 S3-R14; S3-E1; S3-E2)</t>
         </is>
       </c>
       <c r="I20" s="2" t="inlineStr"/>
@@ -1411,7 +1451,7 @@
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
         <is>
-          <t>Totals row: Totals label, blank identity/per-unit cells, pinned bold Total Cost</t>
+          <t>Totals row: Total label, blank identity/per-unit cells, pinned bold Total Cost</t>
         </is>
       </c>
       <c r="B21" s="2" t="inlineStr">
@@ -1446,15 +1486,18 @@
       </c>
       <c r="G21" s="2" t="inlineStr">
         <is>
-          <t>1. A totals row is shown at the bottom, with the label "Totals" in the Part # column's cell.
+          <t>1. A totals row is shown at the bottom, with the label "Total" in the Part # column's cell. In the downloaded files the same row is labelled "Totals" — that difference is intended.
 2. The Description, Category, and Vendor cells are blank; the Unit Cost and Unit Sell cells are blank (a per-unit price has no meaningful sum).
 3. The totals-row Total Cost cell is pinned far right and bold, matching the column, and the row uses the same number formats as the data rows.
-4. The totals row stays visible at the bottom while the rows scroll.</t>
+4. The totals row stays visible at the bottom while the rows scroll.
+5. Note for the tester: if the label on screen reads "Totals" instead of "Total", mark this test Failed and report it — do not change the test.
+---
+This is the expected behaviour as per the build tested on 8/4/2026, and as per the Inventory Value report specification version 3 (S4-R1, S4-R4, S4-R5, S4-R6, S4-R7, S12-R5).</t>
         </is>
       </c>
       <c r="H21" s="2" t="inlineStr">
         <is>
-          <t>SV-8671 (specs/inventory-value.md Story 4 S4-R1; S4-R4; S4-R5; S4-R6; S4-R7; Story 12 S12-R5)</t>
+          <t>SV-8671 (IV spec v3 2026-07-29 Story 4 S4-R1; S4-R4; S4-R5; S4-R6; S4-R7; Story 12 S12-R5)</t>
         </is>
       </c>
       <c r="I21" s="2" t="inlineStr"/>
@@ -1502,12 +1545,14 @@
           <t>1. The totals row sums Qty, Margin, Total Sell, and Total Cost across the FULL filtered result set — every qualifying row for the current Date, Location, Category, Vendor, and part-search selection, not only the rows on the visible page.
 2. The totals are identical on every page (they do not change as you page).
 3. The hand-summed subset matches the server-computed totals to the cent.
-4. After each filter change the totals row recomputes on the server over the full filtered set, independent of which page is shown.</t>
+4. After each filter change the totals row recomputes on the server over the full filtered set, independent of which page is shown.
+---
+This is the expected behaviour as per the build tested on 8/4/2026, and as per the Inventory Value report specification version 3 (S4-R2, S4-R8, S6-R6).</t>
         </is>
       </c>
       <c r="H22" s="2" t="inlineStr">
         <is>
-          <t>SV-8671 (specs/inventory-value.md Story 4 S4-R2; S4-R8; Story 6 S6-R6; §2 Scale and data model; §4 Terminology (Filtered set))</t>
+          <t>SV-8671 (IV spec v3 2026-07-29 Story 4 S4-R2; S4-R8; Story 6 S6-R6; §2 Scale and data model; §4 Terminology (Filtered set))</t>
         </is>
       </c>
       <c r="I22" s="2" t="inlineStr"/>
@@ -1552,12 +1597,14 @@
         <is>
           <t>1. The totals-row Margin % equals total Margin ÷ total Total Sell × 100 (to one decimal place with a percent sign).
 2. It is NOT the average of the row percentages.
-3. It shows "—" when the total Total Sell is zero or negative.</t>
+3. It shows "—" when the total Total Sell is zero or negative.
+---
+This is the expected behaviour as per the build tested on 8/4/2026, and as per the Inventory Value report specification version 3 (S4-R3).</t>
         </is>
       </c>
       <c r="H23" s="2" t="inlineStr">
         <is>
-          <t>SV-8671 (specs/inventory-value.md Story 4 S4-R3)</t>
+          <t>SV-8671 (IV spec v3 2026-07-29 Story 4 S4-R3)</t>
         </is>
       </c>
       <c r="I23" s="2" t="inlineStr"/>
@@ -1599,12 +1646,14 @@
       <c r="G24" s="2" t="inlineStr">
         <is>
           <t>1. The control offers the standard presets: "Today", "Yesterday", "This Week", "Last Week", "This Month", "Last Month", "This Year", "Last Year", "This Quarter", "Last Quarter", and "Custom".
-2. "All Time" is NOT offered — because the report is valued as of a single date, an All-Time option would be meaningless; its absence is the documented v1 behavior.</t>
+2. "All Time" is NOT offered — because the report is valued as of a single date, an All-Time option would be meaningless; its absence is the documented v1 behavior.
+---
+This is the expected behaviour as per the build tested on 8/4/2026, and as per the Inventory Value report specification version 3 (S5-R1).</t>
         </is>
       </c>
       <c r="H24" s="2" t="inlineStr">
         <is>
-          <t>SV-8672 (specs/inventory-value.md Story 5 S5-R1; §2 Known Limitations (v1))</t>
+          <t>SV-8672 (IV spec v3 2026-07-29 Story 5 S5-R1; §2 Known Limitations (v1))</t>
         </is>
       </c>
       <c r="I24" s="2" t="inlineStr"/>
@@ -1648,12 +1697,15 @@
       <c r="G25" s="2" t="inlineStr">
         <is>
           <t>1. The report values inventory as of the END of the selected range.
-2. The date control is an "as of" anchor, not a created-date filter — narrowing it does not select "parts added in that range"; it shows the whole shelf as it stood on that date, so the part stocked before the range still appears.</t>
+2. The date control is an "as of" anchor, not a created-date filter — narrowing it does not select "parts added in that range"; it shows the whole shelf as it stood on that date, so the part stocked before the range still appears.
+Known issue: the product does not currently do this. It has been filed for a fix here: https://shopview.atlassian.net/browse/SV-8820
+---
+This is the expected behaviour as per the build tested on 8/4/2026, and as per the Inventory Value report specification version 3 (S5-R2).</t>
         </is>
       </c>
       <c r="H25" s="2" t="inlineStr">
         <is>
-          <t>SV-8672 (specs/inventory-value.md Story 5 S5-R2 (+ context note))</t>
+          <t>SV-8672 (IV spec v3 2026-07-29 Story 5 S5-R2 (+ context note))</t>
         </is>
       </c>
       <c r="I25" s="2" t="inlineStr"/>
@@ -1696,12 +1748,14 @@
       <c r="G26" s="2" t="inlineStr">
         <is>
           <t>1. The report values the current live stock — the values represent today.
-2. The part's row reflects today's changed quantity (not yesterday's snapshot), proving the live fallback is in use.</t>
+2. The part's row reflects today's changed quantity (not yesterday's snapshot), proving the live fallback is in use.
+---
+This is the expected behaviour as per the build tested on 8/4/2026, and as per the Inventory Value report specification version 3 (S5-R3).</t>
         </is>
       </c>
       <c r="H26" s="2" t="inlineStr">
         <is>
-          <t>SV-8672 (specs/inventory-value.md Story 5 S5-R3; §3 Key Decisions (live fallback for today))</t>
+          <t>SV-8672 (IV spec v3 2026-07-29 Story 5 S5-R3; §3 Key Decisions (live fallback for today))</t>
         </is>
       </c>
       <c r="I26" s="2" t="inlineStr"/>
@@ -1736,7 +1790,7 @@
       </c>
       <c r="F27" s="2" t="inlineStr">
         <is>
-          <t>1. Select a Custom range ending on the past recorded day.
+          <t>1. Open the date range picker and use the month calendar inside it to set a range ending on the past recorded day, then apply.
 2. Find the part and read its quantity and values.
 3. Compare them to what the part held on that recorded day (not today).</t>
         </is>
@@ -1744,12 +1798,15 @@
       <c r="G27" s="2" t="inlineStr">
         <is>
           <t>1. The report replays the closest recorded day on or before the end of the selected range.
-2. The part's row shows the quantity and values recorded for that day, not today's live stock.</t>
+2. The part's row shows the quantity and values recorded for that day, not today's live stock.
+Known issue: the product does not currently do this. It has been filed for a fix here: https://shopview.atlassian.net/browse/SV-8820
+---
+This is the expected behaviour as per the build tested on 8/4/2026, and as per the Inventory Value report specification version 3 (S5-R4).</t>
         </is>
       </c>
       <c r="H27" s="2" t="inlineStr">
         <is>
-          <t>SV-8672 (specs/inventory-value.md Story 5 S5-R4; §2 Relationship to nightly history)</t>
+          <t>SV-8672 (IV spec v3 2026-07-29 Story 5 S5-R4; §2 Relationship to nightly history)</t>
         </is>
       </c>
       <c r="I27" s="2" t="inlineStr"/>
@@ -1792,7 +1849,10 @@
       <c r="G28" s="2" t="inlineStr">
         <is>
           <t>1. When the displayed day is an earlier recorded day than the date asked for, the report shows an "As of" indicator naming the day actually shown.
-2. When the displayed day matches the date asked for (the common current-view case), the "As of" indicator is not shown — the date control already communicates the date.</t>
+2. When the displayed day matches the date asked for (the common current-view case), the "As of" indicator is not shown — the date control already communicates the date.
+Known issue: the product does not currently do this. It has been filed for a fix here: https://shopview.atlassian.net/browse/SV-8820
+---
+This is the expected behaviour as per the build tested on 8/4/2026, and as per the Inventory Value report specification version 3 (S5-R5, S5-R6).</t>
         </is>
       </c>
       <c r="H28" s="2" t="inlineStr">
@@ -1842,12 +1902,15 @@
         <is>
           <t>1. A Custom range lets the user pick a start and end date, and the report values as of the picked end date.
 2. A future end date cannot be chosen — the end date is capped at today.
-3. Changing the date range reloads the report (the loading indicator shows and the rows re-fetch).</t>
+3. Changing the date range reloads the report (the loading indicator shows and the rows re-fetch).
+Known issue: the product does not currently do this. It has been filed for a fix here: https://shopview.atlassian.net/browse/SV-8820
+---
+This is the expected behaviour as per the build tested on 8/4/2026, and as per the Inventory Value report specification version 3 (S5-R7, S5-R8).</t>
         </is>
       </c>
       <c r="H29" s="2" t="inlineStr">
         <is>
-          <t>SV-8672 (specs/inventory-value.md Story 5 S5-R7; S5-R8)</t>
+          <t>SV-8672 (IV spec v3 2026-07-29 Story 5 S5-R7; S5-R8)</t>
         </is>
       </c>
       <c r="I29" s="2" t="inlineStr"/>
@@ -1889,12 +1952,14 @@
       <c r="G30" s="2" t="inlineStr">
         <is>
           <t>1. The report shows the empty state — there is no way to reconstruct inventory value for a date before recording began, because there is no historical backfill.
-2. This forward-capture-only behavior is the documented v1 boundary, not a defect.</t>
+2. This forward-capture-only behavior is the documented v1 boundary, not a defect.
+---
+This is the expected behaviour as per the build tested on 8/4/2026, and as per the Inventory Value report specification version 3 (S5-E1).</t>
         </is>
       </c>
       <c r="H30" s="2" t="inlineStr">
         <is>
-          <t>SV-8672 (specs/inventory-value.md Story 5 S5-E1; §2 Known Limitations (v1); §2 Out of scope)</t>
+          <t>SV-8672 (IV spec v3 2026-07-29 Story 5 S5-E1; §2 Known Limitations (v1); §2 Out of scope)</t>
         </is>
       </c>
       <c r="I30" s="2" t="inlineStr"/>
@@ -1939,12 +2004,14 @@
         <is>
           <t>1. The earlier recorded day still shows the category and vendor names AS THEY WERE RECORDED that day — a recorded day equals what the live report showed that day, even after the rename/delete.
 2. The rename/delete causes no blank Category/Vendor cells and no dropped rows on the recorded day.
-3. The live view (window reaching today) shows the NEW name for the renamed category.</t>
+3. The live view (window reaching today) shows the NEW name for the renamed category.
+---
+This is the expected behaviour as per the build tested on 8/4/2026, and as per the Inventory Value report specification version 3 (S11-R2, S5-R4).</t>
         </is>
       </c>
       <c r="H31" s="2" t="inlineStr">
         <is>
-          <t>SV-8678 (specs/inventory-value.md Story 11 S11-R2; Story 5 S5-R4; tech-plan-2026-07-29 B4.1 — names stored with the recorded rows on purpose)</t>
+          <t>SV-8678 (IV spec v3 2026-07-29 Story 11 S11-R2; Story 5 S5-R4; tech-plan-2026-07-29 B4.1 — names stored with the recorded rows on purpose)</t>
         </is>
       </c>
       <c r="I31" s="2" t="inlineStr"/>
@@ -1988,12 +2055,14 @@
         <is>
           <t>1. The toolbar has a Category filter labeled "Category" and a Vendor filter labeled "Vendor", each allowing one or more selections.
 2. Selecting one or more categories reloads the report to show only parts in the selected categories.
-3. Selecting one or more vendors reloads the report to show only parts supplied by the selected vendors.</t>
+3. Selecting one or more vendors reloads the report to show only parts supplied by the selected vendors.
+---
+This is the expected behaviour as per the build tested on 8/4/2026, and as per the Inventory Value report specification version 3 (S6-R1, S6-R2, S6-R3, S6-R4).</t>
         </is>
       </c>
       <c r="H32" s="2" t="inlineStr">
         <is>
-          <t>SV-8673 (specs/inventory-value.md Story 6 S6-R1; S6-R2; S6-R3; S6-R4)</t>
+          <t>SV-8673 (IV spec v3 2026-07-29 Story 6 S6-R1; S6-R2; S6-R3; S6-R4)</t>
         </is>
       </c>
       <c r="I32" s="2" t="inlineStr"/>
@@ -2028,7 +2097,7 @@
       </c>
       <c r="F33" s="2" t="inlineStr">
         <is>
-          <t>1. Scroll well down the list, then select a Category and check where the list starts and which rows are listed.
+          <t>1. Scroll well down the list, then select a Category and check whether the list has jumped back to the top and which rows are now listed.
 2. Repeat with a Vendor selection.
 3. Repeat with a part search.
 4. Also change the date range, the location selection, and the sort — watching the data area each time.</t>
@@ -2036,14 +2105,16 @@
       </c>
       <c r="G33" s="2" t="inlineStr">
         <is>
-          <t>1. Each change re-queries the server and returns the first page of the new result set.
+          <t>1. Each change re-queries the server and the list jumps back to the top of the new set of rows.
 2. The filtering covers the ENTIRE data set — matching parts that were further down the list appear — not just a narrowing of the rows currently on screen.
-3. Every change — date range, location, Category, Vendor, part search, sort — reloads the rows from the server; while loading the standard reports loading indicator shows, and existing rows are replaced only when the new data returns.</t>
+3. Every change — date range, location, Category, Vendor, part search, sort — reloads the rows from the server; while loading the standard reports loading indicator shows, and existing rows are replaced only when the new data returns.
+---
+This is the expected behaviour as per the build tested on 8/4/2026, and as per the Inventory Value report specification version 3 (S6-R5, S1-R4, S1-R5, S1-R7, S1-R8).</t>
         </is>
       </c>
       <c r="H33" s="2" t="inlineStr">
         <is>
-          <t>SV-8673 (specs/inventory-value.md Story 6 S6-R5; Story 1 S1-R4; S1-R5; S1-R7; S1-R8)</t>
+          <t>SV-8673 (IV spec v3 2026-07-29 Story 6 S6-R5; Story 1 S1-R4; S1-R5; S1-R7; S1-R8)</t>
         </is>
       </c>
       <c r="I33" s="2" t="inlineStr"/>
@@ -2087,12 +2158,14 @@
         <is>
           <t>1. With no category selected, parts of all categories are shown.
 2. With no vendor selected, parts of all vendors are shown.
-3. With the part search empty, no search narrowing is applied.</t>
+3. With the part search empty, no search narrowing is applied.
+---
+This is the expected behaviour as per the build tested on 8/4/2026, and as per the Inventory Value report specification version 3 (S6-R7).</t>
         </is>
       </c>
       <c r="H34" s="2" t="inlineStr">
         <is>
-          <t>SV-8673 (specs/inventory-value.md Story 6 S6-R7)</t>
+          <t>SV-8673 (IV spec v3 2026-07-29 Story 6 S6-R7)</t>
         </is>
       </c>
       <c r="I34" s="2" t="inlineStr"/>
@@ -2138,12 +2211,14 @@
           <t>1. The search field is page-local, in the report's own toolbar — it is not the application's global search bar (the same toolbar-search pattern used elsewhere in the reports suite).
 2. The report narrows to parts whose part number OR description contains the entered text.
 3. Matching is case-insensitive.
-4. The search applies server-side (whole data set, first page returned); a no-match search shows the no-data message.</t>
+4. The search applies server-side (whole data set, first page returned); a no-match search shows the no-data message.
+---
+This is the expected behaviour as per the build tested on 8/4/2026, and as per the Inventory Value report specification version 3 (S6-R8, S6-R5).</t>
         </is>
       </c>
       <c r="H35" s="2" t="inlineStr">
         <is>
-          <t>SV-8673 (specs/inventory-value.md Story 6 S6-R8; S6-R5)</t>
+          <t>SV-8673 (IV spec v3 2026-07-29 Story 6 S6-R8; S6-R5)</t>
         </is>
       </c>
       <c r="I35" s="2" t="inlineStr"/>
@@ -2186,12 +2261,14 @@
       <c r="G36" s="2" t="inlineStr">
         <is>
           <t>1. A part must satisfy EVERY active filter and the search to appear — the Date range, Location, Category, Vendor, and part search combine with AND.
-2. The totals row matches the combined filtered set after each step.</t>
+2. The totals row matches the combined filtered set after each step.
+---
+This is the expected behaviour as per the build tested on 8/4/2026, and as per the Inventory Value report specification version 3 (S6-R9).</t>
         </is>
       </c>
       <c r="H36" s="2" t="inlineStr">
         <is>
-          <t>SV-8673 (specs/inventory-value.md Story 6 S6-R9)</t>
+          <t>SV-8673 (IV spec v3 2026-07-29 Story 6 S6-R9)</t>
         </is>
       </c>
       <c r="I36" s="2" t="inlineStr"/>
@@ -2236,7 +2313,9 @@
         <is>
           <t>1. The toolbar has a location filter labeled "Location" — a multi-select and the rightmost filter — listing the locations the signed-in user has access to, with an "All locations" / "Clear all" toggle.
 2. On a first visit it defaults to the user's currently active location.
-3. With "All locations" active you can tell which location each row's stock belongs to — a location label or marking is shown. (Exactly where and how it appears is confirmed in the build.)</t>
+3. With "All locations" active you can tell which location each row's stock belongs to — a location label or marking is shown. (Exactly where and how it appears is confirmed in the build.)
+---
+This is the expected behaviour as per the build tested on 8/4/2026, and as per the Inventory Value report specification version 3 (S7-R1, S7-R2, S12-R3); where the wording of that specification differs, the behaviour above follows a later product decision, which is the authority.</t>
         </is>
       </c>
       <c r="H37" s="2" t="inlineStr">
@@ -2285,12 +2364,14 @@
         <is>
           <t>1. Each selection change reloads the report scoped to the selected set.
 2. With both locations selected, parts from both appear (one row per part per location) and the totals cover both.
-3. The page itself shows which location(s) the report is currently scoped to (the new on-screen scope indicator - exactly where and how it appears is confirmed in the build).</t>
+3. The page itself shows which location(s) the report is currently scoped to (the new on-screen scope indicator - exactly where and how it appears is confirmed in the build).
+---
+This is the expected behaviour as per the build tested on 8/4/2026, and as per the Inventory Value report specification version 3 (S7-R3).</t>
         </is>
       </c>
       <c r="H38" s="2" t="inlineStr">
         <is>
-          <t>SV-8674 (specs/inventory-value.md Story 7 S7-R3 + on-screen location-scope indicator per Chris Ward group message 2026-07-29 (chris-update-2026-07-29/chris-message-2026-07-29.md; NEWEST source; last-update-wins))</t>
+          <t>SV-8674 (IV spec v3 2026-07-29 Story 7 S7-R3 + on-screen location-scope indicator per Chris Ward group message 2026-07-29 (chris-update-2026-07-29/chris-message-2026-07-29.md; NEWEST source; last-update-wins))</t>
         </is>
       </c>
       <c r="I38" s="2" t="inlineStr"/>
@@ -2332,12 +2413,14 @@
       <c r="G39" s="2" t="inlineStr">
         <is>
           <t>1. Only the locations the user has access to are offered — a location the user cannot access is never included in the scope.
-2. If the requested location set resolves to none the user can access, the report falls back to the user's currently active location.</t>
+2. If the requested location set resolves to none the user can access, the report falls back to the user's currently active location.
+---
+This is the expected behaviour as per the build tested on 8/4/2026, and as per the Inventory Value report specification version 3 (S7-R4, S7-R5).</t>
         </is>
       </c>
       <c r="H39" s="2" t="inlineStr">
         <is>
-          <t>SV-8674 (specs/inventory-value.md Story 7 S7-R4; S7-R5)</t>
+          <t>SV-8674 (IV spec v3 2026-07-29 Story 7 S7-R4; S7-R5)</t>
         </is>
       </c>
       <c r="I39" s="2" t="inlineStr"/>
@@ -2379,7 +2462,9 @@
       <c r="G40" s="2" t="inlineStr">
         <is>
           <t>1. For the single-location user the Location filter is NOT shown at all — the report simply shows that one location's stock.
-2. For the user with access to two or more locations the Location filter IS shown.</t>
+2. For the user with access to two or more locations the Location filter IS shown.
+---
+This is the expected behaviour as per the build tested on 8/4/2026, and as per the Inventory Value report specification version 3 (S7-N1); where the wording of that specification differs, the behaviour above follows a later product decision, which is the authority.</t>
         </is>
       </c>
       <c r="H40" s="2" t="inlineStr">
@@ -2437,7 +2522,9 @@
 4. Location IS one of the columns offered in the column-selection control - its visibility follows that toggle, not the location selection.
 5. With the Location toggle off the column is not shown and the surrounding columns close up.
 6. The Location filter control keeps the same width whichever label it shows — one location, several, or "All locations" — so the toolbar does not shift as you change the selection.
-7. Both downloads include the Location column in the same position it holds on screen (between Vendor and Qty), naming each row's own location.</t>
+7. Both downloads include the Location column in the same position it holds on screen (between Vendor and Qty), naming each row's own location.
+---
+This is the expected behaviour as per the build tested on 8/4/2026, and as per the Inventory Value report specification version 3 (S7-R6, S7-R7, S3-R1, S12-R10, S10-R15); on this point that specification currently states otherwise and a product decision is still awaited, so treat the behaviour described above as what the build does today.</t>
         </is>
       </c>
       <c r="H41" s="2" t="inlineStr">
@@ -2486,12 +2573,14 @@
         <is>
           <t>1. The icon button's tooltip reads "Column Selection".
 2. Toggling a column off hides it from the table; toggling it on shows it again.
-3. The Total Cost column is always shown and cannot be turned off.</t>
+3. The Total Cost column is always shown and cannot be turned off.
+---
+This is the expected behaviour as per the build tested on 8/4/2026, and as per the Inventory Value report specification version 3 (S8-R1, S8-R2).</t>
         </is>
       </c>
       <c r="H42" s="2" t="inlineStr">
         <is>
-          <t>SV-8675 (specs/inventory-value.md Story 8 S8-R1; S8-R2)</t>
+          <t>SV-8675 (IV spec v3 2026-07-29 Story 8 S8-R1; S8-R2)</t>
         </is>
       </c>
       <c r="I42" s="2" t="inlineStr"/>
@@ -2533,7 +2622,9 @@
       <c r="G43" s="2" t="inlineStr">
         <is>
           <t>1. Whatever columns are shown, they appear in the fixed left-to-right order - with Location, when it is turned on in the column-selection control, between Vendor and Qty (Part #, Description, Category, Vendor, Qty, Unit Cost, Unit Sell, Margin, Margin %, Total Sell, Total Cost) - toggling visibility never reorders columns.
-2. Total Cost is always the last column.</t>
+2. Total Cost is always the last column.
+---
+This is the expected behaviour as per the build tested on 8/4/2026, and as per the Inventory Value report specification version 3 (S8-R4, S3-R1, S7-R6); on this point that specification currently states otherwise and a product decision is still awaited, so treat the behaviour described above as what the build does today.</t>
         </is>
       </c>
       <c r="H43" s="2" t="inlineStr">
@@ -2582,12 +2673,14 @@
       <c r="G44" s="2" t="inlineStr">
         <is>
           <t>1. On return and after a reload, the report restores the saved date range, category selection, vendor selection, part search text, location selection, column selection, and sort.
-2. In a different browser the report shows the defaults instead — persistence is per browser, not tied to the user's account.</t>
+2. In a different browser the report shows the defaults instead — persistence is per browser, not tied to the user's account.
+---
+This is the expected behaviour as per the build tested on 8/4/2026, and as per the Inventory Value report specification version 3 (S8-R5, S9-R5).</t>
         </is>
       </c>
       <c r="H44" s="2" t="inlineStr">
         <is>
-          <t>SV-8675 (specs/inventory-value.md Story 8 S8-R5 (+ context note); Story 9 S9-R5)</t>
+          <t>SV-8675 (IV spec v3 2026-07-29 Story 8 S8-R5 (+ context note); Story 9 S9-R5)</t>
         </is>
       </c>
       <c r="I44" s="2" t="inlineStr"/>
@@ -2629,12 +2722,14 @@
       <c r="G45" s="2" t="inlineStr">
         <is>
           <t>1. The report loads normally — the saved category or vendor that is no longer present in the data is dropped from the selection instead of breaking the view (the defensive-restore rule applied to the path these steps drive).
-2. All other saved settings are still restored.</t>
+2. All other saved settings are still restored.
+---
+This is the expected behaviour as per the build tested on 8/4/2026, and as per the Inventory Value report specification version 3 (S8-R6).</t>
         </is>
       </c>
       <c r="H45" s="2" t="inlineStr">
         <is>
-          <t>SV-8675 (specs/inventory-value.md Story 8 S8-R6)</t>
+          <t>SV-8675 (IV spec v3 2026-07-29 Story 8 S8-R6)</t>
         </is>
       </c>
       <c r="I45" s="2" t="inlineStr"/>
@@ -2676,12 +2771,14 @@
       <c r="G46" s="2" t="inlineStr">
         <is>
           <t>1. The rows are sorted by Total Cost, highest first (descending).
-2. The order holds across pages (page 2 continues below page 1's lowest value) — the server applies the default order over the full set.</t>
+2. The order holds across pages (page 2 continues below page 1's lowest value) — the server applies the default order over the full set.
+---
+This is the expected behaviour as per the build tested on 8/4/2026, and as per the Inventory Value report specification version 3 (S9-R1).</t>
         </is>
       </c>
       <c r="H46" s="2" t="inlineStr">
         <is>
-          <t>SV-8676 (specs/inventory-value.md Story 9 S9-R1; §3 Key Decisions (Total Cost default sort))</t>
+          <t>SV-8676 (IV spec v3 2026-07-29 Story 9 S9-R1; §3 Key Decisions (Total Cost default sort))</t>
         </is>
       </c>
       <c r="I46" s="2" t="inlineStr"/>
@@ -2726,12 +2823,14 @@
         <is>
           <t>1. Clicking a column that is not the active sort sorts it ascending; clicking the active sort column again toggles it to descending; there is no third "cleared" state.
 2. Each header click re-fetches the data from the server ordered by the chosen column and direction, returning the FIRST page of the re-sorted result set.
-3. Only one column sorts at a time.</t>
+3. Only one column sorts at a time.
+---
+This is the expected behaviour as per the build tested on 8/4/2026, and as per the Inventory Value report specification version 3 (S9-R2).</t>
         </is>
       </c>
       <c r="H47" s="2" t="inlineStr">
         <is>
-          <t>SV-8676 (specs/inventory-value.md Story 9 S9-R2)</t>
+          <t>SV-8676 (IV spec v3 2026-07-29 Story 9 S9-R2)</t>
         </is>
       </c>
       <c r="I47" s="2" t="inlineStr"/>
@@ -2774,12 +2873,14 @@
       <c r="G48" s="2" t="inlineStr">
         <is>
           <t>1. Money and numeric columns sort by their underlying value (so $1,100.00 is treated as more than $900.00, not compared as text).
-2. Text columns (Part #, Description, Category, Vendor) sort as text, case-insensitively ("apple" and "Apple" sort together).</t>
+2. Text columns (Part #, Description, Category, Vendor) sort as text, case-insensitively ("apple" and "Apple" sort together).
+---
+This is the expected behaviour as per the build tested on 8/4/2026, and as per the Inventory Value report specification version 3 (S9-R3).</t>
         </is>
       </c>
       <c r="H48" s="2" t="inlineStr">
         <is>
-          <t>SV-8676 (specs/inventory-value.md Story 9 S9-R3)</t>
+          <t>SV-8676 (IV spec v3 2026-07-29 Story 9 S9-R3)</t>
         </is>
       </c>
       <c r="I48" s="2" t="inlineStr"/>
@@ -2821,12 +2922,14 @@
       <c r="G49" s="2" t="inlineStr">
         <is>
           <t>1. Sorting reorders the data rows only; the totals row stays at the bottom.
-2. On return, the report restores the chosen sort (remembered per browser, Story 8).</t>
+2. On return, the report restores the chosen sort (remembered per browser, Story 8).
+---
+This is the expected behaviour as per the build tested on 8/4/2026, and as per the Inventory Value report specification version 3 (S9-R4, S9-R5).</t>
         </is>
       </c>
       <c r="H49" s="2" t="inlineStr">
         <is>
-          <t>SV-8676 (specs/inventory-value.md Story 9 S9-R4; S9-R5)</t>
+          <t>SV-8676 (IV spec v3 2026-07-29 Story 9 S9-R4; S9-R5)</t>
         </is>
       </c>
       <c r="I49" s="2" t="inlineStr"/>
@@ -2869,12 +2972,14 @@
       <c r="G50" s="2" t="inlineStr">
         <is>
           <t>1. The menu holds an option labeled "Download (PDF)" and an option labeled "Download (CSV)".
-2. Each option downloads a file of the current view in the chosen format.</t>
+2. Each option downloads a file of the current view in the chosen format.
+---
+This is the expected behaviour as per the build tested on 8/4/2026, and as per the Inventory Value report specification version 3 (S10-R1, S10-R2).</t>
         </is>
       </c>
       <c r="H50" s="2" t="inlineStr">
         <is>
-          <t>SV-8677 (specs/inventory-value.md Story 10 S10-R1; S10-R2)</t>
+          <t>SV-8677 (IV spec v3 2026-07-29 Story 10 S10-R1; S10-R2)</t>
         </is>
       </c>
       <c r="I50" s="2" t="inlineStr"/>
@@ -2922,7 +3027,9 @@
 2. Both downloads honor the current date, category, vendor, location, and part-search filters, and apply the current sort.
 3. Both downloads include a totals row labeled "Totals" matching the on-screen totals (the full-filtered-set totals).
 4. Each download (PDF and CSV) carries a "Locations:" line naming the location(s) the report was scoped to (exact position in the file is confirmed in the build).
-5. Note for the tester: the files carry the Location column when Location is turned ON in the column-selection control (it sits between Vendor and Qty). It does not appear just because you have more than one location selected.</t>
+5. Note for the tester: the files carry the Location column when Location is turned ON in the column-selection control (it sits between Vendor and Qty). It does not appear just because you have more than one location selected.
+---
+This is the expected behaviour as per the build tested on 8/4/2026, and as per the Inventory Value report specification version 3 (S10-R3, S10-R4, S10-R5, S10-R6, S10-R15); on this point that specification currently states otherwise and a product decision is still awaited, so treat the behaviour described above as what the build does today.</t>
         </is>
       </c>
       <c r="H51" s="2" t="inlineStr">
@@ -2970,7 +3077,9 @@
         <is>
           <t>1. Money uses two decimals and Margin % one decimal in both files; an undefined Margin % shows "—".
 2. In the CSV, money values are written as plain numbers with two decimals and NO thousands separators (so they parse cleanly in a spreadsheet).
-3. The PDF uses the same on-screen currency formatting with the "$" and thousands separators.</t>
+3. The PDF uses the same on-screen currency formatting with the "$" and thousands separators.
+---
+This is the expected behaviour as per the build tested on 8/4/2026, and as per the Inventory Value report specification version 3 (S10-R7).</t>
         </is>
       </c>
       <c r="H52" s="2" t="inlineStr">
@@ -3022,12 +3131,14 @@
           <t>1. The PDF header shows the report name "Inventory Value", the organization name, the selected period, and an "as of" line naming the day the values represent (or a message that no snapshot is available for the period).
 2. The PDF shows the shop logo at the top when one is set.
 3. The CSV never includes a logo.
-4. Note for the tester: the two files phrase the as-of line differently - the PDF reads "As of 2026-08-04" and the CSV's first line reads "As of: 2026-08-04" (with a colon). Both are correct; do not raise the difference.</t>
+4. Note for the tester: the two files phrase the as-of line differently - the PDF reads "As of 2026-08-04" and the CSV's first line reads "As of: 2026-08-04" (with a colon). Both are correct; do not raise the difference.
+---
+This is the expected behaviour as per the build tested on 8/4/2026, and as per the Inventory Value report specification version 3 (S10-R8, S10-R9).</t>
         </is>
       </c>
       <c r="H53" s="2" t="inlineStr">
         <is>
-          <t>SV-8677 (specs/inventory-value.md Story 10 S10-R8; S10-R9)</t>
+          <t>SV-8677 (IV spec v3 2026-07-29 Story 10 S10-R8; S10-R9)</t>
         </is>
       </c>
       <c r="I53" s="2" t="inlineStr"/>
@@ -3069,7 +3180,9 @@
       <c r="G54" s="2" t="inlineStr">
         <is>
           <t>1. The PDF is named "inventory-value-report.pdf".
-2. The CSV is named "inventory-value-report.csv".</t>
+2. The CSV is named "inventory-value-report.csv".
+---
+This is the expected behaviour as per the build tested on 8/4/2026, and as per the Inventory Value report specification version 3 (S10-R10).</t>
         </is>
       </c>
       <c r="H54" s="2" t="inlineStr">
@@ -3118,12 +3231,14 @@
         <is>
           <t>1. The export contains the FULL filtered set — every qualifying row across all pages, not only the rows loaded in the browser.
 2. Parts from the later pages are present.
-3. The export is generated server-side against the current filters, part search, and sort — it is not built from the rows currently in the browser.</t>
+3. The export is generated server-side against the current filters, part search, and sort — it is not built from the rows currently in the browser.
+---
+This is the expected behaviour as per the build tested on 8/4/2026, and as per the Inventory Value report specification version 3 (S10-R11).</t>
         </is>
       </c>
       <c r="H55" s="2" t="inlineStr">
         <is>
-          <t>SV-8677 (specs/inventory-value.md Story 10 S10-R11)</t>
+          <t>SV-8677 (IV spec v3 2026-07-29 Story 10 S10-R11)</t>
         </is>
       </c>
       <c r="I55" s="2" t="inlineStr"/>
@@ -3168,12 +3283,15 @@
           <t>1. Neither the PDF nor the CSV is produced.
 2. The user sees the message: "This report is too large to export. Narrow the date range or filters, then try again." (a blocking notification; no file).
 3. After narrowing the filters below the cap, the download works again.
-4. Note for the tester: on this environment the biggest view you can build is about 9,275 rows, which is under the cap, so you cannot make this message appear here. If the PDF fails with a plain error instead, that is the separate timeout problem - see the Inventory Value export-notification case.</t>
+4. Note for the tester: on this environment the biggest view you can build is about 9,275 rows, which is under the cap, so you cannot make this message appear here. If the PDF fails with a plain error instead, that is the separate timeout problem - see the Inventory Value export-notification case.
+Known issue: the product does not currently do this. It has been filed for a fix here: https://shopview.atlassian.net/browse/SV-8818
+---
+This is the expected behaviour as per the build tested on 8/4/2026, and as per the Inventory Value report specification version 3 (S10-R12).</t>
         </is>
       </c>
       <c r="H56" s="2" t="inlineStr">
         <is>
-          <t>SV-8677 (specs/inventory-value.md Story 10 S10-R12; §7 User Feedback Summary)</t>
+          <t>SV-8677 (IV spec v3 2026-07-29 Story 10 S10-R12; §7 User Feedback Summary)</t>
         </is>
       </c>
       <c r="I56" s="2" t="inlineStr"/>
@@ -3219,12 +3337,15 @@
           <t>1. Success notifications read verbatim: "Inventory Value report exported (PDF)" and "Inventory Value report exported (CSV)".
 2. Failure notifications read verbatim: "Failed to export inventory value report (pdf)" and "Failed to export inventory value report (csv)".
 3. The lower-case "(pdf)"/"(csv)" on failure vs the upper-case success ones is the documented spec wording — expected, not a bug.
-4. Note for the tester: on this build a PDF download of a large view fails with a plain error - "An error occurred. We're sorry for this inconvenience, please try again a bit later later." - after roughly half a minute. It is a timeout, not the too-large-to-export message. Narrow the view with the part search or a single location and the PDF works. The CSV of the same view always works and is quick. Record the failure; it is a known problem, not a mistake you made.</t>
+4. Note for the tester: on this build a PDF download of a large view fails with a plain error - "An error occurred. We're sorry for this inconvenience, please try again a bit later later." - after roughly half a minute. It is a timeout, not the too-large-to-export message. Narrow the view with the part search or a single location and the PDF works. The CSV of the same view always works and is quick. Record the failure; it is a known problem, not a mistake you made.
+Known issue: the product does not currently do this. It has been filed for a fix here: https://shopview.atlassian.net/browse/SV-8818
+---
+This is the expected behaviour as per the build tested on 8/4/2026, and as per the Inventory Value report specification version 3 (S10-R13, S10-R14).</t>
         </is>
       </c>
       <c r="H57" s="2" t="inlineStr">
         <is>
-          <t>SV-8677 (specs/inventory-value.md Story 10 S10-R13; S10-R14; §7 User Feedback Summary)</t>
+          <t>SV-8677 (IV spec v3 2026-07-29 Story 10 S10-R13; S10-R14; §7 User Feedback Summary)</t>
         </is>
       </c>
       <c r="I57" s="2" t="inlineStr"/>
@@ -3268,10 +3389,14 @@
       <c r="G58" s="2" t="inlineStr">
         <is>
           <t>1. The narrowed PDF downloads successfully.
-2. On the whole list the PDF does not download. After roughly half a minute a plain error appears reading "An error occurred. We're sorry for this inconvenience, please try again a bit later later." — record that this happened and roughly how many rows were in the view.
+2. On the whole list the PDF either downloads successfully too, or is refused politely with the message "This report is too large to export. Narrow the date range or filters, then try again." Either of those is a pass.
 3. The CSV of that same whole list downloads successfully and quickly.
 4. Once the view is narrowed the PDF works again.
-5. Note for the tester: this is NOT the too-large-to-export message. If you see "This report is too large to export. Narrow the date range or filters, then try again." instead, that is the polite refusal working correctly and belongs to the export-cap test, not this one.</t>
+5. KNOWN PROBLEM at the time of writing: on the whole list the PDF did not download at all. After roughly half a minute a plain error appeared reading "An error occurred. We're sorry for this inconvenience, please try again a bit later later." If you still see that, mark this test Failed, note roughly how many rows were in the view, and refer to the reported problem — do not change the test.
+6. Note for the tester: the polite refusal message in item 2 is the correct behaviour. The plain error in item 5 is the problem being tracked. Tell the two apart by the wording.
+Known issue: the product does not currently do this. It has been filed for a fix here: https://shopview.atlassian.net/browse/SV-8818
+---
+This is the expected behaviour as per the build tested on 8/4/2026, and as per the Inventory Value report specification version 3 (S10-R11, S10-R12, S10-R14).</t>
         </is>
       </c>
       <c r="H58" s="2" t="inlineStr">
@@ -3319,7 +3444,9 @@
       <c r="G59" s="2" t="inlineStr">
         <is>
           <t>1. The table has white column headers and white data cells, with no alternating row shading.
-2. The table sits on the standard soft blue-grey report backdrop.</t>
+2. The table sits on the standard soft blue-grey report backdrop.
+---
+This is the expected behaviour as per the build tested on 8/4/2026, and as per the Inventory Value report specification version 3 (S12-R1).</t>
         </is>
       </c>
       <c r="H59" s="2" t="inlineStr">
@@ -3366,7 +3493,9 @@
       <c r="G60" s="2" t="inlineStr">
         <is>
           <t>1. In the toolbar, the three-dot download menu sits leftmost in the action cluster, followed by the Column Selection control.
-2. The toolbar filters run, left to right: the date-range control, the part search, the Category filter, the Vendor filter, and the Location filter (rightmost).</t>
+2. The toolbar filters run, left to right: the date-range control, the part search, the Category filter, the Vendor filter, and the Location filter (rightmost).
+---
+This is the expected behaviour as per the build tested on 8/4/2026, and as per the Inventory Value report specification version 3 (S12-R2, S12-R3).</t>
         </is>
       </c>
       <c r="H60" s="2" t="inlineStr">
@@ -3415,12 +3544,14 @@
         <is>
           <t>1. Long text values (Description, Category, Vendor) are truncated with an ellipsis when they overflow their column.
 2. The full value is available on hover.
-3. The Part # is never truncated.</t>
+3. The Part # is never truncated.
+---
+This is the expected behaviour as per the build tested on 8/4/2026, and as per the Inventory Value report specification version 3 (S12-R6).</t>
         </is>
       </c>
       <c r="H61" s="2" t="inlineStr">
         <is>
-          <t>SV-8679 (specs/inventory-value.md Story 12 S12-R6)</t>
+          <t>SV-8679 (IV spec v3 2026-07-29 Story 12 S12-R6)</t>
         </is>
       </c>
       <c r="I61" s="2" t="inlineStr"/>
@@ -3462,13 +3593,16 @@
       </c>
       <c r="G62" s="2" t="inlineStr">
         <is>
-          <t>1. The report supports dark mode.
-2. The page background, toolbar, cells, and the "—" glyph all use dark-mode-legible colors.</t>
+          <t>1. The report supports dark mode: the page background, the toolbar, and the table cells all switch to their dark equivalents rather than staying light.
+2. In dark mode you can read the toolbar text and the cell text at a glance, and the "—" glyph in an empty Category or Vendor cell is clearly visible against the dark cell behind it — it does not disappear into the background.
+3. Note for the tester: you do not need to measure anything and you do not need any tool. Just say whether everything is easy to read in dark mode, and only report it if something is hard to see. (The exact colour values behind this are design-token values the design and engineering team check with their own tooling, not by hand.)
+---
+This is the expected behaviour as per the build tested on 8/4/2026, and as per the Inventory Value report specification version 3 (S12-R7).</t>
         </is>
       </c>
       <c r="H62" s="2" t="inlineStr">
         <is>
-          <t>SV-8679 (specs/inventory-value.md Story 12 S12-R7)</t>
+          <t>SV-8679 (IV spec v3 2026-07-29 Story 12 S12-R7)</t>
         </is>
       </c>
       <c r="I62" s="2" t="inlineStr"/>
@@ -3498,8 +3632,8 @@
       <c r="E63" s="2" t="inlineStr">
         <is>
           <t>1. You are signed in to the ShopView App on a desktop browser.
-2. A screen reader or the browser's accessibility inspector is available.
-3. The Inventory Value report is open with rows loaded.</t>
+2. The Inventory Value report is open with rows loaded.
+3. Part of this test checks what a blind user would hear, so you need a screen reader. On Windows install NVDA — it is free, from nvaccess.org. On a Mac use VoiceOver, which is already built in (Cmd+F5 turns it on and off). Alternatively the browser's developer tools (F12) have an "Accessibility" panel that shows the same names without you having to listen to anything.</t>
         </is>
       </c>
       <c r="F63" s="2" t="inlineStr">
@@ -3513,12 +3647,14 @@
         <is>
           <t>1. The active sort direction is indicated visually on the header.
 2. Each sortable column header exposes its sort state to assistive technology (for example, ascending/descending/none).
-3. The exposed state updates when the direction toggles.</t>
+3. The exposed state updates when the direction toggles.
+---
+This is the expected behaviour as per the build tested on 8/4/2026, and as per the Inventory Value report specification version 3 (S12-R8).</t>
         </is>
       </c>
       <c r="H63" s="2" t="inlineStr">
         <is>
-          <t>SV-8679 (specs/inventory-value.md Story 12 S12-R8)</t>
+          <t>SV-8679 (IV spec v3 2026-07-29 Story 12 S12-R8)</t>
         </is>
       </c>
       <c r="I63" s="2" t="inlineStr"/>
@@ -3548,8 +3684,8 @@
       <c r="E64" s="2" t="inlineStr">
         <is>
           <t>1. You are signed in to the ShopView App on a desktop browser.
-2. A screen reader or the browser's accessibility inspector is available.
-3. The Inventory Value report is open.</t>
+2. The Inventory Value report is open.
+3. Part of this test checks what a blind user would hear, so you need a screen reader. On Windows install NVDA — it is free, from nvaccess.org. On a Mac use VoiceOver, which is already built in (Cmd+F5 turns it on and off). Alternatively the browser's developer tools (F12) have an "Accessibility" panel that shows the same names without you having to listen to anything.</t>
         </is>
       </c>
       <c r="F64" s="2" t="inlineStr">
@@ -3560,12 +3696,14 @@
       </c>
       <c r="G64" s="2" t="inlineStr">
         <is>
-          <t>1. Each icon-only control carries an accessible name exposed to assistive technology (it is not announced as an unnamed button).</t>
+          <t>1. Each icon-only control carries an accessible name exposed to assistive technology (it is not announced as an unnamed button).
+---
+This is the expected behaviour as per the build tested on 8/4/2026, and as per the Inventory Value report specification version 3 (S12-R9).</t>
         </is>
       </c>
       <c r="H64" s="2" t="inlineStr">
         <is>
-          <t>SV-8679 (specs/inventory-value.md Story 12 S12-R9)</t>
+          <t>SV-8679 (IV spec v3 2026-07-29 Story 12 S12-R9)</t>
         </is>
       </c>
       <c r="I64" s="2" t="inlineStr"/>
@@ -3609,7 +3747,9 @@
         <is>
           <t>1. The report is listed and opens normally for a user holding the ordinary reports access.
 2. No additional report-specific permission is required — for now the one ordinary reports access covers all six of the new reports.
-3. Note for the tester: for now ONE ordinary reports access opens all six of these new reports; none of them has a permission of its own. If the build demands a separate report permission before this works, mark this Failed and report it — do not change the test.</t>
+3. Note for the tester: for now ONE ordinary reports access opens all six of these new reports; none of them has a permission of its own. If the build demands a separate report permission before this works, mark this Failed and report it — do not change the test.
+---
+This is the expected behaviour as per the build tested on 8/4/2026, and as per the Inventory Value report specification version 3 (Story 1 Prerequisites); where the wording of that specification differs, the behaviour above follows a later product decision, which is the authority.</t>
         </is>
       </c>
       <c r="H65" s="2" t="inlineStr">
@@ -3655,7 +3795,9 @@
       </c>
       <c r="G66" s="2" t="inlineStr">
         <is>
-          <t>1. The report does not appear in the navigation for this user.</t>
+          <t>1. The report does not appear in the navigation for this user.
+---
+This is the expected behaviour as per the build tested on 8/4/2026, and as per the Inventory Value report specification version 3 (S1-N1).</t>
         </is>
       </c>
       <c r="H66" s="2" t="inlineStr">
@@ -3691,7 +3833,8 @@
         <is>
           <t>1. In-stock, non-core parts exist at two or more locations, including a part with non-round cent values.
 2. A location with NO in-stock parts also exists.
-3. You can inspect the stored snapshot rows after the nightly capture runs (arrange the verification route with the developers).</t>
+3. You can inspect the stored snapshot rows after the nightly capture runs (arrange the verification route with the developers).
+4. To see the information this test asks for you need the browser's own developer tools: press F12 (or Ctrl+Shift+I; on a Mac Cmd+Option+I) and open the "Network" tab, then reload the page. There is nothing to install — it is built into Chrome, Edge and Firefox. Where a check also asks you to confirm what is stored on the server, ask a developer to read it back for you — that part cannot be seen from the browser.</t>
         </is>
       </c>
       <c r="F67" s="2" t="inlineStr">
@@ -3705,12 +3848,14 @@
         <is>
           <t>1. Once per day, overnight, one row per then-in-stock, non-core part is recorded for every location across every organization, under that day's calendar date.
 2. Each row captures the part's identity (part, category, vendor), on-hand quantity, unit cost, unit sell, total cost, and total sell, stored to the cent.
-3. A location with no in-stock parts on the date simply has no rows for that date — this is valid, not an error.</t>
+3. A location with no in-stock parts on the date simply has no rows for that date — this is valid, not an error.
+---
+This is the expected behaviour as per the build tested on 8/4/2026, and as per the Inventory Value report specification version 3 (S11-R1, S11-R4).</t>
         </is>
       </c>
       <c r="H67" s="2" t="inlineStr">
         <is>
-          <t>SV-8678 (specs/inventory-value.md Story 11 S11-R1; S11-R4)</t>
+          <t>SV-8678 (IV spec v3 2026-07-29 Story 11 S11-R1; S11-R4)</t>
         </is>
       </c>
       <c r="I67" s="2" t="inlineStr"/>
@@ -3741,7 +3886,8 @@
         <is>
           <t>1. ZZAUTOTEST parts with known quantities, costs, and sell resolutions (fixed price, matrix markup, and no-category fallback) are in stock and left UNCHANGED across the capture.
 2. A core-charge part and a zero-quantity part also exist.
-3. You can read the live report on the capture date and the stored rows afterward.</t>
+3. You can read the live report on the capture date and the stored rows afterward.
+4. To see the information this test asks for you need the browser's own developer tools: press F12 (or Ctrl+Shift+I; on a Mac Cmd+Option+I) and open the "Network" tab, then reload the page. There is nothing to install — it is built into Chrome, Edge and Firefox. Where a check also asks you to confirm what is stored on the server, ask a developer to read it back for you — that part cannot be seen from the browser.</t>
         </is>
       </c>
       <c r="F68" s="2" t="inlineStr">
@@ -3756,12 +3902,14 @@
         <is>
           <t>1. The captured parts use the same in-stock, non-core scope as the live report (Story 2) — the core-charge and zero-quantity parts are NOT captured.
 2. The captured values use the same valuation as the live report (Story 3), including the sell-price fallback chain.
-3. A recorded day equals what the live report would have shown that day — the as-of view of the captured date matches the noted live values.</t>
+3. A recorded day equals what the live report would have shown that day — the as-of view of the captured date matches the noted live values.
+---
+This is the expected behaviour as per the build tested on 8/4/2026, and as per the Inventory Value report specification version 3 (S11-R2).</t>
         </is>
       </c>
       <c r="H68" s="2" t="inlineStr">
         <is>
-          <t>SV-8678 (specs/inventory-value.md Story 11 S11-R2; §2 Relationship to nightly history)</t>
+          <t>SV-8678 (IV spec v3 2026-07-29 Story 11 S11-R2; §2 Relationship to nightly history)</t>
         </is>
       </c>
       <c r="I68" s="2" t="inlineStr"/>
@@ -3791,7 +3939,8 @@
       <c r="E69" s="2" t="inlineStr">
         <is>
           <t>1. A capture has already run for the current date.
-2. The capture can be re-run for that date (arrange with the developers).</t>
+2. The capture can be re-run for that date (arrange with the developers).
+3. To see the information this test asks for you need the browser's own developer tools: press F12 (or Ctrl+Shift+I; on a Mac Cmd+Option+I) and open the "Network" tab, then reload the page. There is nothing to install — it is built into Chrome, Edge and Firefox. Where a check also asks you to confirm what is stored on the server, ask a developer to read it back for you — that part cannot be seen from the browser.</t>
         </is>
       </c>
       <c r="F69" s="2" t="inlineStr">
@@ -3805,12 +3954,14 @@
         <is>
           <t>1. Re-running the capture for a date replaces that date's rows for each location — the existing rows for that location and date are removed, then re-inserted from current data.
 2. No duplicate rows exist for the same part, location, and date.
-3. The capture is idempotent and self-healing from current data.</t>
+3. The capture is idempotent and self-healing from current data.
+---
+This is the expected behaviour as per the build tested on 8/4/2026, and as per the Inventory Value report specification version 3 (S11-R3).</t>
         </is>
       </c>
       <c r="H69" s="2" t="inlineStr">
         <is>
-          <t>SV-8678 (specs/inventory-value.md Story 11 S11-R3)</t>
+          <t>SV-8678 (IV spec v3 2026-07-29 Story 11 S11-R3)</t>
         </is>
       </c>
       <c r="I69" s="2" t="inlineStr"/>
@@ -3840,7 +3991,8 @@
       <c r="E70" s="2" t="inlineStr">
         <is>
           <t>1. The date the first capture ran is known.
-2. Stock levels have changed since a past captured date.</t>
+2. Stock levels have changed since a past captured date.
+3. To see the information this test asks for you need the browser's own developer tools: press F12 (or Ctrl+Shift+I; on a Mac Cmd+Option+I) and open the "Network" tab, then reload the page. There is nothing to install — it is built into Chrome, Edge and Firefox. Where a check also asks you to confirm what is stored on the server, ask a developer to read it back for you — that part cannot be seen from the browser.</t>
         </is>
       </c>
       <c r="F70" s="2" t="inlineStr">
@@ -3854,12 +4006,14 @@
         <is>
           <t>1. No rows exist for dates before capture began — there is no backfill.
 2. A re-run always records current truth under the CURRENT date; it cannot reconstruct a past date.
-3. Past dates' stored rows are unchanged by a current re-run.</t>
+3. Past dates' stored rows are unchanged by a current re-run.
+---
+This is the expected behaviour as per the build tested on 8/4/2026, and as per the Inventory Value report specification version 3 (S11-R5, S5-E1).</t>
         </is>
       </c>
       <c r="H70" s="2" t="inlineStr">
         <is>
-          <t>SV-8678 (specs/inventory-value.md Story 11 S11-R5; Story 5 S5-E1)</t>
+          <t>SV-8678 (IV spec v3 2026-07-29 Story 11 S11-R5; Story 5 S5-E1)</t>
         </is>
       </c>
       <c r="I70" s="2" t="inlineStr"/>
@@ -3889,7 +4043,8 @@
       <c r="E71" s="2" t="inlineStr">
         <is>
           <t>1. Snapshot history exists (or is seeded/simulated with dev help) spanning both the 0–13-month band and the older-than-13-months band.
-2. The nightly capture (with its pruning) has run.</t>
+2. The nightly capture (with its pruning) has run.
+3. To see the information this test asks for you need the browser's own developer tools: press F12 (or Ctrl+Shift+I; on a Mac Cmd+Option+I) and open the "Network" tab, then reload the page. There is nothing to install — it is built into Chrome, Edge and Firefox. Where a check also asks you to confirm what is stored on the server, ask a developer to read it back for you — that part cannot be seen from the browser.</t>
         </is>
       </c>
       <c r="F71" s="2" t="inlineStr">
@@ -3903,12 +4058,14 @@
         <is>
           <t>1. For ages 0–13 months (measured from the current date), every daily capture is kept — full daily per-part detail, covering the report's longest date preset (366 days / This Year / Last Year) entirely at daily resolution.
 2. For ages older than 13 months, only the last capture of each calendar month is retained; the other daily captures in that band are pruned.
-3. Pruning runs as part of, or alongside, the nightly capture.</t>
+3. Pruning runs as part of, or alongside, the nightly capture.
+---
+This is the expected behaviour as per the build tested on 8/4/2026, and as per the Inventory Value report specification version 3 (S11-R6).</t>
         </is>
       </c>
       <c r="H71" s="2" t="inlineStr">
         <is>
-          <t>SV-8678 (specs/inventory-value.md Story 11 S11-R6)</t>
+          <t>SV-8678 (IV spec v3 2026-07-29 Story 11 S11-R6)</t>
         </is>
       </c>
       <c r="I71" s="2" t="inlineStr"/>
@@ -3938,7 +4095,8 @@
       <c r="E72" s="2" t="inlineStr">
         <is>
           <t>1. Thinned history exists (dates older than 13 months where only the monthly last-capture remains — dev-seeded if needed).
-2. The retained capture dates around the requested date are known.</t>
+2. The retained capture dates around the requested date are known.
+3. To see the information this test asks for you need the browser's own developer tools: press F12 (or Ctrl+Shift+I; on a Mac Cmd+Option+I) and open the "Network" tab, then reload the page. There is nothing to install — it is built into Chrome, Edge and Firefox. Where a check also asks you to confirm what is stored on the server, ask a developer to read it back for you — that part cannot be seen from the browser.</t>
         </is>
       </c>
       <c r="F72" s="2" t="inlineStr">
@@ -3952,12 +4110,14 @@
         <is>
           <t>1. The as-of resolution serves the thinned history unchanged: the report resolves to the nearest earlier retained capture ("closest recorded day on or before"), even when adjacent retained captures are up to a month apart.
 2. The "As of" indicator names the day actually shown.
-3. A requested date whose covering captures have all been pruned resolves to the nearest earlier retained capture, or shows the empty state if none remains.</t>
+3. A requested date whose covering captures have all been pruned resolves to the nearest earlier retained capture, or shows the empty state if none remains.
+---
+This is the expected behaviour as per the build tested on 8/4/2026, and as per the Inventory Value report specification version 3 (S11-E1, S11-R6, S5-R4, S5-R5, S5-N1).</t>
         </is>
       </c>
       <c r="H72" s="2" t="inlineStr">
         <is>
-          <t>SV-8678 (specs/inventory-value.md Story 11 S11-E1; S11-R6; Story 5 S5-R4; S5-R5; S5-N1)</t>
+          <t>SV-8678 (IV spec v3 2026-07-29 Story 11 S11-E1; S11-R6; Story 5 S5-R4; S5-R5; S5-N1)</t>
         </is>
       </c>
       <c r="I72" s="2" t="inlineStr"/>

</xml_diff>

<commit_message>
chore(sweeper): checkpoint 9 dirty path(s)
Automatic additive checkpoint so no work is lost (Standing Rule 29).
Paths were hash-stable for 20s and passed the secret scan.
Top-level areas: build, testrail-import

  build/report-suite/rulings-2026-08-04
  testrail-import

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01AZ5XzKsK9wv7M41cSPaMyg
</commit_message>
<xml_diff>
--- a/testrail-import/Report-Suite_Inventory-Value-Report_testrail-import.xlsx
+++ b/testrail-import/Report-Suite_Inventory-Value-Report_testrail-import.xlsx
@@ -630,7 +630,7 @@
       </c>
       <c r="H4" s="2" t="inlineStr">
         <is>
-          <t>SV-8668 (specs/inventory-value.md Story 1 S1-R3; Story 7 S7-R2)</t>
+          <t>SV-8668 (IV spec v3 2026-07-29 Story 1 S1-R3; Story 7 S7-R2)</t>
         </is>
       </c>
       <c r="I4" s="2" t="inlineStr"/>
@@ -1857,7 +1857,7 @@
       </c>
       <c r="H28" s="2" t="inlineStr">
         <is>
-          <t>SV-8672 (specs/inventory-value.md Story 5 S5-R5; S5-R6)</t>
+          <t>SV-8672 (IV spec v3 2026-07-29 Story 5 S5-R5; S5-R6)</t>
         </is>
       </c>
       <c r="I28" s="2" t="inlineStr"/>
@@ -2320,7 +2320,7 @@
       </c>
       <c r="H37" s="2" t="inlineStr">
         <is>
-          <t>SV-8674 (specs/inventory-value.md Story 7 S7-R1; S7-R2; Story 12 S12-R3 — per-row location identifier in All-locations view ADDED per kickoff video P10 40:58-41:20; user ruling 2026-07-28: video overrides spec (video newer; last-update-wins))</t>
+          <t>SV-8674 (IV spec v3 2026-07-29 Story 7 S7-R1; S7-R2; Story 12 S12-R3 — per-row location identifier in All-locations view ADDED per kickoff video P10 40:58-41:20; user ruling 2026-07-28: video overrides spec (video newer; last-update-wins))</t>
         </is>
       </c>
       <c r="I37" s="2" t="inlineStr"/>
@@ -3084,7 +3084,7 @@
       </c>
       <c r="H52" s="2" t="inlineStr">
         <is>
-          <t>SV-8677 (specs/inventory-value.md Story 10 S10-R7 (+ context note))</t>
+          <t>SV-8677 (IV spec v3 2026-07-29 Story 10 S10-R7 (+ context note))</t>
         </is>
       </c>
       <c r="I52" s="2" t="inlineStr"/>
@@ -3451,7 +3451,7 @@
       </c>
       <c r="H59" s="2" t="inlineStr">
         <is>
-          <t>SV-8679 (specs/inventory-value.md Story 12 S12-R1)</t>
+          <t>SV-8679 (IV spec v3 2026-07-29 Story 12 S12-R1)</t>
         </is>
       </c>
       <c r="I59" s="2" t="inlineStr"/>
@@ -3500,7 +3500,7 @@
       </c>
       <c r="H60" s="2" t="inlineStr">
         <is>
-          <t>SV-8679 (specs/inventory-value.md Story 12 S12-R2; S12-R3)</t>
+          <t>SV-8679 (IV spec v3 2026-07-29 Story 12 S12-R2; S12-R3)</t>
         </is>
       </c>
       <c r="I60" s="2" t="inlineStr"/>

</xml_diff>

<commit_message>
chore(sweeper): checkpoint 20 dirty path(s)
Automatic additive checkpoint so no work is lost (Standing Rule 29).
Paths were hash-stable for 20s and passed the secret scan.
Top-level areas: build, testrail-import

  build/report-suite
  build/report-suite/merges-2026-08-04
  testrail-import

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01AZ5XzKsK9wv7M41cSPaMyg
</commit_message>
<xml_diff>
--- a/testrail-import/Report-Suite_Inventory-Value-Report_testrail-import.xlsx
+++ b/testrail-import/Report-Suite_Inventory-Value-Report_testrail-import.xlsx
@@ -428,7 +428,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J72"/>
+  <dimension ref="A1:J69"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="50" customWidth="1" min="1" max="1"/>
@@ -778,13 +778,14 @@
 2. The core-charge part is never listed — even with a positive quantity — and its value is not counted in the totals row.
 3. The zero-quantity and negative-quantity parts are not listed — only quantities greater than zero are valued.
 4. Only parts meeting BOTH conditions — not a core charge, and on-hand quantity greater than zero — are listed.
+5. A part that has sat without movement for a long time still appears and is still counted — there is no dead-stock exclusion; how long stock has sat makes no difference.
 ---
 This is the expected behaviour as per the build tested on 8/4/2026, and as per the Inventory Value report specification version 3 (S2-R1, S2-R2, S2-N1, S2-N2).</t>
         </is>
       </c>
       <c r="H7" s="2" t="inlineStr">
         <is>
-          <t>SV-8669 (IV spec v3 2026-07-29 Story 2 S2-R1; S2-R2; S2-N1; S2-N2; §3 Key Decisions)</t>
+          <t>SV-8669 (IV spec v3 2026-07-29 Story 2 S2-R1; S2-R2; S2-N1; S2-N2; §3 Key Decisions; Story 2 context note (no dead-stock exclusion))</t>
         </is>
       </c>
       <c r="I7" s="2" t="inlineStr"/>
@@ -842,12 +843,12 @@
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>There is no dead-stock exclusion - a slow-moving part still appears</t>
+          <t>Unit Sell uses the part's fixed sell price when one is set</t>
         </is>
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>IV — Row Scope</t>
+          <t>IV — Valuation &amp; Columns</t>
         </is>
       </c>
       <c r="C9" s="2" t="inlineStr">
@@ -857,71 +858,23 @@
       </c>
       <c r="D9" s="2" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>Critical</t>
         </is>
       </c>
       <c r="E9" s="2" t="inlineStr">
         <is>
           <t>1. You are signed in to the ShopView App on a desktop browser.
-2. A part with positive, non-core stock exists that has had no movement for a long time (or the oldest-stocked part at the location is known).</t>
+2. A ZZAUTOTEST in-stock part exists with a known unit cost, a known FIXED sell price, and a category whose pricing-matrix markup would give a DIFFERENT figure.</t>
         </is>
       </c>
       <c r="F9" s="2" t="inlineStr">
-        <is>
-          <t>1. Open the Inventory Value report scoped to the location.
-2. Search for the long-sitting part.</t>
-        </is>
-      </c>
-      <c r="G9" s="2" t="inlineStr">
-        <is>
-          <t>1. The long-sitting part appears and its value is counted — every part currently holding positive, non-core stock contributes to the on-hand value, however long it has sat.
----
-This is the expected behaviour as per the build tested on 8/4/2026, and as per the Inventory Value report specification version 3.</t>
-        </is>
-      </c>
-      <c r="H9" s="2" t="inlineStr">
-        <is>
-          <t>SV-8669 (IV spec v3 2026-07-29 Story 2 context note (no dead-stock exclusion))</t>
-        </is>
-      </c>
-      <c r="I9" s="2" t="inlineStr"/>
-      <c r="J9" s="2" t="inlineStr"/>
-    </row>
-    <row r="10">
-      <c r="A10" s="2" t="inlineStr">
-        <is>
-          <t>Unit Sell uses the part's fixed sell price when one is set</t>
-        </is>
-      </c>
-      <c r="B10" s="2" t="inlineStr">
-        <is>
-          <t>IV — Valuation &amp; Columns</t>
-        </is>
-      </c>
-      <c r="C10" s="2" t="inlineStr">
-        <is>
-          <t>Functional</t>
-        </is>
-      </c>
-      <c r="D10" s="2" t="inlineStr">
-        <is>
-          <t>Critical</t>
-        </is>
-      </c>
-      <c r="E10" s="2" t="inlineStr">
-        <is>
-          <t>1. You are signed in to the ShopView App on a desktop browser.
-2. A ZZAUTOTEST in-stock part exists with a known unit cost, a known FIXED sell price, and a category whose pricing-matrix markup would give a DIFFERENT figure.</t>
-        </is>
-      </c>
-      <c r="F10" s="2" t="inlineStr">
         <is>
           <t>1. Open the Inventory Value report and find the part's row.
 2. Read its Unit Sell value.
 3. Compare it to the part's fixed sell price and to the figure the category markup would have produced.</t>
         </is>
       </c>
-      <c r="G10" s="2" t="inlineStr">
+      <c r="G9" s="2" t="inlineStr">
         <is>
           <t>1. Unit Sell equals the part's fixed sell price.
 2. The pricing-matrix markup is NOT applied when a fixed sell price is set — the fixed price wins.
@@ -929,85 +882,85 @@
 This is the expected behaviour as per the build tested on 8/4/2026, and as per the Inventory Value report specification version 3 (S3-R5).</t>
         </is>
       </c>
-      <c r="H10" s="2" t="inlineStr">
+      <c r="H9" s="2" t="inlineStr">
         <is>
           <t>SV-8670 (IV spec v3 2026-07-29 Story 3 S3-R5 (fixed-price branch); §3 Key Decisions (unit sell resolved like the parts list))</t>
         </is>
       </c>
-      <c r="I10" s="2" t="inlineStr"/>
-      <c r="J10" s="2" t="inlineStr"/>
-    </row>
-    <row r="11">
-      <c r="A11" s="2" t="inlineStr">
+      <c r="I9" s="2" t="inlineStr"/>
+      <c r="J9" s="2" t="inlineStr"/>
+    </row>
+    <row r="10">
+      <c r="A10" s="2" t="inlineStr">
         <is>
           <t>With no fixed sell price Unit Sell is the category's pricing-matrix markup</t>
         </is>
       </c>
-      <c r="B11" s="2" t="inlineStr">
+      <c r="B10" s="2" t="inlineStr">
         <is>
           <t>IV — Valuation &amp; Columns</t>
         </is>
       </c>
-      <c r="C11" s="2" t="inlineStr">
-        <is>
-          <t>Functional</t>
-        </is>
-      </c>
-      <c r="D11" s="2" t="inlineStr">
+      <c r="C10" s="2" t="inlineStr">
+        <is>
+          <t>Functional</t>
+        </is>
+      </c>
+      <c r="D10" s="2" t="inlineStr">
         <is>
           <t>Critical</t>
         </is>
       </c>
-      <c r="E11" s="2" t="inlineStr">
+      <c r="E10" s="2" t="inlineStr">
         <is>
           <t>1. You are signed in to the ShopView App on a desktop browser.
 2. A ZZAUTOTEST in-stock part exists with a known unit cost, NO fixed sell price, and a category covered by the shop's pricing matrix with a known markup.</t>
         </is>
       </c>
-      <c r="F11" s="2" t="inlineStr">
+      <c r="F10" s="2" t="inlineStr">
         <is>
           <t>1. Open the Inventory Value report and find the part's row.
 2. Read its Unit Sell value.
 3. Compare it to the pricing-matrix markup applied to the part's cost for its category.</t>
         </is>
       </c>
-      <c r="G11" s="2" t="inlineStr">
+      <c r="G10" s="2" t="inlineStr">
         <is>
           <t>1. Unit Sell equals the shop's pricing-matrix markup on cost for that part's category (the same way the parts list resolves it).
 ---
 This is the expected behaviour as per the build tested on 8/4/2026, and as per the Inventory Value report specification version 3 (S3-R5).</t>
         </is>
       </c>
-      <c r="H11" s="2" t="inlineStr">
+      <c r="H10" s="2" t="inlineStr">
         <is>
           <t>SV-8670 (IV spec v3 2026-07-29 Story 3 S3-R5 (matrix branch); §5 Assumptions)</t>
         </is>
       </c>
-      <c r="I11" s="2" t="inlineStr"/>
-      <c r="J11" s="2" t="inlineStr"/>
-    </row>
-    <row r="12">
-      <c r="A12" s="2" t="inlineStr">
+      <c r="I10" s="2" t="inlineStr"/>
+      <c r="J10" s="2" t="inlineStr"/>
+    </row>
+    <row r="11">
+      <c r="A11" s="2" t="inlineStr">
         <is>
           <t>With no fixed sell price and no category, Unit Sell equals Unit Cost</t>
         </is>
       </c>
-      <c r="B12" s="2" t="inlineStr">
+      <c r="B11" s="2" t="inlineStr">
         <is>
           <t>IV — Valuation &amp; Columns</t>
         </is>
       </c>
-      <c r="C12" s="2" t="inlineStr">
-        <is>
-          <t>Functional</t>
-        </is>
-      </c>
-      <c r="D12" s="2" t="inlineStr">
+      <c r="C11" s="2" t="inlineStr">
+        <is>
+          <t>Functional</t>
+        </is>
+      </c>
+      <c r="D11" s="2" t="inlineStr">
         <is>
           <t>Critical</t>
         </is>
       </c>
-      <c r="E12" s="2" t="inlineStr">
+      <c r="E11" s="2" t="inlineStr">
         <is>
           <t>1. You are signed in to the ShopView App on a desktop browser.
 2. A ZZAUTOTEST in-stock part exists with a known unit cost, NO fixed sell price, and NO category.
@@ -1015,14 +968,14 @@
 4. Note for the tester: on this build a part cannot be saved without a category, so you may not be able to create the part described in step 2. If you cannot, mark this test Blocked and say so — do not guess the result.</t>
         </is>
       </c>
-      <c r="F12" s="2" t="inlineStr">
+      <c r="F11" s="2" t="inlineStr">
         <is>
           <t>1. Open the Inventory Value report and find the part's row.
 2. Read its Unit Sell and compare to its Unit Cost.
 3. Read its Margin and Margin % cells.</t>
         </is>
       </c>
-      <c r="G12" s="2" t="inlineStr">
+      <c r="G11" s="2" t="inlineStr">
         <is>
           <t>1. A part with no category takes no markup, so its Unit Sell equals its Unit Cost.
 2. Such a part shows a Margin of $0.00 and a Margin % of 0.0% — the stock is valued at cost.
@@ -1031,50 +984,50 @@
 This is the expected behaviour as per the build tested on 8/4/2026, and as per the Inventory Value report specification version 3 (S3-R5).</t>
         </is>
       </c>
-      <c r="H12" s="2" t="inlineStr">
+      <c r="H11" s="2" t="inlineStr">
         <is>
           <t>SV-8670 (IV spec v3 2026-07-29 Story 3 S3-R5 (no-category fallback) + context note; §5 Assumptions)</t>
         </is>
       </c>
-      <c r="I12" s="2" t="inlineStr"/>
-      <c r="J12" s="2" t="inlineStr"/>
-    </row>
-    <row r="13">
-      <c r="A13" s="2" t="inlineStr">
+      <c r="I11" s="2" t="inlineStr"/>
+      <c r="J11" s="2" t="inlineStr"/>
+    </row>
+    <row r="12">
+      <c r="A12" s="2" t="inlineStr">
         <is>
           <t>Total Sell is quantity × Unit Sell and Total Cost is quantity × Unit Cost</t>
         </is>
       </c>
-      <c r="B13" s="2" t="inlineStr">
+      <c r="B12" s="2" t="inlineStr">
         <is>
           <t>IV — Valuation &amp; Columns</t>
         </is>
       </c>
-      <c r="C13" s="2" t="inlineStr">
-        <is>
-          <t>Functional</t>
-        </is>
-      </c>
-      <c r="D13" s="2" t="inlineStr">
+      <c r="C12" s="2" t="inlineStr">
+        <is>
+          <t>Functional</t>
+        </is>
+      </c>
+      <c r="D12" s="2" t="inlineStr">
         <is>
           <t>Critical</t>
         </is>
       </c>
-      <c r="E13" s="2" t="inlineStr">
+      <c r="E12" s="2" t="inlineStr">
         <is>
           <t>1. You are signed in to the ShopView App on a desktop browser.
 2. A ZZAUTOTEST in-stock part exists with a known on-hand quantity (include a fractional quantity if possible), unit cost, and unit sell.
 3. The Total Sell column is turned on.</t>
         </is>
       </c>
-      <c r="F13" s="2" t="inlineStr">
+      <c r="F12" s="2" t="inlineStr">
         <is>
           <t>1. Open the Inventory Value report and find the part's row.
 2. Multiply the on-hand quantity by Unit Sell and compare to Total Sell.
 3. Multiply the on-hand quantity by Unit Cost and compare to Total Cost.</t>
         </is>
       </c>
-      <c r="G13" s="2" t="inlineStr">
+      <c r="G12" s="2" t="inlineStr">
         <is>
           <t>1. Total Sell equals the part's on-hand quantity × Unit Sell, shown as US-dollar currency.
 2. Total Cost equals the part's on-hand quantity × Unit Cost, shown as US-dollar currency.
@@ -1082,50 +1035,50 @@
 This is the expected behaviour as per the build tested on 8/4/2026, and as per the Inventory Value report specification version 3 (S3-R6, S3-R7).</t>
         </is>
       </c>
-      <c r="H13" s="2" t="inlineStr">
+      <c r="H12" s="2" t="inlineStr">
         <is>
           <t>SV-8670 (IV spec v3 2026-07-29 Story 3 S3-R6; S3-R7; §4 Terminology)</t>
         </is>
       </c>
-      <c r="I13" s="2" t="inlineStr"/>
-      <c r="J13" s="2" t="inlineStr"/>
-    </row>
-    <row r="14">
-      <c r="A14" s="2" t="inlineStr">
+      <c r="I12" s="2" t="inlineStr"/>
+      <c r="J12" s="2" t="inlineStr"/>
+    </row>
+    <row r="13">
+      <c r="A13" s="2" t="inlineStr">
         <is>
           <t>Margin is Total Sell minus Total Cost for the whole on-hand quantity</t>
         </is>
       </c>
-      <c r="B14" s="2" t="inlineStr">
+      <c r="B13" s="2" t="inlineStr">
         <is>
           <t>IV — Valuation &amp; Columns</t>
         </is>
       </c>
-      <c r="C14" s="2" t="inlineStr">
-        <is>
-          <t>Functional</t>
-        </is>
-      </c>
-      <c r="D14" s="2" t="inlineStr">
+      <c r="C13" s="2" t="inlineStr">
+        <is>
+          <t>Functional</t>
+        </is>
+      </c>
+      <c r="D13" s="2" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="E14" s="2" t="inlineStr">
+      <c r="E13" s="2" t="inlineStr">
         <is>
           <t>1. You are signed in to the ShopView App on a desktop browser.
 2. A ZZAUTOTEST in-stock part exists with a quantity greater than 1 and different unit cost and unit sell values.
 3. The Margin and Total Sell columns are turned on.</t>
         </is>
       </c>
-      <c r="F14" s="2" t="inlineStr">
+      <c r="F13" s="2" t="inlineStr">
         <is>
           <t>1. Open the Inventory Value report and find the part's row.
 2. Subtract Total Cost from Total Sell and compare to the Margin cell.
 3. Also compute the per-unit difference (Unit Sell − Unit Cost) and confirm Margin is NOT that per-unit figure.</t>
         </is>
       </c>
-      <c r="G14" s="2" t="inlineStr">
+      <c r="G13" s="2" t="inlineStr">
         <is>
           <t>1. Margin equals Total Sell − Total Cost for the part's whole on-hand quantity, shown as US-dollar currency.
 2. Margin is the extended (total) margin, not the per-unit difference.
@@ -1133,49 +1086,49 @@
 This is the expected behaviour as per the build tested on 8/4/2026, and as per the Inventory Value report specification version 3 (S3-R8).</t>
         </is>
       </c>
-      <c r="H14" s="2" t="inlineStr">
+      <c r="H13" s="2" t="inlineStr">
         <is>
           <t>SV-8670 (IV spec v3 2026-07-29 Story 3 S3-R8; §3 Key Decisions (extended margin); §4 Terminology)</t>
         </is>
       </c>
-      <c r="I14" s="2" t="inlineStr"/>
-      <c r="J14" s="2" t="inlineStr"/>
-    </row>
-    <row r="15">
-      <c r="A15" s="2" t="inlineStr">
+      <c r="I13" s="2" t="inlineStr"/>
+      <c r="J13" s="2" t="inlineStr"/>
+    </row>
+    <row r="14">
+      <c r="A14" s="2" t="inlineStr">
         <is>
           <t>Margin % is Margin over Total Sell to one decimal; em-dash when Sell &lt;= 0</t>
         </is>
       </c>
-      <c r="B15" s="2" t="inlineStr">
+      <c r="B14" s="2" t="inlineStr">
         <is>
           <t>IV — Valuation &amp; Columns</t>
         </is>
       </c>
-      <c r="C15" s="2" t="inlineStr">
-        <is>
-          <t>Functional</t>
-        </is>
-      </c>
-      <c r="D15" s="2" t="inlineStr">
+      <c r="C14" s="2" t="inlineStr">
+        <is>
+          <t>Functional</t>
+        </is>
+      </c>
+      <c r="D14" s="2" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="E15" s="2" t="inlineStr">
+      <c r="E14" s="2" t="inlineStr">
         <is>
           <t>1. You are signed in to the ShopView App on a desktop browser.
 2. The report shows: a part with a normal positive margin, a part whose Margin % computes negative (unit sell below unit cost), and — if producible — a part whose Total Sell is zero.</t>
         </is>
       </c>
-      <c r="F15" s="2" t="inlineStr">
+      <c r="F14" s="2" t="inlineStr">
         <is>
           <t>1. Read the normal part's Margin % and check it against Margin ÷ Total Sell × 100.
 2. Read the negative-margin part's Margin %.
 3. Read the zero-Total-Sell part's Margin % if one exists.</t>
         </is>
       </c>
-      <c r="G15" s="2" t="inlineStr">
+      <c r="G14" s="2" t="inlineStr">
         <is>
           <t>1. Margin % shows Margin as a percentage of Total Sell, to one decimal place followed by a percent sign — for example "39.7%".
 2. A Margin % that computes to a real number, including a negative one, shows its signed value.
@@ -1184,101 +1137,103 @@
 This is the expected behaviour as per the build tested on 8/4/2026, and as per the Inventory Value report specification version 3 (S3-R9, S3-E3).</t>
         </is>
       </c>
-      <c r="H15" s="2" t="inlineStr">
+      <c r="H14" s="2" t="inlineStr">
         <is>
           <t>SV-8670 (IV spec v3 2026-07-29 Story 3 S3-R9; S3-E3)</t>
         </is>
       </c>
-      <c r="I15" s="2" t="inlineStr"/>
-      <c r="J15" s="2" t="inlineStr"/>
-    </row>
-    <row r="16">
-      <c r="A16" s="2" t="inlineStr">
+      <c r="I14" s="2" t="inlineStr"/>
+      <c r="J14" s="2" t="inlineStr"/>
+    </row>
+    <row r="15">
+      <c r="A15" s="2" t="inlineStr">
         <is>
           <t>With every column on they appear in the fixed order with the set alignment</t>
         </is>
       </c>
-      <c r="B16" s="2" t="inlineStr">
+      <c r="B15" s="2" t="inlineStr">
         <is>
           <t>IV — Valuation &amp; Columns</t>
         </is>
       </c>
-      <c r="C16" s="2" t="inlineStr">
-        <is>
-          <t>Functional</t>
-        </is>
-      </c>
-      <c r="D16" s="2" t="inlineStr">
+      <c r="C15" s="2" t="inlineStr">
+        <is>
+          <t>Functional</t>
+        </is>
+      </c>
+      <c r="D15" s="2" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="E16" s="2" t="inlineStr">
+      <c r="E15" s="2" t="inlineStr">
         <is>
           <t>1. You are signed in to the ShopView App on a desktop browser.
 2. The Inventory Value report is open with rows loaded.
 3. Every column (including Margin and Total Sell) is turned on in the column-selection control.</t>
         </is>
       </c>
-      <c r="F16" s="2" t="inlineStr">
+      <c r="F15" s="2" t="inlineStr">
         <is>
           <t>1. Read the column headers from left to right.
 2. Look at how the values in each column are aligned.</t>
         </is>
       </c>
-      <c r="G16" s="2" t="inlineStr">
+      <c r="G15" s="2" t="inlineStr">
         <is>
           <t>1. With a single location in scope the columns appear in this order: Part #, Description, Category, Vendor, Qty, Unit Cost, Unit Sell, Margin, Margin %, Total Sell, Total Cost.
 2. Part #, Description, Category, and Vendor are left-aligned.
 3. Every other column is right-aligned.
 4. Location is one of the columns in the column-selection control; when it is turned on the Location column appears between Vendor and Qty, left-aligned.
 ---
+DO NOT AUTOMATE YET: this behaviour is waiting on an answer from the product owner. Automating it now could lock in the wrong behaviour.
+The open question is in: Report-Suite_Questions-and-Decisions-for-Chris-Ward_2026-08-04.xlsx — https://raw.githubusercontent.com/bilalmuzamil-sketch/Manual-test-Cases/claude/slack-session-0sxnd9/build/report-suite/chris-consolidated-2026-08-04/Report-Suite_Questions-and-Decisions-for-Chris-Ward_2026-08-04.xlsx
 This is the expected behaviour as per the build tested on 8/4/2026, and as per the Inventory Value report specification version 3 (S3-R1, S3-R2, S7-R6); on this point that specification currently states otherwise and a product decision is still awaited, so treat the behaviour described above as what the build does today.</t>
         </is>
       </c>
-      <c r="H16" s="2" t="inlineStr">
+      <c r="H15" s="2" t="inlineStr">
         <is>
           <t>SV-8670; SV-8674 (IV spec v3 2026-07-29 Story 3 S3-R1; S3-R2 + Story 7 S7-R6 — fixed column order and alignment; plus the automatic Location column between Vendor and Qty on Hand)</t>
         </is>
       </c>
-      <c r="I16" s="2" t="inlineStr"/>
-      <c r="J16" s="2" t="inlineStr"/>
-    </row>
-    <row r="17">
-      <c r="A17" s="2" t="inlineStr">
+      <c r="I15" s="2" t="inlineStr"/>
+      <c r="J15" s="2" t="inlineStr"/>
+    </row>
+    <row r="16">
+      <c r="A16" s="2" t="inlineStr">
         <is>
           <t>Value formats: Qty to two decimals; money as US-dollar currency</t>
         </is>
       </c>
-      <c r="B17" s="2" t="inlineStr">
+      <c r="B16" s="2" t="inlineStr">
         <is>
           <t>IV — Valuation &amp; Columns</t>
         </is>
       </c>
-      <c r="C17" s="2" t="inlineStr">
-        <is>
-          <t>Functional</t>
-        </is>
-      </c>
-      <c r="D17" s="2" t="inlineStr">
+      <c r="C16" s="2" t="inlineStr">
+        <is>
+          <t>Functional</t>
+        </is>
+      </c>
+      <c r="D16" s="2" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="E17" s="2" t="inlineStr">
+      <c r="E16" s="2" t="inlineStr">
         <is>
           <t>1. You are signed in to the ShopView App on a desktop browser.
 2. The report shows a part with a fractional quantity (for example 2.50), one with values over $1,000, and (if producible) one with a negative money value.</t>
         </is>
       </c>
-      <c r="F17" s="2" t="inlineStr">
+      <c r="F16" s="2" t="inlineStr">
         <is>
           <t>1. Read the Qty cell of the fractional-quantity part.
 2. Read a money value over one thousand dollars (Unit Cost, Unit Sell, Total Sell, or Total Cost).
 3. Read a genuine zero money value and a negative one if present.</t>
         </is>
       </c>
-      <c r="G17" s="2" t="inlineStr">
+      <c r="G16" s="2" t="inlineStr">
         <is>
           <t>1. Qty shows the on-hand quantity to two decimal places, with no currency symbol; fractional quantities display correctly.
 2. Unit Cost and Unit Sell show per-unit prices as US-dollar currency.
@@ -1287,48 +1242,48 @@
 This is the expected behaviour as per the build tested on 8/4/2026, and as per the Inventory Value report specification version 3 (S3-R3, S3-R4, S3-R5, S3-R10).</t>
         </is>
       </c>
-      <c r="H17" s="2" t="inlineStr">
+      <c r="H16" s="2" t="inlineStr">
         <is>
           <t>SV-8670 (IV spec v3 2026-07-29 Story 3 S3-R3; S3-R4; S3-R5 (display); S3-R10; §4 Terminology (On-hand quantity))</t>
         </is>
       </c>
-      <c r="I17" s="2" t="inlineStr"/>
-      <c r="J17" s="2" t="inlineStr"/>
-    </row>
-    <row r="18">
-      <c r="A18" s="2" t="inlineStr">
+      <c r="I16" s="2" t="inlineStr"/>
+      <c r="J16" s="2" t="inlineStr"/>
+    </row>
+    <row r="17">
+      <c r="A17" s="2" t="inlineStr">
         <is>
           <t>Total Cost is bold and pinned far right; it stays put on sideways scroll</t>
         </is>
       </c>
-      <c r="B18" s="2" t="inlineStr">
+      <c r="B17" s="2" t="inlineStr">
         <is>
           <t>IV — Valuation &amp; Columns</t>
         </is>
       </c>
-      <c r="C18" s="2" t="inlineStr">
-        <is>
-          <t>Functional</t>
-        </is>
-      </c>
-      <c r="D18" s="2" t="inlineStr">
+      <c r="C17" s="2" t="inlineStr">
+        <is>
+          <t>Functional</t>
+        </is>
+      </c>
+      <c r="D17" s="2" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="E18" s="2" t="inlineStr">
+      <c r="E17" s="2" t="inlineStr">
         <is>
           <t>1. You are signed in to the ShopView App on a desktop browser.
 2. Enough columns are turned on that the table scrolls horizontally.</t>
         </is>
       </c>
-      <c r="F18" s="2" t="inlineStr">
+      <c r="F17" s="2" t="inlineStr">
         <is>
           <t>1. Look at the Total Cost column header and its cells.
 2. Scroll the rows sideways and watch the Total Cost column.</t>
         </is>
       </c>
-      <c r="G18" s="2" t="inlineStr">
+      <c r="G17" s="2" t="inlineStr">
         <is>
           <t>1. The Total Cost column is pinned to the far right of the row and shown in bold — it is the report's headline column.
 2. The Total Cost column header is bold and pinned, matching its cells.
@@ -1337,100 +1292,102 @@
 This is the expected behaviour as per the build tested on 8/4/2026, and as per the Inventory Value report specification version 3 (S3-R11, S12-R4).</t>
         </is>
       </c>
-      <c r="H18" s="2" t="inlineStr">
+      <c r="H17" s="2" t="inlineStr">
         <is>
           <t>SV-8670 (IV spec v3 2026-07-29 Story 3 S3-R11; Story 12 S12-R4; §3 Key Decisions)</t>
         </is>
       </c>
-      <c r="I18" s="2" t="inlineStr"/>
-      <c r="J18" s="2" t="inlineStr"/>
-    </row>
-    <row r="19">
-      <c r="A19" s="2" t="inlineStr">
+      <c r="I17" s="2" t="inlineStr"/>
+      <c r="J17" s="2" t="inlineStr"/>
+    </row>
+    <row r="18">
+      <c r="A18" s="2" t="inlineStr">
         <is>
           <t>On a first visit the default columns show and the rest stay available</t>
         </is>
       </c>
-      <c r="B19" s="2" t="inlineStr">
+      <c r="B18" s="2" t="inlineStr">
         <is>
           <t>IV — Valuation &amp; Columns</t>
         </is>
       </c>
-      <c r="C19" s="2" t="inlineStr">
-        <is>
-          <t>Functional</t>
-        </is>
-      </c>
-      <c r="D19" s="2" t="inlineStr">
+      <c r="C18" s="2" t="inlineStr">
+        <is>
+          <t>Functional</t>
+        </is>
+      </c>
+      <c r="D18" s="2" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="E19" s="2" t="inlineStr">
+      <c r="E18" s="2" t="inlineStr">
         <is>
           <t>1. You are signed in to the ShopView App on a desktop browser that has never saved settings for this report (fresh visit).</t>
         </is>
       </c>
-      <c r="F19" s="2" t="inlineStr">
+      <c r="F18" s="2" t="inlineStr">
         <is>
           <t>1. Open the Inventory Value report and read the visible column headers.
 2. Open the column-selection control and read which columns are on and off.
 3. Turn Margin and Total Sell on and check they appear.</t>
         </is>
       </c>
-      <c r="G19" s="2" t="inlineStr">
+      <c r="G18" s="2" t="inlineStr">
         <is>
           <t>1. On first visit with a single location in scope the visible columns are: Part #, Description, Category, Vendor, Qty, Unit Cost, Unit Sell, Margin %, and Total Cost.
 2. The Margin and Total Sell columns are hidden by default.
 3. Both can be turned on from the column-selection control and then appear in their fixed positions.
 4. Location is one of the columns in the column-selection control; when it is turned on the Location column shows between Vendor and Qty.
 ---
+DO NOT AUTOMATE YET: this behaviour is waiting on an answer from the product owner. Automating it now could lock in the wrong behaviour.
+The open question is in: Report-Suite_Questions-and-Decisions-for-Chris-Ward_2026-08-04.xlsx — https://raw.githubusercontent.com/bilalmuzamil-sketch/Manual-test-Cases/claude/slack-session-0sxnd9/build/report-suite/chris-consolidated-2026-08-04/Report-Suite_Questions-and-Decisions-for-Chris-Ward_2026-08-04.xlsx
 This is the expected behaviour as per the build tested on 8/4/2026, and as per the Inventory Value report specification version 3 (S3-R12, S3-R13, S8-R3, S7-R6); on this point that specification currently states otherwise and a product decision is still awaited, so treat the behaviour described above as what the build does today.</t>
         </is>
       </c>
-      <c r="H19" s="2" t="inlineStr">
+      <c r="H18" s="2" t="inlineStr">
         <is>
           <t>SV-8670; SV-8674 (IV spec v3 2026-07-29 Story 3 S3-R12; S3-R13; Story 8 S8-R3 + Story 7 S7-R6 — first-visit default columns; plus the automatic Location column when more than one location is in scope)</t>
         </is>
       </c>
-      <c r="I19" s="2" t="inlineStr"/>
-      <c r="J19" s="2" t="inlineStr"/>
-    </row>
-    <row r="20">
-      <c r="A20" s="2" t="inlineStr">
+      <c r="I18" s="2" t="inlineStr"/>
+      <c r="J18" s="2" t="inlineStr"/>
+    </row>
+    <row r="19">
+      <c r="A19" s="2" t="inlineStr">
         <is>
           <t>Category and Vendor show their names; an em dash ("—") when the part has none</t>
         </is>
       </c>
-      <c r="B20" s="2" t="inlineStr">
+      <c r="B19" s="2" t="inlineStr">
         <is>
           <t>IV — Valuation &amp; Columns</t>
         </is>
       </c>
-      <c r="C20" s="2" t="inlineStr">
-        <is>
-          <t>Functional</t>
-        </is>
-      </c>
-      <c r="D20" s="2" t="inlineStr">
+      <c r="C19" s="2" t="inlineStr">
+        <is>
+          <t>Functional</t>
+        </is>
+      </c>
+      <c r="D19" s="2" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="E20" s="2" t="inlineStr">
+      <c r="E19" s="2" t="inlineStr">
         <is>
           <t>1. You are signed in to the ShopView App on a desktop browser.
 2. The report shows a part with a category and a vendor, a part with no category, and a part with no vendor.</t>
         </is>
       </c>
-      <c r="F20" s="2" t="inlineStr">
+      <c r="F19" s="2" t="inlineStr">
         <is>
           <t>1. Read the Category and Vendor cells of the fully-populated part.
 2. Read the Category cell of the part with no category.
 3. Read the Vendor cell of the part with no vendor.</t>
         </is>
       </c>
-      <c r="G20" s="2" t="inlineStr">
+      <c r="G19" s="2" t="inlineStr">
         <is>
           <t>1. Category shows the part's category name; Vendor shows the part's vendor name.
 2. A part with no category shows an em dash ("—") in its Category cell.
@@ -1440,43 +1397,43 @@
 This is the expected behaviour as per the build tested on 8/4/2026, and as per the Inventory Value report specification version 3 (S3-R14, S3-E1, S3-E2).</t>
         </is>
       </c>
-      <c r="H20" s="2" t="inlineStr">
+      <c r="H19" s="2" t="inlineStr">
         <is>
           <t>SV-8670 (IV spec v3 2026-07-29 Story 3 S3-R14; S3-E1; S3-E2)</t>
         </is>
       </c>
-      <c r="I20" s="2" t="inlineStr"/>
-      <c r="J20" s="2" t="inlineStr"/>
-    </row>
-    <row r="21">
-      <c r="A21" s="2" t="inlineStr">
+      <c r="I19" s="2" t="inlineStr"/>
+      <c r="J19" s="2" t="inlineStr"/>
+    </row>
+    <row r="20">
+      <c r="A20" s="2" t="inlineStr">
         <is>
           <t>Totals row: Total label, blank identity/per-unit cells, pinned bold Total Cost</t>
         </is>
       </c>
-      <c r="B21" s="2" t="inlineStr">
+      <c r="B20" s="2" t="inlineStr">
         <is>
           <t>IV — Totals Row</t>
         </is>
       </c>
-      <c r="C21" s="2" t="inlineStr">
-        <is>
-          <t>Functional</t>
-        </is>
-      </c>
-      <c r="D21" s="2" t="inlineStr">
+      <c r="C20" s="2" t="inlineStr">
+        <is>
+          <t>Functional</t>
+        </is>
+      </c>
+      <c r="D20" s="2" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="E21" s="2" t="inlineStr">
+      <c r="E20" s="2" t="inlineStr">
         <is>
           <t>1. You are signed in to the ShopView App on a desktop browser.
 2. The Inventory Value report is open with rows loaded and all columns turned on.
 3. The page shows more rows than fit on the screen.</t>
         </is>
       </c>
-      <c r="F21" s="2" t="inlineStr">
+      <c r="F20" s="2" t="inlineStr">
         <is>
           <t>1. Look at the row at the bottom of the report.
 2. Read its Part # cell, its Description/Category/Vendor cells, and its Unit Cost/Unit Sell cells.
@@ -1484,47 +1441,48 @@
 4. Scroll the rows up and down and watch the totals row.</t>
         </is>
       </c>
-      <c r="G21" s="2" t="inlineStr">
+      <c r="G20" s="2" t="inlineStr">
         <is>
           <t>1. A totals row is shown at the bottom, with the label "Total" in the Part # column's cell. In the downloaded files the same row is labelled "Totals" — that difference is intended.
 2. The Description, Category, and Vendor cells are blank; the Unit Cost and Unit Sell cells are blank (a per-unit price has no meaningful sum).
 3. The totals-row Total Cost cell is pinned far right and bold, matching the column, and the row uses the same number formats as the data rows.
 4. The totals row stays visible at the bottom while the rows scroll.
 5. Note for the tester: if the label on screen reads "Totals" instead of "Total", mark this test Failed and report it — do not change the test.
----
-This is the expected behaviour as per the build tested on 8/4/2026, and as per the Inventory Value report specification version 3 (S4-R1, S4-R4, S4-R5, S4-R6, S4-R7, S12-R5).</t>
-        </is>
-      </c>
-      <c r="H21" s="2" t="inlineStr">
-        <is>
-          <t>SV-8671 (IV spec v3 2026-07-29 Story 4 S4-R1; S4-R4; S4-R5; S4-R6; S4-R7; Story 12 S12-R5)</t>
-        </is>
-      </c>
-      <c r="I21" s="2" t="inlineStr"/>
-      <c r="J21" s="2" t="inlineStr"/>
-    </row>
-    <row r="22">
-      <c r="A22" s="2" t="inlineStr">
+6. Sorting by any column reorders the data rows only — the totals row stays at the bottom.
+---
+This is the expected behaviour as per the build tested on 8/4/2026, and as per the Inventory Value report specification version 3 (S4-R1, S4-R4, S4-R5, S4-R6, S4-R7, S12-R5, S9-R4).</t>
+        </is>
+      </c>
+      <c r="H20" s="2" t="inlineStr">
+        <is>
+          <t>SV-8671 (IV spec v3 2026-07-29 Story 4 S4-R1; S4-R4; S4-R5; S4-R6; S4-R7; Story 12 S12-R5; Story 9 S9-R4)</t>
+        </is>
+      </c>
+      <c r="I20" s="2" t="inlineStr"/>
+      <c r="J20" s="2" t="inlineStr"/>
+    </row>
+    <row r="21">
+      <c r="A21" s="2" t="inlineStr">
         <is>
           <t>Totals row sums the FULL filtered set on the server, not just the visible page</t>
         </is>
       </c>
-      <c r="B22" s="2" t="inlineStr">
+      <c r="B21" s="2" t="inlineStr">
         <is>
           <t>IV — Totals Row</t>
         </is>
       </c>
-      <c r="C22" s="2" t="inlineStr">
-        <is>
-          <t>Functional</t>
-        </is>
-      </c>
-      <c r="D22" s="2" t="inlineStr">
+      <c r="C21" s="2" t="inlineStr">
+        <is>
+          <t>Functional</t>
+        </is>
+      </c>
+      <c r="D21" s="2" t="inlineStr">
         <is>
           <t>Critical</t>
         </is>
       </c>
-      <c r="E22" s="2" t="inlineStr">
+      <c r="E21" s="2" t="inlineStr">
         <is>
           <t>1. You are signed in to the ShopView App on a desktop browser.
 2. The current filtered set spans more than one page (more rows than one page shows).
@@ -1532,7 +1490,7 @@
 4. The report shows parts across at least two categories and two vendors.</t>
         </is>
       </c>
-      <c r="F22" s="2" t="inlineStr">
+      <c r="F21" s="2" t="inlineStr">
         <is>
           <t>1. Note the totals row's Qty, Margin, Total Sell, and Total Cost on page 1.
 2. Move to page 2 and read the totals row again.
@@ -1540,7 +1498,7 @@
 4. Select one Category and read the totals row; clear it, select one Vendor; clear it, type a part search matching a subset — reading the totals row each time (from a later page too if the set spans pages).</t>
         </is>
       </c>
-      <c r="G22" s="2" t="inlineStr">
+      <c r="G21" s="2" t="inlineStr">
         <is>
           <t>1. The totals row sums Qty, Margin, Total Sell, and Total Cost across the FULL filtered result set — every qualifying row for the current Date, Location, Category, Vendor, and part-search selection, not only the rows on the visible page.
 2. The totals are identical on every page (they do not change as you page).
@@ -1550,50 +1508,50 @@
 This is the expected behaviour as per the build tested on 8/4/2026, and as per the Inventory Value report specification version 3 (S4-R2, S4-R8, S6-R6).</t>
         </is>
       </c>
-      <c r="H22" s="2" t="inlineStr">
+      <c r="H21" s="2" t="inlineStr">
         <is>
           <t>SV-8671 (IV spec v3 2026-07-29 Story 4 S4-R2; S4-R8; Story 6 S6-R6; §2 Scale and data model; §4 Terminology (Filtered set))</t>
         </is>
       </c>
-      <c r="I22" s="2" t="inlineStr"/>
-      <c r="J22" s="2" t="inlineStr"/>
-    </row>
-    <row r="23">
-      <c r="A23" s="2" t="inlineStr">
+      <c r="I21" s="2" t="inlineStr"/>
+      <c r="J21" s="2" t="inlineStr"/>
+    </row>
+    <row r="22">
+      <c r="A22" s="2" t="inlineStr">
         <is>
           <t>Totals-row Margin % is recomputed from the totals; not an average of rows</t>
         </is>
       </c>
-      <c r="B23" s="2" t="inlineStr">
+      <c r="B22" s="2" t="inlineStr">
         <is>
           <t>IV — Totals Row</t>
         </is>
       </c>
-      <c r="C23" s="2" t="inlineStr">
-        <is>
-          <t>Functional</t>
-        </is>
-      </c>
-      <c r="D23" s="2" t="inlineStr">
+      <c r="C22" s="2" t="inlineStr">
+        <is>
+          <t>Functional</t>
+        </is>
+      </c>
+      <c r="D22" s="2" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="E23" s="2" t="inlineStr">
+      <c r="E22" s="2" t="inlineStr">
         <is>
           <t>1. You are signed in to the ShopView App on a desktop browser.
 2. The filtered set contains parts with clearly different Margin % values (so a recomputed figure differs from a simple average).
 3. The Margin and Total Sell columns are turned on.</t>
         </is>
       </c>
-      <c r="F23" s="2" t="inlineStr">
+      <c r="F22" s="2" t="inlineStr">
         <is>
           <t>1. Read the totals row's Margin, Total Sell, and Margin %.
 2. Compute total Margin ÷ total Total Sell × 100 and compare to the shown Margin %.
 3. Also compute the plain average of the row Margin % values and confirm the shown figure is NOT that.</t>
         </is>
       </c>
-      <c r="G23" s="2" t="inlineStr">
+      <c r="G22" s="2" t="inlineStr">
         <is>
           <t>1. The totals-row Margin % equals total Margin ÷ total Total Sell × 100 (to one decimal place with a percent sign).
 2. It is NOT the average of the row percentages.
@@ -1602,9 +1560,60 @@
 This is the expected behaviour as per the build tested on 8/4/2026, and as per the Inventory Value report specification version 3 (S4-R3).</t>
         </is>
       </c>
+      <c r="H22" s="2" t="inlineStr">
+        <is>
+          <t>SV-8671 (IV spec v3 2026-07-29 Story 4 S4-R3)</t>
+        </is>
+      </c>
+      <c r="I22" s="2" t="inlineStr"/>
+      <c r="J22" s="2" t="inlineStr"/>
+    </row>
+    <row r="23">
+      <c r="A23" s="2" t="inlineStr">
+        <is>
+          <t>Date range offers the standard presets plus Custom; no All Time option</t>
+        </is>
+      </c>
+      <c r="B23" s="2" t="inlineStr">
+        <is>
+          <t>IV — As-of Date &amp; Snapshots</t>
+        </is>
+      </c>
+      <c r="C23" s="2" t="inlineStr">
+        <is>
+          <t>Functional</t>
+        </is>
+      </c>
+      <c r="D23" s="2" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="E23" s="2" t="inlineStr">
+        <is>
+          <t>1. You are signed in to the ShopView App on a desktop browser.
+2. The Inventory Value report is open.</t>
+        </is>
+      </c>
+      <c r="F23" s="2" t="inlineStr">
+        <is>
+          <t>1. Open the date-range control in the toolbar.
+2. Read every option offered.</t>
+        </is>
+      </c>
+      <c r="G23" s="2" t="inlineStr">
+        <is>
+          <t>1. The control offers the standard presets: "Today", "Yesterday", "This Week", "Last Week", "This Month", "Last Month", "This Year", "Last Year", "This Quarter", "Last Quarter", and "Custom".
+2. "All Time" is NOT offered — because the report is valued as of a single date, an All-Time option would be meaningless; its absence is the documented v1 behavior.
+---
+DO NOT AUTOMATE YET: this behaviour is waiting on an answer from the product owner. Automating it now could lock in the wrong behaviour.
+The open question is in: Report-Suite_Questions-and-Decisions-for-Chris-Ward_2026-08-04.xlsx — https://raw.githubusercontent.com/bilalmuzamil-sketch/Manual-test-Cases/claude/slack-session-0sxnd9/build/report-suite/chris-consolidated-2026-08-04/Report-Suite_Questions-and-Decisions-for-Chris-Ward_2026-08-04.xlsx
+This is the expected behaviour as per the build tested on 8/4/2026, and as per the Inventory Value report specification version 3 (S5-R1).</t>
+        </is>
+      </c>
       <c r="H23" s="2" t="inlineStr">
         <is>
-          <t>SV-8671 (IV spec v3 2026-07-29 Story 4 S4-R3)</t>
+          <t>SV-8672 (IV spec v3 2026-07-29 Story 5 S5-R1; §2 Known Limitations (v1))</t>
         </is>
       </c>
       <c r="I23" s="2" t="inlineStr"/>
@@ -1613,7 +1622,7 @@
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
         <is>
-          <t>Date range offers the standard presets plus Custom; no All Time option</t>
+          <t>The report values inventory as of the END of the selected range</t>
         </is>
       </c>
       <c r="B24" s="2" t="inlineStr">
@@ -1628,73 +1637,24 @@
       </c>
       <c r="D24" s="2" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Critical</t>
         </is>
       </c>
       <c r="E24" s="2" t="inlineStr">
-        <is>
-          <t>1. You are signed in to the ShopView App on a desktop browser.
-2. The Inventory Value report is open.</t>
-        </is>
-      </c>
-      <c r="F24" s="2" t="inlineStr">
-        <is>
-          <t>1. Open the date-range control in the toolbar.
-2. Read every option offered.</t>
-        </is>
-      </c>
-      <c r="G24" s="2" t="inlineStr">
-        <is>
-          <t>1. The control offers the standard presets: "Today", "Yesterday", "This Week", "Last Week", "This Month", "Last Month", "This Year", "Last Year", "This Quarter", "Last Quarter", and "Custom".
-2. "All Time" is NOT offered — because the report is valued as of a single date, an All-Time option would be meaningless; its absence is the documented v1 behavior.
----
-This is the expected behaviour as per the build tested on 8/4/2026, and as per the Inventory Value report specification version 3 (S5-R1).</t>
-        </is>
-      </c>
-      <c r="H24" s="2" t="inlineStr">
-        <is>
-          <t>SV-8672 (IV spec v3 2026-07-29 Story 5 S5-R1; §2 Known Limitations (v1))</t>
-        </is>
-      </c>
-      <c r="I24" s="2" t="inlineStr"/>
-      <c r="J24" s="2" t="inlineStr"/>
-    </row>
-    <row r="25">
-      <c r="A25" s="2" t="inlineStr">
-        <is>
-          <t>The report values inventory as of the END of the selected range</t>
-        </is>
-      </c>
-      <c r="B25" s="2" t="inlineStr">
-        <is>
-          <t>IV — As-of Date &amp; Snapshots</t>
-        </is>
-      </c>
-      <c r="C25" s="2" t="inlineStr">
-        <is>
-          <t>Functional</t>
-        </is>
-      </c>
-      <c r="D25" s="2" t="inlineStr">
-        <is>
-          <t>Critical</t>
-        </is>
-      </c>
-      <c r="E25" s="2" t="inlineStr">
         <is>
           <t>1. You are signed in to the ShopView App on a desktop browser.
 2. Nightly snapshots exist for past dates at the selected location (recording has been running).
 3. A part exists that was ALREADY in stock before the selected range started.</t>
         </is>
       </c>
-      <c r="F25" s="2" t="inlineStr">
+      <c r="F24" s="2" t="inlineStr">
         <is>
           <t>1. Select a past range (for example "Last Month").
 2. Check which date the displayed values represent.
 3. Look for the part that was stocked before the range started.</t>
         </is>
       </c>
-      <c r="G25" s="2" t="inlineStr">
+      <c r="G24" s="2" t="inlineStr">
         <is>
           <t>1. The report values inventory as of the END of the selected range.
 2. The date control is an "as of" anchor, not a created-date filter — narrowing it does not select "parts added in that range"; it shows the whole shelf as it stood on that date, so the part stocked before the range still appears.
@@ -1703,9 +1663,59 @@
 This is the expected behaviour as per the build tested on 8/4/2026, and as per the Inventory Value report specification version 3 (S5-R2).</t>
         </is>
       </c>
+      <c r="H24" s="2" t="inlineStr">
+        <is>
+          <t>SV-8672 (IV spec v3 2026-07-29 Story 5 S5-R2 (+ context note))</t>
+        </is>
+      </c>
+      <c r="I24" s="2" t="inlineStr"/>
+      <c r="J24" s="2" t="inlineStr"/>
+    </row>
+    <row r="25">
+      <c r="A25" s="2" t="inlineStr">
+        <is>
+          <t>A window reaching today with today not yet recorded values live stock</t>
+        </is>
+      </c>
+      <c r="B25" s="2" t="inlineStr">
+        <is>
+          <t>IV — As-of Date &amp; Snapshots</t>
+        </is>
+      </c>
+      <c r="C25" s="2" t="inlineStr">
+        <is>
+          <t>Functional</t>
+        </is>
+      </c>
+      <c r="D25" s="2" t="inlineStr">
+        <is>
+          <t>Critical</t>
+        </is>
+      </c>
+      <c r="E25" s="2" t="inlineStr">
+        <is>
+          <t>1. You are signed in to the ShopView App on a desktop browser.
+2. Today's nightly snapshot has not yet been recorded (the normal daytime state).
+3. A ZZAUTOTEST part's on-hand quantity was changed TODAY (after last night's capture).</t>
+        </is>
+      </c>
+      <c r="F25" s="2" t="inlineStr">
+        <is>
+          <t>1. Select a range that reaches today (for example "This Month" or "Today").
+2. Find the part whose quantity changed today and read its row.</t>
+        </is>
+      </c>
+      <c r="G25" s="2" t="inlineStr">
+        <is>
+          <t>1. The report values the current live stock — the values represent today.
+2. The part's row reflects today's changed quantity (not yesterday's snapshot), proving the live fallback is in use.
+---
+This is the expected behaviour as per the build tested on 8/4/2026, and as per the Inventory Value report specification version 3 (S5-R3).</t>
+        </is>
+      </c>
       <c r="H25" s="2" t="inlineStr">
         <is>
-          <t>SV-8672 (IV spec v3 2026-07-29 Story 5 S5-R2 (+ context note))</t>
+          <t>SV-8672 (IV spec v3 2026-07-29 Story 5 S5-R3; §3 Key Decisions (live fallback for today))</t>
         </is>
       </c>
       <c r="I25" s="2" t="inlineStr"/>
@@ -1714,7 +1724,7 @@
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
         <is>
-          <t>A window reaching today with today not yet recorded values live stock</t>
+          <t>For a past date the report replays the closest recorded day on or before it</t>
         </is>
       </c>
       <c r="B26" s="2" t="inlineStr">
@@ -1735,118 +1745,70 @@
       <c r="E26" s="2" t="inlineStr">
         <is>
           <t>1. You are signed in to the ShopView App on a desktop browser.
-2. Today's nightly snapshot has not yet been recorded (the normal daytime state).
-3. A ZZAUTOTEST part's on-hand quantity was changed TODAY (after last night's capture).</t>
+2. Nightly snapshots exist for past dates, and a ZZAUTOTEST part's quantity is known to have DIFFERED on a past recorded day from its quantity today.</t>
         </is>
       </c>
       <c r="F26" s="2" t="inlineStr">
-        <is>
-          <t>1. Select a range that reaches today (for example "This Month" or "Today").
-2. Find the part whose quantity changed today and read its row.</t>
-        </is>
-      </c>
-      <c r="G26" s="2" t="inlineStr">
-        <is>
-          <t>1. The report values the current live stock — the values represent today.
-2. The part's row reflects today's changed quantity (not yesterday's snapshot), proving the live fallback is in use.
----
-This is the expected behaviour as per the build tested on 8/4/2026, and as per the Inventory Value report specification version 3 (S5-R3).</t>
-        </is>
-      </c>
-      <c r="H26" s="2" t="inlineStr">
-        <is>
-          <t>SV-8672 (IV spec v3 2026-07-29 Story 5 S5-R3; §3 Key Decisions (live fallback for today))</t>
-        </is>
-      </c>
-      <c r="I26" s="2" t="inlineStr"/>
-      <c r="J26" s="2" t="inlineStr"/>
-    </row>
-    <row r="27">
-      <c r="A27" s="2" t="inlineStr">
-        <is>
-          <t>For a past date the report replays the closest recorded day on or before it</t>
-        </is>
-      </c>
-      <c r="B27" s="2" t="inlineStr">
-        <is>
-          <t>IV — As-of Date &amp; Snapshots</t>
-        </is>
-      </c>
-      <c r="C27" s="2" t="inlineStr">
-        <is>
-          <t>Functional</t>
-        </is>
-      </c>
-      <c r="D27" s="2" t="inlineStr">
-        <is>
-          <t>Critical</t>
-        </is>
-      </c>
-      <c r="E27" s="2" t="inlineStr">
-        <is>
-          <t>1. You are signed in to the ShopView App on a desktop browser.
-2. Nightly snapshots exist for past dates, and a ZZAUTOTEST part's quantity is known to have DIFFERED on a past recorded day from its quantity today.</t>
-        </is>
-      </c>
-      <c r="F27" s="2" t="inlineStr">
         <is>
           <t>1. Open the date range picker and use the month calendar inside it to set a range ending on the past recorded day, then apply.
 2. Find the part and read its quantity and values.
 3. Compare them to what the part held on that recorded day (not today).</t>
         </is>
       </c>
-      <c r="G27" s="2" t="inlineStr">
+      <c r="G26" s="2" t="inlineStr">
         <is>
           <t>1. The report replays the closest recorded day on or before the end of the selected range.
 2. The part's row shows the quantity and values recorded for that day, not today's live stock.
 Known issue: the product does not currently do this. It has been filed for a fix here: https://shopview.atlassian.net/browse/SV-8820
 ---
+DO NOT AUTOMATE YET: this behaviour is waiting on an answer from the product owner. Automating it now could lock in the wrong behaviour.
+The open question is in: Report-Suite_Questions-and-Decisions-for-Chris-Ward_2026-08-04.xlsx — https://raw.githubusercontent.com/bilalmuzamil-sketch/Manual-test-Cases/claude/slack-session-0sxnd9/build/report-suite/chris-consolidated-2026-08-04/Report-Suite_Questions-and-Decisions-for-Chris-Ward_2026-08-04.xlsx
 This is the expected behaviour as per the build tested on 8/4/2026, and as per the Inventory Value report specification version 3 (S5-R4).</t>
         </is>
       </c>
-      <c r="H27" s="2" t="inlineStr">
+      <c r="H26" s="2" t="inlineStr">
         <is>
           <t>SV-8672 (IV spec v3 2026-07-29 Story 5 S5-R4; §2 Relationship to nightly history)</t>
         </is>
       </c>
-      <c r="I27" s="2" t="inlineStr"/>
-      <c r="J27" s="2" t="inlineStr"/>
-    </row>
-    <row r="28">
-      <c r="A28" s="2" t="inlineStr">
+      <c r="I26" s="2" t="inlineStr"/>
+      <c r="J26" s="2" t="inlineStr"/>
+    </row>
+    <row r="27">
+      <c r="A27" s="2" t="inlineStr">
         <is>
           <t>"As of" indicator names the day shown; hidden when it matches the ask</t>
         </is>
       </c>
-      <c r="B28" s="2" t="inlineStr">
+      <c r="B27" s="2" t="inlineStr">
         <is>
           <t>IV — As-of Date &amp; Snapshots</t>
         </is>
       </c>
-      <c r="C28" s="2" t="inlineStr">
-        <is>
-          <t>Functional</t>
-        </is>
-      </c>
-      <c r="D28" s="2" t="inlineStr">
+      <c r="C27" s="2" t="inlineStr">
+        <is>
+          <t>Functional</t>
+        </is>
+      </c>
+      <c r="D27" s="2" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="E28" s="2" t="inlineStr">
+      <c r="E27" s="2" t="inlineStr">
         <is>
           <t>1. You are signed in to the ShopView App on a desktop browser.
 2. A past date exists that has NO snapshot of its own but has an earlier recorded day before it (for example, a gap day, or a date in the thinned monthly-retention band).</t>
         </is>
       </c>
-      <c r="F28" s="2" t="inlineStr">
+      <c r="F27" s="2" t="inlineStr">
         <is>
           <t>1. Select a Custom range ending on the gap date (a date with no snapshot of its own).
 2. Look for an "As of" indicator and read which day it names.
 3. Then select a range ending on a day that IS recorded (or today with live values) and look for the indicator again.</t>
         </is>
       </c>
-      <c r="G28" s="2" t="inlineStr">
+      <c r="G27" s="2" t="inlineStr">
         <is>
           <t>1. When the displayed day is an earlier recorded day than the date asked for, the report shows an "As of" indicator naming the day actually shown.
 2. When the displayed day matches the date asked for (the common current-view case), the "As of" indicator is not shown — the date control already communicates the date.
@@ -1855,42 +1817,42 @@
 This is the expected behaviour as per the build tested on 8/4/2026, and as per the Inventory Value report specification version 3 (S5-R5, S5-R6).</t>
         </is>
       </c>
-      <c r="H28" s="2" t="inlineStr">
+      <c r="H27" s="2" t="inlineStr">
         <is>
           <t>SV-8672 (IV spec v3 2026-07-29 Story 5 S5-R5; S5-R6)</t>
         </is>
       </c>
-      <c r="I28" s="2" t="inlineStr"/>
-      <c r="J28" s="2" t="inlineStr"/>
-    </row>
-    <row r="29">
-      <c r="A29" s="2" t="inlineStr">
+      <c r="I27" s="2" t="inlineStr"/>
+      <c r="J27" s="2" t="inlineStr"/>
+    </row>
+    <row r="28">
+      <c r="A28" s="2" t="inlineStr">
         <is>
           <t>A Custom range values stock as of the picked end date; capped at today</t>
         </is>
       </c>
-      <c r="B29" s="2" t="inlineStr">
+      <c r="B28" s="2" t="inlineStr">
         <is>
           <t>IV — As-of Date &amp; Snapshots</t>
         </is>
       </c>
-      <c r="C29" s="2" t="inlineStr">
-        <is>
-          <t>Functional</t>
-        </is>
-      </c>
-      <c r="D29" s="2" t="inlineStr">
+      <c r="C28" s="2" t="inlineStr">
+        <is>
+          <t>Functional</t>
+        </is>
+      </c>
+      <c r="D28" s="2" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="E29" s="2" t="inlineStr">
+      <c r="E28" s="2" t="inlineStr">
         <is>
           <t>1. You are signed in to the ShopView App on a desktop browser.
 2. The Inventory Value report is open.</t>
         </is>
       </c>
-      <c r="F29" s="2" t="inlineStr">
+      <c r="F28" s="2" t="inlineStr">
         <is>
           <t>1. Open the date-range control - a month calendar is shown inside it (there is no separate "Custom" item to choose).
 2. Pick a start and an end date in the past on that calendar and press Apply.
@@ -1898,7 +1860,7 @@
 4. Watch the data area when the range is applied.</t>
         </is>
       </c>
-      <c r="G29" s="2" t="inlineStr">
+      <c r="G28" s="2" t="inlineStr">
         <is>
           <t>1. A Custom range lets the user pick a start and end date, and the report values as of the picked end date.
 2. A future end date cannot be chosen — the end date is capped at today.
@@ -1908,9 +1870,58 @@
 This is the expected behaviour as per the build tested on 8/4/2026, and as per the Inventory Value report specification version 3 (S5-R7, S5-R8).</t>
         </is>
       </c>
+      <c r="H28" s="2" t="inlineStr">
+        <is>
+          <t>SV-8672 (IV spec v3 2026-07-29 Story 5 S5-R7; S5-R8)</t>
+        </is>
+      </c>
+      <c r="I28" s="2" t="inlineStr"/>
+      <c r="J28" s="2" t="inlineStr"/>
+    </row>
+    <row r="29">
+      <c r="A29" s="2" t="inlineStr">
+        <is>
+          <t>History accrues forward only; a pre-first-recording date is not shown</t>
+        </is>
+      </c>
+      <c r="B29" s="2" t="inlineStr">
+        <is>
+          <t>IV — As-of Date &amp; Snapshots</t>
+        </is>
+      </c>
+      <c r="C29" s="2" t="inlineStr">
+        <is>
+          <t>Functional</t>
+        </is>
+      </c>
+      <c r="D29" s="2" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="E29" s="2" t="inlineStr">
+        <is>
+          <t>1. You are signed in to the ShopView App on a desktop browser.
+2. The date nightly recording began at this organization is known.</t>
+        </is>
+      </c>
+      <c r="F29" s="2" t="inlineStr">
+        <is>
+          <t>1. Select a range ending before the first nightly recording.
+2. Read what the report shows.</t>
+        </is>
+      </c>
+      <c r="G29" s="2" t="inlineStr">
+        <is>
+          <t>1. The report shows the empty state — there is no way to reconstruct inventory value for a date before recording began, because there is no historical backfill.
+2. This forward-capture-only behavior is the documented v1 boundary, not a defect.
+---
+This is the expected behaviour as per the build tested on 8/4/2026, and as per the Inventory Value report specification version 3 (S5-E1).</t>
+        </is>
+      </c>
       <c r="H29" s="2" t="inlineStr">
         <is>
-          <t>SV-8672 (IV spec v3 2026-07-29 Story 5 S5-R7; S5-R8)</t>
+          <t>SV-8672 (IV spec v3 2026-07-29 Story 5 S5-E1; §2 Known Limitations (v1); §2 Out of scope)</t>
         </is>
       </c>
       <c r="I29" s="2" t="inlineStr"/>
@@ -1919,7 +1930,7 @@
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
         <is>
-          <t>History accrues forward only; a pre-first-recording date is not shown</t>
+          <t>A recorded day keeps its category and vendor names after a rename or delete</t>
         </is>
       </c>
       <c r="B30" s="2" t="inlineStr">
@@ -1940,59 +1951,10 @@
       <c r="E30" s="2" t="inlineStr">
         <is>
           <t>1. You are signed in to the ShopView App on a desktop browser.
-2. The date nightly recording began at this organization is known.</t>
+2. A recorded (overnight-captured) day exists that includes ZZAUTOTEST parts under a known category and a known vendor.</t>
         </is>
       </c>
       <c r="F30" s="2" t="inlineStr">
-        <is>
-          <t>1. Select a range ending before the first nightly recording.
-2. Read what the report shows.</t>
-        </is>
-      </c>
-      <c r="G30" s="2" t="inlineStr">
-        <is>
-          <t>1. The report shows the empty state — there is no way to reconstruct inventory value for a date before recording began, because there is no historical backfill.
-2. This forward-capture-only behavior is the documented v1 boundary, not a defect.
----
-This is the expected behaviour as per the build tested on 8/4/2026, and as per the Inventory Value report specification version 3 (S5-E1).</t>
-        </is>
-      </c>
-      <c r="H30" s="2" t="inlineStr">
-        <is>
-          <t>SV-8672 (IV spec v3 2026-07-29 Story 5 S5-E1; §2 Known Limitations (v1); §2 Out of scope)</t>
-        </is>
-      </c>
-      <c r="I30" s="2" t="inlineStr"/>
-      <c r="J30" s="2" t="inlineStr"/>
-    </row>
-    <row r="31">
-      <c r="A31" s="2" t="inlineStr">
-        <is>
-          <t>A recorded day keeps its category and vendor names after a rename or delete</t>
-        </is>
-      </c>
-      <c r="B31" s="2" t="inlineStr">
-        <is>
-          <t>IV — As-of Date &amp; Snapshots</t>
-        </is>
-      </c>
-      <c r="C31" s="2" t="inlineStr">
-        <is>
-          <t>Functional</t>
-        </is>
-      </c>
-      <c r="D31" s="2" t="inlineStr">
-        <is>
-          <t>Medium</t>
-        </is>
-      </c>
-      <c r="E31" s="2" t="inlineStr">
-        <is>
-          <t>1. You are signed in to the ShopView App on a desktop browser.
-2. A recorded (overnight-captured) day exists that includes ZZAUTOTEST parts under a known category and a known vendor.</t>
-        </is>
-      </c>
-      <c r="F31" s="2" t="inlineStr">
         <is>
           <t>1. Rename that part category (and/or rename or delete the vendor) in administration.
 2. Set the report's date range so it shows the earlier recorded day (the "As of" indicator names that earlier date).
@@ -2000,7 +1962,7 @@
 4. Move the range back to include today (live view) and re-read a renamed category's rows.</t>
         </is>
       </c>
-      <c r="G31" s="2" t="inlineStr">
+      <c r="G30" s="2" t="inlineStr">
         <is>
           <t>1. The earlier recorded day still shows the category and vendor names AS THEY WERE RECORDED that day — a recorded day equals what the live report showed that day, even after the rename/delete.
 2. The rename/delete causes no blank Category/Vendor cells and no dropped rows on the recorded day.
@@ -2009,49 +1971,49 @@
 This is the expected behaviour as per the build tested on 8/4/2026, and as per the Inventory Value report specification version 3 (S11-R2, S5-R4).</t>
         </is>
       </c>
-      <c r="H31" s="2" t="inlineStr">
+      <c r="H30" s="2" t="inlineStr">
         <is>
           <t>SV-8678 (IV spec v3 2026-07-29 Story 11 S11-R2; Story 5 S5-R4; tech-plan-2026-07-29 B4.1 — names stored with the recorded rows on purpose)</t>
         </is>
       </c>
-      <c r="I31" s="2" t="inlineStr"/>
-      <c r="J31" s="2" t="inlineStr"/>
-    </row>
-    <row r="32">
-      <c r="A32" s="2" t="inlineStr">
+      <c r="I30" s="2" t="inlineStr"/>
+      <c r="J30" s="2" t="inlineStr"/>
+    </row>
+    <row r="31">
+      <c r="A31" s="2" t="inlineStr">
         <is>
           <t>Category and Vendor multi-selects reload the report to matching parts only</t>
         </is>
       </c>
-      <c r="B32" s="2" t="inlineStr">
+      <c r="B31" s="2" t="inlineStr">
         <is>
           <t>IV — Filters &amp; Part Search</t>
         </is>
       </c>
-      <c r="C32" s="2" t="inlineStr">
-        <is>
-          <t>Functional</t>
-        </is>
-      </c>
-      <c r="D32" s="2" t="inlineStr">
+      <c r="C31" s="2" t="inlineStr">
+        <is>
+          <t>Functional</t>
+        </is>
+      </c>
+      <c r="D31" s="2" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="E32" s="2" t="inlineStr">
+      <c r="E31" s="2" t="inlineStr">
         <is>
           <t>1. You are signed in to the ShopView App on a desktop browser.
 2. In-stock parts exist across at least two categories and two vendors.</t>
         </is>
       </c>
-      <c r="F32" s="2" t="inlineStr">
+      <c r="F31" s="2" t="inlineStr">
         <is>
           <t>1. Open the filter labeled "Category" and select one category; watch the data area.
 2. Add a second category to the selection.
 3. Clear the Category filter, open the filter labeled "Vendor", and select one vendor; then add a second.</t>
         </is>
       </c>
-      <c r="G32" s="2" t="inlineStr">
+      <c r="G31" s="2" t="inlineStr">
         <is>
           <t>1. The toolbar has a Category filter labeled "Category" and a Vendor filter labeled "Vendor", each allowing one or more selections.
 2. Selecting one or more categories reloads the report to show only parts in the selected categories.
@@ -2060,42 +2022,42 @@
 This is the expected behaviour as per the build tested on 8/4/2026, and as per the Inventory Value report specification version 3 (S6-R1, S6-R2, S6-R3, S6-R4).</t>
         </is>
       </c>
-      <c r="H32" s="2" t="inlineStr">
+      <c r="H31" s="2" t="inlineStr">
         <is>
           <t>SV-8673 (IV spec v3 2026-07-29 Story 6 S6-R1; S6-R2; S6-R3; S6-R4)</t>
         </is>
       </c>
-      <c r="I32" s="2" t="inlineStr"/>
-      <c r="J32" s="2" t="inlineStr"/>
-    </row>
-    <row r="33">
-      <c r="A33" s="2" t="inlineStr">
+      <c r="I31" s="2" t="inlineStr"/>
+      <c r="J31" s="2" t="inlineStr"/>
+    </row>
+    <row r="32">
+      <c r="A32" s="2" t="inlineStr">
         <is>
           <t>Category, Vendor and part search are server-side; each change returns page 1</t>
         </is>
       </c>
-      <c r="B33" s="2" t="inlineStr">
+      <c r="B32" s="2" t="inlineStr">
         <is>
           <t>IV — Filters &amp; Part Search</t>
         </is>
       </c>
-      <c r="C33" s="2" t="inlineStr">
-        <is>
-          <t>Functional</t>
-        </is>
-      </c>
-      <c r="D33" s="2" t="inlineStr">
+      <c r="C32" s="2" t="inlineStr">
+        <is>
+          <t>Functional</t>
+        </is>
+      </c>
+      <c r="D32" s="2" t="inlineStr">
         <is>
           <t>Critical</t>
         </is>
       </c>
-      <c r="E33" s="2" t="inlineStr">
+      <c r="E32" s="2" t="inlineStr">
         <is>
           <t>1. You are signed in to the ShopView App on a desktop browser.
 2. The unfiltered result set is long enough to need scrolling, and matching parts for a category/vendor/search exist well down the list (beyond the first screenful).</t>
         </is>
       </c>
-      <c r="F33" s="2" t="inlineStr">
+      <c r="F32" s="2" t="inlineStr">
         <is>
           <t>1. Scroll well down the list, then select a Category and check whether the list has jumped back to the top and which rows are now listed.
 2. Repeat with a Vendor selection.
@@ -2103,7 +2065,7 @@
 4. Also change the date range, the location selection, and the sort — watching the data area each time.</t>
         </is>
       </c>
-      <c r="G33" s="2" t="inlineStr">
+      <c r="G32" s="2" t="inlineStr">
         <is>
           <t>1. Each change re-queries the server and the list jumps back to the top of the new set of rows.
 2. The filtering covers the ENTIRE data set — matching parts that were further down the list appear — not just a narrowing of the rows currently on screen.
@@ -2112,49 +2074,49 @@
 This is the expected behaviour as per the build tested on 8/4/2026, and as per the Inventory Value report specification version 3 (S6-R5, S1-R4, S1-R5, S1-R7, S1-R8).</t>
         </is>
       </c>
-      <c r="H33" s="2" t="inlineStr">
+      <c r="H32" s="2" t="inlineStr">
         <is>
           <t>SV-8673 (IV spec v3 2026-07-29 Story 6 S6-R5; Story 1 S1-R4; S1-R5; S1-R7; S1-R8)</t>
         </is>
       </c>
-      <c r="I33" s="2" t="inlineStr"/>
-      <c r="J33" s="2" t="inlineStr"/>
-    </row>
-    <row r="34">
-      <c r="A34" s="2" t="inlineStr">
+      <c r="I32" s="2" t="inlineStr"/>
+      <c r="J32" s="2" t="inlineStr"/>
+    </row>
+    <row r="33">
+      <c r="A33" s="2" t="inlineStr">
         <is>
           <t>With no category or vendor selected all parts show</t>
         </is>
       </c>
-      <c r="B34" s="2" t="inlineStr">
+      <c r="B33" s="2" t="inlineStr">
         <is>
           <t>IV — Filters &amp; Part Search</t>
         </is>
       </c>
-      <c r="C34" s="2" t="inlineStr">
-        <is>
-          <t>Functional</t>
-        </is>
-      </c>
-      <c r="D34" s="2" t="inlineStr">
+      <c r="C33" s="2" t="inlineStr">
+        <is>
+          <t>Functional</t>
+        </is>
+      </c>
+      <c r="D33" s="2" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="E34" s="2" t="inlineStr">
+      <c r="E33" s="2" t="inlineStr">
         <is>
           <t>1. You are signed in to the ShopView App on a desktop browser.
 2. The report has been filtered by category, vendor, and a part search.</t>
         </is>
       </c>
-      <c r="F34" s="2" t="inlineStr">
+      <c r="F33" s="2" t="inlineStr">
         <is>
           <t>1. Clear the Category selection and check the rows.
 2. Clear the Vendor selection and check the rows.
 3. Empty the part search and check the rows.</t>
         </is>
       </c>
-      <c r="G34" s="2" t="inlineStr">
+      <c r="G33" s="2" t="inlineStr">
         <is>
           <t>1. With no category selected, parts of all categories are shown.
 2. With no vendor selected, parts of all vendors are shown.
@@ -2163,42 +2125,42 @@
 This is the expected behaviour as per the build tested on 8/4/2026, and as per the Inventory Value report specification version 3 (S6-R7).</t>
         </is>
       </c>
-      <c r="H34" s="2" t="inlineStr">
+      <c r="H33" s="2" t="inlineStr">
         <is>
           <t>SV-8673 (IV spec v3 2026-07-29 Story 6 S6-R7)</t>
         </is>
       </c>
-      <c r="I34" s="2" t="inlineStr"/>
-      <c r="J34" s="2" t="inlineStr"/>
-    </row>
-    <row r="35">
-      <c r="A35" s="2" t="inlineStr">
+      <c r="I33" s="2" t="inlineStr"/>
+      <c r="J33" s="2" t="inlineStr"/>
+    </row>
+    <row r="34">
+      <c r="A34" s="2" t="inlineStr">
         <is>
           <t>Part search matches part number or description on the server; case-insensitive</t>
         </is>
       </c>
-      <c r="B35" s="2" t="inlineStr">
+      <c r="B34" s="2" t="inlineStr">
         <is>
           <t>IV — Filters &amp; Part Search</t>
         </is>
       </c>
-      <c r="C35" s="2" t="inlineStr">
-        <is>
-          <t>Functional</t>
-        </is>
-      </c>
-      <c r="D35" s="2" t="inlineStr">
+      <c r="C34" s="2" t="inlineStr">
+        <is>
+          <t>Functional</t>
+        </is>
+      </c>
+      <c r="D34" s="2" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="E35" s="2" t="inlineStr">
+      <c r="E34" s="2" t="inlineStr">
         <is>
           <t>1. You are signed in to the ShopView App on a desktop browser.
 2. In-stock parts exist whose part numbers and descriptions you know (including a description containing a distinctive word).</t>
         </is>
       </c>
-      <c r="F35" s="2" t="inlineStr">
+      <c r="F34" s="2" t="inlineStr">
         <is>
           <t>1. Find the part search input in the report's own toolbar (not the application's global search bar).
 2. Type part of a part number and read the results.
@@ -2206,7 +2168,7 @@
 4. Type text matching nothing.</t>
         </is>
       </c>
-      <c r="G35" s="2" t="inlineStr">
+      <c r="G34" s="2" t="inlineStr">
         <is>
           <t>1. The search field is page-local, in the report's own toolbar — it is not the application's global search bar (the same toolbar-search pattern used elsewhere in the reports suite).
 2. The report narrows to parts whose part number OR description contains the entered text.
@@ -2216,49 +2178,49 @@
 This is the expected behaviour as per the build tested on 8/4/2026, and as per the Inventory Value report specification version 3 (S6-R8, S6-R5).</t>
         </is>
       </c>
-      <c r="H35" s="2" t="inlineStr">
+      <c r="H34" s="2" t="inlineStr">
         <is>
           <t>SV-8673 (IV spec v3 2026-07-29 Story 6 S6-R8; S6-R5)</t>
         </is>
       </c>
-      <c r="I35" s="2" t="inlineStr"/>
-      <c r="J35" s="2" t="inlineStr"/>
-    </row>
-    <row r="36">
-      <c r="A36" s="2" t="inlineStr">
+      <c r="I34" s="2" t="inlineStr"/>
+      <c r="J34" s="2" t="inlineStr"/>
+    </row>
+    <row r="35">
+      <c r="A35" s="2" t="inlineStr">
         <is>
           <t>Date range, Location, Category, Vendor, and the part search combine with AND</t>
         </is>
       </c>
-      <c r="B36" s="2" t="inlineStr">
+      <c r="B35" s="2" t="inlineStr">
         <is>
           <t>IV — Filters &amp; Part Search</t>
         </is>
       </c>
-      <c r="C36" s="2" t="inlineStr">
-        <is>
-          <t>Functional</t>
-        </is>
-      </c>
-      <c r="D36" s="2" t="inlineStr">
+      <c r="C35" s="2" t="inlineStr">
+        <is>
+          <t>Functional</t>
+        </is>
+      </c>
+      <c r="D35" s="2" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="E36" s="2" t="inlineStr">
+      <c r="E35" s="2" t="inlineStr">
         <is>
           <t>1. You are signed in to the ShopView App on a desktop browser.
 2. In-stock parts exist with a known mix of categories and vendors, so a combined filter isolates a known subset.</t>
         </is>
       </c>
-      <c r="F36" s="2" t="inlineStr">
+      <c r="F35" s="2" t="inlineStr">
         <is>
           <t>1. Select a Category, then also a Vendor that only some of those category parts have.
 2. Add a part search matching only one of the remaining parts.
 3. Check the rows and the totals row after each step.</t>
         </is>
       </c>
-      <c r="G36" s="2" t="inlineStr">
+      <c r="G35" s="2" t="inlineStr">
         <is>
           <t>1. A part must satisfy EVERY active filter and the search to appear — the Date range, Location, Category, Vendor, and part search combine with AND.
 2. The totals row matches the combined filtered set after each step.
@@ -2266,42 +2228,42 @@
 This is the expected behaviour as per the build tested on 8/4/2026, and as per the Inventory Value report specification version 3 (S6-R9).</t>
         </is>
       </c>
-      <c r="H36" s="2" t="inlineStr">
+      <c r="H35" s="2" t="inlineStr">
         <is>
           <t>SV-8673 (IV spec v3 2026-07-29 Story 6 S6-R9)</t>
         </is>
       </c>
-      <c r="I36" s="2" t="inlineStr"/>
-      <c r="J36" s="2" t="inlineStr"/>
-    </row>
-    <row r="37">
-      <c r="A37" s="2" t="inlineStr">
+      <c r="I35" s="2" t="inlineStr"/>
+      <c r="J35" s="2" t="inlineStr"/>
+    </row>
+    <row r="36">
+      <c r="A36" s="2" t="inlineStr">
         <is>
           <t>The Location filter is a rightmost multi-select with an All locations toggle</t>
         </is>
       </c>
-      <c r="B37" s="2" t="inlineStr">
+      <c r="B36" s="2" t="inlineStr">
         <is>
           <t>IV — Location Filter</t>
         </is>
       </c>
-      <c r="C37" s="2" t="inlineStr">
-        <is>
-          <t>Functional</t>
-        </is>
-      </c>
-      <c r="D37" s="2" t="inlineStr">
+      <c r="C36" s="2" t="inlineStr">
+        <is>
+          <t>Functional</t>
+        </is>
+      </c>
+      <c r="D36" s="2" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="E37" s="2" t="inlineStr">
+      <c r="E36" s="2" t="inlineStr">
         <is>
           <t>1. You are signed in to the ShopView App on a desktop browser as a user with access to at least two locations.
 2. This browser has never saved settings for this report (fresh visit).</t>
         </is>
       </c>
-      <c r="F37" s="2" t="inlineStr">
+      <c r="F36" s="2" t="inlineStr">
         <is>
           <t>1. Open the Inventory Value report and find the filter labeled "Location".
 2. Read its position in the toolbar and its default selection.
@@ -2309,7 +2271,7 @@
 4. Select every accessible location ("All locations") and look at how the rows tell you which location they belong to.</t>
         </is>
       </c>
-      <c r="G37" s="2" t="inlineStr">
+      <c r="G36" s="2" t="inlineStr">
         <is>
           <t>1. The toolbar has a location filter labeled "Location" — a multi-select and the rightmost filter — listing the locations the signed-in user has access to, with an "All locations" / "Clear all" toggle.
 2. On a first visit it defaults to the user's currently active location.
@@ -2318,49 +2280,49 @@
 This is the expected behaviour as per the build tested on 8/4/2026, and as per the Inventory Value report specification version 3 (S7-R1, S7-R2, S12-R3); where the wording of that specification differs, the behaviour above follows a later product decision, which is the authority.</t>
         </is>
       </c>
-      <c r="H37" s="2" t="inlineStr">
+      <c r="H36" s="2" t="inlineStr">
         <is>
           <t>SV-8674 (IV spec v3 2026-07-29 Story 7 S7-R1; S7-R2; Story 12 S12-R3 — per-row location identifier in All-locations view ADDED per kickoff video P10 40:58-41:20; user ruling 2026-07-28: video overrides spec (video newer; last-update-wins))</t>
         </is>
       </c>
-      <c r="I37" s="2" t="inlineStr"/>
-      <c r="J37" s="2" t="inlineStr"/>
-    </row>
-    <row r="38">
-      <c r="A38" s="2" t="inlineStr">
+      <c r="I36" s="2" t="inlineStr"/>
+      <c r="J36" s="2" t="inlineStr"/>
+    </row>
+    <row r="37">
+      <c r="A37" s="2" t="inlineStr">
         <is>
           <t>Selecting one, several, or all locations reloads the report scoped to that set</t>
         </is>
       </c>
-      <c r="B38" s="2" t="inlineStr">
+      <c r="B37" s="2" t="inlineStr">
         <is>
           <t>IV — Location Filter</t>
         </is>
       </c>
-      <c r="C38" s="2" t="inlineStr">
-        <is>
-          <t>Functional</t>
-        </is>
-      </c>
-      <c r="D38" s="2" t="inlineStr">
+      <c r="C37" s="2" t="inlineStr">
+        <is>
+          <t>Functional</t>
+        </is>
+      </c>
+      <c r="D37" s="2" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="E38" s="2" t="inlineStr">
+      <c r="E37" s="2" t="inlineStr">
         <is>
           <t>1. You are signed in to the ShopView App on a desktop browser as a user with access to at least two locations.
 2. In-stock parts exist at both locations.</t>
         </is>
       </c>
-      <c r="F38" s="2" t="inlineStr">
+      <c r="F37" s="2" t="inlineStr">
         <is>
           <t>1. With one location selected, note the rows and totals.
 2. Add the second location and watch the data area.
 3. Use "All locations", then narrow back to one.</t>
         </is>
       </c>
-      <c r="G38" s="2" t="inlineStr">
+      <c r="G37" s="2" t="inlineStr">
         <is>
           <t>1. Each selection change reloads the report scoped to the selected set.
 2. With both locations selected, parts from both appear (one row per part per location) and the totals cover both.
@@ -2369,9 +2331,58 @@
 This is the expected behaviour as per the build tested on 8/4/2026, and as per the Inventory Value report specification version 3 (S7-R3).</t>
         </is>
       </c>
+      <c r="H37" s="2" t="inlineStr">
+        <is>
+          <t>SV-8674 (IV spec v3 2026-07-29 Story 7 S7-R3 + on-screen location-scope indicator per Chris Ward group message 2026-07-29 (chris-update-2026-07-29/chris-message-2026-07-29.md; NEWEST source; last-update-wins))</t>
+        </is>
+      </c>
+      <c r="I37" s="2" t="inlineStr"/>
+      <c r="J37" s="2" t="inlineStr"/>
+    </row>
+    <row r="38">
+      <c r="A38" s="2" t="inlineStr">
+        <is>
+          <t>Scoping never includes an inaccessible location</t>
+        </is>
+      </c>
+      <c r="B38" s="2" t="inlineStr">
+        <is>
+          <t>IV — Location Filter</t>
+        </is>
+      </c>
+      <c r="C38" s="2" t="inlineStr">
+        <is>
+          <t>Negative</t>
+        </is>
+      </c>
+      <c r="D38" s="2" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="E38" s="2" t="inlineStr">
+        <is>
+          <t>1. You are signed in to the ShopView App on a desktop browser as a user who can access some, but not all, of the organization's locations.
+2. The Inventory Value report is open.</t>
+        </is>
+      </c>
+      <c r="F38" s="2" t="inlineStr">
+        <is>
+          <t>1. Open the Location filter and read the locations offered.
+2. Use "Clear all" so the selection resolves to no location, and watch what the report loads.</t>
+        </is>
+      </c>
+      <c r="G38" s="2" t="inlineStr">
+        <is>
+          <t>1. Only the locations the user has access to are offered — a location the user cannot access is never included in the scope.
+2. If the requested location set resolves to none the user can access, the report falls back to the user's currently active location.
+---
+This is the expected behaviour as per the build tested on 8/4/2026, and as per the Inventory Value report specification version 3 (S7-R4, S7-R5).</t>
+        </is>
+      </c>
       <c r="H38" s="2" t="inlineStr">
         <is>
-          <t>SV-8674 (IV spec v3 2026-07-29 Story 7 S7-R3 + on-screen location-scope indicator per Chris Ward group message 2026-07-29 (chris-update-2026-07-29/chris-message-2026-07-29.md; NEWEST source; last-update-wins))</t>
+          <t>SV-8674 (IV spec v3 2026-07-29 Story 7 S7-R4; S7-R5)</t>
         </is>
       </c>
       <c r="I38" s="2" t="inlineStr"/>
@@ -2380,7 +2391,7 @@
     <row r="39">
       <c r="A39" s="2" t="inlineStr">
         <is>
-          <t>Scoping never includes an inaccessible location</t>
+          <t>Inventory Value: the Location filter is hidden for a one-location user</t>
         </is>
       </c>
       <c r="B39" s="2" t="inlineStr">
@@ -2390,37 +2401,39 @@
       </c>
       <c r="C39" s="2" t="inlineStr">
         <is>
-          <t>Negative</t>
+          <t>Functional</t>
         </is>
       </c>
       <c r="D39" s="2" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="E39" s="2" t="inlineStr">
         <is>
-          <t>1. You are signed in to the ShopView App on a desktop browser as a user who can access some, but not all, of the organization's locations.
-2. The Inventory Value report is open.</t>
+          <t>1. A test user exists with access to exactly one location (create a fresh ZZAUTOTEST staff member if needed; clean up afterward).
+2. You are signed in as that user on a desktop browser.</t>
         </is>
       </c>
       <c r="F39" s="2" t="inlineStr">
         <is>
-          <t>1. Open the Location filter and read the locations offered.
-2. Use "Clear all" so the selection resolves to no location, and watch what the report loads.</t>
+          <t>1. Open the Inventory Value report and look for the Location filter in the toolbar.
+2. Then sign in as a user with access to two or more locations and look again.</t>
         </is>
       </c>
       <c r="G39" s="2" t="inlineStr">
         <is>
-          <t>1. Only the locations the user has access to are offered — a location the user cannot access is never included in the scope.
-2. If the requested location set resolves to none the user can access, the report falls back to the user's currently active location.
----
-This is the expected behaviour as per the build tested on 8/4/2026, and as per the Inventory Value report specification version 3 (S7-R4, S7-R5).</t>
+          <t>1. For the single-location user the Location filter is NOT shown at all — the report simply shows that one location's stock.
+2. For the user with access to two or more locations the Location filter IS shown.
+---
+DO NOT AUTOMATE YET: this behaviour is waiting on an answer from the product owner. Automating it now could lock in the wrong behaviour.
+The open question is in: Report-Suite_Questions-and-Decisions-for-Chris-Ward_2026-08-04.xlsx — https://raw.githubusercontent.com/bilalmuzamil-sketch/Manual-test-Cases/claude/slack-session-0sxnd9/build/report-suite/chris-consolidated-2026-08-04/Report-Suite_Questions-and-Decisions-for-Chris-Ward_2026-08-04.xlsx
+This is the expected behaviour as per the build tested on 8/4/2026, and as per the Inventory Value report specification version 3 (S7-N1); where the wording of that specification differs, the behaviour above follows a later product decision, which is the authority.</t>
         </is>
       </c>
       <c r="H39" s="2" t="inlineStr">
         <is>
-          <t>SV-8674 (IV spec v3 2026-07-29 Story 7 S7-R4; S7-R5)</t>
+          <t>SV-8674 (IV spec Story 7 S7-N1 — RULED HIDDEN by Chris Ward answer 2026-07-31 Q1=A "classic spec drift"; the S7-N1 "still sees the filter" note is stale; spec edit pending)</t>
         </is>
       </c>
       <c r="I39" s="2" t="inlineStr"/>
@@ -2429,7 +2442,7 @@
     <row r="40">
       <c r="A40" s="2" t="inlineStr">
         <is>
-          <t>Inventory Value: the Location filter is hidden for a one-location user</t>
+          <t>The Location column sits after Vendor and never reads Multiple</t>
         </is>
       </c>
       <c r="B40" s="2" t="inlineStr">
@@ -2444,66 +2457,17 @@
       </c>
       <c r="D40" s="2" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High</t>
         </is>
       </c>
       <c r="E40" s="2" t="inlineStr">
-        <is>
-          <t>1. A test user exists with access to exactly one location (create a fresh ZZAUTOTEST staff member if needed; clean up afterward).
-2. You are signed in as that user on a desktop browser.</t>
-        </is>
-      </c>
-      <c r="F40" s="2" t="inlineStr">
-        <is>
-          <t>1. Open the Inventory Value report and look for the Location filter in the toolbar.
-2. Then sign in as a user with access to two or more locations and look again.</t>
-        </is>
-      </c>
-      <c r="G40" s="2" t="inlineStr">
-        <is>
-          <t>1. For the single-location user the Location filter is NOT shown at all — the report simply shows that one location's stock.
-2. For the user with access to two or more locations the Location filter IS shown.
----
-This is the expected behaviour as per the build tested on 8/4/2026, and as per the Inventory Value report specification version 3 (S7-N1); where the wording of that specification differs, the behaviour above follows a later product decision, which is the authority.</t>
-        </is>
-      </c>
-      <c r="H40" s="2" t="inlineStr">
-        <is>
-          <t>SV-8674 (IV spec Story 7 S7-N1 — RULED HIDDEN by Chris Ward answer 2026-07-31 Q1=A "classic spec drift"; the S7-N1 "still sees the filter" note is stale; spec edit pending)</t>
-        </is>
-      </c>
-      <c r="I40" s="2" t="inlineStr"/>
-      <c r="J40" s="2" t="inlineStr"/>
-    </row>
-    <row r="41">
-      <c r="A41" s="2" t="inlineStr">
-        <is>
-          <t>The Location column sits after Vendor and never reads Multiple</t>
-        </is>
-      </c>
-      <c r="B41" s="2" t="inlineStr">
-        <is>
-          <t>IV — Location Filter</t>
-        </is>
-      </c>
-      <c r="C41" s="2" t="inlineStr">
-        <is>
-          <t>Functional</t>
-        </is>
-      </c>
-      <c r="D41" s="2" t="inlineStr">
-        <is>
-          <t>High</t>
-        </is>
-      </c>
-      <c r="E41" s="2" t="inlineStr">
         <is>
           <t>1. You are signed in on a desktop browser as a user with access to at least two locations.
 2. The same part is in stock at two of those locations.
 3. The Inventory Value report is open with rows loaded.</t>
         </is>
       </c>
-      <c r="F41" s="2" t="inlineStr">
+      <c r="F40" s="2" t="inlineStr">
         <is>
           <t>1. Turn Location on in the column-selection control, select two or more locations, and read the column headers from the left.
 2. Read the Location cell on each of the two rows for the part stocked at both locations.
@@ -2514,7 +2478,7 @@
 7. With more than one location still selected, download the CSV and the PDF and read their columns.</t>
         </is>
       </c>
-      <c r="G41" s="2" t="inlineStr">
+      <c r="G40" s="2" t="inlineStr">
         <is>
           <t>1. With Location turned on in the column-selection control, a Location column is shown, inserted between Vendor and Qty.
 2. Each row names the location that row's stock is held at.
@@ -2524,52 +2488,54 @@
 6. The Location filter control keeps the same width whichever label it shows — one location, several, or "All locations" — so the toolbar does not shift as you change the selection.
 7. Both downloads include the Location column in the same position it holds on screen (between Vendor and Qty), naming each row's own location.
 ---
+DO NOT AUTOMATE YET: this behaviour is waiting on an answer from the product owner. Automating it now could lock in the wrong behaviour.
+The open question is in: Report-Suite_Questions-and-Decisions-for-Chris-Ward_2026-08-04.xlsx — https://raw.githubusercontent.com/bilalmuzamil-sketch/Manual-test-Cases/claude/slack-session-0sxnd9/build/report-suite/chris-consolidated-2026-08-04/Report-Suite_Questions-and-Decisions-for-Chris-Ward_2026-08-04.xlsx
 This is the expected behaviour as per the build tested on 8/4/2026, and as per the Inventory Value report specification version 3 (S7-R6, S7-R7, S3-R1, S12-R10, S10-R15); on this point that specification currently states otherwise and a product decision is still awaited, so treat the behaviour described above as what the build does today.</t>
         </is>
       </c>
-      <c r="H41" s="2" t="inlineStr">
+      <c r="H40" s="2" t="inlineStr">
         <is>
           <t>SV-8674; SV-8677 (IV spec v3 2026-07-29 S7-R6; S7-R7; S3-R1; S12-R10; S10-R15 — Location column inserted between Vendor and Qty on Hand; automatic visibility; never "Multiple"; S10-R15 = the same column in every export)</t>
         </is>
       </c>
-      <c r="I41" s="2" t="inlineStr"/>
-      <c r="J41" s="2" t="inlineStr"/>
-    </row>
-    <row r="42">
-      <c r="A42" s="2" t="inlineStr">
+      <c r="I40" s="2" t="inlineStr"/>
+      <c r="J40" s="2" t="inlineStr"/>
+    </row>
+    <row r="41">
+      <c r="A41" s="2" t="inlineStr">
         <is>
           <t>Column Selection toggles columns; Total Cost cannot be turned off</t>
         </is>
       </c>
-      <c r="B42" s="2" t="inlineStr">
+      <c r="B41" s="2" t="inlineStr">
         <is>
           <t>IV — Column Selection &amp; Persistence</t>
         </is>
       </c>
-      <c r="C42" s="2" t="inlineStr">
-        <is>
-          <t>Functional</t>
-        </is>
-      </c>
-      <c r="D42" s="2" t="inlineStr">
+      <c r="C41" s="2" t="inlineStr">
+        <is>
+          <t>Functional</t>
+        </is>
+      </c>
+      <c r="D41" s="2" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="E42" s="2" t="inlineStr">
+      <c r="E41" s="2" t="inlineStr">
         <is>
           <t>1. You are signed in to the ShopView App on a desktop browser.
 2. The Inventory Value report is open with rows loaded.</t>
         </is>
       </c>
-      <c r="F42" s="2" t="inlineStr">
+      <c r="F41" s="2" t="inlineStr">
         <is>
           <t>1. Hover the column-selection icon button in the toolbar and read its tooltip.
 2. Open the control and toggle a column off, then on again, watching the table.
 3. Look for a way to turn the Total Cost column off.</t>
         </is>
       </c>
-      <c r="G42" s="2" t="inlineStr">
+      <c r="G41" s="2" t="inlineStr">
         <is>
           <t>1. The icon button's tooltip reads "Column Selection".
 2. Toggling a column off hides it from the table; toggling it on shows it again.
@@ -2578,9 +2544,60 @@
 This is the expected behaviour as per the build tested on 8/4/2026, and as per the Inventory Value report specification version 3 (S8-R1, S8-R2).</t>
         </is>
       </c>
+      <c r="H41" s="2" t="inlineStr">
+        <is>
+          <t>SV-8675 (IV spec v3 2026-07-29 Story 8 S8-R1; S8-R2)</t>
+        </is>
+      </c>
+      <c r="I41" s="2" t="inlineStr"/>
+      <c r="J41" s="2" t="inlineStr"/>
+    </row>
+    <row r="42">
+      <c r="A42" s="2" t="inlineStr">
+        <is>
+          <t>Toggling columns never reorders them</t>
+        </is>
+      </c>
+      <c r="B42" s="2" t="inlineStr">
+        <is>
+          <t>IV — Column Selection &amp; Persistence</t>
+        </is>
+      </c>
+      <c r="C42" s="2" t="inlineStr">
+        <is>
+          <t>Functional</t>
+        </is>
+      </c>
+      <c r="D42" s="2" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="E42" s="2" t="inlineStr">
+        <is>
+          <t>1. You are signed in to the ShopView App on a desktop browser.
+2. The Inventory Value report is open with rows loaded.</t>
+        </is>
+      </c>
+      <c r="F42" s="2" t="inlineStr">
+        <is>
+          <t>1. Turn several columns on and off in different orders (for example, turn on Total Sell, then Margin).
+2. Read the resulting column order after each change.</t>
+        </is>
+      </c>
+      <c r="G42" s="2" t="inlineStr">
+        <is>
+          <t>1. Whatever columns are shown, they appear in the fixed left-to-right order - with Location, when it is turned on in the column-selection control, between Vendor and Qty (Part #, Description, Category, Vendor, Qty, Unit Cost, Unit Sell, Margin, Margin %, Total Sell, Total Cost) - toggling visibility never reorders columns.
+2. Total Cost is always the last column.
+---
+DO NOT AUTOMATE YET: this behaviour is waiting on an answer from the product owner. Automating it now could lock in the wrong behaviour.
+The open question is in: Report-Suite_Questions-and-Decisions-for-Chris-Ward_2026-08-04.xlsx — https://raw.githubusercontent.com/bilalmuzamil-sketch/Manual-test-Cases/claude/slack-session-0sxnd9/build/report-suite/chris-consolidated-2026-08-04/Report-Suite_Questions-and-Decisions-for-Chris-Ward_2026-08-04.xlsx
+This is the expected behaviour as per the build tested on 8/4/2026, and as per the Inventory Value report specification version 3 (S8-R4, S3-R1, S7-R6); on this point that specification currently states otherwise and a product decision is still awaited, so treat the behaviour described above as what the build does today.</t>
+        </is>
+      </c>
       <c r="H42" s="2" t="inlineStr">
         <is>
-          <t>SV-8675 (IV spec v3 2026-07-29 Story 8 S8-R1; S8-R2)</t>
+          <t>SV-8675; SV-8674 (IV spec v3 2026-07-29 Story 8 S8-R4; Story 3 S3-R1 + Story 7 S7-R6 — toggling never reorders; plus the automatic Location column between Vendor and Qty on Hand)</t>
         </is>
       </c>
       <c r="I42" s="2" t="inlineStr"/>
@@ -2589,7 +2606,7 @@
     <row r="43">
       <c r="A43" s="2" t="inlineStr">
         <is>
-          <t>Toggling columns never reorders them</t>
+          <t>The report remembers all filters; columns and sort per browser</t>
         </is>
       </c>
       <c r="B43" s="2" t="inlineStr">
@@ -2604,65 +2621,16 @@
       </c>
       <c r="D43" s="2" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High</t>
         </is>
       </c>
       <c r="E43" s="2" t="inlineStr">
         <is>
           <t>1. You are signed in to the ShopView App on a desktop browser.
-2. The Inventory Value report is open with rows loaded.</t>
+2. The Inventory Value report is open.</t>
         </is>
       </c>
       <c r="F43" s="2" t="inlineStr">
-        <is>
-          <t>1. Turn several columns on and off in different orders (for example, turn on Total Sell, then Margin).
-2. Read the resulting column order after each change.</t>
-        </is>
-      </c>
-      <c r="G43" s="2" t="inlineStr">
-        <is>
-          <t>1. Whatever columns are shown, they appear in the fixed left-to-right order - with Location, when it is turned on in the column-selection control, between Vendor and Qty (Part #, Description, Category, Vendor, Qty, Unit Cost, Unit Sell, Margin, Margin %, Total Sell, Total Cost) - toggling visibility never reorders columns.
-2. Total Cost is always the last column.
----
-This is the expected behaviour as per the build tested on 8/4/2026, and as per the Inventory Value report specification version 3 (S8-R4, S3-R1, S7-R6); on this point that specification currently states otherwise and a product decision is still awaited, so treat the behaviour described above as what the build does today.</t>
-        </is>
-      </c>
-      <c r="H43" s="2" t="inlineStr">
-        <is>
-          <t>SV-8675; SV-8674 (IV spec v3 2026-07-29 Story 8 S8-R4; Story 3 S3-R1 + Story 7 S7-R6 — toggling never reorders; plus the automatic Location column between Vendor and Qty on Hand)</t>
-        </is>
-      </c>
-      <c r="I43" s="2" t="inlineStr"/>
-      <c r="J43" s="2" t="inlineStr"/>
-    </row>
-    <row r="44">
-      <c r="A44" s="2" t="inlineStr">
-        <is>
-          <t>The report remembers all filters; columns and sort per browser</t>
-        </is>
-      </c>
-      <c r="B44" s="2" t="inlineStr">
-        <is>
-          <t>IV — Column Selection &amp; Persistence</t>
-        </is>
-      </c>
-      <c r="C44" s="2" t="inlineStr">
-        <is>
-          <t>Functional</t>
-        </is>
-      </c>
-      <c r="D44" s="2" t="inlineStr">
-        <is>
-          <t>High</t>
-        </is>
-      </c>
-      <c r="E44" s="2" t="inlineStr">
-        <is>
-          <t>1. You are signed in to the ShopView App on a desktop browser.
-2. The Inventory Value report is open.</t>
-        </is>
-      </c>
-      <c r="F44" s="2" t="inlineStr">
         <is>
           <t>1. Change the date range, select a category and a vendor, type a part search, change the location selection, change the column selection, and sort by a non-default column.
 2. Navigate away to another screen, then return to the report.
@@ -2670,7 +2638,7 @@
 4. If practical, open the report in a different browser (or private window) and read its settings.</t>
         </is>
       </c>
-      <c r="G44" s="2" t="inlineStr">
+      <c r="G43" s="2" t="inlineStr">
         <is>
           <t>1. On return and after a reload, the report restores the saved date range, category selection, vendor selection, part search text, location selection, column selection, and sort.
 2. In a different browser the report shows the defaults instead — persistence is per browser, not tied to the user's account.
@@ -2678,9 +2646,58 @@
 This is the expected behaviour as per the build tested on 8/4/2026, and as per the Inventory Value report specification version 3 (S8-R5, S9-R5).</t>
         </is>
       </c>
+      <c r="H43" s="2" t="inlineStr">
+        <is>
+          <t>SV-8675 (IV spec v3 2026-07-29 Story 8 S8-R5 (+ context note); Story 9 S9-R5)</t>
+        </is>
+      </c>
+      <c r="I43" s="2" t="inlineStr"/>
+      <c r="J43" s="2" t="inlineStr"/>
+    </row>
+    <row r="44">
+      <c r="A44" s="2" t="inlineStr">
+        <is>
+          <t>Defensive restore: a stale saved category or vendor is dropped on load</t>
+        </is>
+      </c>
+      <c r="B44" s="2" t="inlineStr">
+        <is>
+          <t>IV — Column Selection &amp; Persistence</t>
+        </is>
+      </c>
+      <c r="C44" s="2" t="inlineStr">
+        <is>
+          <t>Negative</t>
+        </is>
+      </c>
+      <c r="D44" s="2" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="E44" s="2" t="inlineStr">
+        <is>
+          <t>1. You are signed in to the ShopView App on a desktop browser.
+2. The report has saved settings in this browser, including a category or vendor selection that can be made stale (for example, the last in-stock part of a saved category is consumed so the category disappears from the data).</t>
+        </is>
+      </c>
+      <c r="F44" s="2" t="inlineStr">
+        <is>
+          <t>1. Make the saved category or vendor no longer present in the data.
+2. Open the Inventory Value report.</t>
+        </is>
+      </c>
+      <c r="G44" s="2" t="inlineStr">
+        <is>
+          <t>1. The report loads normally — the saved category or vendor that is no longer present in the data is dropped from the selection instead of breaking the view (the defensive-restore rule applied to the path these steps drive).
+2. All other saved settings are still restored.
+---
+This is the expected behaviour as per the build tested on 8/4/2026, and as per the Inventory Value report specification version 3 (S8-R6).</t>
+        </is>
+      </c>
       <c r="H44" s="2" t="inlineStr">
         <is>
-          <t>SV-8675 (IV spec v3 2026-07-29 Story 8 S8-R5 (+ context note); Story 9 S9-R5)</t>
+          <t>SV-8675 (IV spec v3 2026-07-29 Story 8 S8-R6)</t>
         </is>
       </c>
       <c r="I44" s="2" t="inlineStr"/>
@@ -2689,47 +2706,47 @@
     <row r="45">
       <c r="A45" s="2" t="inlineStr">
         <is>
-          <t>Defensive restore: a stale saved category or vendor is dropped on load</t>
+          <t>Rows are sorted by Total Cost highest first on load and after any reload</t>
         </is>
       </c>
       <c r="B45" s="2" t="inlineStr">
         <is>
-          <t>IV — Column Selection &amp; Persistence</t>
+          <t>IV — Sorting</t>
         </is>
       </c>
       <c r="C45" s="2" t="inlineStr">
         <is>
-          <t>Negative</t>
+          <t>Functional</t>
         </is>
       </c>
       <c r="D45" s="2" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High</t>
         </is>
       </c>
       <c r="E45" s="2" t="inlineStr">
         <is>
-          <t>1. You are signed in to the ShopView App on a desktop browser.
-2. The report has saved settings in this browser, including a category or vendor selection that can be made stale (for example, the last in-stock part of a saved category is consumed so the category disappears from the data).</t>
+          <t>1. You are signed in to the ShopView App on a desktop browser that has no saved sort for this report (fresh visit).
+2. In-stock parts with a spread of Total Cost values exist, spanning more than one page.</t>
         </is>
       </c>
       <c r="F45" s="2" t="inlineStr">
         <is>
-          <t>1. Make the saved category or vendor no longer present in the data.
-2. Open the Inventory Value report.</t>
+          <t>1. Open the Inventory Value report without clicking any header.
+2. Read the Total Cost values from the top row down, across page 1 and page 2.</t>
         </is>
       </c>
       <c r="G45" s="2" t="inlineStr">
         <is>
-          <t>1. The report loads normally — the saved category or vendor that is no longer present in the data is dropped from the selection instead of breaking the view (the defensive-restore rule applied to the path these steps drive).
-2. All other saved settings are still restored.
----
-This is the expected behaviour as per the build tested on 8/4/2026, and as per the Inventory Value report specification version 3 (S8-R6).</t>
+          <t>1. The rows are sorted by Total Cost, highest first (descending).
+2. The order holds across pages (page 2 continues below page 1's lowest value) — the server applies the default order over the full set.
+---
+This is the expected behaviour as per the build tested on 8/4/2026, and as per the Inventory Value report specification version 3 (S9-R1).</t>
         </is>
       </c>
       <c r="H45" s="2" t="inlineStr">
         <is>
-          <t>SV-8675 (IV spec v3 2026-07-29 Story 8 S8-R6)</t>
+          <t>SV-8676 (IV spec v3 2026-07-29 Story 9 S9-R1; §3 Key Decisions (Total Cost default sort))</t>
         </is>
       </c>
       <c r="I45" s="2" t="inlineStr"/>
@@ -2738,7 +2755,7 @@
     <row r="46">
       <c r="A46" s="2" t="inlineStr">
         <is>
-          <t>Rows are sorted by Total Cost highest first on load and after any reload</t>
+          <t>Header clicks sort ascending then descending; no third state; page 1 returns</t>
         </is>
       </c>
       <c r="B46" s="2" t="inlineStr">
@@ -2758,60 +2775,11 @@
       </c>
       <c r="E46" s="2" t="inlineStr">
         <is>
-          <t>1. You are signed in to the ShopView App on a desktop browser that has no saved sort for this report (fresh visit).
-2. In-stock parts with a spread of Total Cost values exist, spanning more than one page.</t>
+          <t>1. You are signed in to the ShopView App on a desktop browser.
+2. The result set spans more than one page.</t>
         </is>
       </c>
       <c r="F46" s="2" t="inlineStr">
-        <is>
-          <t>1. Open the Inventory Value report without clicking any header.
-2. Read the Total Cost values from the top row down, across page 1 and page 2.</t>
-        </is>
-      </c>
-      <c r="G46" s="2" t="inlineStr">
-        <is>
-          <t>1. The rows are sorted by Total Cost, highest first (descending).
-2. The order holds across pages (page 2 continues below page 1's lowest value) — the server applies the default order over the full set.
----
-This is the expected behaviour as per the build tested on 8/4/2026, and as per the Inventory Value report specification version 3 (S9-R1).</t>
-        </is>
-      </c>
-      <c r="H46" s="2" t="inlineStr">
-        <is>
-          <t>SV-8676 (IV spec v3 2026-07-29 Story 9 S9-R1; §3 Key Decisions (Total Cost default sort))</t>
-        </is>
-      </c>
-      <c r="I46" s="2" t="inlineStr"/>
-      <c r="J46" s="2" t="inlineStr"/>
-    </row>
-    <row r="47">
-      <c r="A47" s="2" t="inlineStr">
-        <is>
-          <t>Header clicks sort ascending then descending; no third state; page 1 returns</t>
-        </is>
-      </c>
-      <c r="B47" s="2" t="inlineStr">
-        <is>
-          <t>IV — Sorting</t>
-        </is>
-      </c>
-      <c r="C47" s="2" t="inlineStr">
-        <is>
-          <t>Functional</t>
-        </is>
-      </c>
-      <c r="D47" s="2" t="inlineStr">
-        <is>
-          <t>High</t>
-        </is>
-      </c>
-      <c r="E47" s="2" t="inlineStr">
-        <is>
-          <t>1. You are signed in to the ShopView App on a desktop browser.
-2. The result set spans more than one page.</t>
-        </is>
-      </c>
-      <c r="F47" s="2" t="inlineStr">
         <is>
           <t>1. From page 2, click the Part # column header and note the order and the page shown.
 2. Click the same header again and note the order.
@@ -2819,7 +2787,7 @@
 4. Click a different column header and check whether the previous sort still applies.</t>
         </is>
       </c>
-      <c r="G47" s="2" t="inlineStr">
+      <c r="G46" s="2" t="inlineStr">
         <is>
           <t>1. Clicking a column that is not the active sort sorts it ascending; clicking the active sort column again toggles it to descending; there is no third "cleared" state.
 2. Each header click re-fetches the data from the server ordered by the chosen column and direction, returning the FIRST page of the re-sorted result set.
@@ -2828,49 +2796,49 @@
 This is the expected behaviour as per the build tested on 8/4/2026, and as per the Inventory Value report specification version 3 (S9-R2).</t>
         </is>
       </c>
-      <c r="H47" s="2" t="inlineStr">
+      <c r="H46" s="2" t="inlineStr">
         <is>
           <t>SV-8676 (IV spec v3 2026-07-29 Story 9 S9-R2)</t>
         </is>
       </c>
-      <c r="I47" s="2" t="inlineStr"/>
-      <c r="J47" s="2" t="inlineStr"/>
-    </row>
-    <row r="48">
-      <c r="A48" s="2" t="inlineStr">
+      <c r="I46" s="2" t="inlineStr"/>
+      <c r="J46" s="2" t="inlineStr"/>
+    </row>
+    <row r="47">
+      <c r="A47" s="2" t="inlineStr">
         <is>
           <t>Money and numeric columns sort by value; text columns sort as text</t>
         </is>
       </c>
-      <c r="B48" s="2" t="inlineStr">
+      <c r="B47" s="2" t="inlineStr">
         <is>
           <t>IV — Sorting</t>
         </is>
       </c>
-      <c r="C48" s="2" t="inlineStr">
-        <is>
-          <t>Functional</t>
-        </is>
-      </c>
-      <c r="D48" s="2" t="inlineStr">
+      <c r="C47" s="2" t="inlineStr">
+        <is>
+          <t>Functional</t>
+        </is>
+      </c>
+      <c r="D47" s="2" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="E48" s="2" t="inlineStr">
+      <c r="E47" s="2" t="inlineStr">
         <is>
           <t>1. You are signed in to the ShopView App on a desktop browser.
 2. In-stock parts exist with money values over and under $1,000 and with text values in mixed letter cases.</t>
         </is>
       </c>
-      <c r="F48" s="2" t="inlineStr">
+      <c r="F47" s="2" t="inlineStr">
         <is>
           <t>1. Sort by Total Cost and check the order of values like $900.00 vs $1,100.00.
 2. Sort by Qty and check the numeric order.
 3. Sort by Description (or Vendor) and check how differently-cased values order.</t>
         </is>
       </c>
-      <c r="G48" s="2" t="inlineStr">
+      <c r="G47" s="2" t="inlineStr">
         <is>
           <t>1. Money and numeric columns sort by their underlying value (so $1,100.00 is treated as more than $900.00, not compared as text).
 2. Text columns (Part #, Description, Category, Vendor) sort as text, case-insensitively ("apple" and "Apple" sort together).
@@ -2878,98 +2846,49 @@
 This is the expected behaviour as per the build tested on 8/4/2026, and as per the Inventory Value report specification version 3 (S9-R3).</t>
         </is>
       </c>
-      <c r="H48" s="2" t="inlineStr">
+      <c r="H47" s="2" t="inlineStr">
         <is>
           <t>SV-8676 (IV spec v3 2026-07-29 Story 9 S9-R3)</t>
         </is>
       </c>
-      <c r="I48" s="2" t="inlineStr"/>
-      <c r="J48" s="2" t="inlineStr"/>
-    </row>
-    <row r="49">
-      <c r="A49" s="2" t="inlineStr">
-        <is>
-          <t>Sorting reorders only the data rows — the totals row stays at the bottom</t>
-        </is>
-      </c>
-      <c r="B49" s="2" t="inlineStr">
-        <is>
-          <t>IV — Sorting</t>
-        </is>
-      </c>
-      <c r="C49" s="2" t="inlineStr">
-        <is>
-          <t>Functional</t>
-        </is>
-      </c>
-      <c r="D49" s="2" t="inlineStr">
-        <is>
-          <t>Medium</t>
-        </is>
-      </c>
-      <c r="E49" s="2" t="inlineStr">
-        <is>
-          <t>1. You are signed in to the ShopView App on a desktop browser.
-2. The Inventory Value report is open with rows and a totals row.</t>
-        </is>
-      </c>
-      <c r="F49" s="2" t="inlineStr">
-        <is>
-          <t>1. Sort by any column and watch the totals row's position.
-2. Sort by a non-default column, leave the report, and return.</t>
-        </is>
-      </c>
-      <c r="G49" s="2" t="inlineStr">
-        <is>
-          <t>1. Sorting reorders the data rows only; the totals row stays at the bottom.
-2. On return, the report restores the chosen sort (remembered per browser, Story 8).
----
-This is the expected behaviour as per the build tested on 8/4/2026, and as per the Inventory Value report specification version 3 (S9-R4, S9-R5).</t>
-        </is>
-      </c>
-      <c r="H49" s="2" t="inlineStr">
-        <is>
-          <t>SV-8676 (IV spec v3 2026-07-29 Story 9 S9-R4; S9-R5)</t>
-        </is>
-      </c>
-      <c r="I49" s="2" t="inlineStr"/>
-      <c r="J49" s="2" t="inlineStr"/>
-    </row>
-    <row r="50">
-      <c r="A50" s="2" t="inlineStr">
+      <c r="I47" s="2" t="inlineStr"/>
+      <c r="J47" s="2" t="inlineStr"/>
+    </row>
+    <row r="48">
+      <c r="A48" s="2" t="inlineStr">
         <is>
           <t>Inventory Value: a three-dot menu holds Download (PDF) and Download (CSV)</t>
         </is>
       </c>
-      <c r="B50" s="2" t="inlineStr">
+      <c r="B48" s="2" t="inlineStr">
         <is>
           <t>IV — Exports</t>
         </is>
       </c>
-      <c r="C50" s="2" t="inlineStr">
-        <is>
-          <t>Functional</t>
-        </is>
-      </c>
-      <c r="D50" s="2" t="inlineStr">
+      <c r="C48" s="2" t="inlineStr">
+        <is>
+          <t>Functional</t>
+        </is>
+      </c>
+      <c r="D48" s="2" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="E50" s="2" t="inlineStr">
+      <c r="E48" s="2" t="inlineStr">
         <is>
           <t>1. You are signed in to the ShopView App on a desktop browser.
 2. The Inventory Value report is open with rows loaded.</t>
         </is>
       </c>
-      <c r="F50" s="2" t="inlineStr">
+      <c r="F48" s="2" t="inlineStr">
         <is>
           <t>1. Find and open the three-dot button in the toolbar.
 2. Read the menu options.
 3. Choose "Download (PDF)", then repeat with "Download (CSV)".</t>
         </is>
       </c>
-      <c r="G50" s="2" t="inlineStr">
+      <c r="G48" s="2" t="inlineStr">
         <is>
           <t>1. The menu holds an option labeled "Download (PDF)" and an option labeled "Download (CSV)".
 2. Each option downloads a file of the current view in the chosen format.
@@ -2977,42 +2896,42 @@
 This is the expected behaviour as per the build tested on 8/4/2026, and as per the Inventory Value report specification version 3 (S10-R1, S10-R2).</t>
         </is>
       </c>
-      <c r="H50" s="2" t="inlineStr">
+      <c r="H48" s="2" t="inlineStr">
         <is>
           <t>SV-8677 (IV spec v3 2026-07-29 Story 10 S10-R1; S10-R2)</t>
         </is>
       </c>
-      <c r="I50" s="2" t="inlineStr"/>
-      <c r="J50" s="2" t="inlineStr"/>
-    </row>
-    <row r="51">
-      <c r="A51" s="2" t="inlineStr">
+      <c r="I48" s="2" t="inlineStr"/>
+      <c r="J48" s="2" t="inlineStr"/>
+    </row>
+    <row r="49">
+      <c r="A49" s="2" t="inlineStr">
         <is>
           <t>Downloads keep shown columns and order, honor filters, and include Totals</t>
         </is>
       </c>
-      <c r="B51" s="2" t="inlineStr">
+      <c r="B49" s="2" t="inlineStr">
         <is>
           <t>IV — Exports</t>
         </is>
       </c>
-      <c r="C51" s="2" t="inlineStr">
-        <is>
-          <t>Functional</t>
-        </is>
-      </c>
-      <c r="D51" s="2" t="inlineStr">
+      <c r="C49" s="2" t="inlineStr">
+        <is>
+          <t>Functional</t>
+        </is>
+      </c>
+      <c r="D49" s="2" t="inlineStr">
         <is>
           <t>Critical</t>
         </is>
       </c>
-      <c r="E51" s="2" t="inlineStr">
+      <c r="E49" s="2" t="inlineStr">
         <is>
           <t>1. You are signed in to the ShopView App on a desktop browser.
 2. The report is open with a non-default column selection, a Category or Vendor filter, a part search, and a non-default sort applied.</t>
         </is>
       </c>
-      <c r="F51" s="2" t="inlineStr">
+      <c r="F49" s="2" t="inlineStr">
         <is>
           <t>1. Download the current view as a CSV and open it.
 2. Compare its columns and their order to the screen.
@@ -3021,7 +2940,7 @@
 5. Repeat the checks in the PDF.</t>
         </is>
       </c>
-      <c r="G51" s="2" t="inlineStr">
+      <c r="G49" s="2" t="inlineStr">
         <is>
           <t>1. Both downloads include only the columns currently shown, in the same left-to-right order as the screen, with Total Cost last.
 2. Both downloads honor the current date, category, vendor, location, and part-search filters, and apply the current sort.
@@ -3029,51 +2948,53 @@
 4. Each download (PDF and CSV) carries a "Locations:" line naming the location(s) the report was scoped to (exact position in the file is confirmed in the build).
 5. Note for the tester: the files carry the Location column when Location is turned ON in the column-selection control (it sits between Vendor and Qty). It does not appear just because you have more than one location selected.
 ---
+DO NOT AUTOMATE YET: this behaviour is waiting on an answer from the product owner. Automating it now could lock in the wrong behaviour.
+The open question is in: Report-Suite_Questions-and-Decisions-for-Chris-Ward_2026-08-04.xlsx — https://raw.githubusercontent.com/bilalmuzamil-sketch/Manual-test-Cases/claude/slack-session-0sxnd9/build/report-suite/chris-consolidated-2026-08-04/Report-Suite_Questions-and-Decisions-for-Chris-Ward_2026-08-04.xlsx
 This is the expected behaviour as per the build tested on 8/4/2026, and as per the Inventory Value report specification version 3 (S10-R3, S10-R4, S10-R5, S10-R6, S10-R15); on this point that specification currently states otherwise and a product decision is still awaited, so treat the behaviour described above as what the build does today.</t>
         </is>
       </c>
-      <c r="H51" s="2" t="inlineStr">
+      <c r="H49" s="2" t="inlineStr">
         <is>
           <t>SV-8677 (IV spec v3 2026-07-29 Story 10 S10-R3; S10-R4; S10-R5; S10-R6; S10-R15 — downloads keep the shown columns and order; honour the filters; include the Totals row; S10-R15 = the "Locations:" line and the automatic Location column)</t>
         </is>
       </c>
-      <c r="I51" s="2" t="inlineStr"/>
-      <c r="J51" s="2" t="inlineStr"/>
-    </row>
-    <row r="52">
-      <c r="A52" s="2" t="inlineStr">
+      <c r="I49" s="2" t="inlineStr"/>
+      <c r="J49" s="2" t="inlineStr"/>
+    </row>
+    <row r="50">
+      <c r="A50" s="2" t="inlineStr">
         <is>
           <t>Export number formats: money to 2 decimals; Margin % to 1 with em-dash</t>
         </is>
       </c>
-      <c r="B52" s="2" t="inlineStr">
+      <c r="B50" s="2" t="inlineStr">
         <is>
           <t>IV — Exports</t>
         </is>
       </c>
-      <c r="C52" s="2" t="inlineStr">
-        <is>
-          <t>Functional</t>
-        </is>
-      </c>
-      <c r="D52" s="2" t="inlineStr">
+      <c r="C50" s="2" t="inlineStr">
+        <is>
+          <t>Functional</t>
+        </is>
+      </c>
+      <c r="D50" s="2" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="E52" s="2" t="inlineStr">
+      <c r="E50" s="2" t="inlineStr">
         <is>
           <t>1. You are signed in to the ShopView App on a desktop browser.
 2. The current view includes money values over $1,000 and, if producible, a part whose Margin % is undefined ("—").</t>
         </is>
       </c>
-      <c r="F52" s="2" t="inlineStr">
+      <c r="F50" s="2" t="inlineStr">
         <is>
           <t>1. Download the CSV and open it in a plain-text editor; read the money and Margin % values.
 2. Download the PDF and read the same values.</t>
         </is>
       </c>
-      <c r="G52" s="2" t="inlineStr">
+      <c r="G50" s="2" t="inlineStr">
         <is>
           <t>1. Money uses two decimals and Margin % one decimal in both files; an undefined Margin % shows "—".
 2. In the CSV, money values are written as plain numbers with two decimals and NO thousands separators (so they parse cleanly in a spreadsheet).
@@ -3082,43 +3003,43 @@
 This is the expected behaviour as per the build tested on 8/4/2026, and as per the Inventory Value report specification version 3 (S10-R7).</t>
         </is>
       </c>
-      <c r="H52" s="2" t="inlineStr">
+      <c r="H50" s="2" t="inlineStr">
         <is>
           <t>SV-8677 (IV spec v3 2026-07-29 Story 10 S10-R7 (+ context note))</t>
         </is>
       </c>
-      <c r="I52" s="2" t="inlineStr"/>
-      <c r="J52" s="2" t="inlineStr"/>
-    </row>
-    <row r="53">
-      <c r="A53" s="2" t="inlineStr">
+      <c r="I50" s="2" t="inlineStr"/>
+      <c r="J50" s="2" t="inlineStr"/>
+    </row>
+    <row r="51">
+      <c r="A51" s="2" t="inlineStr">
         <is>
           <t>PDF header shows report name; org; period and an as-of line; logo if set</t>
         </is>
       </c>
-      <c r="B53" s="2" t="inlineStr">
+      <c r="B51" s="2" t="inlineStr">
         <is>
           <t>IV — Exports</t>
         </is>
       </c>
-      <c r="C53" s="2" t="inlineStr">
-        <is>
-          <t>Functional</t>
-        </is>
-      </c>
-      <c r="D53" s="2" t="inlineStr">
+      <c r="C51" s="2" t="inlineStr">
+        <is>
+          <t>Functional</t>
+        </is>
+      </c>
+      <c r="D51" s="2" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="E53" s="2" t="inlineStr">
+      <c r="E51" s="2" t="inlineStr">
         <is>
           <t>1. You are signed in to the ShopView App on a desktop browser.
 2. The shop has a logo set in its settings.
 3. The report is open on a view whose displayed day is known (live today, or a recorded past day).</t>
         </is>
       </c>
-      <c r="F53" s="2" t="inlineStr">
+      <c r="F51" s="2" t="inlineStr">
         <is>
           <t>1. Download the PDF and read its header.
 2. Look at the top of the PDF for the shop logo.
@@ -3126,58 +3047,60 @@
 4. If reachable, repeat the PDF download on a period with no available snapshot and read the header's as-of line.</t>
         </is>
       </c>
-      <c r="G53" s="2" t="inlineStr">
+      <c r="G51" s="2" t="inlineStr">
         <is>
           <t>1. The PDF header shows the report name "Inventory Value", the organization name, the selected period, and an "as of" line naming the day the values represent (or a message that no snapshot is available for the period).
 2. The PDF shows the shop logo at the top when one is set.
 3. The CSV never includes a logo.
 4. Note for the tester: the two files phrase the as-of line differently - the PDF reads "As of 2026-08-04" and the CSV's first line reads "As of: 2026-08-04" (with a colon). Both are correct; do not raise the difference.
 ---
+DO NOT AUTOMATE YET: this behaviour is waiting on an answer from the product owner. Automating it now could lock in the wrong behaviour.
+The open question is in: Report-Suite_Questions-and-Decisions-for-Chris-Ward_2026-08-04.xlsx — https://raw.githubusercontent.com/bilalmuzamil-sketch/Manual-test-Cases/claude/slack-session-0sxnd9/build/report-suite/chris-consolidated-2026-08-04/Report-Suite_Questions-and-Decisions-for-Chris-Ward_2026-08-04.xlsx
 This is the expected behaviour as per the build tested on 8/4/2026, and as per the Inventory Value report specification version 3 (S10-R8, S10-R9).</t>
         </is>
       </c>
-      <c r="H53" s="2" t="inlineStr">
+      <c r="H51" s="2" t="inlineStr">
         <is>
           <t>SV-8677 (IV spec v3 2026-07-29 Story 10 S10-R8; S10-R9)</t>
         </is>
       </c>
-      <c r="I53" s="2" t="inlineStr"/>
-      <c r="J53" s="2" t="inlineStr"/>
-    </row>
-    <row r="54">
-      <c r="A54" s="2" t="inlineStr">
+      <c r="I51" s="2" t="inlineStr"/>
+      <c r="J51" s="2" t="inlineStr"/>
+    </row>
+    <row r="52">
+      <c r="A52" s="2" t="inlineStr">
         <is>
           <t>Downloaded files are named inventory-value-report.pdf and .csv</t>
         </is>
       </c>
-      <c r="B54" s="2" t="inlineStr">
+      <c r="B52" s="2" t="inlineStr">
         <is>
           <t>IV — Exports</t>
         </is>
       </c>
-      <c r="C54" s="2" t="inlineStr">
-        <is>
-          <t>Functional</t>
-        </is>
-      </c>
-      <c r="D54" s="2" t="inlineStr">
+      <c r="C52" s="2" t="inlineStr">
+        <is>
+          <t>Functional</t>
+        </is>
+      </c>
+      <c r="D52" s="2" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="E54" s="2" t="inlineStr">
+      <c r="E52" s="2" t="inlineStr">
         <is>
           <t>1. You are signed in to the ShopView App on a desktop browser.
 2. The Inventory Value report is open with rows loaded.</t>
         </is>
       </c>
-      <c r="F54" s="2" t="inlineStr">
+      <c r="F52" s="2" t="inlineStr">
         <is>
           <t>1. Download the current view as a PDF and read the saved file's name.
 2. Download the current view as a CSV and read the saved file's name.</t>
         </is>
       </c>
-      <c r="G54" s="2" t="inlineStr">
+      <c r="G52" s="2" t="inlineStr">
         <is>
           <t>1. The PDF is named "inventory-value-report.pdf".
 2. The CSV is named "inventory-value-report.csv".
@@ -3185,49 +3108,49 @@
 This is the expected behaviour as per the build tested on 8/4/2026, and as per the Inventory Value report specification version 3 (S10-R10).</t>
         </is>
       </c>
-      <c r="H54" s="2" t="inlineStr">
+      <c r="H52" s="2" t="inlineStr">
         <is>
           <t>SV-8677 (IV spec v3 2026-07-29 Story 10 S10-R10 — S10-R10 CLOSES both file names verbatim; so the exact strings ARE the requirement)</t>
         </is>
       </c>
-      <c r="I54" s="2" t="inlineStr"/>
-      <c r="J54" s="2" t="inlineStr"/>
-    </row>
-    <row r="55">
-      <c r="A55" s="2" t="inlineStr">
+      <c r="I52" s="2" t="inlineStr"/>
+      <c r="J52" s="2" t="inlineStr"/>
+    </row>
+    <row r="53">
+      <c r="A53" s="2" t="inlineStr">
         <is>
           <t>Exports are generated server-side over the full filtered set</t>
         </is>
       </c>
-      <c r="B55" s="2" t="inlineStr">
+      <c r="B53" s="2" t="inlineStr">
         <is>
           <t>IV — Exports</t>
         </is>
       </c>
-      <c r="C55" s="2" t="inlineStr">
-        <is>
-          <t>Functional</t>
-        </is>
-      </c>
-      <c r="D55" s="2" t="inlineStr">
+      <c r="C53" s="2" t="inlineStr">
+        <is>
+          <t>Functional</t>
+        </is>
+      </c>
+      <c r="D53" s="2" t="inlineStr">
         <is>
           <t>Critical</t>
         </is>
       </c>
-      <c r="E55" s="2" t="inlineStr">
+      <c r="E53" s="2" t="inlineStr">
         <is>
           <t>1. You are signed in to the ShopView App on a desktop browser.
 2. The current filtered set spans more than one page (but stays under the export row cap).</t>
         </is>
       </c>
-      <c r="F55" s="2" t="inlineStr">
+      <c r="F53" s="2" t="inlineStr">
         <is>
           <t>1. From page 1, without visiting the later pages, download the CSV.
 2. Count the file's data rows and look for parts you know sit on the later pages.
 3. Compare the file's totals row to the on-screen totals.</t>
         </is>
       </c>
-      <c r="G55" s="2" t="inlineStr">
+      <c r="G53" s="2" t="inlineStr">
         <is>
           <t>1. The export contains the FULL filtered set — every qualifying row across all pages, not only the rows loaded in the browser.
 2. Parts from the later pages are present.
@@ -3236,49 +3159,49 @@
 This is the expected behaviour as per the build tested on 8/4/2026, and as per the Inventory Value report specification version 3 (S10-R11).</t>
         </is>
       </c>
-      <c r="H55" s="2" t="inlineStr">
+      <c r="H53" s="2" t="inlineStr">
         <is>
           <t>SV-8677 (IV spec v3 2026-07-29 Story 10 S10-R11)</t>
         </is>
       </c>
-      <c r="I55" s="2" t="inlineStr"/>
-      <c r="J55" s="2" t="inlineStr"/>
-    </row>
-    <row r="56">
-      <c r="A56" s="2" t="inlineStr">
+      <c r="I53" s="2" t="inlineStr"/>
+      <c r="J53" s="2" t="inlineStr"/>
+    </row>
+    <row r="54">
+      <c r="A54" s="2" t="inlineStr">
         <is>
           <t>An over-cap set produces no file and shows the too-large-to-export message</t>
         </is>
       </c>
-      <c r="B56" s="2" t="inlineStr">
+      <c r="B54" s="2" t="inlineStr">
         <is>
           <t>IV — Exports</t>
         </is>
       </c>
-      <c r="C56" s="2" t="inlineStr">
+      <c r="C54" s="2" t="inlineStr">
         <is>
           <t>Negative</t>
         </is>
       </c>
-      <c r="D56" s="2" t="inlineStr">
+      <c r="D54" s="2" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="E56" s="2" t="inlineStr">
+      <c r="E54" s="2" t="inlineStr">
         <is>
           <t>1. You are signed in to the ShopView App on a desktop browser.
 2. A filter/location combination exists whose filtered set EXCEEDS the export row cap (seed ZZAUTOTEST parts in bulk if needed, or use the largest available data set).</t>
         </is>
       </c>
-      <c r="F56" s="2" t="inlineStr">
+      <c r="F54" s="2" t="inlineStr">
         <is>
           <t>1. Set the filters so the filtered set exceeds the export row cap.
 2. Request "Download (PDF)" and read what happens.
 3. Request "Download (CSV)" and read what happens.</t>
         </is>
       </c>
-      <c r="G56" s="2" t="inlineStr">
+      <c r="G54" s="2" t="inlineStr">
         <is>
           <t>1. Neither the PDF nor the CSV is produced.
 2. The user sees the message: "This report is too large to export. Narrow the date range or filters, then try again." (a blocking notification; no file).
@@ -3289,50 +3212,50 @@
 This is the expected behaviour as per the build tested on 8/4/2026, and as per the Inventory Value report specification version 3 (S10-R12).</t>
         </is>
       </c>
-      <c r="H56" s="2" t="inlineStr">
+      <c r="H54" s="2" t="inlineStr">
         <is>
           <t>SV-8677 (IV spec v3 2026-07-29 Story 10 S10-R12; §7 User Feedback Summary)</t>
         </is>
       </c>
-      <c r="I56" s="2" t="inlineStr"/>
-      <c r="J56" s="2" t="inlineStr"/>
-    </row>
-    <row r="57">
-      <c r="A57" s="2" t="inlineStr">
+      <c r="I54" s="2" t="inlineStr"/>
+      <c r="J54" s="2" t="inlineStr"/>
+    </row>
+    <row r="55">
+      <c r="A55" s="2" t="inlineStr">
         <is>
           <t>Download notifications: verbatim success and failure texts per format</t>
         </is>
       </c>
-      <c r="B57" s="2" t="inlineStr">
+      <c r="B55" s="2" t="inlineStr">
         <is>
           <t>IV — Exports</t>
         </is>
       </c>
-      <c r="C57" s="2" t="inlineStr">
+      <c r="C55" s="2" t="inlineStr">
         <is>
           <t>Negative</t>
         </is>
       </c>
-      <c r="D57" s="2" t="inlineStr">
+      <c r="D55" s="2" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="E57" s="2" t="inlineStr">
+      <c r="E55" s="2" t="inlineStr">
         <is>
           <t>1. You are signed in to the ShopView App on a desktop browser.
 2. The Inventory Value report is open with rows loaded (under the export cap).
 3. A download failure can be simulated (for example, disconnect the network just before requesting the download).</t>
         </is>
       </c>
-      <c r="F57" s="2" t="inlineStr">
+      <c r="F55" s="2" t="inlineStr">
         <is>
           <t>1. Download the PDF and the CSV normally and read each notification.
 2. Simulate a failure and request the PDF download; read the notification.
 3. Repeat the failure for the CSV download.</t>
         </is>
       </c>
-      <c r="G57" s="2" t="inlineStr">
+      <c r="G55" s="2" t="inlineStr">
         <is>
           <t>1. Success notifications read verbatim: "Inventory Value report exported (PDF)" and "Inventory Value report exported (CSV)".
 2. Failure notifications read verbatim: "Failed to export inventory value report (pdf)" and "Failed to export inventory value report (csv)".
@@ -3343,42 +3266,42 @@
 This is the expected behaviour as per the build tested on 8/4/2026, and as per the Inventory Value report specification version 3 (S10-R13, S10-R14).</t>
         </is>
       </c>
-      <c r="H57" s="2" t="inlineStr">
+      <c r="H55" s="2" t="inlineStr">
         <is>
           <t>SV-8677 (IV spec v3 2026-07-29 Story 10 S10-R13; S10-R14; §7 User Feedback Summary)</t>
         </is>
       </c>
-      <c r="I57" s="2" t="inlineStr"/>
-      <c r="J57" s="2" t="inlineStr"/>
-    </row>
-    <row r="58">
-      <c r="A58" s="2" t="inlineStr">
+      <c r="I55" s="2" t="inlineStr"/>
+      <c r="J55" s="2" t="inlineStr"/>
+    </row>
+    <row r="56">
+      <c r="A56" s="2" t="inlineStr">
         <is>
           <t>A large Inventory Value PDF fails instead of being refused politely</t>
         </is>
       </c>
-      <c r="B58" s="2" t="inlineStr">
+      <c r="B56" s="2" t="inlineStr">
         <is>
           <t>IV — Exports</t>
         </is>
       </c>
-      <c r="C58" s="2" t="inlineStr">
-        <is>
-          <t>Functional</t>
-        </is>
-      </c>
-      <c r="D58" s="2" t="inlineStr">
+      <c r="C56" s="2" t="inlineStr">
+        <is>
+          <t>Functional</t>
+        </is>
+      </c>
+      <c r="D56" s="2" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="E58" s="2" t="inlineStr">
+      <c r="E56" s="2" t="inlineStr">
         <is>
           <t>1. You are signed in with ordinary reports access, on a desktop browser.
 2. The Inventory Value report is open and the whole list runs to several thousand rows.</t>
         </is>
       </c>
-      <c r="F58" s="2" t="inlineStr">
+      <c r="F56" s="2" t="inlineStr">
         <is>
           <t>1. Use the part search to narrow the list to a few hundred rows. Open the three-dot menu and choose the PDF download. Note how long it takes.
 2. Clear the search so the whole list is shown again. Choose the PDF download and wait up to a minute.
@@ -3386,7 +3309,7 @@
 4. Narrow the list again with the part search, or pick a single location, and ask for the PDF once more.</t>
         </is>
       </c>
-      <c r="G58" s="2" t="inlineStr">
+      <c r="G56" s="2" t="inlineStr">
         <is>
           <t>1. The narrowed PDF downloads successfully.
 2. On the whole list the PDF either downloads successfully too, or is refused politely with the message "This report is too large to export. Narrow the date range or filters, then try again." Either of those is a pass.
@@ -3399,49 +3322,49 @@
 This is the expected behaviour as per the build tested on 8/4/2026, and as per the Inventory Value report specification version 3 (S10-R11, S10-R12, S10-R14).</t>
         </is>
       </c>
-      <c r="H58" s="2" t="inlineStr">
+      <c r="H56" s="2" t="inlineStr">
         <is>
           <t>SV-8677 (IV spec v3 2026-07-29 S10-R11; S10-R12; S10-R14 — the observed failure path is a roughly 30-second server-side timeout and not the S10-R12 row cap; observed on build v3.4.1-0ed4433)</t>
         </is>
       </c>
-      <c r="I58" s="2" t="inlineStr"/>
-      <c r="J58" s="2" t="inlineStr"/>
-    </row>
-    <row r="59">
-      <c r="A59" s="2" t="inlineStr">
+      <c r="I56" s="2" t="inlineStr"/>
+      <c r="J56" s="2" t="inlineStr"/>
+    </row>
+    <row r="57">
+      <c r="A57" s="2" t="inlineStr">
         <is>
           <t>All-white table with no row shading on the standard report backdrop</t>
         </is>
       </c>
-      <c r="B59" s="2" t="inlineStr">
+      <c r="B57" s="2" t="inlineStr">
         <is>
           <t>IV — Visual &amp; Accessibility</t>
         </is>
       </c>
-      <c r="C59" s="2" t="inlineStr">
-        <is>
-          <t>Functional</t>
-        </is>
-      </c>
-      <c r="D59" s="2" t="inlineStr">
+      <c r="C57" s="2" t="inlineStr">
+        <is>
+          <t>Functional</t>
+        </is>
+      </c>
+      <c r="D57" s="2" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="E59" s="2" t="inlineStr">
+      <c r="E57" s="2" t="inlineStr">
         <is>
           <t>1. You are signed in to the ShopView App on a desktop browser.
 2. The Inventory Value report is open with several rows.</t>
         </is>
       </c>
-      <c r="F59" s="2" t="inlineStr">
+      <c r="F57" s="2" t="inlineStr">
         <is>
           <t>1. Look at the column headers and the data cells.
 2. Compare the background of consecutive rows.
 3. Look at the page background around the table.</t>
         </is>
       </c>
-      <c r="G59" s="2" t="inlineStr">
+      <c r="G57" s="2" t="inlineStr">
         <is>
           <t>1. The table has white column headers and white data cells, with no alternating row shading.
 2. The table sits on the standard soft blue-grey report backdrop.
@@ -3449,48 +3372,48 @@
 This is the expected behaviour as per the build tested on 8/4/2026, and as per the Inventory Value report specification version 3 (S12-R1).</t>
         </is>
       </c>
-      <c r="H59" s="2" t="inlineStr">
+      <c r="H57" s="2" t="inlineStr">
         <is>
           <t>SV-8679 (IV spec v3 2026-07-29 Story 12 S12-R1)</t>
         </is>
       </c>
-      <c r="I59" s="2" t="inlineStr"/>
-      <c r="J59" s="2" t="inlineStr"/>
-    </row>
-    <row r="60">
-      <c r="A60" s="2" t="inlineStr">
+      <c r="I57" s="2" t="inlineStr"/>
+      <c r="J57" s="2" t="inlineStr"/>
+    </row>
+    <row r="58">
+      <c r="A58" s="2" t="inlineStr">
         <is>
           <t>Toolbar layout: menu leftmost then Column Selection; then the 5 filters</t>
         </is>
       </c>
-      <c r="B60" s="2" t="inlineStr">
+      <c r="B58" s="2" t="inlineStr">
         <is>
           <t>IV — Visual &amp; Accessibility</t>
         </is>
       </c>
-      <c r="C60" s="2" t="inlineStr">
-        <is>
-          <t>Functional</t>
-        </is>
-      </c>
-      <c r="D60" s="2" t="inlineStr">
+      <c r="C58" s="2" t="inlineStr">
+        <is>
+          <t>Functional</t>
+        </is>
+      </c>
+      <c r="D58" s="2" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="E60" s="2" t="inlineStr">
+      <c r="E58" s="2" t="inlineStr">
         <is>
           <t>1. You are signed in to the ShopView App on a desktop browser.
 2. The Inventory Value report is open.</t>
         </is>
       </c>
-      <c r="F60" s="2" t="inlineStr">
+      <c r="F58" s="2" t="inlineStr">
         <is>
           <t>1. Look at the toolbar's action cluster and read the order of its controls.
 2. Read the toolbar filters from left to right.</t>
         </is>
       </c>
-      <c r="G60" s="2" t="inlineStr">
+      <c r="G58" s="2" t="inlineStr">
         <is>
           <t>1. In the toolbar, the three-dot download menu sits leftmost in the action cluster, followed by the Column Selection control.
 2. The toolbar filters run, left to right: the date-range control, the part search, the Category filter, the Vendor filter, and the Location filter (rightmost).
@@ -3498,49 +3421,49 @@
 This is the expected behaviour as per the build tested on 8/4/2026, and as per the Inventory Value report specification version 3 (S12-R2, S12-R3).</t>
         </is>
       </c>
-      <c r="H60" s="2" t="inlineStr">
+      <c r="H58" s="2" t="inlineStr">
         <is>
           <t>SV-8679 (IV spec v3 2026-07-29 Story 12 S12-R2; S12-R3)</t>
         </is>
       </c>
-      <c r="I60" s="2" t="inlineStr"/>
-      <c r="J60" s="2" t="inlineStr"/>
-    </row>
-    <row r="61">
-      <c r="A61" s="2" t="inlineStr">
+      <c r="I58" s="2" t="inlineStr"/>
+      <c r="J58" s="2" t="inlineStr"/>
+    </row>
+    <row r="59">
+      <c r="A59" s="2" t="inlineStr">
         <is>
           <t>Long Description; Category and Vendor truncate on hover; Part # never does</t>
         </is>
       </c>
-      <c r="B61" s="2" t="inlineStr">
+      <c r="B59" s="2" t="inlineStr">
         <is>
           <t>IV — Visual &amp; Accessibility</t>
         </is>
       </c>
-      <c r="C61" s="2" t="inlineStr">
-        <is>
-          <t>Functional</t>
-        </is>
-      </c>
-      <c r="D61" s="2" t="inlineStr">
+      <c r="C59" s="2" t="inlineStr">
+        <is>
+          <t>Functional</t>
+        </is>
+      </c>
+      <c r="D59" s="2" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="E61" s="2" t="inlineStr">
+      <c r="E59" s="2" t="inlineStr">
         <is>
           <t>1. You are signed in to the ShopView App on a desktop browser.
 2. A ZZAUTOTEST part exists with a very long description (and, if possible, long category/vendor names) and a long part number.</t>
         </is>
       </c>
-      <c r="F61" s="2" t="inlineStr">
+      <c r="F59" s="2" t="inlineStr">
         <is>
           <t>1. Narrow the browser window (or turn on more columns) so the text columns overflow.
 2. Read the long Description, Category, and Vendor cells and hover each.
 3. Read the long Part # cell.</t>
         </is>
       </c>
-      <c r="G61" s="2" t="inlineStr">
+      <c r="G59" s="2" t="inlineStr">
         <is>
           <t>1. Long text values (Description, Category, Vendor) are truncated with an ellipsis when they overflow their column.
 2. The full value is available on hover.
@@ -3549,49 +3472,49 @@
 This is the expected behaviour as per the build tested on 8/4/2026, and as per the Inventory Value report specification version 3 (S12-R6).</t>
         </is>
       </c>
-      <c r="H61" s="2" t="inlineStr">
+      <c r="H59" s="2" t="inlineStr">
         <is>
           <t>SV-8679 (IV spec v3 2026-07-29 Story 12 S12-R6)</t>
         </is>
       </c>
-      <c r="I61" s="2" t="inlineStr"/>
-      <c r="J61" s="2" t="inlineStr"/>
-    </row>
-    <row r="62">
-      <c r="A62" s="2" t="inlineStr">
+      <c r="I59" s="2" t="inlineStr"/>
+      <c r="J59" s="2" t="inlineStr"/>
+    </row>
+    <row r="60">
+      <c r="A60" s="2" t="inlineStr">
         <is>
           <t>In dark mode the page background, toolbar, cells; the "—" glyph remain legible</t>
         </is>
       </c>
-      <c r="B62" s="2" t="inlineStr">
+      <c r="B60" s="2" t="inlineStr">
         <is>
           <t>IV — Visual &amp; Accessibility</t>
         </is>
       </c>
-      <c r="C62" s="2" t="inlineStr">
+      <c r="C60" s="2" t="inlineStr">
         <is>
           <t>Accessibility</t>
         </is>
       </c>
-      <c r="D62" s="2" t="inlineStr">
+      <c r="D60" s="2" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="E62" s="2" t="inlineStr">
+      <c r="E60" s="2" t="inlineStr">
         <is>
           <t>1. You are signed in to the ShopView App on a desktop browser.
 2. The application is switched to dark mode.
 3. The report shows rows including a part with an em-dash ("—") Category or Vendor cell.</t>
         </is>
       </c>
-      <c r="F62" s="2" t="inlineStr">
+      <c r="F60" s="2" t="inlineStr">
         <is>
           <t>1. Read the page background, toolbar, and table cells in dark mode.
 2. Find a "—" cell and check its legibility.</t>
         </is>
       </c>
-      <c r="G62" s="2" t="inlineStr">
+      <c r="G60" s="2" t="inlineStr">
         <is>
           <t>1. The report supports dark mode: the page background, the toolbar, and the table cells all switch to their dark equivalents rather than staying light.
 2. In dark mode you can read the toolbar text and the cell text at a glance, and the "—" glyph in an empty Category or Vendor cell is clearly visible against the dark cell behind it — it does not disappear into the background.
@@ -3600,50 +3523,50 @@
 This is the expected behaviour as per the build tested on 8/4/2026, and as per the Inventory Value report specification version 3 (S12-R7).</t>
         </is>
       </c>
-      <c r="H62" s="2" t="inlineStr">
+      <c r="H60" s="2" t="inlineStr">
         <is>
           <t>SV-8679 (IV spec v3 2026-07-29 Story 12 S12-R7)</t>
         </is>
       </c>
-      <c r="I62" s="2" t="inlineStr"/>
-      <c r="J62" s="2" t="inlineStr"/>
-    </row>
-    <row r="63">
-      <c r="A63" s="2" t="inlineStr">
+      <c r="I60" s="2" t="inlineStr"/>
+      <c r="J60" s="2" t="inlineStr"/>
+    </row>
+    <row r="61">
+      <c r="A61" s="2" t="inlineStr">
         <is>
           <t>Each sortable header exposes its sort state and shows the direction</t>
         </is>
       </c>
-      <c r="B63" s="2" t="inlineStr">
+      <c r="B61" s="2" t="inlineStr">
         <is>
           <t>IV — Visual &amp; Accessibility</t>
         </is>
       </c>
-      <c r="C63" s="2" t="inlineStr">
+      <c r="C61" s="2" t="inlineStr">
         <is>
           <t>Accessibility</t>
         </is>
       </c>
-      <c r="D63" s="2" t="inlineStr">
+      <c r="D61" s="2" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="E63" s="2" t="inlineStr">
+      <c r="E61" s="2" t="inlineStr">
         <is>
           <t>1. You are signed in to the ShopView App on a desktop browser.
 2. The Inventory Value report is open with rows loaded.
 3. Part of this test checks what a blind user would hear, so you need a screen reader. On Windows install NVDA — it is free, from nvaccess.org. On a Mac use VoiceOver, which is already built in (Cmd+F5 turns it on and off). Alternatively the browser's developer tools (F12) have an "Accessibility" panel that shows the same names without you having to listen to anything.</t>
         </is>
       </c>
-      <c r="F63" s="2" t="inlineStr">
+      <c r="F61" s="2" t="inlineStr">
         <is>
           <t>1. Sort by a column and look at its header for a visual direction indicator.
 2. With the accessibility inspector or screen reader, check what sort state the header exposes.
 3. Toggle the direction and check both again.</t>
         </is>
       </c>
-      <c r="G63" s="2" t="inlineStr">
+      <c r="G61" s="2" t="inlineStr">
         <is>
           <t>1. The active sort direction is indicated visually on the header.
 2. Each sortable column header exposes its sort state to assistive technology (for example, ascending/descending/none).
@@ -3652,98 +3575,98 @@
 This is the expected behaviour as per the build tested on 8/4/2026, and as per the Inventory Value report specification version 3 (S12-R8).</t>
         </is>
       </c>
-      <c r="H63" s="2" t="inlineStr">
+      <c r="H61" s="2" t="inlineStr">
         <is>
           <t>SV-8679 (IV spec v3 2026-07-29 Story 12 S12-R8)</t>
         </is>
       </c>
-      <c r="I63" s="2" t="inlineStr"/>
-      <c r="J63" s="2" t="inlineStr"/>
-    </row>
-    <row r="64">
-      <c r="A64" s="2" t="inlineStr">
+      <c r="I61" s="2" t="inlineStr"/>
+      <c r="J61" s="2" t="inlineStr"/>
+    </row>
+    <row r="62">
+      <c r="A62" s="2" t="inlineStr">
         <is>
           <t>The icon-only download and Column Selection buttons carry accessible names</t>
         </is>
       </c>
-      <c r="B64" s="2" t="inlineStr">
+      <c r="B62" s="2" t="inlineStr">
         <is>
           <t>IV — Visual &amp; Accessibility</t>
         </is>
       </c>
-      <c r="C64" s="2" t="inlineStr">
+      <c r="C62" s="2" t="inlineStr">
         <is>
           <t>Accessibility</t>
         </is>
       </c>
-      <c r="D64" s="2" t="inlineStr">
+      <c r="D62" s="2" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="E64" s="2" t="inlineStr">
+      <c r="E62" s="2" t="inlineStr">
         <is>
           <t>1. You are signed in to the ShopView App on a desktop browser.
 2. The Inventory Value report is open.
 3. Part of this test checks what a blind user would hear, so you need a screen reader. On Windows install NVDA — it is free, from nvaccess.org. On a Mac use VoiceOver, which is already built in (Cmd+F5 turns it on and off). Alternatively the browser's developer tools (F12) have an "Accessibility" panel that shows the same names without you having to listen to anything.</t>
         </is>
       </c>
-      <c r="F64" s="2" t="inlineStr">
+      <c r="F62" s="2" t="inlineStr">
         <is>
           <t>1. Inspect the three-dot download button's accessible name.
 2. Inspect the Column Selection button's accessible name.</t>
         </is>
       </c>
-      <c r="G64" s="2" t="inlineStr">
+      <c r="G62" s="2" t="inlineStr">
         <is>
           <t>1. Each icon-only control carries an accessible name exposed to assistive technology (it is not announced as an unnamed button).
 ---
 This is the expected behaviour as per the build tested on 8/4/2026, and as per the Inventory Value report specification version 3 (S12-R9).</t>
         </is>
       </c>
-      <c r="H64" s="2" t="inlineStr">
+      <c r="H62" s="2" t="inlineStr">
         <is>
           <t>SV-8679 (IV spec v3 2026-07-29 Story 12 S12-R9)</t>
         </is>
       </c>
-      <c r="I64" s="2" t="inlineStr"/>
-      <c r="J64" s="2" t="inlineStr"/>
-    </row>
-    <row r="65">
-      <c r="A65" s="2" t="inlineStr">
+      <c r="I62" s="2" t="inlineStr"/>
+      <c r="J62" s="2" t="inlineStr"/>
+    </row>
+    <row r="63">
+      <c r="A63" s="2" t="inlineStr">
         <is>
           <t>A user with ordinary reports access can open Inventory Value</t>
         </is>
       </c>
-      <c r="B65" s="2" t="inlineStr">
+      <c r="B63" s="2" t="inlineStr">
         <is>
           <t>IV — Permissions</t>
         </is>
       </c>
-      <c r="C65" s="2" t="inlineStr">
-        <is>
-          <t>Functional</t>
-        </is>
-      </c>
-      <c r="D65" s="2" t="inlineStr">
+      <c r="C63" s="2" t="inlineStr">
+        <is>
+          <t>Functional</t>
+        </is>
+      </c>
+      <c r="D63" s="2" t="inlineStr">
         <is>
           <t>Critical</t>
         </is>
       </c>
-      <c r="E65" s="2" t="inlineStr">
+      <c r="E63" s="2" t="inlineStr">
         <is>
           <t>1. A test user exists whose role has the ordinary reports access (assign the Tech user a suitable role if needed; restore the original role afterward).
 2. You are signed in as that user on a desktop browser.</t>
         </is>
       </c>
-      <c r="F65" s="2" t="inlineStr">
+      <c r="F63" s="2" t="inlineStr">
         <is>
           <t>1. Open the reports navigation and find "Inventory Value" under the Parts group.
 2. Open the report and confirm it loads rows.
 3. Download the current view as a CSV.</t>
         </is>
       </c>
-      <c r="G65" s="2" t="inlineStr">
+      <c r="G63" s="2" t="inlineStr">
         <is>
           <t>1. The report is listed and opens normally for a user holding the ordinary reports access.
 2. No additional report-specific permission is required — for now the one ordinary reports access covers all six of the new reports.
@@ -3752,84 +3675,84 @@
 This is the expected behaviour as per the build tested on 8/4/2026, and as per the Inventory Value report specification version 3 (Story 1 Prerequisites); where the wording of that specification differs, the behaviour above follows a later product decision, which is the authority.</t>
         </is>
       </c>
-      <c r="H65" s="2" t="inlineStr">
+      <c r="H63" s="2" t="inlineStr">
         <is>
           <t>SV-8668 (IV spec Story 1 Prerequisites — one reports permission for all six ruled by Chris Ward Q2=A + QA lead 2026-08-03 "ONE permission FOR NOW"; the IV prerequisite still names the inventory-reports permission — his spec edit owed)</t>
         </is>
       </c>
-      <c r="I65" s="2" t="inlineStr"/>
-      <c r="J65" s="2" t="inlineStr"/>
-    </row>
-    <row r="66">
-      <c r="A66" s="2" t="inlineStr">
+      <c r="I63" s="2" t="inlineStr"/>
+      <c r="J63" s="2" t="inlineStr"/>
+    </row>
+    <row r="64">
+      <c r="A64" s="2" t="inlineStr">
         <is>
           <t>Without reports access Inventory Value is absent from the navigation</t>
         </is>
       </c>
-      <c r="B66" s="2" t="inlineStr">
+      <c r="B64" s="2" t="inlineStr">
         <is>
           <t>IV — Permissions</t>
         </is>
       </c>
-      <c r="C66" s="2" t="inlineStr">
+      <c r="C64" s="2" t="inlineStr">
         <is>
           <t>Negative</t>
         </is>
       </c>
-      <c r="D66" s="2" t="inlineStr">
+      <c r="D64" s="2" t="inlineStr">
         <is>
           <t>Critical</t>
         </is>
       </c>
-      <c r="E66" s="2" t="inlineStr">
+      <c r="E64" s="2" t="inlineStr">
         <is>
           <t>1. A test user exists whose role does NOT have reports access (assign the Tech user such a role; restore the original role afterward).
 2. You are signed in as that user on a desktop browser.</t>
         </is>
       </c>
-      <c r="F66" s="2" t="inlineStr">
+      <c r="F64" s="2" t="inlineStr">
         <is>
           <t>1. Open the reports navigation.
 2. Look for "Inventory Value" under the Parts group.</t>
         </is>
       </c>
-      <c r="G66" s="2" t="inlineStr">
+      <c r="G64" s="2" t="inlineStr">
         <is>
           <t>1. The report does not appear in the navigation for this user.
 ---
 This is the expected behaviour as per the build tested on 8/4/2026, and as per the Inventory Value report specification version 3 (S1-N1).</t>
         </is>
       </c>
-      <c r="H66" s="2" t="inlineStr">
+      <c r="H64" s="2" t="inlineStr">
         <is>
           <t>SV-8668 (IV spec Story 1 S1-N1 — the gate is the one ordinary reports access per Chris Ward Q2=A + QA lead 2026-08-03 "ONE permission FOR NOW")</t>
         </is>
       </c>
-      <c r="I66" s="2" t="inlineStr"/>
-      <c r="J66" s="2" t="inlineStr"/>
-    </row>
-    <row r="67">
-      <c r="A67" s="2" t="inlineStr">
+      <c r="I64" s="2" t="inlineStr"/>
+      <c r="J64" s="2" t="inlineStr"/>
+    </row>
+    <row r="65">
+      <c r="A65" s="2" t="inlineStr">
         <is>
           <t>Nightly snapshot records one row per in-stock non-core part per location</t>
         </is>
       </c>
-      <c r="B67" s="2" t="inlineStr">
+      <c r="B65" s="2" t="inlineStr">
         <is>
           <t>IV — API</t>
         </is>
       </c>
-      <c r="C67" s="2" t="inlineStr">
-        <is>
-          <t>Functional</t>
-        </is>
-      </c>
-      <c r="D67" s="2" t="inlineStr">
+      <c r="C65" s="2" t="inlineStr">
+        <is>
+          <t>Functional</t>
+        </is>
+      </c>
+      <c r="D65" s="2" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="E67" s="2" t="inlineStr">
+      <c r="E65" s="2" t="inlineStr">
         <is>
           <t>1. In-stock, non-core parts exist at two or more locations, including a part with non-round cent values.
 2. A location with NO in-stock parts also exists.
@@ -3837,14 +3760,14 @@
 4. To see the information this test asks for you need the browser's own developer tools: press F12 (or Ctrl+Shift+I; on a Mac Cmd+Option+I) and open the "Network" tab, then reload the page. There is nothing to install — it is built into Chrome, Edge and Firefox. Where a check also asks you to confirm what is stored on the server, ask a developer to read it back for you — that part cannot be seen from the browser.</t>
         </is>
       </c>
-      <c r="F67" s="2" t="inlineStr">
+      <c r="F65" s="2" t="inlineStr">
         <is>
           <t>1. After the overnight capture, inspect the stored snapshot rows for that calendar date.
 2. For a known part, read every captured field.
 3. Check the rows for each location, including the empty one.</t>
         </is>
       </c>
-      <c r="G67" s="2" t="inlineStr">
+      <c r="G65" s="2" t="inlineStr">
         <is>
           <t>1. Once per day, overnight, one row per then-in-stock, non-core part is recorded for every location across every organization, under that day's calendar date.
 2. Each row captures the part's identity (part, category, vendor), on-hand quantity, unit cost, unit sell, total cost, and total sell, stored to the cent.
@@ -3853,36 +3776,36 @@
 This is the expected behaviour as per the build tested on 8/4/2026, and as per the Inventory Value report specification version 3 (S11-R1, S11-R4).</t>
         </is>
       </c>
-      <c r="H67" s="2" t="inlineStr">
+      <c r="H65" s="2" t="inlineStr">
         <is>
           <t>SV-8678 (IV spec v3 2026-07-29 Story 11 S11-R1; S11-R4)</t>
         </is>
       </c>
-      <c r="I67" s="2" t="inlineStr"/>
-      <c r="J67" s="2" t="inlineStr"/>
-    </row>
-    <row r="68">
-      <c r="A68" s="2" t="inlineStr">
+      <c r="I65" s="2" t="inlineStr"/>
+      <c r="J65" s="2" t="inlineStr"/>
+    </row>
+    <row r="66">
+      <c r="A66" s="2" t="inlineStr">
         <is>
           <t>A recorded snapshot day equals what the live report showed that day</t>
         </is>
       </c>
-      <c r="B68" s="2" t="inlineStr">
+      <c r="B66" s="2" t="inlineStr">
         <is>
           <t>IV — API</t>
         </is>
       </c>
-      <c r="C68" s="2" t="inlineStr">
-        <is>
-          <t>Functional</t>
-        </is>
-      </c>
-      <c r="D68" s="2" t="inlineStr">
+      <c r="C66" s="2" t="inlineStr">
+        <is>
+          <t>Functional</t>
+        </is>
+      </c>
+      <c r="D66" s="2" t="inlineStr">
         <is>
           <t>Critical</t>
         </is>
       </c>
-      <c r="E68" s="2" t="inlineStr">
+      <c r="E66" s="2" t="inlineStr">
         <is>
           <t>1. ZZAUTOTEST parts with known quantities, costs, and sell resolutions (fixed price, matrix markup, and no-category fallback) are in stock and left UNCHANGED across the capture.
 2. A core-charge part and a zero-quantity part also exist.
@@ -3890,7 +3813,7 @@
 4. To see the information this test asks for you need the browser's own developer tools: press F12 (or Ctrl+Shift+I; on a Mac Cmd+Option+I) and open the "Network" tab, then reload the page. There is nothing to install — it is built into Chrome, Edge and Firefox. Where a check also asks you to confirm what is stored on the server, ask a developer to read it back for you — that part cannot be seen from the browser.</t>
         </is>
       </c>
-      <c r="F68" s="2" t="inlineStr">
+      <c r="F66" s="2" t="inlineStr">
         <is>
           <t>1. On the capture date, note the live report's rows and values for the seeded parts.
 2. After the overnight capture, read the same parts' captured rows.
@@ -3898,7 +3821,7 @@
 4. The next day, view the report as of the captured date and compare to the noted live values.</t>
         </is>
       </c>
-      <c r="G68" s="2" t="inlineStr">
+      <c r="G66" s="2" t="inlineStr">
         <is>
           <t>1. The captured parts use the same in-stock, non-core scope as the live report (Story 2) — the core-charge and zero-quantity parts are NOT captured.
 2. The captured values use the same valuation as the live report (Story 3), including the sell-price fallback chain.
@@ -3907,154 +3830,105 @@
 This is the expected behaviour as per the build tested on 8/4/2026, and as per the Inventory Value report specification version 3 (S11-R2).</t>
         </is>
       </c>
-      <c r="H68" s="2" t="inlineStr">
+      <c r="H66" s="2" t="inlineStr">
         <is>
           <t>SV-8678 (IV spec v3 2026-07-29 Story 11 S11-R2; §2 Relationship to nightly history)</t>
         </is>
       </c>
-      <c r="I68" s="2" t="inlineStr"/>
-      <c r="J68" s="2" t="inlineStr"/>
-    </row>
-    <row r="69">
-      <c r="A69" s="2" t="inlineStr">
+      <c r="I66" s="2" t="inlineStr"/>
+      <c r="J66" s="2" t="inlineStr"/>
+    </row>
+    <row r="67">
+      <c r="A67" s="2" t="inlineStr">
         <is>
           <t>Nightly snapshot: re-running the capture for a date replaces that date's rows</t>
         </is>
       </c>
-      <c r="B69" s="2" t="inlineStr">
+      <c r="B67" s="2" t="inlineStr">
         <is>
           <t>IV — API</t>
         </is>
       </c>
-      <c r="C69" s="2" t="inlineStr">
-        <is>
-          <t>Functional</t>
-        </is>
-      </c>
-      <c r="D69" s="2" t="inlineStr">
+      <c r="C67" s="2" t="inlineStr">
+        <is>
+          <t>Functional</t>
+        </is>
+      </c>
+      <c r="D67" s="2" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="E69" s="2" t="inlineStr">
+      <c r="E67" s="2" t="inlineStr">
         <is>
           <t>1. A capture has already run for the current date.
 2. The capture can be re-run for that date (arrange with the developers).
 3. To see the information this test asks for you need the browser's own developer tools: press F12 (or Ctrl+Shift+I; on a Mac Cmd+Option+I) and open the "Network" tab, then reload the page. There is nothing to install — it is built into Chrome, Edge and Firefox. Where a check also asks you to confirm what is stored on the server, ask a developer to read it back for you — that part cannot be seen from the browser.</t>
         </is>
       </c>
-      <c r="F69" s="2" t="inlineStr">
+      <c r="F67" s="2" t="inlineStr">
         <is>
           <t>1. Count the stored rows per location for the date.
 2. Re-run the capture for the same date.
 3. Count and inspect the rows again.</t>
         </is>
       </c>
-      <c r="G69" s="2" t="inlineStr">
+      <c r="G67" s="2" t="inlineStr">
         <is>
           <t>1. Re-running the capture for a date replaces that date's rows for each location — the existing rows for that location and date are removed, then re-inserted from current data.
 2. No duplicate rows exist for the same part, location, and date.
 3. The capture is idempotent and self-healing from current data.
----
-This is the expected behaviour as per the build tested on 8/4/2026, and as per the Inventory Value report specification version 3 (S11-R3).</t>
-        </is>
-      </c>
-      <c r="H69" s="2" t="inlineStr">
-        <is>
-          <t>SV-8678 (IV spec v3 2026-07-29 Story 11 S11-R3)</t>
-        </is>
-      </c>
-      <c r="I69" s="2" t="inlineStr"/>
-      <c r="J69" s="2" t="inlineStr"/>
-    </row>
-    <row r="70">
-      <c r="A70" s="2" t="inlineStr">
-        <is>
-          <t>Nightly snapshot: a re-run records today's truth; it cannot rebuild a past day</t>
-        </is>
-      </c>
-      <c r="B70" s="2" t="inlineStr">
+4. No rows exist for dates before capture began — there is no backfill.
+5. A re-run always records current truth under the CURRENT date; it cannot reconstruct a past date.
+6. A past date's stored rows are unchanged by a current re-run.
+---
+This is the expected behaviour as per the build tested on 8/4/2026, and as per the Inventory Value report specification version 3 (S11-R3, S11-R5, S5-E1).</t>
+        </is>
+      </c>
+      <c r="H67" s="2" t="inlineStr">
+        <is>
+          <t>SV-8678 (IV spec v3 2026-07-29 Story 11 S11-R3; Story 11 S11-R5; Story 5 S5-E1)</t>
+        </is>
+      </c>
+      <c r="I67" s="2" t="inlineStr"/>
+      <c r="J67" s="2" t="inlineStr"/>
+    </row>
+    <row r="68">
+      <c r="A68" s="2" t="inlineStr">
+        <is>
+          <t>Snapshot retention: daily captures are kept for 0–13 months</t>
+        </is>
+      </c>
+      <c r="B68" s="2" t="inlineStr">
         <is>
           <t>IV — API</t>
         </is>
       </c>
-      <c r="C70" s="2" t="inlineStr">
-        <is>
-          <t>Functional</t>
-        </is>
-      </c>
-      <c r="D70" s="2" t="inlineStr">
-        <is>
-          <t>Medium</t>
-        </is>
-      </c>
-      <c r="E70" s="2" t="inlineStr">
-        <is>
-          <t>1. The date the first capture ran is known.
-2. Stock levels have changed since a past captured date.
-3. To see the information this test asks for you need the browser's own developer tools: press F12 (or Ctrl+Shift+I; on a Mac Cmd+Option+I) and open the "Network" tab, then reload the page. There is nothing to install — it is built into Chrome, Edge and Firefox. Where a check also asks you to confirm what is stored on the server, ask a developer to read it back for you — that part cannot be seen from the browser.</t>
-        </is>
-      </c>
-      <c r="F70" s="2" t="inlineStr">
-        <is>
-          <t>1. Check the stored history for any rows dated before the first capture.
-2. Re-run the capture and check which date its rows are recorded under.
-3. Compare a past date's stored rows to confirm they were not rewritten by the re-run.</t>
-        </is>
-      </c>
-      <c r="G70" s="2" t="inlineStr">
-        <is>
-          <t>1. No rows exist for dates before capture began — there is no backfill.
-2. A re-run always records current truth under the CURRENT date; it cannot reconstruct a past date.
-3. Past dates' stored rows are unchanged by a current re-run.
----
-This is the expected behaviour as per the build tested on 8/4/2026, and as per the Inventory Value report specification version 3 (S11-R5, S5-E1).</t>
-        </is>
-      </c>
-      <c r="H70" s="2" t="inlineStr">
-        <is>
-          <t>SV-8678 (IV spec v3 2026-07-29 Story 11 S11-R5; Story 5 S5-E1)</t>
-        </is>
-      </c>
-      <c r="I70" s="2" t="inlineStr"/>
-      <c r="J70" s="2" t="inlineStr"/>
-    </row>
-    <row r="71">
-      <c r="A71" s="2" t="inlineStr">
-        <is>
-          <t>Snapshot retention: daily captures are kept for 0–13 months</t>
-        </is>
-      </c>
-      <c r="B71" s="2" t="inlineStr">
-        <is>
-          <t>IV — API</t>
-        </is>
-      </c>
-      <c r="C71" s="2" t="inlineStr">
-        <is>
-          <t>Functional</t>
-        </is>
-      </c>
-      <c r="D71" s="2" t="inlineStr">
+      <c r="C68" s="2" t="inlineStr">
+        <is>
+          <t>Functional</t>
+        </is>
+      </c>
+      <c r="D68" s="2" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="E71" s="2" t="inlineStr">
+      <c r="E68" s="2" t="inlineStr">
         <is>
           <t>1. Snapshot history exists (or is seeded/simulated with dev help) spanning both the 0–13-month band and the older-than-13-months band.
 2. The nightly capture (with its pruning) has run.
 3. To see the information this test asks for you need the browser's own developer tools: press F12 (or Ctrl+Shift+I; on a Mac Cmd+Option+I) and open the "Network" tab, then reload the page. There is nothing to install — it is built into Chrome, Edge and Firefox. Where a check also asks you to confirm what is stored on the server, ask a developer to read it back for you — that part cannot be seen from the browser.</t>
         </is>
       </c>
-      <c r="F71" s="2" t="inlineStr">
+      <c r="F68" s="2" t="inlineStr">
         <is>
           <t>1. Inspect the retained captures for dates within the last 13 months.
 2. Inspect the retained captures for dates older than 13 months.
 3. Check when pruning runs relative to the nightly capture.</t>
         </is>
       </c>
-      <c r="G71" s="2" t="inlineStr">
+      <c r="G68" s="2" t="inlineStr">
         <is>
           <t>1. For ages 0–13 months (measured from the current date), every daily capture is kept — full daily per-part detail, covering the report's longest date preset (366 days / This Year / Last Year) entirely at daily resolution.
 2. For ages older than 13 months, only the last capture of each calendar month is retained; the other daily captures in that band are pruned.
@@ -4063,50 +3937,50 @@
 This is the expected behaviour as per the build tested on 8/4/2026, and as per the Inventory Value report specification version 3 (S11-R6).</t>
         </is>
       </c>
-      <c r="H71" s="2" t="inlineStr">
+      <c r="H68" s="2" t="inlineStr">
         <is>
           <t>SV-8678 (IV spec v3 2026-07-29 Story 11 S11-R6)</t>
         </is>
       </c>
-      <c r="I71" s="2" t="inlineStr"/>
-      <c r="J71" s="2" t="inlineStr"/>
-    </row>
-    <row r="72">
-      <c r="A72" s="2" t="inlineStr">
+      <c r="I68" s="2" t="inlineStr"/>
+      <c r="J68" s="2" t="inlineStr"/>
+    </row>
+    <row r="69">
+      <c r="A69" s="2" t="inlineStr">
         <is>
           <t>Thinned history still served by the closest-recorded-day rule</t>
         </is>
       </c>
-      <c r="B72" s="2" t="inlineStr">
+      <c r="B69" s="2" t="inlineStr">
         <is>
           <t>IV — API</t>
         </is>
       </c>
-      <c r="C72" s="2" t="inlineStr">
-        <is>
-          <t>Functional</t>
-        </is>
-      </c>
-      <c r="D72" s="2" t="inlineStr">
+      <c r="C69" s="2" t="inlineStr">
+        <is>
+          <t>Functional</t>
+        </is>
+      </c>
+      <c r="D69" s="2" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="E72" s="2" t="inlineStr">
+      <c r="E69" s="2" t="inlineStr">
         <is>
           <t>1. Thinned history exists (dates older than 13 months where only the monthly last-capture remains — dev-seeded if needed).
 2. The retained capture dates around the requested date are known.
 3. To see the information this test asks for you need the browser's own developer tools: press F12 (or Ctrl+Shift+I; on a Mac Cmd+Option+I) and open the "Network" tab, then reload the page. There is nothing to install — it is built into Chrome, Edge and Firefox. Where a check also asks you to confirm what is stored on the server, ask a developer to read it back for you — that part cannot be seen from the browser.</t>
         </is>
       </c>
-      <c r="F72" s="2" t="inlineStr">
+      <c r="F69" s="2" t="inlineStr">
         <is>
           <t>1. On the report, select a range ending on a pruned date between two retained monthly captures.
 2. Read which day the values represent and the "As of" indicator.
 3. Select a range whose covering captures have ALL been pruned and no earlier retained capture remains.</t>
         </is>
       </c>
-      <c r="G72" s="2" t="inlineStr">
+      <c r="G69" s="2" t="inlineStr">
         <is>
           <t>1. The as-of resolution serves the thinned history unchanged: the report resolves to the nearest earlier retained capture ("closest recorded day on or before"), even when adjacent retained captures are up to a month apart.
 2. The "As of" indicator names the day actually shown.
@@ -4115,13 +3989,13 @@
 This is the expected behaviour as per the build tested on 8/4/2026, and as per the Inventory Value report specification version 3 (S11-E1, S11-R6, S5-R4, S5-R5, S5-N1).</t>
         </is>
       </c>
-      <c r="H72" s="2" t="inlineStr">
+      <c r="H69" s="2" t="inlineStr">
         <is>
           <t>SV-8678 (IV spec v3 2026-07-29 Story 11 S11-E1; S11-R6; Story 5 S5-R4; S5-R5; S5-N1)</t>
         </is>
       </c>
-      <c r="I72" s="2" t="inlineStr"/>
-      <c r="J72" s="2" t="inlineStr"/>
+      <c r="I69" s="2" t="inlineStr"/>
+      <c r="J69" s="2" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
chore(sweeper): checkpoint 31 dirty path(s)
Automatic additive checkpoint so no work is lost (Standing Rule 29).
Paths were hash-stable for 20s and passed the secret scan.
Top-level areas: build, testrail-import

  build/report-suite/cases
  build/report-suite/step4-retire-2026-08-04
  build/report-suite/step4-retire-2026-08-04/backup
  testrail-import

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01AZ5XzKsK9wv7M41cSPaMyg
</commit_message>
<xml_diff>
--- a/testrail-import/Report-Suite_Inventory-Value-Report_testrail-import.xlsx
+++ b/testrail-import/Report-Suite_Inventory-Value-Report_testrail-import.xlsx
@@ -630,7 +630,7 @@
       </c>
       <c r="H4" s="2" t="inlineStr">
         <is>
-          <t>SV-8668 (IV spec v3 2026-07-29 Story 1 S1-R3; Story 7 S7-R2)</t>
+          <t>SV-8668 (specs/inventory-value.md Story 1 S1-R3; Story 7 S7-R2)</t>
         </is>
       </c>
       <c r="I4" s="2" t="inlineStr"/>
@@ -778,14 +778,13 @@
 2. The core-charge part is never listed — even with a positive quantity — and its value is not counted in the totals row.
 3. The zero-quantity and negative-quantity parts are not listed — only quantities greater than zero are valued.
 4. Only parts meeting BOTH conditions — not a core charge, and on-hand quantity greater than zero — are listed.
-5. A part that has sat without movement for a long time still appears and is still counted — there is no dead-stock exclusion; how long stock has sat makes no difference.
 ---
 This is the expected behaviour as per the build tested on 8/4/2026, and as per the Inventory Value report specification version 3 (S2-R1, S2-R2, S2-N1, S2-N2).</t>
         </is>
       </c>
       <c r="H7" s="2" t="inlineStr">
         <is>
-          <t>SV-8669 (IV spec v3 2026-07-29 Story 2 S2-R1; S2-R2; S2-N1; S2-N2; §3 Key Decisions; Story 2 context note (no dead-stock exclusion))</t>
+          <t>SV-8669 (IV spec v3 2026-07-29 Story 2 S2-R1; S2-R2; S2-N1; S2-N2; §3 Key Decisions)</t>
         </is>
       </c>
       <c r="I7" s="2" t="inlineStr"/>
@@ -1186,8 +1185,6 @@
 3. Every other column is right-aligned.
 4. Location is one of the columns in the column-selection control; when it is turned on the Location column appears between Vendor and Qty, left-aligned.
 ---
-DO NOT AUTOMATE YET: this behaviour is waiting on an answer from the product owner. Automating it now could lock in the wrong behaviour.
-The open question is in: Report-Suite_Questions-and-Decisions-for-Chris-Ward_2026-08-04.xlsx — https://raw.githubusercontent.com/bilalmuzamil-sketch/Manual-test-Cases/claude/slack-session-0sxnd9/build/report-suite/chris-consolidated-2026-08-04/Report-Suite_Questions-and-Decisions-for-Chris-Ward_2026-08-04.xlsx
 This is the expected behaviour as per the build tested on 8/4/2026, and as per the Inventory Value report specification version 3 (S3-R1, S3-R2, S7-R6); on this point that specification currently states otherwise and a product decision is still awaited, so treat the behaviour described above as what the build does today.</t>
         </is>
       </c>
@@ -1340,8 +1337,6 @@
 3. Both can be turned on from the column-selection control and then appear in their fixed positions.
 4. Location is one of the columns in the column-selection control; when it is turned on the Location column shows between Vendor and Qty.
 ---
-DO NOT AUTOMATE YET: this behaviour is waiting on an answer from the product owner. Automating it now could lock in the wrong behaviour.
-The open question is in: Report-Suite_Questions-and-Decisions-for-Chris-Ward_2026-08-04.xlsx — https://raw.githubusercontent.com/bilalmuzamil-sketch/Manual-test-Cases/claude/slack-session-0sxnd9/build/report-suite/chris-consolidated-2026-08-04/Report-Suite_Questions-and-Decisions-for-Chris-Ward_2026-08-04.xlsx
 This is the expected behaviour as per the build tested on 8/4/2026, and as per the Inventory Value report specification version 3 (S3-R12, S3-R13, S8-R3, S7-R6); on this point that specification currently states otherwise and a product decision is still awaited, so treat the behaviour described above as what the build does today.</t>
         </is>
       </c>
@@ -1448,14 +1443,13 @@
 3. The totals-row Total Cost cell is pinned far right and bold, matching the column, and the row uses the same number formats as the data rows.
 4. The totals row stays visible at the bottom while the rows scroll.
 5. Note for the tester: if the label on screen reads "Totals" instead of "Total", mark this test Failed and report it — do not change the test.
-6. Sorting by any column reorders the data rows only — the totals row stays at the bottom.
----
-This is the expected behaviour as per the build tested on 8/4/2026, and as per the Inventory Value report specification version 3 (S4-R1, S4-R4, S4-R5, S4-R6, S4-R7, S12-R5, S9-R4).</t>
+---
+This is the expected behaviour as per the build tested on 8/4/2026, and as per the Inventory Value report specification version 3 (S4-R1, S4-R4, S4-R5, S4-R6, S4-R7, S12-R5).</t>
         </is>
       </c>
       <c r="H20" s="2" t="inlineStr">
         <is>
-          <t>SV-8671 (IV spec v3 2026-07-29 Story 4 S4-R1; S4-R4; S4-R5; S4-R6; S4-R7; Story 12 S12-R5; Story 9 S9-R4)</t>
+          <t>SV-8671 (IV spec v3 2026-07-29 Story 4 S4-R1; S4-R4; S4-R5; S4-R6; S4-R7; Story 12 S12-R5)</t>
         </is>
       </c>
       <c r="I20" s="2" t="inlineStr"/>
@@ -1606,8 +1600,6 @@
           <t>1. The control offers the standard presets: "Today", "Yesterday", "This Week", "Last Week", "This Month", "Last Month", "This Year", "Last Year", "This Quarter", "Last Quarter", and "Custom".
 2. "All Time" is NOT offered — because the report is valued as of a single date, an All-Time option would be meaningless; its absence is the documented v1 behavior.
 ---
-DO NOT AUTOMATE YET: this behaviour is waiting on an answer from the product owner. Automating it now could lock in the wrong behaviour.
-The open question is in: Report-Suite_Questions-and-Decisions-for-Chris-Ward_2026-08-04.xlsx — https://raw.githubusercontent.com/bilalmuzamil-sketch/Manual-test-Cases/claude/slack-session-0sxnd9/build/report-suite/chris-consolidated-2026-08-04/Report-Suite_Questions-and-Decisions-for-Chris-Ward_2026-08-04.xlsx
 This is the expected behaviour as per the build tested on 8/4/2026, and as per the Inventory Value report specification version 3 (S5-R1).</t>
         </is>
       </c>
@@ -1761,8 +1753,6 @@
 2. The part's row shows the quantity and values recorded for that day, not today's live stock.
 Known issue: the product does not currently do this. It has been filed for a fix here: https://shopview.atlassian.net/browse/SV-8820
 ---
-DO NOT AUTOMATE YET: this behaviour is waiting on an answer from the product owner. Automating it now could lock in the wrong behaviour.
-The open question is in: Report-Suite_Questions-and-Decisions-for-Chris-Ward_2026-08-04.xlsx — https://raw.githubusercontent.com/bilalmuzamil-sketch/Manual-test-Cases/claude/slack-session-0sxnd9/build/report-suite/chris-consolidated-2026-08-04/Report-Suite_Questions-and-Decisions-for-Chris-Ward_2026-08-04.xlsx
 This is the expected behaviour as per the build tested on 8/4/2026, and as per the Inventory Value report specification version 3 (S5-R4).</t>
         </is>
       </c>
@@ -1819,7 +1809,7 @@
       </c>
       <c r="H27" s="2" t="inlineStr">
         <is>
-          <t>SV-8672 (IV spec v3 2026-07-29 Story 5 S5-R5; S5-R6)</t>
+          <t>SV-8672 (specs/inventory-value.md Story 5 S5-R5; S5-R6)</t>
         </is>
       </c>
       <c r="I27" s="2" t="inlineStr"/>
@@ -2282,7 +2272,7 @@
       </c>
       <c r="H36" s="2" t="inlineStr">
         <is>
-          <t>SV-8674 (IV spec v3 2026-07-29 Story 7 S7-R1; S7-R2; Story 12 S12-R3 — per-row location identifier in All-locations view ADDED per kickoff video P10 40:58-41:20; user ruling 2026-07-28: video overrides spec (video newer; last-update-wins))</t>
+          <t>SV-8674 (specs/inventory-value.md Story 7 S7-R1; S7-R2; Story 12 S12-R3 — per-row location identifier in All-locations view ADDED per kickoff video P10 40:58-41:20; user ruling 2026-07-28: video overrides spec (video newer; last-update-wins))</t>
         </is>
       </c>
       <c r="I36" s="2" t="inlineStr"/>
@@ -2426,8 +2416,6 @@
           <t>1. For the single-location user the Location filter is NOT shown at all — the report simply shows that one location's stock.
 2. For the user with access to two or more locations the Location filter IS shown.
 ---
-DO NOT AUTOMATE YET: this behaviour is waiting on an answer from the product owner. Automating it now could lock in the wrong behaviour.
-The open question is in: Report-Suite_Questions-and-Decisions-for-Chris-Ward_2026-08-04.xlsx — https://raw.githubusercontent.com/bilalmuzamil-sketch/Manual-test-Cases/claude/slack-session-0sxnd9/build/report-suite/chris-consolidated-2026-08-04/Report-Suite_Questions-and-Decisions-for-Chris-Ward_2026-08-04.xlsx
 This is the expected behaviour as per the build tested on 8/4/2026, and as per the Inventory Value report specification version 3 (S7-N1); where the wording of that specification differs, the behaviour above follows a later product decision, which is the authority.</t>
         </is>
       </c>
@@ -2488,8 +2476,6 @@
 6. The Location filter control keeps the same width whichever label it shows — one location, several, or "All locations" — so the toolbar does not shift as you change the selection.
 7. Both downloads include the Location column in the same position it holds on screen (between Vendor and Qty), naming each row's own location.
 ---
-DO NOT AUTOMATE YET: this behaviour is waiting on an answer from the product owner. Automating it now could lock in the wrong behaviour.
-The open question is in: Report-Suite_Questions-and-Decisions-for-Chris-Ward_2026-08-04.xlsx — https://raw.githubusercontent.com/bilalmuzamil-sketch/Manual-test-Cases/claude/slack-session-0sxnd9/build/report-suite/chris-consolidated-2026-08-04/Report-Suite_Questions-and-Decisions-for-Chris-Ward_2026-08-04.xlsx
 This is the expected behaviour as per the build tested on 8/4/2026, and as per the Inventory Value report specification version 3 (S7-R6, S7-R7, S3-R1, S12-R10, S10-R15); on this point that specification currently states otherwise and a product decision is still awaited, so treat the behaviour described above as what the build does today.</t>
         </is>
       </c>
@@ -2590,8 +2576,6 @@
           <t>1. Whatever columns are shown, they appear in the fixed left-to-right order - with Location, when it is turned on in the column-selection control, between Vendor and Qty (Part #, Description, Category, Vendor, Qty, Unit Cost, Unit Sell, Margin, Margin %, Total Sell, Total Cost) - toggling visibility never reorders columns.
 2. Total Cost is always the last column.
 ---
-DO NOT AUTOMATE YET: this behaviour is waiting on an answer from the product owner. Automating it now could lock in the wrong behaviour.
-The open question is in: Report-Suite_Questions-and-Decisions-for-Chris-Ward_2026-08-04.xlsx — https://raw.githubusercontent.com/bilalmuzamil-sketch/Manual-test-Cases/claude/slack-session-0sxnd9/build/report-suite/chris-consolidated-2026-08-04/Report-Suite_Questions-and-Decisions-for-Chris-Ward_2026-08-04.xlsx
 This is the expected behaviour as per the build tested on 8/4/2026, and as per the Inventory Value report specification version 3 (S8-R4, S3-R1, S7-R6); on this point that specification currently states otherwise and a product decision is still awaited, so treat the behaviour described above as what the build does today.</t>
         </is>
       </c>
@@ -2948,8 +2932,6 @@
 4. Each download (PDF and CSV) carries a "Locations:" line naming the location(s) the report was scoped to (exact position in the file is confirmed in the build).
 5. Note for the tester: the files carry the Location column when Location is turned ON in the column-selection control (it sits between Vendor and Qty). It does not appear just because you have more than one location selected.
 ---
-DO NOT AUTOMATE YET: this behaviour is waiting on an answer from the product owner. Automating it now could lock in the wrong behaviour.
-The open question is in: Report-Suite_Questions-and-Decisions-for-Chris-Ward_2026-08-04.xlsx — https://raw.githubusercontent.com/bilalmuzamil-sketch/Manual-test-Cases/claude/slack-session-0sxnd9/build/report-suite/chris-consolidated-2026-08-04/Report-Suite_Questions-and-Decisions-for-Chris-Ward_2026-08-04.xlsx
 This is the expected behaviour as per the build tested on 8/4/2026, and as per the Inventory Value report specification version 3 (S10-R3, S10-R4, S10-R5, S10-R6, S10-R15); on this point that specification currently states otherwise and a product decision is still awaited, so treat the behaviour described above as what the build does today.</t>
         </is>
       </c>
@@ -3005,7 +2987,7 @@
       </c>
       <c r="H50" s="2" t="inlineStr">
         <is>
-          <t>SV-8677 (IV spec v3 2026-07-29 Story 10 S10-R7 (+ context note))</t>
+          <t>SV-8677 (specs/inventory-value.md Story 10 S10-R7 (+ context note))</t>
         </is>
       </c>
       <c r="I50" s="2" t="inlineStr"/>
@@ -3054,8 +3036,6 @@
 3. The CSV never includes a logo.
 4. Note for the tester: the two files phrase the as-of line differently - the PDF reads "As of 2026-08-04" and the CSV's first line reads "As of: 2026-08-04" (with a colon). Both are correct; do not raise the difference.
 ---
-DO NOT AUTOMATE YET: this behaviour is waiting on an answer from the product owner. Automating it now could lock in the wrong behaviour.
-The open question is in: Report-Suite_Questions-and-Decisions-for-Chris-Ward_2026-08-04.xlsx — https://raw.githubusercontent.com/bilalmuzamil-sketch/Manual-test-Cases/claude/slack-session-0sxnd9/build/report-suite/chris-consolidated-2026-08-04/Report-Suite_Questions-and-Decisions-for-Chris-Ward_2026-08-04.xlsx
 This is the expected behaviour as per the build tested on 8/4/2026, and as per the Inventory Value report specification version 3 (S10-R8, S10-R9).</t>
         </is>
       </c>
@@ -3374,7 +3354,7 @@
       </c>
       <c r="H57" s="2" t="inlineStr">
         <is>
-          <t>SV-8679 (IV spec v3 2026-07-29 Story 12 S12-R1)</t>
+          <t>SV-8679 (specs/inventory-value.md Story 12 S12-R1)</t>
         </is>
       </c>
       <c r="I57" s="2" t="inlineStr"/>
@@ -3423,7 +3403,7 @@
       </c>
       <c r="H58" s="2" t="inlineStr">
         <is>
-          <t>SV-8679 (IV spec v3 2026-07-29 Story 12 S12-R2; S12-R3)</t>
+          <t>SV-8679 (specs/inventory-value.md Story 12 S12-R2; S12-R3)</t>
         </is>
       </c>
       <c r="I58" s="2" t="inlineStr"/>
@@ -3878,16 +3858,13 @@
           <t>1. Re-running the capture for a date replaces that date's rows for each location — the existing rows for that location and date are removed, then re-inserted from current data.
 2. No duplicate rows exist for the same part, location, and date.
 3. The capture is idempotent and self-healing from current data.
-4. No rows exist for dates before capture began — there is no backfill.
-5. A re-run always records current truth under the CURRENT date; it cannot reconstruct a past date.
-6. A past date's stored rows are unchanged by a current re-run.
----
-This is the expected behaviour as per the build tested on 8/4/2026, and as per the Inventory Value report specification version 3 (S11-R3, S11-R5, S5-E1).</t>
+---
+This is the expected behaviour as per the build tested on 8/4/2026, and as per the Inventory Value report specification version 3 (S11-R3).</t>
         </is>
       </c>
       <c r="H67" s="2" t="inlineStr">
         <is>
-          <t>SV-8678 (IV spec v3 2026-07-29 Story 11 S11-R3; Story 11 S11-R5; Story 5 S5-E1)</t>
+          <t>SV-8678 (IV spec v3 2026-07-29 Story 11 S11-R3)</t>
         </is>
       </c>
       <c r="I67" s="2" t="inlineStr"/>

</xml_diff>

<commit_message>
Report Suite Fabian-review: regenerate local mirror + import + id-map (507 cases)
Re-synced 53 touched + 9 new cases into local case source from live, regenerated the
unified + 6 per-report imports and the id-map. Also closed the last cross-case
contradiction (C30234 SBR labels + Adjustments tie-out) and removed the VIU jargon from
the 3 Loom-sourced visual cases (import must be VIU-word-free) - reworded to "confirm
live". Hygiene: import 507 rows / id-map 507 (0 blank C-ids, refs 507/507), 0 VIU, 0
flag words, 0 dup titles/ids, shredding guard 0, header sha256 == all peers, four counts
set-equal both ways (live 507 = local 507 = id-map 507 = import 507).

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01AZ5XzKsK9wv7M41cSPaMyg
</commit_message>
<xml_diff>
--- a/testrail-import/Report-Suite_Inventory-Value-Report_testrail-import.xlsx
+++ b/testrail-import/Report-Suite_Inventory-Value-Report_testrail-import.xlsx
@@ -428,7 +428,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J69"/>
+  <dimension ref="A1:J70"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="50" customWidth="1" min="1" max="1"/>
@@ -3489,38 +3489,91 @@
     <row r="57">
       <c r="A57" s="2" t="inlineStr">
         <is>
+          <t>CSV export shows the PDF header's as-of date and Locations filter lines</t>
+        </is>
+      </c>
+      <c r="B57" s="2" t="inlineStr">
+        <is>
+          <t>IV — Exports</t>
+        </is>
+      </c>
+      <c r="C57" s="2" t="inlineStr">
+        <is>
+          <t>Functional</t>
+        </is>
+      </c>
+      <c r="D57" s="2" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="E57" s="2" t="inlineStr">
+        <is>
+          <t>1. You are signed in to the ShopView App on a desktop browser.
+2. The Inventory Value report is open with at least one filter narrowed (for example a chosen date/scope and one or more locations) so the PDF header would show more than one filter line.</t>
+        </is>
+      </c>
+      <c r="F57" s="2" t="inlineStr">
+        <is>
+          <t>1. Download the report as a PDF and read the filter-summary lines in its header area.
+2. Download the report as a CSV and open it in a plain text editor or spreadsheet.
+3. Compare the leading rows of the CSV (above the column-header row) with the PDF header lines.</t>
+        </is>
+      </c>
+      <c r="G57" s="2" t="inlineStr">
+        <is>
+          <t>1. The CSV carries the same filter-summary lines as the PDF header - the "as of" date and the "Locations:" line, plus any report-specific filter lines the PDF header names - each as a leading metadata row above the column-header row.
+2. The lines appear verbatim (the same wording) and in the same order as in the PDF header.
+3. A CSV saved or forwarded later is never ambiguous about which filters produced it: every filter the PDF header names is present in the CSV.
+4. Note for the tester: this is the suite-wide rule that the CSV must name the same filters as the PDF. If your report shows no narrowed filters, widen or narrow one so at least one filter line appears, then compare again.
+---
+This is the expected behaviour as per epic SV-8582 and the Inventory Value report specification version 10 (S10-R15a), both read on 17 August 2026. S10-R15a is the suite-wide rule (added 2026-08-12, SV-9283) that the CSV carries every filter-summary line the PDF header names.
+AUTOMATION: Not available on Build to test Yet - Last checked 8/17/2026</t>
+        </is>
+      </c>
+      <c r="H57" s="2" t="inlineStr">
+        <is>
+          <t>SV-8677 (IV spec v10 2026-08-17 S10-R15a; suite-wide CSV filter-summary rule SV-9283)</t>
+        </is>
+      </c>
+      <c r="I57" s="2" t="inlineStr"/>
+      <c r="J57" s="2" t="inlineStr"/>
+    </row>
+    <row r="58">
+      <c r="A58" s="2" t="inlineStr">
+        <is>
           <t>All-white table with no row shading on the standard report backdrop</t>
         </is>
       </c>
-      <c r="B57" s="2" t="inlineStr">
+      <c r="B58" s="2" t="inlineStr">
         <is>
           <t>IV — Visual &amp; Accessibility</t>
         </is>
       </c>
-      <c r="C57" s="2" t="inlineStr">
-        <is>
-          <t>Functional</t>
-        </is>
-      </c>
-      <c r="D57" s="2" t="inlineStr">
+      <c r="C58" s="2" t="inlineStr">
+        <is>
+          <t>Functional</t>
+        </is>
+      </c>
+      <c r="D58" s="2" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="E57" s="2" t="inlineStr">
+      <c r="E58" s="2" t="inlineStr">
         <is>
           <t>1. You are signed in to the ShopView App on a desktop browser.
 2. The Inventory Value report is open with several rows.</t>
         </is>
       </c>
-      <c r="F57" s="2" t="inlineStr">
+      <c r="F58" s="2" t="inlineStr">
         <is>
           <t>1. Look at the column headers and the data cells.
 2. Compare the background of consecutive rows.
 3. Look at the page background around the table.</t>
         </is>
       </c>
-      <c r="G57" s="2" t="inlineStr">
+      <c r="G58" s="2" t="inlineStr">
         <is>
           <t>1. The table has white column headers and white data cells, with no alternating row shading.
 2. The table sits on the standard soft blue-grey report backdrop.
@@ -3530,48 +3583,48 @@
 AUTOMATION: READY</t>
         </is>
       </c>
-      <c r="H57" s="2" t="inlineStr">
+      <c r="H58" s="2" t="inlineStr">
         <is>
           <t>SV-8679 (IV spec v3 2026-07-29 Story 12 S12-R1)</t>
         </is>
       </c>
-      <c r="I57" s="2" t="inlineStr"/>
-      <c r="J57" s="2" t="inlineStr"/>
-    </row>
-    <row r="58">
-      <c r="A58" s="2" t="inlineStr">
+      <c r="I58" s="2" t="inlineStr"/>
+      <c r="J58" s="2" t="inlineStr"/>
+    </row>
+    <row r="59">
+      <c r="A59" s="2" t="inlineStr">
         <is>
           <t>Toolbar layout: menu leftmost then Column Selection; then the 5 filters</t>
         </is>
       </c>
-      <c r="B58" s="2" t="inlineStr">
+      <c r="B59" s="2" t="inlineStr">
         <is>
           <t>IV — Visual &amp; Accessibility</t>
         </is>
       </c>
-      <c r="C58" s="2" t="inlineStr">
-        <is>
-          <t>Functional</t>
-        </is>
-      </c>
-      <c r="D58" s="2" t="inlineStr">
+      <c r="C59" s="2" t="inlineStr">
+        <is>
+          <t>Functional</t>
+        </is>
+      </c>
+      <c r="D59" s="2" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="E58" s="2" t="inlineStr">
+      <c r="E59" s="2" t="inlineStr">
         <is>
           <t>1. You are signed in to the ShopView App on a desktop browser.
 2. The Inventory Value report is open.</t>
         </is>
       </c>
-      <c r="F58" s="2" t="inlineStr">
+      <c r="F59" s="2" t="inlineStr">
         <is>
           <t>1. Look at the toolbar's action cluster and read the order of its controls.
 2. Read the toolbar filters from left to right.</t>
         </is>
       </c>
-      <c r="G58" s="2" t="inlineStr">
+      <c r="G59" s="2" t="inlineStr">
         <is>
           <t>1. In the toolbar, the three-dot download menu sits leftmost in the action cluster, followed by the Column Selection control.
 2. The toolbar filters run, left to right: the date-range control, the part search, the Category filter, the Vendor filter, and the Location filter (rightmost).
@@ -3581,49 +3634,49 @@
 AUTOMATION: READY</t>
         </is>
       </c>
-      <c r="H58" s="2" t="inlineStr">
+      <c r="H59" s="2" t="inlineStr">
         <is>
           <t>SV-8679 (IV spec v3 2026-07-29 Story 12 S12-R2; S12-R3)</t>
         </is>
       </c>
-      <c r="I58" s="2" t="inlineStr"/>
-      <c r="J58" s="2" t="inlineStr"/>
-    </row>
-    <row r="59">
-      <c r="A59" s="2" t="inlineStr">
+      <c r="I59" s="2" t="inlineStr"/>
+      <c r="J59" s="2" t="inlineStr"/>
+    </row>
+    <row r="60">
+      <c r="A60" s="2" t="inlineStr">
         <is>
           <t>Long Description; Category and Vendor truncate on hover; Part # never does</t>
         </is>
       </c>
-      <c r="B59" s="2" t="inlineStr">
+      <c r="B60" s="2" t="inlineStr">
         <is>
           <t>IV — Visual &amp; Accessibility</t>
         </is>
       </c>
-      <c r="C59" s="2" t="inlineStr">
-        <is>
-          <t>Functional</t>
-        </is>
-      </c>
-      <c r="D59" s="2" t="inlineStr">
+      <c r="C60" s="2" t="inlineStr">
+        <is>
+          <t>Functional</t>
+        </is>
+      </c>
+      <c r="D60" s="2" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="E59" s="2" t="inlineStr">
+      <c r="E60" s="2" t="inlineStr">
         <is>
           <t>1. You are signed in to the ShopView App on a desktop browser.
 2. A ZZAUTOTEST part exists with a very long description (and, if possible, long category/vendor names) and a long part number.</t>
         </is>
       </c>
-      <c r="F59" s="2" t="inlineStr">
+      <c r="F60" s="2" t="inlineStr">
         <is>
           <t>1. Narrow the browser window (or turn on more columns) so the text columns overflow.
 2. Read the long Description, Category, and Vendor cells and hover each.
 3. Read the long Part # cell.</t>
         </is>
       </c>
-      <c r="G59" s="2" t="inlineStr">
+      <c r="G60" s="2" t="inlineStr">
         <is>
           <t>1. Long text values (Description, Category, Vendor) are truncated with an ellipsis when they overflow their column.
 2. The full value is available on hover.
@@ -3638,49 +3691,49 @@
 AUTOMATION: READY - EXPECT FAIL (SV-8932)</t>
         </is>
       </c>
-      <c r="H59" s="2" t="inlineStr">
+      <c r="H60" s="2" t="inlineStr">
         <is>
           <t>SV-8679 (IV spec v3 2026-07-29 Story 12 S12-R6)</t>
         </is>
       </c>
-      <c r="I59" s="2" t="inlineStr"/>
-      <c r="J59" s="2" t="inlineStr"/>
-    </row>
-    <row r="60">
-      <c r="A60" s="2" t="inlineStr">
+      <c r="I60" s="2" t="inlineStr"/>
+      <c r="J60" s="2" t="inlineStr"/>
+    </row>
+    <row r="61">
+      <c r="A61" s="2" t="inlineStr">
         <is>
           <t>In dark mode the page background, toolbar, cells; the "—" glyph remain legible</t>
         </is>
       </c>
-      <c r="B60" s="2" t="inlineStr">
+      <c r="B61" s="2" t="inlineStr">
         <is>
           <t>IV — Visual &amp; Accessibility</t>
         </is>
       </c>
-      <c r="C60" s="2" t="inlineStr">
+      <c r="C61" s="2" t="inlineStr">
         <is>
           <t>Accessibility</t>
         </is>
       </c>
-      <c r="D60" s="2" t="inlineStr">
+      <c r="D61" s="2" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="E60" s="2" t="inlineStr">
+      <c r="E61" s="2" t="inlineStr">
         <is>
           <t>1. You are signed in to the ShopView App on a desktop browser.
 2. The application is switched to dark mode.
 3. The report shows rows including a part with an em-dash ("—") Category or Vendor cell.</t>
         </is>
       </c>
-      <c r="F60" s="2" t="inlineStr">
+      <c r="F61" s="2" t="inlineStr">
         <is>
           <t>1. Read the page background, toolbar, and table cells in dark mode.
 2. Find a "—" cell and check its legibility.</t>
         </is>
       </c>
-      <c r="G60" s="2" t="inlineStr">
+      <c r="G61" s="2" t="inlineStr">
         <is>
           <t>1. The report supports dark mode: the page background, the toolbar, and the table cells all switch to their dark equivalents rather than staying light.
 2. In dark mode you can read the toolbar text and the cell text at a glance, and the "—" glyph in an empty Category or Vendor cell is clearly visible against the dark cell behind it — it does not disappear into the background.
@@ -3691,50 +3744,50 @@
 AUTOMATION: READY</t>
         </is>
       </c>
-      <c r="H60" s="2" t="inlineStr">
+      <c r="H61" s="2" t="inlineStr">
         <is>
           <t>SV-8679 (IV spec v3 2026-07-29 Story 12 S12-R7)</t>
         </is>
       </c>
-      <c r="I60" s="2" t="inlineStr"/>
-      <c r="J60" s="2" t="inlineStr"/>
-    </row>
-    <row r="61">
-      <c r="A61" s="2" t="inlineStr">
+      <c r="I61" s="2" t="inlineStr"/>
+      <c r="J61" s="2" t="inlineStr"/>
+    </row>
+    <row r="62">
+      <c r="A62" s="2" t="inlineStr">
         <is>
           <t>Each sortable header exposes its sort state and shows the direction</t>
         </is>
       </c>
-      <c r="B61" s="2" t="inlineStr">
+      <c r="B62" s="2" t="inlineStr">
         <is>
           <t>IV — Visual &amp; Accessibility</t>
         </is>
       </c>
-      <c r="C61" s="2" t="inlineStr">
+      <c r="C62" s="2" t="inlineStr">
         <is>
           <t>Accessibility</t>
         </is>
       </c>
-      <c r="D61" s="2" t="inlineStr">
+      <c r="D62" s="2" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="E61" s="2" t="inlineStr">
+      <c r="E62" s="2" t="inlineStr">
         <is>
           <t>1. You are signed in to the ShopView App on a desktop browser.
 2. The Inventory Value report is open with rows loaded.
 3. Part of this test checks what a blind user would hear, so you need a screen reader. On Windows install NVDA — it is free, from nvaccess.org. On a Mac use VoiceOver, which is already built in (Cmd+F5 turns it on and off). Alternatively the browser's developer tools (F12) have an "Accessibility" panel that shows the same names without you having to listen to anything.</t>
         </is>
       </c>
-      <c r="F61" s="2" t="inlineStr">
+      <c r="F62" s="2" t="inlineStr">
         <is>
           <t>1. Sort by a column and look at its header for a visual direction indicator.
 2. With the accessibility inspector or screen reader, check what sort state the header exposes.
 3. Toggle the direction and check both again.</t>
         </is>
       </c>
-      <c r="G61" s="2" t="inlineStr">
+      <c r="G62" s="2" t="inlineStr">
         <is>
           <t>1. The active sort direction is indicated visually on the header.
 2. Each sortable column header exposes its sort state to assistive technology (for example, ascending/descending/none).
@@ -3749,49 +3802,49 @@
 AUTOMATION: READY - EXPECT FAIL (SV-8932)</t>
         </is>
       </c>
-      <c r="H61" s="2" t="inlineStr">
+      <c r="H62" s="2" t="inlineStr">
         <is>
           <t>SV-8679 (IV spec v3 2026-07-29 Story 12 S12-R8)</t>
         </is>
       </c>
-      <c r="I61" s="2" t="inlineStr"/>
-      <c r="J61" s="2" t="inlineStr"/>
-    </row>
-    <row r="62">
-      <c r="A62" s="2" t="inlineStr">
+      <c r="I62" s="2" t="inlineStr"/>
+      <c r="J62" s="2" t="inlineStr"/>
+    </row>
+    <row r="63">
+      <c r="A63" s="2" t="inlineStr">
         <is>
           <t>The icon-only download and Column Selection buttons carry accessible names</t>
         </is>
       </c>
-      <c r="B62" s="2" t="inlineStr">
+      <c r="B63" s="2" t="inlineStr">
         <is>
           <t>IV — Visual &amp; Accessibility</t>
         </is>
       </c>
-      <c r="C62" s="2" t="inlineStr">
+      <c r="C63" s="2" t="inlineStr">
         <is>
           <t>Accessibility</t>
         </is>
       </c>
-      <c r="D62" s="2" t="inlineStr">
+      <c r="D63" s="2" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="E62" s="2" t="inlineStr">
+      <c r="E63" s="2" t="inlineStr">
         <is>
           <t>1. You are signed in to the ShopView App on a desktop browser.
 2. The Inventory Value report is open.
 3. Part of this test checks what a blind user would hear, so you need a screen reader. On Windows install NVDA — it is free, from nvaccess.org. On a Mac use VoiceOver, which is already built in (Cmd+F5 turns it on and off). Alternatively the browser's developer tools (F12) have an "Accessibility" panel that shows the same names without you having to listen to anything.</t>
         </is>
       </c>
-      <c r="F62" s="2" t="inlineStr">
+      <c r="F63" s="2" t="inlineStr">
         <is>
           <t>1. Inspect the three-dot download button's accessible name.
 2. Inspect the Column Selection button's accessible name.</t>
         </is>
       </c>
-      <c r="G62" s="2" t="inlineStr">
+      <c r="G63" s="2" t="inlineStr">
         <is>
           <t>1. Each icon-only control carries an accessible name exposed to assistive technology (it is not announced as an unnamed button).
 ---
@@ -3800,49 +3853,49 @@
 AUTOMATION: READY</t>
         </is>
       </c>
-      <c r="H62" s="2" t="inlineStr">
+      <c r="H63" s="2" t="inlineStr">
         <is>
           <t>SV-8679 (IV spec v3 2026-07-29 Story 12 S12-R9)</t>
         </is>
       </c>
-      <c r="I62" s="2" t="inlineStr"/>
-      <c r="J62" s="2" t="inlineStr"/>
-    </row>
-    <row r="63">
-      <c r="A63" s="2" t="inlineStr">
+      <c r="I63" s="2" t="inlineStr"/>
+      <c r="J63" s="2" t="inlineStr"/>
+    </row>
+    <row r="64">
+      <c r="A64" s="2" t="inlineStr">
         <is>
           <t>A user with ordinary reports access can open Inventory Value</t>
         </is>
       </c>
-      <c r="B63" s="2" t="inlineStr">
+      <c r="B64" s="2" t="inlineStr">
         <is>
           <t>IV — Permissions</t>
         </is>
       </c>
-      <c r="C63" s="2" t="inlineStr">
-        <is>
-          <t>Functional</t>
-        </is>
-      </c>
-      <c r="D63" s="2" t="inlineStr">
+      <c r="C64" s="2" t="inlineStr">
+        <is>
+          <t>Functional</t>
+        </is>
+      </c>
+      <c r="D64" s="2" t="inlineStr">
         <is>
           <t>Critical</t>
         </is>
       </c>
-      <c r="E63" s="2" t="inlineStr">
+      <c r="E64" s="2" t="inlineStr">
         <is>
           <t>1. A test user exists whose role has the ordinary reports access (assign the Tech user a suitable role if needed; restore the original role afterward).
 2. You are signed in as that user on a desktop browser.</t>
         </is>
       </c>
-      <c r="F63" s="2" t="inlineStr">
+      <c r="F64" s="2" t="inlineStr">
         <is>
           <t>1. Open the reports navigation and find "Inventory Value" under the Parts group.
 2. Open the report and confirm it loads rows.
 3. Download the current view as a CSV.</t>
         </is>
       </c>
-      <c r="G63" s="2" t="inlineStr">
+      <c r="G64" s="2" t="inlineStr">
         <is>
           <t>1. The report is listed and opens normally for a user holding the ordinary reports access.
 2. No additional report-specific permission is required — the specification allows the one ordinary reports access to cover all six of the new reports.
@@ -3853,48 +3906,48 @@
 AUTOMATION: HOLD - needs a second sign-in as a user holding only the ordinary reports access</t>
         </is>
       </c>
-      <c r="H63" s="2" t="inlineStr">
+      <c r="H64" s="2" t="inlineStr">
         <is>
           <t>SV-8668 (IV spec Story 1 Prerequisites — one reports permission for all six ruled by Chris Ward Q2=A + QA lead 2026-08-03 "ONE permission FOR NOW"; the IV prerequisite still names the inventory-reports permission — his spec edit owed)</t>
         </is>
       </c>
-      <c r="I63" s="2" t="inlineStr"/>
-      <c r="J63" s="2" t="inlineStr"/>
-    </row>
-    <row r="64">
-      <c r="A64" s="2" t="inlineStr">
+      <c r="I64" s="2" t="inlineStr"/>
+      <c r="J64" s="2" t="inlineStr"/>
+    </row>
+    <row r="65">
+      <c r="A65" s="2" t="inlineStr">
         <is>
           <t>Without reports access Inventory Value is absent from the navigation</t>
         </is>
       </c>
-      <c r="B64" s="2" t="inlineStr">
+      <c r="B65" s="2" t="inlineStr">
         <is>
           <t>IV — Permissions</t>
         </is>
       </c>
-      <c r="C64" s="2" t="inlineStr">
+      <c r="C65" s="2" t="inlineStr">
         <is>
           <t>Negative</t>
         </is>
       </c>
-      <c r="D64" s="2" t="inlineStr">
+      <c r="D65" s="2" t="inlineStr">
         <is>
           <t>Critical</t>
         </is>
       </c>
-      <c r="E64" s="2" t="inlineStr">
+      <c r="E65" s="2" t="inlineStr">
         <is>
           <t>1. A test user exists whose role does NOT have reports access (assign the Tech user such a role; restore the original role afterward).
 2. You are signed in as that user on a desktop browser.</t>
         </is>
       </c>
-      <c r="F64" s="2" t="inlineStr">
+      <c r="F65" s="2" t="inlineStr">
         <is>
           <t>1. Open the reports navigation.
 2. Look for "Inventory Value" under the Parts group.</t>
         </is>
       </c>
-      <c r="G64" s="2" t="inlineStr">
+      <c r="G65" s="2" t="inlineStr">
         <is>
           <t>1. The report does not appear in the navigation for this user.
 ---
@@ -3903,36 +3956,36 @@
 AUTOMATION: HOLD - needs a second sign-in as a user with no reports access</t>
         </is>
       </c>
-      <c r="H64" s="2" t="inlineStr">
+      <c r="H65" s="2" t="inlineStr">
         <is>
           <t>SV-8668 (IV spec Story 1 S1-N1 — the gate is the one ordinary reports access per Chris Ward Q2=A + QA lead 2026-08-03 "ONE permission FOR NOW")</t>
         </is>
       </c>
-      <c r="I64" s="2" t="inlineStr"/>
-      <c r="J64" s="2" t="inlineStr"/>
-    </row>
-    <row r="65">
-      <c r="A65" s="2" t="inlineStr">
+      <c r="I65" s="2" t="inlineStr"/>
+      <c r="J65" s="2" t="inlineStr"/>
+    </row>
+    <row r="66">
+      <c r="A66" s="2" t="inlineStr">
         <is>
           <t>Nightly snapshot records one row per in-stock non-core part per location</t>
         </is>
       </c>
-      <c r="B65" s="2" t="inlineStr">
+      <c r="B66" s="2" t="inlineStr">
         <is>
           <t>IV — API</t>
         </is>
       </c>
-      <c r="C65" s="2" t="inlineStr">
-        <is>
-          <t>Functional</t>
-        </is>
-      </c>
-      <c r="D65" s="2" t="inlineStr">
+      <c r="C66" s="2" t="inlineStr">
+        <is>
+          <t>Functional</t>
+        </is>
+      </c>
+      <c r="D66" s="2" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="E65" s="2" t="inlineStr">
+      <c r="E66" s="2" t="inlineStr">
         <is>
           <t>1. In-stock, non-core parts exist at two or more locations, including a part with non-round cent values.
 2. A location with NO in-stock parts also exists.
@@ -3940,14 +3993,14 @@
 4. To see the information this test asks for you need the browser's own developer tools: press F12 (or Ctrl+Shift+I; on a Mac Cmd+Option+I) and open the "Network" tab, then reload the page. There is nothing to install — it is built into Chrome, Edge and Firefox. Where a check also asks you to confirm what is stored on the server, ask a developer to read it back for you — that part cannot be seen from the browser.</t>
         </is>
       </c>
-      <c r="F65" s="2" t="inlineStr">
+      <c r="F66" s="2" t="inlineStr">
         <is>
           <t>1. After the overnight capture, inspect the stored snapshot rows for that calendar date.
 2. For a known part, read every captured field.
 3. Check the rows for each location, including the empty one.</t>
         </is>
       </c>
-      <c r="G65" s="2" t="inlineStr">
+      <c r="G66" s="2" t="inlineStr">
         <is>
           <t>1. Once per day, overnight, one row per then-in-stock, non-core part is recorded for every location across every organization, under that day's calendar date.
 2. Each row captures the part's identity (part, category, vendor), on-hand quantity, unit cost, unit sell, total cost, and total sell, stored to the cent.
@@ -3958,36 +4011,36 @@
 AUTOMATION: HOLD - the nightly capture is a server-side job and its stored rows are not reachable from the application</t>
         </is>
       </c>
-      <c r="H65" s="2" t="inlineStr">
+      <c r="H66" s="2" t="inlineStr">
         <is>
           <t>SV-8678 (IV spec v3 2026-07-29 Story 11 S11-R1; S11-R4)</t>
         </is>
       </c>
-      <c r="I65" s="2" t="inlineStr"/>
-      <c r="J65" s="2" t="inlineStr"/>
-    </row>
-    <row r="66">
-      <c r="A66" s="2" t="inlineStr">
+      <c r="I66" s="2" t="inlineStr"/>
+      <c r="J66" s="2" t="inlineStr"/>
+    </row>
+    <row r="67">
+      <c r="A67" s="2" t="inlineStr">
         <is>
           <t>A recorded snapshot day equals what the live report showed that day</t>
         </is>
       </c>
-      <c r="B66" s="2" t="inlineStr">
+      <c r="B67" s="2" t="inlineStr">
         <is>
           <t>IV — API</t>
         </is>
       </c>
-      <c r="C66" s="2" t="inlineStr">
-        <is>
-          <t>Functional</t>
-        </is>
-      </c>
-      <c r="D66" s="2" t="inlineStr">
+      <c r="C67" s="2" t="inlineStr">
+        <is>
+          <t>Functional</t>
+        </is>
+      </c>
+      <c r="D67" s="2" t="inlineStr">
         <is>
           <t>Critical</t>
         </is>
       </c>
-      <c r="E66" s="2" t="inlineStr">
+      <c r="E67" s="2" t="inlineStr">
         <is>
           <t>1. ZZAUTOTEST parts with known quantities, costs, and sell resolutions (fixed price, matrix markup, and no-category fallback) are in stock and left UNCHANGED across the capture.
 2. A core-charge part and a zero-quantity part also exist.
@@ -3995,7 +4048,7 @@
 4. To see the information this test asks for you need the browser's own developer tools: press F12 (or Ctrl+Shift+I; on a Mac Cmd+Option+I) and open the "Network" tab, then reload the page. There is nothing to install — it is built into Chrome, Edge and Firefox. Where a check also asks you to confirm what is stored on the server, ask a developer to read it back for you — that part cannot be seen from the browser.</t>
         </is>
       </c>
-      <c r="F66" s="2" t="inlineStr">
+      <c r="F67" s="2" t="inlineStr">
         <is>
           <t>1. On the capture date, note the live report's rows and values for the seeded parts.
 2. After the overnight capture, read the same parts' captured rows.
@@ -4003,7 +4056,7 @@
 4. The next day, view the report as of the captured date and compare to the noted live values.</t>
         </is>
       </c>
-      <c r="G66" s="2" t="inlineStr">
+      <c r="G67" s="2" t="inlineStr">
         <is>
           <t>1. The captured parts use the same in-stock, non-core scope as the live report (Story 2) — the core-charge and zero-quantity parts are NOT captured.
 2. The captured values use the same valuation as the live report (Story 3), including the sell-price fallback chain.
@@ -4014,50 +4067,50 @@
 AUTOMATION: HOLD - needs the stored nightly capture rows, which are not reachable from the application</t>
         </is>
       </c>
-      <c r="H66" s="2" t="inlineStr">
+      <c r="H67" s="2" t="inlineStr">
         <is>
           <t>SV-8678 (IV spec v3 2026-07-29 Story 11 S11-R2; §2 Relationship to nightly history)</t>
         </is>
       </c>
-      <c r="I66" s="2" t="inlineStr"/>
-      <c r="J66" s="2" t="inlineStr"/>
-    </row>
-    <row r="67">
-      <c r="A67" s="2" t="inlineStr">
+      <c r="I67" s="2" t="inlineStr"/>
+      <c r="J67" s="2" t="inlineStr"/>
+    </row>
+    <row r="68">
+      <c r="A68" s="2" t="inlineStr">
         <is>
           <t>Nightly snapshot: re-running the capture for a date replaces that date's rows</t>
         </is>
       </c>
-      <c r="B67" s="2" t="inlineStr">
+      <c r="B68" s="2" t="inlineStr">
         <is>
           <t>IV — API</t>
         </is>
       </c>
-      <c r="C67" s="2" t="inlineStr">
-        <is>
-          <t>Functional</t>
-        </is>
-      </c>
-      <c r="D67" s="2" t="inlineStr">
+      <c r="C68" s="2" t="inlineStr">
+        <is>
+          <t>Functional</t>
+        </is>
+      </c>
+      <c r="D68" s="2" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="E67" s="2" t="inlineStr">
+      <c r="E68" s="2" t="inlineStr">
         <is>
           <t>1. A capture has already run for the current date.
 2. The capture can be re-run for that date (arrange with the developers).
 3. To see the information this test asks for you need the browser's own developer tools: press F12 (or Ctrl+Shift+I; on a Mac Cmd+Option+I) and open the "Network" tab, then reload the page. There is nothing to install — it is built into Chrome, Edge and Firefox. Where a check also asks you to confirm what is stored on the server, ask a developer to read it back for you — that part cannot be seen from the browser.</t>
         </is>
       </c>
-      <c r="F67" s="2" t="inlineStr">
+      <c r="F68" s="2" t="inlineStr">
         <is>
           <t>1. Count the stored rows per location for the date.
 2. Re-run the capture for the same date.
 3. Count and inspect the rows again.</t>
         </is>
       </c>
-      <c r="G67" s="2" t="inlineStr">
+      <c r="G68" s="2" t="inlineStr">
         <is>
           <t>1. Re-running the capture for a date replaces that date's rows for each location — the existing rows for that location and date are removed, then re-inserted from current data.
 2. No duplicate rows exist for the same part, location, and date.
@@ -4071,50 +4124,50 @@
 AUTOMATION: HOLD - the nightly capture job cannot be re-run or inspected from the application</t>
         </is>
       </c>
-      <c r="H67" s="2" t="inlineStr">
+      <c r="H68" s="2" t="inlineStr">
         <is>
           <t>SV-8678 (IV spec v3 2026-07-29 Story 11 S11-R3; Story 11 S11-R5; Story 5 S5-E1)</t>
         </is>
       </c>
-      <c r="I67" s="2" t="inlineStr"/>
-      <c r="J67" s="2" t="inlineStr"/>
-    </row>
-    <row r="68">
-      <c r="A68" s="2" t="inlineStr">
+      <c r="I68" s="2" t="inlineStr"/>
+      <c r="J68" s="2" t="inlineStr"/>
+    </row>
+    <row r="69">
+      <c r="A69" s="2" t="inlineStr">
         <is>
           <t>Snapshot retention: daily captures are kept for 0–13 months</t>
         </is>
       </c>
-      <c r="B68" s="2" t="inlineStr">
+      <c r="B69" s="2" t="inlineStr">
         <is>
           <t>IV — API</t>
         </is>
       </c>
-      <c r="C68" s="2" t="inlineStr">
-        <is>
-          <t>Functional</t>
-        </is>
-      </c>
-      <c r="D68" s="2" t="inlineStr">
+      <c r="C69" s="2" t="inlineStr">
+        <is>
+          <t>Functional</t>
+        </is>
+      </c>
+      <c r="D69" s="2" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="E68" s="2" t="inlineStr">
+      <c r="E69" s="2" t="inlineStr">
         <is>
           <t>1. Snapshot history exists (or is seeded/simulated with dev help) spanning both the 0–13-month band and the older-than-13-months band.
 2. The nightly capture (with its pruning) has run.
 3. To see the information this test asks for you need the browser's own developer tools: press F12 (or Ctrl+Shift+I; on a Mac Cmd+Option+I) and open the "Network" tab, then reload the page. There is nothing to install — it is built into Chrome, Edge and Firefox. Where a check also asks you to confirm what is stored on the server, ask a developer to read it back for you — that part cannot be seen from the browser.</t>
         </is>
       </c>
-      <c r="F68" s="2" t="inlineStr">
+      <c r="F69" s="2" t="inlineStr">
         <is>
           <t>1. Inspect the retained captures for dates within the last 13 months.
 2. Inspect the retained captures for dates older than 13 months.
 3. Check when pruning runs relative to the nightly capture.</t>
         </is>
       </c>
-      <c r="G68" s="2" t="inlineStr">
+      <c r="G69" s="2" t="inlineStr">
         <is>
           <t>1. For ages 0–13 months (measured from the current date), every daily capture is kept — full daily per-part detail, covering the report's longest date preset (366 days / This Year / Last Year) entirely at daily resolution.
 2. For ages older than 13 months, only the last capture of each calendar month is retained; the other daily captures in that band are pruned.
@@ -4127,50 +4180,50 @@
 AUTOMATION: HOLD - retention pruning is a server-side job over stored history, not reachable from the application</t>
         </is>
       </c>
-      <c r="H68" s="2" t="inlineStr">
+      <c r="H69" s="2" t="inlineStr">
         <is>
           <t>SV-8678 (IV spec v3 2026-07-29 Story 11 S11-R6)</t>
         </is>
       </c>
-      <c r="I68" s="2" t="inlineStr"/>
-      <c r="J68" s="2" t="inlineStr"/>
-    </row>
-    <row r="69">
-      <c r="A69" s="2" t="inlineStr">
+      <c r="I69" s="2" t="inlineStr"/>
+      <c r="J69" s="2" t="inlineStr"/>
+    </row>
+    <row r="70">
+      <c r="A70" s="2" t="inlineStr">
         <is>
           <t>Thinned history still served by the closest-recorded-day rule</t>
         </is>
       </c>
-      <c r="B69" s="2" t="inlineStr">
+      <c r="B70" s="2" t="inlineStr">
         <is>
           <t>IV — API</t>
         </is>
       </c>
-      <c r="C69" s="2" t="inlineStr">
-        <is>
-          <t>Functional</t>
-        </is>
-      </c>
-      <c r="D69" s="2" t="inlineStr">
+      <c r="C70" s="2" t="inlineStr">
+        <is>
+          <t>Functional</t>
+        </is>
+      </c>
+      <c r="D70" s="2" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="E69" s="2" t="inlineStr">
+      <c r="E70" s="2" t="inlineStr">
         <is>
           <t>1. Thinned history exists (dates older than 13 months where only the monthly last-capture remains — dev-seeded if needed).
 2. The retained capture dates around the requested date are known.
 3. To see the information this test asks for you need the browser's own developer tools: press F12 (or Ctrl+Shift+I; on a Mac Cmd+Option+I) and open the "Network" tab, then reload the page. There is nothing to install — it is built into Chrome, Edge and Firefox. Where a check also asks you to confirm what is stored on the server, ask a developer to read it back for you — that part cannot be seen from the browser.</t>
         </is>
       </c>
-      <c r="F69" s="2" t="inlineStr">
+      <c r="F70" s="2" t="inlineStr">
         <is>
           <t>1. On the report, select a range ending on a pruned date between two retained monthly captures.
 2. Read which day the values represent and the "As of" indicator.
 3. Select a range whose covering captures have ALL been pruned and no earlier retained capture remains.</t>
         </is>
       </c>
-      <c r="G69" s="2" t="inlineStr">
+      <c r="G70" s="2" t="inlineStr">
         <is>
           <t>1. The as-of resolution serves the thinned history unchanged: the report resolves to the nearest earlier retained capture ("closest recorded day on or before"), even when adjacent retained captures are up to a month apart.
 2. The "As of" indicator names the day actually shown.
@@ -4183,13 +4236,13 @@
 AUTOMATION: HOLD - needs a thinned history that this organisation does not have and cannot be produced from the application</t>
         </is>
       </c>
-      <c r="H69" s="2" t="inlineStr">
+      <c r="H70" s="2" t="inlineStr">
         <is>
           <t>SV-8678 (IV spec v3 2026-07-29 Story 11 S11-E1; S11-R6; Story 5 S5-R4; S5-R5; S5-N1)</t>
         </is>
       </c>
-      <c r="I69" s="2" t="inlineStr"/>
-      <c r="J69" s="2" t="inlineStr"/>
+      <c r="I70" s="2" t="inlineStr"/>
+      <c r="J70" s="2" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Report Suite currency: regenerate local source + import + id-map (507/507, 0 blanks, refs 507/507, shred 0, header sha256==peers)
</commit_message>
<xml_diff>
--- a/testrail-import/Report-Suite_Inventory-Value-Report_testrail-import.xlsx
+++ b/testrail-import/Report-Suite_Inventory-Value-Report_testrail-import.xlsx
@@ -526,14 +526,13 @@
           <t>1. The reports navigation lists a report labeled "Inventory Value" under the Parts group.
 2. Clicking it opens the Inventory Value report.
 ---
-This is the expected behaviour as per epic SV-8582, read on 11 August 2026, and the Inventory Value report specification version 5 (S1-R1), read on 11 August 2026.
-Last checked against build v3.5-16cf83f on 8/6/2026.
-AUTOMATION: READY</t>
+This is the expected behaviour as per epic SV-8582, read on 17 August 2026, and the Inventory Value report specification version 10 (S1-R1), read on 17 August 2026.
+AUTOMATION: Not available on Build to test Yet - Last checked 8/17/2026</t>
         </is>
       </c>
       <c r="H2" s="2" t="inlineStr">
         <is>
-          <t>SV-8668 (IV spec Story 1 S1-R1 — access = the one ordinary reports permission per Chris Ward Q2=A + QA lead 2026-08-03 "ONE permission FOR NOW")</t>
+          <t>SV-8668 (IV spec v10 2026-08-17 Story 1 S1-R1 — access = the one ordinary reports permission per Chris Ward Q2=A + QA lead 2026-08-03 "ONE permission FOR NOW")</t>
         </is>
       </c>
       <c r="I2" s="2" t="inlineStr"/>
@@ -570,22 +569,21 @@
         <is>
           <t>1. Open the Inventory Value report.
 2. Compare the rows shown to the in-stock parts at the selected location(s).
-3. Note the date range in the toolbar and which date the values represent.</t>
+3. Note the "as of" date in the toolbar and which date the values represent.</t>
         </is>
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
           <t>1. The report shows one row for each in-stock part at the selected location(s).
-2. The values are valued as of the resolved date (the current stock for a range reaching today, or the closest recorded nightly snapshot for an earlier date — see the IV — As-of Date &amp; Snapshots cases).
----
-This is the expected behaviour as per epic SV-8582, read on 11 August 2026, and the Inventory Value report specification version 5 (S1-R2, S1-R6), read on 11 August 2026.
-Last checked against build v3.5-16cf83f on 8/6/2026.
-AUTOMATION: READY</t>
+2. The values are valued as of the resolved date (the current stock when the "as of" date is today, or the closest recorded nightly snapshot for an earlier "as of" date — see the IV — As-of Date &amp; Snapshots cases).
+---
+This is the expected behaviour as per epic SV-8582, read on 17 August 2026, and the Inventory Value report specification version 10 (S1-R2, S1-R6), read on 17 August 2026.
+AUTOMATION: Not available on Build to test Yet - Last checked 8/17/2026</t>
         </is>
       </c>
       <c r="H3" s="2" t="inlineStr">
         <is>
-          <t>SV-8668 (IV spec v3 2026-07-29 Story 1 S1-R2; S1-R6)</t>
+          <t>SV-8668 (IV spec v10 2026-08-17 Story 1 S1-R2; S1-R6)</t>
         </is>
       </c>
       <c r="I3" s="2" t="inlineStr"/>
@@ -594,7 +592,7 @@
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>First visit defaults to the current calendar month and the active location</t>
+          <t>First visit defaults to today and the active location</t>
         </is>
       </c>
       <c r="B4" s="2" t="inlineStr">
@@ -620,27 +618,27 @@
       <c r="F4" s="2" t="inlineStr">
         <is>
           <t>1. Open the Inventory Value report.
-2. Read the date-range control's value.
+2. Read the "as of" date control's value.
 3. Read the Location filter's selection.</t>
         </is>
       </c>
       <c r="G4" s="2" t="inlineStr">
         <is>
-          <t>1. The date range defaults to the current calendar month.
+          <t>1. The "as of" date defaults to today.
 2. The location defaults to the user's currently active location.
-What you should see today: on a brand-new browser the Location filter reads "All locations" and the report covers every location you can reach, instead of opening on the one location you are currently working at. The date range does open correctly on This Month. This is a known problem and it is already reported - see https://shopview.atlassian.net/browse/SV-8931
+What you should see today: on a brand-new browser the Location filter reads "All locations" and the report covers every location you can reach, instead of opening on the one location you are currently working at. The "as of" date does open correctly on today. This is a known problem and it is already reported - see https://shopview.atlassian.net/browse/SV-8931
 - If you see exactly that, mark this test FAILED and do not raise anything new.
 - If it fails in a DIFFERENT way from what is described above, that is a NEW problem - please report it.
 - If it PASSES, the fix has shipped: tell the QA lead so the ticket can be closed and this note removed.
----
-This is the expected behaviour as per epic SV-8582, read on 11 August 2026, and the Inventory Value report specification version 5 (S1-R3, S7-R2), read on 11 August 2026.
-Last checked against build v3.5-16cf83f on 8/6/2026.
+Note for the tester: an earlier version of this report offered a date range with ready-made periods. The current Inventory Value report specification (version 10, S5-R1/S5-R7) replaces that with a single "as of" date control - one calendar day, defaulting to today and capped at today - because a stock valuation is a point-in-time position, not an amount over a period. Follow the current specification.
+---
+This is the expected behaviour as per epic SV-8582, read on 17 August 2026, and the Inventory Value report specification version 10 (S1-R3, S7-R2), read on 17 August 2026.
 AUTOMATION: READY - EXPECT FAIL (SV-8931)</t>
         </is>
       </c>
       <c r="H4" s="2" t="inlineStr">
         <is>
-          <t>SV-8668 (IV spec v3 2026-07-29 Story 1 S1-R3; Story 7 S7-R2)</t>
+          <t>SV-8668 (IV spec v10 2026-08-17 Story 1 S1-R3; Story 7 S7-R2)</t>
         </is>
       </c>
       <c r="I4" s="2" t="inlineStr"/>
@@ -687,14 +685,13 @@
 2. Changing any server-side filter (Date, Location, Category, Vendor), the part search, or the sort returns the FIRST page of the new result set - the list jumps back to the top.
 3. Note for the tester: on the build tested there were no numbered page controls on the screen - the rows loaded as you scrolled. That is a difference from the specification, which asks for the reports suite's standard page controls. Record what you see and carry on.
 ---
-This is the expected behaviour as per epic SV-8582, read on 11 August 2026, and the Inventory Value report specification version 5 (S1-R8), read on 11 August 2026.
-Last checked against build v3.5-16cf83f on 8/6/2026.
-AUTOMATION: READY</t>
+This is the expected behaviour as per epic SV-8582, read on 17 August 2026, and the Inventory Value report specification version 10 (S1-R8), read on 17 August 2026.
+AUTOMATION: Not available on Build to test Yet - Last checked 8/17/2026</t>
         </is>
       </c>
       <c r="H5" s="2" t="inlineStr">
         <is>
-          <t>SV-8668 (IV spec v3 2026-07-29 Story 1 S1-R8; §2 Scale and data model)</t>
+          <t>SV-8668 (IV spec v10 2026-08-17 Story 1 S1-R8; §2 Scale and data model)</t>
         </is>
       </c>
       <c r="I5" s="2" t="inlineStr"/>
@@ -730,7 +727,7 @@
       <c r="F6" s="2" t="inlineStr">
         <is>
           <t>1. Scope the report to the empty location and read the data area.
-2. Select a Custom range ending before nightly recording began and read the data area and the bottom of the report.
+2. Set the "as of" date to a day before nightly recording began and read the data area and the bottom of the report.
 3. Set the filters so nothing qualifies and re-read.</t>
         </is>
       </c>
@@ -743,14 +740,13 @@
 - If it fails in a DIFFERENT way from what is described above, that is a NEW problem - please report it.
 - If it PASSES, the fix has shipped: tell the QA lead so the ticket can be closed and this note removed.
 ---
-This is the expected behaviour as per epic SV-8582, read on 11 August 2026, and the Inventory Value report specification version 5 (S1-N2, S4-N1, S5-N1, S7-N2), read on 11 August 2026.
-Last checked against build v3.5-16cf83f on 8/6/2026.
+This is the expected behaviour as per epic SV-8582, read on 17 August 2026, and the Inventory Value report specification version 10 (S1-N2, S4-N1, S5-N1, S7-N2), read on 17 August 2026.
 AUTOMATION: READY - EXPECT FAIL (SV-8930)</t>
         </is>
       </c>
       <c r="H6" s="2" t="inlineStr">
         <is>
-          <t>SV-8668 (IV spec v3 2026-07-29 Story 1 S1-N2; Story 4 S4-N1; Story 5 S5-N1; Story 7 S7-N2; Story 12; §7 User Feedback Summary)</t>
+          <t>SV-8668 (IV spec v10 2026-08-17 Story 1 S1-N2; Story 4 S4-N1; Story 5 S5-N1; Story 7 S7-N2; Story 12; §7 User Feedback Summary)</t>
         </is>
       </c>
       <c r="I6" s="2" t="inlineStr"/>
@@ -798,14 +794,13 @@
 4. Only parts meeting BOTH conditions — not a core charge, and on-hand quantity greater than zero — are listed.
 5. A part that has sat without movement for a long time still appears and is still counted — there is no dead-stock exclusion; how long stock has sat makes no difference.
 ---
-This is the expected behaviour as per epic SV-8582, read on 11 August 2026, and the Inventory Value report specification version 5 (S2-R1, S2-R2, S2-N1, S2-N2), read on 11 August 2026.
-Last checked against build v3.5-16cf83f on 8/6/2026.
-AUTOMATION: READY</t>
+This is the expected behaviour as per epic SV-8582, read on 17 August 2026, and the Inventory Value report specification version 10 (S2-R1, S2-R2, S2-N1, S2-N2), read on 17 August 2026.
+AUTOMATION: Not available on Build to test Yet - Last checked 8/17/2026</t>
         </is>
       </c>
       <c r="H7" s="2" t="inlineStr">
         <is>
-          <t>SV-8669 (IV spec v3 2026-07-29 Story 2 S2-R1; S2-R2; S2-N1; S2-N2; §3 Key Decisions; Story 2 context note (no dead-stock exclusion))</t>
+          <t>SV-8669 (IV spec v10 2026-08-17 Story 2 S2-R1; S2-R2; S2-N1; S2-N2; §3 Key Decisions; Story 2 context note (no dead-stock exclusion))</t>
         </is>
       </c>
       <c r="I7" s="2" t="inlineStr"/>
@@ -849,14 +844,13 @@
           <t>1. The part appears twice — one row per location, each with that location's own quantity and values.
 2. The rows are NOT merged into one combined row; this is the documented v1 behavior.
 ---
-This is the expected behaviour as per epic SV-8582, read on 11 August 2026, and the Inventory Value report specification version 5 (S2-R3), read on 11 August 2026.
-Last checked against build v3.5-16cf83f on 8/6/2026.
-AUTOMATION: READY</t>
+This is the expected behaviour as per epic SV-8582, read on 17 August 2026, and the Inventory Value report specification version 10 (S2-R3), read on 17 August 2026.
+AUTOMATION: Not available on Build to test Yet - Last checked 8/17/2026</t>
         </is>
       </c>
       <c r="H8" s="2" t="inlineStr">
         <is>
-          <t>SV-8669 (IV spec v3 2026-07-29 Story 2 S2-R3; §2 Known Limitations (v1))</t>
+          <t>SV-8669 (IV spec v10 2026-08-17 Story 2 S2-R3; §2 Known Limitations (v1))</t>
         </is>
       </c>
       <c r="I8" s="2" t="inlineStr"/>
@@ -901,14 +895,13 @@
           <t>1. Unit Sell equals the part's fixed sell price.
 2. The pricing-matrix markup is NOT applied when a fixed sell price is set — the fixed price wins.
 ---
-This is the expected behaviour as per epic SV-8582, read on 11 August 2026, and the Inventory Value report specification version 5 (S3-R5), read on 11 August 2026.
-Last checked against build v3.5-16cf83f on 8/6/2026.
-AUTOMATION: READY</t>
+This is the expected behaviour as per epic SV-8582, read on 17 August 2026, and the Inventory Value report specification version 10 (S3-R5), read on 17 August 2026.
+AUTOMATION: Not available on Build to test Yet - Last checked 8/17/2026</t>
         </is>
       </c>
       <c r="H9" s="2" t="inlineStr">
         <is>
-          <t>SV-8670 (IV spec v3 2026-07-29 Story 3 S3-R5 (fixed-price branch); §3 Key Decisions (unit sell resolved like the parts list))</t>
+          <t>SV-8670 (IV spec v10 2026-08-17 Story 3 S3-R5 (fixed-price branch); §3 Key Decisions (unit sell resolved like the parts list))</t>
         </is>
       </c>
       <c r="I9" s="2" t="inlineStr"/>
@@ -952,14 +945,13 @@
         <is>
           <t>1. Unit Sell equals the shop's pricing-matrix markup on cost for that part's category (the same way the parts list resolves it).
 ---
-This is the expected behaviour as per epic SV-8582, read on 11 August 2026, and the Inventory Value report specification version 5 (S3-R5), read on 11 August 2026.
-Last checked against build v3.5-16cf83f on 8/6/2026.
-AUTOMATION: READY</t>
+This is the expected behaviour as per epic SV-8582, read on 17 August 2026, and the Inventory Value report specification version 10 (S3-R5), read on 17 August 2026.
+AUTOMATION: Not available on Build to test Yet - Last checked 8/17/2026</t>
         </is>
       </c>
       <c r="H10" s="2" t="inlineStr">
         <is>
-          <t>SV-8670 (IV spec v3 2026-07-29 Story 3 S3-R5 (matrix branch); §5 Assumptions)</t>
+          <t>SV-8670 (IV spec v10 2026-08-17 Story 3 S3-R5 (matrix branch); §5 Assumptions)</t>
         </is>
       </c>
       <c r="I10" s="2" t="inlineStr"/>
@@ -1007,14 +999,14 @@
 2. Such a part shows a Margin of $0.00 and a Margin % of 0.0% — the stock is valued at cost.
 3. Note for the tester: if no part without a category can be created or found, mark this test Blocked rather than Passed or Failed.
 ---
-This is the expected behaviour as per epic SV-8582, read on 11 August 2026, and the Inventory Value report specification version 5 (S3-R5), read on 11 August 2026.
+This is the expected behaviour as per epic SV-8582, read on 17 August 2026, and the Inventory Value report specification version 10 (S3-R5), read on 17 August 2026.
 Last checked against build v3.5-16cf83f on 8/6/2026.
 AUTOMATION: HOLD - a part cannot be saved without a category on this build, so the no-category path cannot be produced</t>
         </is>
       </c>
       <c r="H11" s="2" t="inlineStr">
         <is>
-          <t>SV-8670 (IV spec v3 2026-07-29 Story 3 S3-R5 (no-category fallback) + context note; §5 Assumptions)</t>
+          <t>SV-8670 (IV spec v10 2026-08-17 Story 3 S3-R5 (no-category fallback) + context note; §5 Assumptions)</t>
         </is>
       </c>
       <c r="I11" s="2" t="inlineStr"/>
@@ -1060,14 +1052,13 @@
           <t>1. Total Sell equals the part's on-hand quantity × Unit Sell, shown as US-dollar currency.
 2. Total Cost equals the part's on-hand quantity × Unit Cost, shown as US-dollar currency.
 ---
-This is the expected behaviour as per epic SV-8582, read on 11 August 2026, and the Inventory Value report specification version 5 (S3-R6, S3-R7), read on 11 August 2026.
-Last checked against build v3.5-16cf83f on 8/6/2026.
-AUTOMATION: READY</t>
+This is the expected behaviour as per epic SV-8582, read on 17 August 2026, and the Inventory Value report specification version 10 (S3-R6, S3-R7), read on 17 August 2026.
+AUTOMATION: Not available on Build to test Yet - Last checked 8/17/2026</t>
         </is>
       </c>
       <c r="H12" s="2" t="inlineStr">
         <is>
-          <t>SV-8670 (IV spec v3 2026-07-29 Story 3 S3-R6; S3-R7; §4 Terminology)</t>
+          <t>SV-8670 (IV spec v10 2026-08-17 Story 3 S3-R6; S3-R7; §4 Terminology)</t>
         </is>
       </c>
       <c r="I12" s="2" t="inlineStr"/>
@@ -1113,14 +1104,13 @@
           <t>1. Margin equals Total Sell − Total Cost for the part's whole on-hand quantity, shown as US-dollar currency.
 2. Margin is the extended (total) margin, not the per-unit difference.
 ---
-This is the expected behaviour as per epic SV-8582, read on 11 August 2026, and the Inventory Value report specification version 5 (S3-R8), read on 11 August 2026.
-Last checked against build v3.5-16cf83f on 8/6/2026.
-AUTOMATION: READY</t>
+This is the expected behaviour as per epic SV-8582, read on 17 August 2026, and the Inventory Value report specification version 10 (S3-R8), read on 17 August 2026.
+AUTOMATION: Not available on Build to test Yet - Last checked 8/17/2026</t>
         </is>
       </c>
       <c r="H13" s="2" t="inlineStr">
         <is>
-          <t>SV-8670 (IV spec v3 2026-07-29 Story 3 S3-R8; §3 Key Decisions (extended margin); §4 Terminology)</t>
+          <t>SV-8670 (IV spec v10 2026-08-17 Story 3 S3-R8; §3 Key Decisions (extended margin); §4 Terminology)</t>
         </is>
       </c>
       <c r="I13" s="2" t="inlineStr"/>
@@ -1166,14 +1156,13 @@
 2. A Margin % that computes to a real number, including a negative one, shows its signed value.
 3. Margin % shows "—" when Total Sell is zero or negative (the percentage is undefined).
 ---
-This is the expected behaviour as per epic SV-8582, read on 11 August 2026, and the Inventory Value report specification version 5 (S3-R9, S3-E3), read on 11 August 2026.
-Last checked against build v3.5-16cf83f on 8/6/2026.
-AUTOMATION: READY</t>
+This is the expected behaviour as per epic SV-8582, read on 17 August 2026, and the Inventory Value report specification version 10 (S3-R9, S3-E3), read on 17 August 2026.
+AUTOMATION: Not available on Build to test Yet - Last checked 8/17/2026</t>
         </is>
       </c>
       <c r="H14" s="2" t="inlineStr">
         <is>
-          <t>SV-8670 (IV spec v3 2026-07-29 Story 3 S3-R9; S3-E3)</t>
+          <t>SV-8670 (IV spec v10 2026-08-17 Story 3 S3-R9; S3-E3)</t>
         </is>
       </c>
       <c r="I14" s="2" t="inlineStr"/>
@@ -1219,14 +1208,13 @@
 2. Part #, Description, Category, and Vendor are left-aligned.
 3. Every other column is right-aligned. When it is on, the Location column appears between Vendor and Qty, and it is right-aligned like the other non-identity columns.The question is in the round-3 question sheet: https://raw.githubusercontent.com/bilalmuzamil-sketch/Manual-test-Cases/claude/slack-session-0sxnd9/build/report-suite/rulings-2026-08-05/Questions-for-Chris-Ward_Report-Suite_Round-3_2026-08-05.xlsx
 ---
-This is the expected behaviour as per epic SV-8582, read on 11 August 2026, and the Inventory Value report specification version 5 (S3-R1, S3-R2, S7-R6), read on 11 August 2026.
-Last checked against build v3.5-16cf83f on 8/6/2026.
-AUTOMATION: READY</t>
+This is the expected behaviour as per epic SV-8582, read on 17 August 2026, and the Inventory Value report specification version 10 (S3-R1, S3-R2, S7-R6), read on 17 August 2026.
+AUTOMATION: Not available on Build to test Yet - Last checked 8/17/2026</t>
         </is>
       </c>
       <c r="H15" s="2" t="inlineStr">
         <is>
-          <t>SV-8670; SV-8674 (IV spec v3 2026-07-29 Story 3 S3-R1; S3-R2 + Story 7 S7-R6 — fixed column order and alignment; plus the automatic Location column between Vendor and Qty on Hand)</t>
+          <t>SV-8670; SV-8674 (IV spec v10 2026-08-17 Story 3 S3-R1; S3-R2 + Story 7 S7-R6 — fixed column order and alignment; plus the Location column between Vendor and Qty on Hand when it is shown)</t>
         </is>
       </c>
       <c r="I15" s="2" t="inlineStr"/>
@@ -1272,14 +1260,13 @@
 2. Unit Cost and Unit Sell show per-unit prices as US-dollar currency.
 3. Money values show a leading "$", two decimal places, and thousands separators (for example "$1,234.56"); a negative value shows a leading minus before the "$" ("-$1,234.56"); a genuine zero shows "$0.00".
 ---
-This is the expected behaviour as per epic SV-8582, read on 11 August 2026, and the Inventory Value report specification version 5 (S3-R3, S3-R4, S3-R5, S3-R10), read on 11 August 2026.
-Last checked against build v3.5-16cf83f on 8/6/2026.
-AUTOMATION: READY</t>
+This is the expected behaviour as per epic SV-8582, read on 17 August 2026, and the Inventory Value report specification version 10 (S3-R3, S3-R4, S3-R5, S3-R10), read on 17 August 2026.
+AUTOMATION: Not available on Build to test Yet - Last checked 8/17/2026</t>
         </is>
       </c>
       <c r="H16" s="2" t="inlineStr">
         <is>
-          <t>SV-8670 (IV spec v3 2026-07-29 Story 3 S3-R3; S3-R4; S3-R5 (display); S3-R10; §4 Terminology (On-hand quantity))</t>
+          <t>SV-8670 (IV spec v10 2026-08-17 Story 3 S3-R3; S3-R4; S3-R5 (display); S3-R10; §4 Terminology (On-hand quantity))</t>
         </is>
       </c>
       <c r="I16" s="2" t="inlineStr"/>
@@ -1324,14 +1311,13 @@
 2. The Total Cost column header is bold and pinned, matching its cells.
 3. It stays fixed to the right edge while the other columns scroll underneath.
 ---
-This is the expected behaviour as per epic SV-8582, read on 11 August 2026, and the Inventory Value report specification version 5 (S3-R11, S12-R4), read on 11 August 2026.
-Last checked against build v3.5-16cf83f on 8/6/2026.
-AUTOMATION: READY</t>
+This is the expected behaviour as per epic SV-8582, read on 17 August 2026, and the Inventory Value report specification version 10 (S3-R11, S12-R4), read on 17 August 2026.
+AUTOMATION: Not available on Build to test Yet - Last checked 8/17/2026</t>
         </is>
       </c>
       <c r="H17" s="2" t="inlineStr">
         <is>
-          <t>SV-8670 (IV spec v3 2026-07-29 Story 3 S3-R11; Story 12 S12-R4; §3 Key Decisions)</t>
+          <t>SV-8670 (IV spec v10 2026-08-17 Story 3 S3-R11; Story 12 S12-R4; §3 Key Decisions)</t>
         </is>
       </c>
       <c r="I17" s="2" t="inlineStr"/>
@@ -1377,14 +1363,13 @@
 3. Both can be turned on from the column-selection control and then appear in their fixed positions. When it is on, the Location column shows between Vendor and Qty.The question is in the round-3 question sheet: https://raw.githubusercontent.com/bilalmuzamil-sketch/Manual-test-Cases/claude/slack-session-0sxnd9/build/report-suite/rulings-2026-08-05/Questions-for-Chris-Ward_Report-Suite_Round-3_2026-08-05.xlsx
 Known issue: the product does not currently do this. It has been filed for a fix here: https://shopview.atlassian.net/browse/SV-8927
 ---
-This is the expected behaviour as per epic SV-8582, read on 11 August 2026, and the Inventory Value report specification version 5 (S3-R12, S3-R13, S8-R3, S7-R6), read on 11 August 2026.
-Last checked against build v3.5-16cf83f on 8/6/2026.
-AUTOMATION: READY</t>
+This is the expected behaviour as per epic SV-8582, read on 17 August 2026, and the Inventory Value report specification version 10 (S3-R12, S3-R13, S8-R3, S7-R6), read on 17 August 2026.
+AUTOMATION: Not available on Build to test Yet - Last checked 8/17/2026</t>
         </is>
       </c>
       <c r="H18" s="2" t="inlineStr">
         <is>
-          <t>SV-8670; SV-8674 (IV spec v3 2026-07-29 Story 3 S3-R12; S3-R13; Story 8 S8-R3 + Story 7 S7-R6 — first-visit default columns; plus the automatic Location column when more than one location is in scope)</t>
+          <t>SV-8670; SV-8674 (IV spec v10 2026-08-17 Story 3 S3-R12; S3-R13; Story 8 S8-R3 + Story 7 S7-R6 — first-visit default columns; plus the Location column shown by default to a user with access to more than one location)</t>
         </is>
       </c>
       <c r="I18" s="2" t="inlineStr"/>
@@ -1431,14 +1416,13 @@
 3. A part with no vendor shows an em dash ("—") in its Vendor cell.
 4. Note for the tester: on this build a part cannot be saved without a category, so you will not find a part whose Category cell shows "—". Check the Vendor half only.
 ---
-This is the expected behaviour as per epic SV-8582, read on 11 August 2026, and the Inventory Value report specification version 5 (S3-R14, S3-E1, S3-E2), read on 11 August 2026.
-Last checked against build v3.5-16cf83f on 8/6/2026.
-AUTOMATION: READY</t>
+This is the expected behaviour as per epic SV-8582, read on 17 August 2026, and the Inventory Value report specification version 10 (S3-R14, S3-E1, S3-E2), read on 17 August 2026.
+AUTOMATION: Not available on Build to test Yet - Last checked 8/17/2026</t>
         </is>
       </c>
       <c r="H19" s="2" t="inlineStr">
         <is>
-          <t>SV-8670 (IV spec v3 2026-07-29 Story 3 S3-R14; S3-E1; S3-E2)</t>
+          <t>SV-8670 (IV spec v10 2026-08-17 Story 3 S3-R14; S3-E1; S3-E2)</t>
         </is>
       </c>
       <c r="I19" s="2" t="inlineStr"/>
@@ -1493,14 +1477,14 @@
 - If it fails in a DIFFERENT way from what is described above, that is a NEW problem - please report it.
 - If it PASSES, the fix has shipped: tell the QA lead so the ticket can be closed and this note removed.
 ---
-This is the expected behaviour as per epic SV-8582, read on 11 August 2026, and the Inventory Value report specification version 5 (S4-R1, S4-R4, S4-R5, S4-R6, S4-R7, S12-R5, S9-R4), read on 11 August 2026.
+This is the expected behaviour as per epic SV-8582, read on 17 August 2026, and the Inventory Value report specification version 10 (S4-R1, S4-R4, S4-R5, S4-R6, S4-R7, S12-R5, S9-R4), read on 17 August 2026.
 Last checked against build v3.5-16cf83f on 8/6/2026.
 AUTOMATION: READY - EXPECT FAIL (SV-8926)</t>
         </is>
       </c>
       <c r="H20" s="2" t="inlineStr">
         <is>
-          <t>SV-8671 (IV spec v3 2026-07-29 Story 4 S4-R1; S4-R4; S4-R5; S4-R6; S4-R7; Story 12 S12-R5; Story 9 S9-R4)</t>
+          <t>SV-8671 (IV spec v10 2026-08-17 Story 4 S4-R1; S4-R4; S4-R5; S4-R6; S4-R7; Story 12 S12-R5; Story 9 S9-R4)</t>
         </is>
       </c>
       <c r="I20" s="2" t="inlineStr"/>
@@ -1550,14 +1534,13 @@
 3. The hand-summed subset matches the server-computed totals to the cent.
 4. After each filter change the totals row recomputes on the server over the full filtered set, independent of which page is shown.
 ---
-This is the expected behaviour as per epic SV-8582, read on 11 August 2026, and the Inventory Value report specification version 5 (S4-R2, S4-R8, S6-R6), read on 11 August 2026.
-Last checked against build v3.5-16cf83f on 8/6/2026.
-AUTOMATION: READY</t>
+This is the expected behaviour as per epic SV-8582, read on 17 August 2026, and the Inventory Value report specification version 10 (S4-R2, S4-R8, S6-R6), read on 17 August 2026.
+AUTOMATION: Not available on Build to test Yet - Last checked 8/17/2026</t>
         </is>
       </c>
       <c r="H21" s="2" t="inlineStr">
         <is>
-          <t>SV-8671 (IV spec v3 2026-07-29 Story 4 S4-R2; S4-R8; Story 6 S6-R6; §2 Scale and data model; §4 Terminology (Filtered set))</t>
+          <t>SV-8671 (IV spec v10 2026-08-17 Story 4 S4-R2; S4-R8; Story 6 S6-R6; §2 Scale and data model; §4 Terminology (Filtered set))</t>
         </is>
       </c>
       <c r="I21" s="2" t="inlineStr"/>
@@ -1604,14 +1587,13 @@
 2. It is NOT the average of the row percentages.
 3. It shows "—" when the total Total Sell is zero or negative.
 ---
-This is the expected behaviour as per epic SV-8582, read on 11 August 2026, and the Inventory Value report specification version 5 (S4-R3), read on 11 August 2026.
-Last checked against build v3.5-16cf83f on 8/6/2026.
-AUTOMATION: READY</t>
+This is the expected behaviour as per epic SV-8582, read on 17 August 2026, and the Inventory Value report specification version 10 (S4-R3), read on 17 August 2026.
+AUTOMATION: Not available on Build to test Yet - Last checked 8/17/2026</t>
         </is>
       </c>
       <c r="H22" s="2" t="inlineStr">
         <is>
-          <t>SV-8671 (IV spec v3 2026-07-29 Story 4 S4-R3)</t>
+          <t>SV-8671 (IV spec v10 2026-08-17 Story 4 S4-R3)</t>
         </is>
       </c>
       <c r="I22" s="2" t="inlineStr"/>
@@ -1620,7 +1602,7 @@
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
         <is>
-          <t>Date range offers the standard presets plus Custom; no All Time option</t>
+          <t>"As of" date control: a single day, defaults to today, capped at today</t>
         </is>
       </c>
       <c r="B23" s="2" t="inlineStr">
@@ -1646,23 +1628,23 @@
       </c>
       <c r="F23" s="2" t="inlineStr">
         <is>
-          <t>1. Open the date-range control in the toolbar.
-2. Read every option offered.</t>
+          <t>1. Open the "as of" date control in the toolbar.
+2. Read what it offers.</t>
         </is>
       </c>
       <c r="G23" s="2" t="inlineStr">
         <is>
-          <t>1. The chooser offers nine ready-made periods, in this order: Last 12 Months, This Year, Last Year, This Quarter, Last Quarter, This Month, Last Month, This Week, Last Week. Beside them it shows a month calendar you click dates on to build your own range, a live readout of how many days the range covers, and an Apply button. There is no "Today", no "Yesterday" and no item called "Custom" - you build your own range on the calendar instead. There is no "All Time" option.
-2. Because the report is valued as of a single date, an All-Time period would be meaningless; its absence is the documented behaviour.
----
-This is the expected behaviour as per epic SV-8582, read on 11 August 2026, and Chris Ward's decision of 8/5/2026, recorded in his answers in this file: https://docs.google.com/spreadsheets/d/1x8cuYJlFsDHalVZZTh156_ZCq2gcOaGY/edit?usp=sharing&amp;ouid=106388879401921597782&amp;rtpof=true&amp;sd=true, read on 11 August 2026. Where the Inventory Value report specification version 5 (S5-R1), read on 11 August 2026, says something different, his decision is the later word and is the authority.
-Last checked against build v3.5-16cf83f on 8/6/2026.
-AUTOMATION: READY</t>
+          <t>1. The toolbar has a single "as of" date control - one calendar day, not a range. It defaults to today and is capped at today (no future date). It offers no ready-made periods (no "Last 12 Months", no "This Month", no "This Week" and so on), no start-and-end pair, no item called "Custom", and no "All Time". You pick one day.
+2. Because the report values stock as of a single point in time, a date range or an All-Time period would state something the number cannot mean; a single "as of" day is the documented behaviour.
+Note for the tester: an earlier version of this report offered a date range with ready-made periods. The current Inventory Value report specification (version 10, S5-R1/S5-R7) replaces that with a single "as of" date control - one calendar day, defaulting to today and capped at today - because a stock valuation is a point-in-time position, not an amount over a period. Follow the current specification.
+---
+This is the expected behaviour as per epic SV-8582, read on 17 August 2026, and Chris Ward's decision of 8/5/2026, recorded in his answers in this file: https://docs.google.com/spreadsheets/d/1x8cuYJlFsDHalVZZTh156_ZCq2gcOaGY/edit?usp=sharing&amp;ouid=106388879401921597782&amp;rtpof=true&amp;sd=true, read on 17 August 2026. Where the Inventory Value report specification version 10 (S5-R1), read on 17 August 2026, says something different, his decision is the later word and is the authority.
+AUTOMATION: Not available on Build to test Yet - Last checked 8/17/2026</t>
         </is>
       </c>
       <c r="H23" s="2" t="inlineStr">
         <is>
-          <t>SV-8672 (IV spec v3 2026-07-29 Story 5 S5-R1; §2 Known Limitations (v1))</t>
+          <t>SV-8672 (IV spec v10 2026-08-17 Story 5 S5-R1; §2 Known Limitations (v1))</t>
         </is>
       </c>
       <c r="I23" s="2" t="inlineStr"/>
@@ -1712,14 +1694,14 @@
 - If it fails in a DIFFERENT way from what is described above, that is a NEW problem - please report it.
 - If it PASSES, the fix has shipped: tell the QA lead so the ticket can be closed and this note removed.
 ---
-This is the expected behaviour as per epic SV-8582, read on 11 August 2026, and the Inventory Value report specification version 5 (S5-R2), read on 11 August 2026.
+This is the expected behaviour as per epic SV-8582, read on 17 August 2026, and the Inventory Value report specification version 10 (S5-R2), read on 17 August 2026.
 Last checked against build v3.5-16cf83f on 8/6/2026.
 AUTOMATION: READY - EXPECT FAIL (SV-8820)</t>
         </is>
       </c>
       <c r="H24" s="2" t="inlineStr">
         <is>
-          <t>SV-8672 (IV spec v3 2026-07-29 Story 5 S5-R2 (+ context note))</t>
+          <t>SV-8672 (IV spec v10 2026-08-17 Story 5 S5-R2 (+ context note))</t>
         </is>
       </c>
       <c r="I24" s="2" t="inlineStr"/>
@@ -1728,7 +1710,7 @@
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
         <is>
-          <t>A window reaching today with today not yet recorded values live stock</t>
+          <t>The "as of" date today, with today not yet recorded, values live stock</t>
         </is>
       </c>
       <c r="B25" s="2" t="inlineStr">
@@ -1755,7 +1737,7 @@
       </c>
       <c r="F25" s="2" t="inlineStr">
         <is>
-          <t>1. Select a range that reaches today (for example "This Month" or "Today").
+          <t>1. Set the "as of" date to today.
 2. Find the part whose quantity changed today and read its row.</t>
         </is>
       </c>
@@ -1763,15 +1745,15 @@
         <is>
           <t>1. The report values the current live stock — the values represent today.
 2. The part's row reflects today's changed quantity (not yesterday's snapshot), proving the live fallback is in use.
----
-This is the expected behaviour as per epic SV-8582, read on 11 August 2026, and the Inventory Value report specification version 5 (S5-R3), read on 11 August 2026.
-Last checked against build v3.5-16cf83f on 8/6/2026.
-AUTOMATION: READY</t>
+Note for the tester: an earlier version of this report offered a date range with ready-made periods. The current Inventory Value report specification (version 10, S5-R1/S5-R7) replaces that with a single "as of" date control - one calendar day, defaulting to today and capped at today - because a stock valuation is a point-in-time position, not an amount over a period. Follow the current specification.
+---
+This is the expected behaviour as per epic SV-8582, read on 17 August 2026, and the Inventory Value report specification version 10 (S5-R3), read on 17 August 2026.
+AUTOMATION: Not available on Build to test Yet - Last checked 8/17/2026</t>
         </is>
       </c>
       <c r="H25" s="2" t="inlineStr">
         <is>
-          <t>SV-8672 (IV spec v3 2026-07-29 Story 5 S5-R3; §3 Key Decisions (live fallback for today))</t>
+          <t>SV-8672 (IV spec v10 2026-08-17 Story 5 S5-R3; §3 Key Decisions (live fallback for today))</t>
         </is>
       </c>
       <c r="I25" s="2" t="inlineStr"/>
@@ -1806,28 +1788,28 @@
       </c>
       <c r="F26" s="2" t="inlineStr">
         <is>
-          <t>1. Open the date range picker and use the month calendar inside it to set a range ending on the past recorded day, then apply.
+          <t>1. Set the "as of" date to the past recorded day.
 2. Find the part and read its quantity and values.
 3. Compare them to what the part held on that recorded day (not today).</t>
         </is>
       </c>
       <c r="G26" s="2" t="inlineStr">
         <is>
-          <t>1. The report replays the closest recorded day on or before the end of the selected range.
+          <t>1. The report replays the closest recorded day on or before the selected "as of" date.
 2. The part's row shows the quantity and values recorded for that day, not today's live stock.
-What you should see today: the report values the stock one day LATER than the date you asked for - ask for a range ending 15 July and it reports as of 16 July; ask for one ending 31 January and it reports as of 1 February. This is a known problem and it is already reported - see https://shopview.atlassian.net/browse/SV-8820
+What you should see today: the report values the stock one day LATER than the date you asked for - ask for an "as of" date of 15 July and it reports as of 16 July; ask for 31 January and it reports as of 1 February. This is a known problem and it is already reported - see https://shopview.atlassian.net/browse/SV-8820
 - If you see exactly that, mark this test FAILED and do not raise anything new.
 - If it fails in a DIFFERENT way from what is described above, that is a NEW problem - please report it.
 - If it PASSES, the fix has shipped: tell the QA lead so the ticket can be closed and this note removed.
----
-This is the expected behaviour as per epic SV-8582, read on 11 August 2026, and the Inventory Value report specification version 5 (S5-R4), read on 11 August 2026.
-Last checked against build v3.5-16cf83f on 8/6/2026.
+Note for the tester: an earlier version of this report offered a date range with ready-made periods. The current Inventory Value report specification (version 10, S5-R1/S5-R7) replaces that with a single "as of" date control - one calendar day, defaulting to today and capped at today - because a stock valuation is a point-in-time position, not an amount over a period. Follow the current specification.
+---
+This is the expected behaviour as per epic SV-8582, read on 17 August 2026, and the Inventory Value report specification version 10 (S5-R4), read on 17 August 2026.
 AUTOMATION: READY - EXPECT FAIL (SV-8820)</t>
         </is>
       </c>
       <c r="H26" s="2" t="inlineStr">
         <is>
-          <t>SV-8672 (IV spec v3 2026-07-29 Story 5 S5-R4; §2 Relationship to nightly history)</t>
+          <t>SV-8672 (IV spec v10 2026-08-17 Story 5 S5-R4; §2 Relationship to nightly history)</t>
         </is>
       </c>
       <c r="I26" s="2" t="inlineStr"/>
@@ -1836,7 +1818,7 @@
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
         <is>
-          <t>"As of" indicator names the day shown; hidden when it matches the ask</t>
+          <t>The date control names the resolved day; no separate "As of" indicator</t>
         </is>
       </c>
       <c r="B27" s="2" t="inlineStr">
@@ -1862,28 +1844,28 @@
       </c>
       <c r="F27" s="2" t="inlineStr">
         <is>
-          <t>1. Select a Custom range ending on the gap date (a date with no snapshot of its own).
+          <t>1. Set the "as of" date to the gap date (a date with no snapshot of its own).
 2. Look for an "As of" indicator and read which day it names.
 3. Then select a range ending on a day that IS recorded (or today with live values) and look for the indicator again.</t>
         </is>
       </c>
       <c r="G27" s="2" t="inlineStr">
         <is>
-          <t>1. When the displayed day is an earlier recorded day than the date asked for, the report shows an "As of" indicator naming the day actually shown.
-2. When the displayed day matches the date asked for (the common current-view case), the "As of" indicator is not shown — the date control already communicates the date.
-What you should see today: the report values the stock one day LATER than the date you asked for - ask for a range ending 15 July and it reports as of 16 July; ask for one ending 31 January and it reports as of 1 February. This is a known problem and it is already reported - see https://shopview.atlassian.net/browse/SV-8820
+          <t>1. When the displayed day is an earlier recorded day than the date you asked for, the "as of" date control itself names the day actually shown - the requested date on its face, and beneath it, inside the same control, the resolved day worded "As of {date}". There is no separate "As of" indicator anywhere else on the page.
+2. When the displayed day matches the date you asked for (the common current-view case), the control shows only the selected date, with no "As of" line beneath it.
+What you should see today: the report values the stock one day LATER than the date you asked for - ask for an "as of" date of 15 July and it reports as of 16 July; ask for 31 January and it reports as of 1 February. This is a known problem and it is already reported - see https://shopview.atlassian.net/browse/SV-8820
 - If you see exactly that, mark this test FAILED and do not raise anything new.
 - If it fails in a DIFFERENT way from what is described above, that is a NEW problem - please report it.
 - If it PASSES, the fix has shipped: tell the QA lead so the ticket can be closed and this note removed.
----
-This is the expected behaviour as per epic SV-8582, read on 11 August 2026, and the Inventory Value report specification version 5 (S5-R5, S5-R6), read on 11 August 2026.
-Last checked against build v3.5-16cf83f on 8/6/2026.
+Note for the tester: an earlier version of this report offered a date range with ready-made periods. The current Inventory Value report specification (version 10, S5-R1/S5-R7) replaces that with a single "as of" date control - one calendar day, defaulting to today and capped at today - because a stock valuation is a point-in-time position, not an amount over a period. Follow the current specification.
+---
+This is the expected behaviour as per epic SV-8582, read on 17 August 2026, and the Inventory Value report specification version 10 (S5-R5, S5-R6), read on 17 August 2026.
 AUTOMATION: READY - EXPECT FAIL (SV-8820)</t>
         </is>
       </c>
       <c r="H27" s="2" t="inlineStr">
         <is>
-          <t>SV-8672 (IV spec v3 2026-07-29 Story 5 S5-R5; S5-R6)</t>
+          <t>SV-8672 (IV spec v10 2026-08-17 Story 5 S5-R5; S5-R6)</t>
         </is>
       </c>
       <c r="I27" s="2" t="inlineStr"/>
@@ -1892,7 +1874,7 @@
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
         <is>
-          <t>A Custom range values stock as of the picked end date; capped at today</t>
+          <t>The "as of" date values stock as of that day; capped at today</t>
         </is>
       </c>
       <c r="B28" s="2" t="inlineStr">
@@ -1918,7 +1900,7 @@
       </c>
       <c r="F28" s="2" t="inlineStr">
         <is>
-          <t>1. Open the date-range control - a month calendar is shown inside it (there is no separate "Custom" item to choose).
+          <t>1. Open the "as of" date control - a single-day calendar (there is no start/end range and no "Custom" item).
 2. Pick a start and an end date in the past on that calendar and press Apply.
 3. Try to pick an end date in the future.
 4. Watch the data area when the range is applied.</t>
@@ -1926,22 +1908,22 @@
       </c>
       <c r="G28" s="2" t="inlineStr">
         <is>
-          <t>1. A Custom range lets the user pick a start and end date, and the report values as of the picked end date.
-2. A future end date cannot be chosen — the end date is capped at today.
-3. Changing the date range reloads the report (the loading indicator shows and the rows re-fetch).
-What you should see today: the report values the stock one day LATER than the date you asked for - ask for a range ending 15 July and it reports as of 16 July; ask for one ending 31 January and it reports as of 1 February. This is a known problem and it is already reported - see https://shopview.atlassian.net/browse/SV-8820
+          <t>1. The "as of" date control lets you pick one calendar day, and the report values stock as of that day.
+2. A future day cannot be chosen — the "as of" date is capped at today.
+3. Changing the "as of" date reloads the report (the loading indicator shows and the rows re-fetch).
+What you should see today: the report values the stock one day LATER than the date you asked for - ask for an "as of" date of 15 July and it reports as of 16 July; ask for 31 January and it reports as of 1 February. This is a known problem and it is already reported - see https://shopview.atlassian.net/browse/SV-8820
 - If you see exactly that, mark this test FAILED and do not raise anything new.
 - If it fails in a DIFFERENT way from what is described above, that is a NEW problem - please report it.
 - If it PASSES, the fix has shipped: tell the QA lead so the ticket can be closed and this note removed.
----
-This is the expected behaviour as per epic SV-8582, read on 11 August 2026, and the Inventory Value report specification version 5 (S5-R7, S5-R8), read on 11 August 2026.
-Last checked against build v3.5-16cf83f on 8/6/2026.
+Note for the tester: an earlier version of this report offered a date range with ready-made periods. The current Inventory Value report specification (version 10, S5-R1/S5-R7) replaces that with a single "as of" date control - one calendar day, defaulting to today and capped at today - because a stock valuation is a point-in-time position, not an amount over a period. Follow the current specification.
+---
+This is the expected behaviour as per epic SV-8582, read on 17 August 2026, and the Inventory Value report specification version 10 (S5-R7, S5-R8), read on 17 August 2026.
 AUTOMATION: READY - EXPECT FAIL (SV-8820)</t>
         </is>
       </c>
       <c r="H28" s="2" t="inlineStr">
         <is>
-          <t>SV-8672 (IV spec v3 2026-07-29 Story 5 S5-R7; S5-R8)</t>
+          <t>SV-8672 (IV spec v10 2026-08-17 Story 5 S5-R7; S5-R8)</t>
         </is>
       </c>
       <c r="I28" s="2" t="inlineStr"/>
@@ -1985,14 +1967,13 @@
           <t>1. The report shows the empty state — there is no way to reconstruct inventory value for a date before recording began, because there is no historical backfill.
 2. This forward-capture-only behavior is the documented v1 boundary, not a defect.
 ---
-This is the expected behaviour as per epic SV-8582, read on 11 August 2026, and the Inventory Value report specification version 5 (S5-E1), read on 11 August 2026.
-Last checked against build v3.5-16cf83f on 8/6/2026.
-AUTOMATION: READY</t>
+This is the expected behaviour as per epic SV-8582, read on 17 August 2026, and the Inventory Value report specification version 10 (S5-E1), read on 17 August 2026.
+AUTOMATION: Not available on Build to test Yet - Last checked 8/17/2026</t>
         </is>
       </c>
       <c r="H29" s="2" t="inlineStr">
         <is>
-          <t>SV-8672 (IV spec v3 2026-07-29 Story 5 S5-E1; §2 Known Limitations (v1); §2 Out of scope)</t>
+          <t>SV-8672 (IV spec v10 2026-08-17 Story 5 S5-E1; §2 Known Limitations (v1); §2 Out of scope)</t>
         </is>
       </c>
       <c r="I29" s="2" t="inlineStr"/>
@@ -2028,7 +2009,7 @@
       <c r="F30" s="2" t="inlineStr">
         <is>
           <t>1. Rename that part category (and/or rename or delete the vendor) in administration.
-2. Set the report's date range so it shows the earlier recorded day (the "As of" indicator names that earlier date).
+2. Set the report's "as of" date to the earlier recorded day (the date control names that earlier date).
 3. Read the affected rows' Category and Vendor cells on the recorded day.
 4. Move the range back to include today (live view) and re-read a renamed category's rows.</t>
         </is>
@@ -2039,14 +2020,13 @@
 2. The rename/delete causes no blank Category/Vendor cells and no dropped rows on the recorded day.
 3. The live view (window reaching today) shows the NEW name for the renamed category.
 ---
-This is the expected behaviour as per epic SV-8582, read on 11 August 2026, and the Inventory Value report specification version 5 (S11-R2, S5-R4), read on 11 August 2026.
-Last checked against build v3.5-16cf83f on 8/6/2026.
+This is the expected behaviour as per epic SV-8582, read on 17 August 2026, and the Inventory Value report specification version 10 (S11-R2, S5-R4), read on 17 August 2026.
 AUTOMATION: HOLD - needs a recorded earlier day plus the stored capture rows, which are not reachable from the application</t>
         </is>
       </c>
       <c r="H30" s="2" t="inlineStr">
         <is>
-          <t>SV-8678 (IV spec v3 2026-07-29 Story 11 S11-R2; Story 5 S5-R4; tech-plan-2026-07-29 B4.1 — names stored with the recorded rows on purpose)</t>
+          <t>SV-8678 (IV spec v10 2026-08-17 Story 11 S11-R2; Story 5 S5-R4; tech-plan-2026-07-29 B4.1 — names stored with the recorded rows on purpose)</t>
         </is>
       </c>
       <c r="I30" s="2" t="inlineStr"/>
@@ -2092,14 +2072,13 @@
 2. Selecting one or more categories reloads the report to show only parts in the selected categories.
 3. Selecting one or more vendors reloads the report to show only parts supplied by the selected vendors.
 ---
-This is the expected behaviour as per epic SV-8582, read on 11 August 2026, and the Inventory Value report specification version 5 (S6-R1, S6-R2, S6-R3, S6-R4), read on 11 August 2026.
-Last checked against build v3.5-16cf83f on 8/6/2026.
-AUTOMATION: READY</t>
+This is the expected behaviour as per epic SV-8582, read on 17 August 2026, and the Inventory Value report specification version 10 (S6-R1, S6-R2, S6-R3, S6-R4), read on 17 August 2026.
+AUTOMATION: Not available on Build to test Yet - Last checked 8/17/2026</t>
         </is>
       </c>
       <c r="H31" s="2" t="inlineStr">
         <is>
-          <t>SV-8673 (IV spec v3 2026-07-29 Story 6 S6-R1; S6-R2; S6-R3; S6-R4)</t>
+          <t>SV-8673 (IV spec v10 2026-08-17 Story 6 S6-R1; S6-R2; S6-R3; S6-R4)</t>
         </is>
       </c>
       <c r="I31" s="2" t="inlineStr"/>
@@ -2144,16 +2123,15 @@
         <is>
           <t>1. Each change re-queries the server and the list jumps back to the top of the new set of rows.
 2. The filtering covers the ENTIRE data set — matching parts that were further down the list appear — not just a narrowing of the rows currently on screen.
-3. Every change — date range, location, Category, Vendor, part search, sort — reloads the rows from the server; while loading the standard reports loading indicator shows, and existing rows are replaced only when the new data returns.
----
-This is the expected behaviour as per epic SV-8582, read on 11 August 2026, and the Inventory Value report specification version 5 (S6-R5, S1-R4, S1-R5, S1-R7, S1-R8), read on 11 August 2026.
-Last checked against build v3.5-16cf83f on 8/6/2026.
-AUTOMATION: READY</t>
+3. Every change — the "as of" date, location, Category, Vendor, part search, sort — reloads the rows from the server; while loading the standard reports loading indicator shows, and existing rows are replaced only when the new data returns.
+---
+This is the expected behaviour as per epic SV-8582, read on 17 August 2026, and the Inventory Value report specification version 10 (S6-R5, S1-R4, S1-R5, S1-R7, S1-R8), read on 17 August 2026.
+AUTOMATION: Not available on Build to test Yet - Last checked 8/17/2026</t>
         </is>
       </c>
       <c r="H32" s="2" t="inlineStr">
         <is>
-          <t>SV-8673 (IV spec v3 2026-07-29 Story 6 S6-R5; Story 1 S1-R4; S1-R5; S1-R7; S1-R8)</t>
+          <t>SV-8673 (IV spec v10 2026-08-17 Story 6 S6-R5; Story 1 S1-R4; S1-R5; S1-R7; S1-R8)</t>
         </is>
       </c>
       <c r="I32" s="2" t="inlineStr"/>
@@ -2199,14 +2177,13 @@
 2. With no vendor selected, parts of all vendors are shown.
 3. With the part search empty, no search narrowing is applied.
 ---
-This is the expected behaviour as per epic SV-8582, read on 11 August 2026, and the Inventory Value report specification version 5 (S6-R7), read on 11 August 2026.
-Last checked against build v3.5-16cf83f on 8/6/2026.
-AUTOMATION: READY</t>
+This is the expected behaviour as per epic SV-8582, read on 17 August 2026, and the Inventory Value report specification version 10 (S6-R7), read on 17 August 2026.
+AUTOMATION: Not available on Build to test Yet - Last checked 8/17/2026</t>
         </is>
       </c>
       <c r="H33" s="2" t="inlineStr">
         <is>
-          <t>SV-8673 (IV spec v3 2026-07-29 Story 6 S6-R7)</t>
+          <t>SV-8673 (IV spec v10 2026-08-17 Story 6 S6-R7)</t>
         </is>
       </c>
       <c r="I33" s="2" t="inlineStr"/>
@@ -2254,14 +2231,13 @@
 3. Matching is case-insensitive.
 4. The search applies server-side (whole data set, first page returned); a no-match search shows the no-data message.
 ---
-This is the expected behaviour as per epic SV-8582, read on 11 August 2026, and the Inventory Value report specification version 5 (S6-R8, S6-R5), read on 11 August 2026.
-Last checked against build v3.5-16cf83f on 8/6/2026.
-AUTOMATION: READY</t>
+This is the expected behaviour as per epic SV-8582, read on 17 August 2026, and the Inventory Value report specification version 10 (S6-R8, S6-R5), read on 17 August 2026.
+AUTOMATION: Not available on Build to test Yet - Last checked 8/17/2026</t>
         </is>
       </c>
       <c r="H34" s="2" t="inlineStr">
         <is>
-          <t>SV-8673 (IV spec v3 2026-07-29 Story 6 S6-R8; S6-R5)</t>
+          <t>SV-8673 (IV spec v10 2026-08-17 Story 6 S6-R8; S6-R5)</t>
         </is>
       </c>
       <c r="I34" s="2" t="inlineStr"/>
@@ -2270,7 +2246,7 @@
     <row r="35">
       <c r="A35" s="2" t="inlineStr">
         <is>
-          <t>Date range, Location, Category, Vendor, and the part search combine with AND</t>
+          <t>"As of" date, Location, Category, Vendor and part search combine with AND</t>
         </is>
       </c>
       <c r="B35" s="2" t="inlineStr">
@@ -2303,17 +2279,16 @@
       </c>
       <c r="G35" s="2" t="inlineStr">
         <is>
-          <t>1. A part must satisfy EVERY active filter and the search to appear — the Date range, Location, Category, Vendor, and part search combine with AND.
+          <t>1. A part must satisfy EVERY active filter and the search to appear — the "as of" date, Location, Category, Vendor, and part search combine with AND.
 2. The totals row matches the combined filtered set after each step.
 ---
-This is the expected behaviour as per epic SV-8582, read on 11 August 2026, and the Inventory Value report specification version 5 (S6-R9), read on 11 August 2026.
-Last checked against build v3.5-16cf83f on 8/6/2026.
-AUTOMATION: READY</t>
+This is the expected behaviour as per epic SV-8582, read on 17 August 2026, and the Inventory Value report specification version 10 (S6-R9), read on 17 August 2026.
+AUTOMATION: Not available on Build to test Yet - Last checked 8/17/2026</t>
         </is>
       </c>
       <c r="H35" s="2" t="inlineStr">
         <is>
-          <t>SV-8673 (IV spec v3 2026-07-29 Story 6 S6-R9)</t>
+          <t>SV-8673 (IV spec v10 2026-08-17 Story 6 S6-R9)</t>
         </is>
       </c>
       <c r="I35" s="2" t="inlineStr"/>
@@ -2359,19 +2334,18 @@
           <t>1. The toolbar has a location filter labeled "Location" — a multi-select and the rightmost filter — listing the locations the signed-in user has access to, with an "All locations" / "Clear all" toggle.
 2. On a first visit it defaults to the user's currently active location.
 3. With "All locations" active you can tell which location each row's stock belongs to — a location label or marking is shown.
-What you should see today: on a brand-new browser the Location filter reads "All locations" and the report covers every location you can reach, instead of opening on the one location you are currently working at. The date range does open correctly on This Month. This is a known problem and it is already reported - see https://shopview.atlassian.net/browse/SV-8931
+What you should see today: on a brand-new browser the Location filter reads "All locations" and the report covers every location you can reach, instead of opening on the one location you are currently working at. The "as of" date does open correctly on today. This is a known problem and it is already reported - see https://shopview.atlassian.net/browse/SV-8931
 - If you see exactly that, mark this test FAILED and do not raise anything new.
 - If it fails in a DIFFERENT way from what is described above, that is a NEW problem - please report it.
 - If it PASSES, the fix has shipped: tell the QA lead so the ticket can be closed and this note removed.
 ---
-This is the expected behaviour as per epic SV-8582, read on 11 August 2026, and the Inventory Value report specification version 5 (S7-R1, S7-R2, S12-R3), read on 11 August 2026; where the wording of that specification differs, the behaviour above follows Chris Ward's later decision, recorded in his answers in this file: https://docs.google.com/spreadsheets/d/1x8cuYJlFsDHalVZZTh156_ZCq2gcOaGY/edit?usp=sharing&amp;ouid=106388879401921597782&amp;rtpof=true&amp;sd=true, read on 11 August 2026, which is the authority.
-Last checked against build v3.5-16cf83f on 8/6/2026.
+This is the expected behaviour as per epic SV-8582, read on 17 August 2026, and the Inventory Value report specification version 10 (S7-R1, S7-R2, S12-R3), read on 17 August 2026; where the wording of that specification differs, the behaviour above follows Chris Ward's later decision, recorded in his answers in this file: https://docs.google.com/spreadsheets/d/1x8cuYJlFsDHalVZZTh156_ZCq2gcOaGY/edit?usp=sharing&amp;ouid=106388879401921597782&amp;rtpof=true&amp;sd=true, read on 17 August 2026, which is the authority.
 AUTOMATION: READY - EXPECT FAIL (SV-8931)</t>
         </is>
       </c>
       <c r="H36" s="2" t="inlineStr">
         <is>
-          <t>SV-8674 (IV spec v3 2026-07-29 Story 7 S7-R1; S7-R2; Story 12 S12-R3 — per-row location identifier in All-locations view ADDED per kickoff video P10 40:58-41:20; user ruling 2026-07-28: video overrides spec (video newer; last-update-wins))</t>
+          <t>SV-8674 (IV spec v10 2026-08-17 Story 7 S7-R1; S7-R2; Story 12 S12-R3 — per-row location identifier in All-locations view ADDED per kickoff video P10 40:58-41:20; user ruling 2026-07-28: video overrides spec (video newer; last-update-wins))</t>
         </is>
       </c>
       <c r="I36" s="2" t="inlineStr"/>
@@ -2416,14 +2390,13 @@
           <t>1. Each selection change reloads the report scoped to the selected set.
 2. With both locations selected, parts from both appear (one row per part per location) and the totals cover both.
 ---
-This is the expected behaviour as per epic SV-8582, read on 11 August 2026, and the Inventory Value report specification version 5 (S7-R3), read on 11 August 2026.
-Last checked against build v3.5-16cf83f on 8/6/2026.
-AUTOMATION: READY</t>
+This is the expected behaviour as per epic SV-8582, read on 17 August 2026, and the Inventory Value report specification version 10 (S7-R3), read on 17 August 2026.
+AUTOMATION: Not available on Build to test Yet - Last checked 8/17/2026</t>
         </is>
       </c>
       <c r="H37" s="2" t="inlineStr">
         <is>
-          <t>SV-8674 (IV spec v3 2026-07-29 Story 7 S7-R3 + on-screen location-scope indicator per Chris Ward group message 2026-07-29 (chris-update-2026-07-29/chris-message-2026-07-29.md; NEWEST source; last-update-wins))</t>
+          <t>SV-8674 (IV spec v10 2026-08-17 Story 7 S7-R3 + on-screen location-scope indicator per Chris Ward group message 2026-07-29 (chris-update-2026-07-29/chris-message-2026-07-29.md; NEWEST source; last-update-wins))</t>
         </is>
       </c>
       <c r="I37" s="2" t="inlineStr"/>
@@ -2467,14 +2440,13 @@
           <t>1. Only the locations the user has access to are offered — a location the user cannot access is never included in the scope.
 2. If the requested location set resolves to none the user can access, the report falls back to the user's currently active location.
 ---
-This is the expected behaviour as per epic SV-8582, read on 11 August 2026, and the Inventory Value report specification version 5 (S7-R4, S7-R5), read on 11 August 2026.
-Last checked against build v3.5-16cf83f on 8/6/2026.
-AUTOMATION: READY</t>
+This is the expected behaviour as per epic SV-8582, read on 17 August 2026, and the Inventory Value report specification version 10 (S7-R4, S7-R5), read on 17 August 2026.
+AUTOMATION: Not available on Build to test Yet - Last checked 8/17/2026</t>
         </is>
       </c>
       <c r="H38" s="2" t="inlineStr">
         <is>
-          <t>SV-8674 (IV spec v3 2026-07-29 Story 7 S7-R4; S7-R5)</t>
+          <t>SV-8674 (IV spec v10 2026-08-17 Story 7 S7-R4; S7-R5)</t>
         </is>
       </c>
       <c r="I38" s="2" t="inlineStr"/>
@@ -2518,14 +2490,14 @@
           <t>1. For the single-location user the Location filter is NOT shown at all — the report simply shows that one location's stock.
 2. For the user with access to two or more locations the Location filter IS shown.
 ---
-This is the expected behaviour as per epic SV-8582, read on 11 August 2026, and the Inventory Value report specification version 5 (S7-N1), read on 11 August 2026. Chris Ward confirmed this on 8/5/2026 in his answers in this file: https://docs.google.com/spreadsheets/d/1x8cuYJlFsDHalVZZTh156_ZCq2gcOaGY/edit?usp=sharing&amp;ouid=106388879401921597782&amp;rtpof=true&amp;sd=true, read on 11 August 2026
+This is the expected behaviour as per epic SV-8582, read on 17 August 2026, and the Inventory Value report specification version 10 (S7-N1), read on 17 August 2026. Chris Ward confirmed this on 8/5/2026 in his answers in this file: https://docs.google.com/spreadsheets/d/1x8cuYJlFsDHalVZZTh156_ZCq2gcOaGY/edit?usp=sharing&amp;ouid=106388879401921597782&amp;rtpof=true&amp;sd=true, read on 17 August 2026
 Last checked against build v3.5-16cf83f on 8/6/2026.
 AUTOMATION: HOLD - needs a second sign-in as a user with access to only one location</t>
         </is>
       </c>
       <c r="H39" s="2" t="inlineStr">
         <is>
-          <t>SV-8674 (IV spec Story 7 S7-N1 — RULED HIDDEN by Chris Ward answer 2026-07-31 Q1=A "classic spec drift"; the S7-N1 "still sees the filter" note is stale; spec edit pending)</t>
+          <t>SV-8674 (IV spec v10 2026-08-17 Story 7 S7-N1 — RULED HIDDEN by Chris Ward answer 2026-07-31 Q1=A "classic spec drift"; the S7-N1 "still sees the filter" note is stale; spec edit pending)</t>
         </is>
       </c>
       <c r="I39" s="2" t="inlineStr"/>
@@ -2581,14 +2553,13 @@
 7. Whenever the column is shown on screen, both downloads include it in the same position (between Vendor and Qty on Hand), naming each row's own location.
 Note for the tester: whether this column appears depends on how many locations your login can reach, not on how many you have currently selected. Someone who can reach only one location never sees it and never finds it in the column list. If it stays on screen after you narrow to a single location, that is correct.
 ---
-This is the expected behaviour as per epic SV-8582, read on 11 August 2026, and the Inventory Value report specification version 5 (S7-R6, S7-R7, S3-R1, S12-R10, S10-R15), read on 11 August 2026.
-Last checked against build v3.5-16cf83f on 8/6/2026.
-AUTOMATION: READY</t>
+This is the expected behaviour as per epic SV-8582, read on 17 August 2026, and the Inventory Value report specification version 10 (S7-R6, S7-R7, S3-R1, S12-R10, S10-R15), read on 17 August 2026.
+AUTOMATION: Not available on Build to test Yet - Last checked 8/17/2026</t>
         </is>
       </c>
       <c r="H40" s="2" t="inlineStr">
         <is>
-          <t>SV-8674; SV-8677 (IV spec v3 2026-07-29 S7-R6; S7-R7; S3-R1; S12-R10; S10-R15 — Location column inserted between Vendor and Qty on Hand; automatic visibility; never "Multiple"; S10-R15 = the same column in every export)</t>
+          <t>SV-8674; SV-8677 (IV spec v10 2026-08-17 S7-R6; S7-R7; S3-R1; S12-R10; S10-R15 — Location column access-gated and toggleable in the column-selection control; between Vendor and Qty on Hand; never "Multiple"; S10-R15 = same column in every export)</t>
         </is>
       </c>
       <c r="I40" s="2" t="inlineStr"/>
@@ -2634,14 +2605,13 @@
 2. Toggling a column off hides it from the table; toggling it on shows it again.
 3. The Total Cost column is always shown and cannot be turned off.
 ---
-This is the expected behaviour as per epic SV-8582, read on 11 August 2026, and the Inventory Value report specification version 5 (S8-R1, S8-R2), read on 11 August 2026.
-Last checked against build v3.5-16cf83f on 8/6/2026.
-AUTOMATION: READY</t>
+This is the expected behaviour as per epic SV-8582, read on 17 August 2026, and the Inventory Value report specification version 10 (S8-R1, S8-R2), read on 17 August 2026.
+AUTOMATION: Not available on Build to test Yet - Last checked 8/17/2026</t>
         </is>
       </c>
       <c r="H41" s="2" t="inlineStr">
         <is>
-          <t>SV-8675 (IV spec v3 2026-07-29 Story 8 S8-R1; S8-R2)</t>
+          <t>SV-8675 (IV spec v10 2026-08-17 Story 8 S8-R1; S8-R2)</t>
         </is>
       </c>
       <c r="I41" s="2" t="inlineStr"/>
@@ -2685,14 +2655,13 @@
           <t>1. Whatever columns are shown, they appear in the fixed left-to-right order - with Location, when it is turned on in the column-selection control, between Vendor and Qty (Part #, Description, Category, Vendor, Qty, Unit Cost, Unit Sell, Margin, Margin %, Total Sell, Total Cost) - toggling visibility never reorders columns.
 2. Total Cost is always the last column.
 ---
-This is the expected behaviour as per epic SV-8582, read on 11 August 2026, and the Inventory Value report specification version 5 (S8-R4, S3-R1, S7-R6), read on 11 August 2026. Chris Ward confirmed this on 8/5/2026 in his answers in this file: https://docs.google.com/spreadsheets/d/1x8cuYJlFsDHalVZZTh156_ZCq2gcOaGY/edit?usp=sharing&amp;ouid=106388879401921597782&amp;rtpof=true&amp;sd=true, read on 11 August 2026
-Last checked against build v3.5-16cf83f on 8/6/2026.
-AUTOMATION: READY</t>
+This is the expected behaviour as per epic SV-8582, read on 17 August 2026, and the Inventory Value report specification version 10 (S8-R4, S3-R1, S7-R6), read on 17 August 2026. Chris Ward confirmed this on 8/5/2026 in his answers in this file: https://docs.google.com/spreadsheets/d/1x8cuYJlFsDHalVZZTh156_ZCq2gcOaGY/edit?usp=sharing&amp;ouid=106388879401921597782&amp;rtpof=true&amp;sd=true, read on 17 August 2026
+AUTOMATION: Not available on Build to test Yet - Last checked 8/17/2026</t>
         </is>
       </c>
       <c r="H42" s="2" t="inlineStr">
         <is>
-          <t>SV-8675; SV-8674 (IV spec v3 2026-07-29 Story 8 S8-R4; Story 3 S3-R1 + Story 7 S7-R6 — toggling never reorders; plus the automatic Location column between Vendor and Qty on Hand)</t>
+          <t>SV-8675; SV-8674 (IV spec v10 2026-08-17 Story 8 S8-R4; Story 3 S3-R1 + Story 7 S7-R6 — toggling never reorders; plus the automatic Location column between Vendor and Qty on Hand)</t>
         </is>
       </c>
       <c r="I42" s="2" t="inlineStr"/>
@@ -2727,7 +2696,7 @@
       </c>
       <c r="F43" s="2" t="inlineStr">
         <is>
-          <t>1. Change the date range, select a category and a vendor, type a part search, change the location selection, change the column selection, and sort by a non-default column.
+          <t>1. Change the "as of" date, select a category and a vendor, type a part search, change the location selection, change the column selection, and sort by a non-default column.
 2. Navigate away to another screen, then return to the report.
 3. Reload the browser page and check again.
 4. If practical, open the report in a different browser (or private window) and read its settings.</t>
@@ -2735,21 +2704,20 @@
       </c>
       <c r="G43" s="2" t="inlineStr">
         <is>
-          <t>1. On return and after a reload, the report restores the saved date range, category selection, vendor selection, part search text, location selection, column selection, and sort.
+          <t>1. On return and after a reload, the report restores the saved "as of" date, category selection, vendor selection, part search text, location selection, column selection, and sort.
 2. In a different browser the report shows the defaults instead — persistence is per browser, not tied to the user's account.
 What you should see today: after you type something in the Search parts box, leave the report and come back, the box is empty and the full list is back - even though the sort, the columns, the dates and the locations all came back correctly. This is a known problem and it is already reported - see https://shopview.atlassian.net/browse/SV-8928
 - If you see exactly that, mark this test FAILED and do not raise anything new.
 - If it fails in a DIFFERENT way from what is described above, that is a NEW problem - please report it.
 - If it PASSES, the fix has shipped: tell the QA lead so the ticket can be closed and this note removed.
 ---
-This is the expected behaviour as per epic SV-8582, read on 11 August 2026, and the Inventory Value report specification version 5 (S8-R5, S9-R5), read on 11 August 2026.
-Last checked against build v3.5-16cf83f on 8/6/2026.
+This is the expected behaviour as per epic SV-8582, read on 17 August 2026, and the Inventory Value report specification version 10 (S8-R5, S9-R5), read on 17 August 2026.
 AUTOMATION: READY - EXPECT FAIL (SV-8928)</t>
         </is>
       </c>
       <c r="H43" s="2" t="inlineStr">
         <is>
-          <t>SV-8675 (IV spec v3 2026-07-29 Story 8 S8-R5 (+ context note); Story 9 S9-R5)</t>
+          <t>SV-8675 (IV spec v10 2026-08-17 Story 8 S8-R5 (+ context note); Story 9 S9-R5)</t>
         </is>
       </c>
       <c r="I43" s="2" t="inlineStr"/>
@@ -2797,14 +2765,14 @@
 - If it fails in a DIFFERENT way from what is described above, that is a NEW problem - please report it.
 - If it PASSES, the fix has shipped: tell the QA lead so the ticket can be closed and this note removed.
 ---
-This is the expected behaviour as per epic SV-8582, read on 11 August 2026, and the Inventory Value report specification version 5 (S8-R6), read on 11 August 2026.
+This is the expected behaviour as per epic SV-8582, read on 17 August 2026, and the Inventory Value report specification version 10 (S8-R6), read on 17 August 2026.
 Last checked against build v3.5-16cf83f on 8/6/2026.
 AUTOMATION: READY - EXPECT FAIL (SV-8929)</t>
         </is>
       </c>
       <c r="H44" s="2" t="inlineStr">
         <is>
-          <t>SV-8675 (IV spec v3 2026-07-29 Story 8 S8-R6)</t>
+          <t>SV-8675 (IV spec v10 2026-08-17 Story 8 S8-R6)</t>
         </is>
       </c>
       <c r="I44" s="2" t="inlineStr"/>
@@ -2848,14 +2816,13 @@
           <t>1. The rows are sorted by Total Cost, highest first (descending).
 2. The order holds across pages (page 2 continues below page 1's lowest value) — the server applies the default order over the full set.
 ---
-This is the expected behaviour as per epic SV-8582, read on 11 August 2026, and the Inventory Value report specification version 5 (S9-R1), read on 11 August 2026.
-Last checked against build v3.5-16cf83f on 8/6/2026.
-AUTOMATION: READY</t>
+This is the expected behaviour as per epic SV-8582, read on 17 August 2026, and the Inventory Value report specification version 10 (S9-R1), read on 17 August 2026.
+AUTOMATION: Not available on Build to test Yet - Last checked 8/17/2026</t>
         </is>
       </c>
       <c r="H45" s="2" t="inlineStr">
         <is>
-          <t>SV-8676 (IV spec v3 2026-07-29 Story 9 S9-R1; §3 Key Decisions (Total Cost default sort))</t>
+          <t>SV-8676 (IV spec v10 2026-08-17 Story 9 S9-R1; §3 Key Decisions (Total Cost default sort))</t>
         </is>
       </c>
       <c r="I45" s="2" t="inlineStr"/>
@@ -2902,14 +2869,13 @@
 2. Each header click re-fetches the data from the server ordered by the chosen column and direction, returning the FIRST page of the re-sorted result set.
 3. Only one column sorts at a time.
 ---
-This is the expected behaviour as per epic SV-8582, read on 11 August 2026, and the Inventory Value report specification version 5 (S9-R2), read on 11 August 2026.
-Last checked against build v3.5-16cf83f on 8/6/2026.
-AUTOMATION: READY</t>
+This is the expected behaviour as per epic SV-8582, read on 17 August 2026, and the Inventory Value report specification version 10 (S9-R2), read on 17 August 2026.
+AUTOMATION: Not available on Build to test Yet - Last checked 8/17/2026</t>
         </is>
       </c>
       <c r="H46" s="2" t="inlineStr">
         <is>
-          <t>SV-8676 (IV spec v3 2026-07-29 Story 9 S9-R2)</t>
+          <t>SV-8676 (IV spec v10 2026-08-17 Story 9 S9-R2)</t>
         </is>
       </c>
       <c r="I46" s="2" t="inlineStr"/>
@@ -2954,14 +2920,13 @@
           <t>1. Money and numeric columns sort by their underlying value (so $1,100.00 is treated as more than $900.00, not compared as text).
 2. Text columns (Part #, Description, Category, Vendor) sort as text, case-insensitively ("apple" and "Apple" sort together).
 ---
-This is the expected behaviour as per epic SV-8582, read on 11 August 2026, and the Inventory Value report specification version 5 (S9-R3), read on 11 August 2026.
-Last checked against build v3.5-16cf83f on 8/6/2026.
-AUTOMATION: READY</t>
+This is the expected behaviour as per epic SV-8582, read on 17 August 2026, and the Inventory Value report specification version 10 (S9-R3), read on 17 August 2026.
+AUTOMATION: Not available on Build to test Yet - Last checked 8/17/2026</t>
         </is>
       </c>
       <c r="H47" s="2" t="inlineStr">
         <is>
-          <t>SV-8676 (IV spec v3 2026-07-29 Story 9 S9-R3)</t>
+          <t>SV-8676 (IV spec v10 2026-08-17 Story 9 S9-R3)</t>
         </is>
       </c>
       <c r="I47" s="2" t="inlineStr"/>
@@ -3010,14 +2975,14 @@
 - If it fails in a DIFFERENT way from what is described above, that is a NEW problem - please report it.
 - If it PASSES, the fix has shipped: tell the QA lead so the ticket can be closed and this note removed.
 ---
-This is the expected behaviour as per epic SV-8582, read on 11 August 2026, and the Inventory Value report specification version 5 (S10-R1, S10-R2), read on 11 August 2026.
+This is the expected behaviour as per epic SV-8582, read on 17 August 2026, and the Inventory Value report specification version 10 (S10-R1, S10-R2), read on 17 August 2026.
 Last checked against build v3.5-16cf83f on 8/6/2026.
 AUTOMATION: READY - EXPECT FAIL (SV-8818)</t>
         </is>
       </c>
       <c r="H48" s="2" t="inlineStr">
         <is>
-          <t>SV-8677 (IV spec v3 2026-07-29 Story 10 S10-R1; S10-R2)</t>
+          <t>SV-8677 (IV spec v10 2026-08-17 Story 10 S10-R1; S10-R2)</t>
         </is>
       </c>
       <c r="I48" s="2" t="inlineStr"/>
@@ -3046,37 +3011,43 @@
       </c>
       <c r="E49" s="2" t="inlineStr">
         <is>
-          <t>1. You are signed in to the ShopView App on a desktop browser.
-2. The report is open with a non-default column selection, a Category or Vendor filter, a part search, and a non-default sort applied.</t>
+          <t xml:space="preserve">&lt;ol&gt;
+&lt;li&gt;You are signed in to the ShopView App on a desktop browser.&lt;/li&gt;
+&lt;li&gt;The report is open with a non-default column selection, a Category or Vendor filter, a part search, and a non-default sort applied.&lt;/li&gt;
+&lt;/ol&gt;
+</t>
         </is>
       </c>
       <c r="F49" s="2" t="inlineStr">
         <is>
-          <t>1. Download the current view as a CSV and open it.
-2. Compare its columns and their order to the screen.
-3. Compare its rows to the current filters, search, and sort.
-4. Compare its totals row to the on-screen totals row.
-5. Repeat the checks in the PDF.</t>
+          <t xml:space="preserve">&lt;ol&gt;
+&lt;li&gt;Download the current view as a CSV and open it.&lt;/li&gt;
+&lt;li&gt;Compare its columns and their order to the screen.&lt;/li&gt;
+&lt;li&gt;Compare its rows to the current filters, search, and sort.&lt;/li&gt;
+&lt;li&gt;Compare its totals row to the on-screen totals row.&lt;/li&gt;
+&lt;li&gt;Repeat the checks in the PDF.&lt;/li&gt;
+&lt;/ol&gt;
+</t>
         </is>
       </c>
       <c r="G49" s="2" t="inlineStr">
         <is>
-          <t>1. Both downloads include only the columns currently shown, in the same left-to-right order as the screen, with Total Cost last.
-2. Both downloads honor the current date, category, vendor, location, and part-search filters, and apply the current sort.
-3. Both downloads include a totals row labeled "Totals" matching the on-screen totals (the full-filtered-set totals).
-4. Each download (PDF and CSV) carries a "Locations:" line naming the location(s) the report was scoped to.
-5. Note for the tester: the files carry the Location column whenever it is showing on screen (it sits between Vendor and Qty).
-On this build the spreadsheet file ignores the columns you picked and puts them in a different order from the screen, so point 1 above will not match - record what you see and carry on.
-Known issue: the product does not currently do this. It has been filed for a fix here: https://shopview.atlassian.net/browse/SV-8823
----
-This is the expected behaviour as per epic SV-8582, read on 11 August 2026, and the Inventory Value report specification version 5 (S10-R3, S10-R4, S10-R5, S10-R6, S10-R15), read on 11 August 2026.
-Last checked against build v3.5-16cf83f on 8/6/2026.
-AUTOMATION: READY</t>
+          <t xml:space="preserve">&lt;ol&gt;
+&lt;li&gt;Both downloads include only the columns currently shown, in the same left-to-right order as the screen, with Total Cost last.&lt;/li&gt;
+&lt;li&gt;Both downloads honor the current date, category, vendor, location, and part-search filters, and apply the current sort.&lt;/li&gt;
+&lt;li&gt;Both downloads include a totals row labeled "Totals" matching the on-screen totals (the full-filtered-set totals).&lt;/li&gt;
+&lt;li&gt;Each download (PDF and CSV) carries a "Locations:" line naming the location(s) the report was scoped to.&lt;/li&gt;
+&lt;li&gt;&lt;p&gt;Note for the tester: the files carry the Location column whenever it is showing on screen (it sits between Vendor and Qty).&lt;br /&gt;On this build the spreadsheet file ignores the columns you picked and puts them in a different order from the screen, so point 1 above will not match - record what you see and carry on.&lt;br /&gt;Known issue: the product does not currently do this. It has been filed for a fix here: &lt;a href="https://shopview.atlassian.net/browse/SV-8823"&gt;https://shopview.atlassian.net/browse/SV-8823&lt;/a&gt;&lt;/p&gt;&lt;/li&gt;
+&lt;/ol&gt;
+&lt;hr /&gt;
+&lt;p&gt;This is the expected behaviour as per epic SV-8582, read on 11 August 2026, and the Inventory Value report specification version 5 (S10-R3, S10-R4, S10-R5, S10-R6, S10-R15), read on 11 August 2026.&lt;br /&gt;Last checked against build v3.5-16cf83f on 8/6/2026.&lt;/p&gt;
+&lt;p&gt;AUTOMATION: READY&lt;/p&gt;
+</t>
         </is>
       </c>
       <c r="H49" s="2" t="inlineStr">
         <is>
-          <t>SV-8677 (IV spec v3 2026-07-29 Story 10 S10-R3; S10-R4; S10-R5; S10-R6; S10-R15 — downloads keep the shown columns and order; honour the filters; include the Totals row; S10-R15 = the "Locations:" line and the automatic Location column)</t>
+          <t>SV-8677 (IV spec v5 2026-08-07 Story 10 S10-R3; S10-R4; S10-R5; S10-R6; S10-R15 — downloads keep the shown columns and order; honour the filters; include the Totals row; S10-R15 = the "Locations:" line and the Location column when shown)</t>
         </is>
       </c>
       <c r="I49" s="2" t="inlineStr"/>
@@ -3126,14 +3097,14 @@
 - If it fails in a DIFFERENT way from what is described above, that is a NEW problem - please report it.
 - If it PASSES, the fix has shipped: tell the QA lead so the ticket can be closed and this note removed.
 ---
-This is the expected behaviour as per epic SV-8582, read on 11 August 2026, and the Inventory Value report specification version 5 (S10-R7), read on 11 August 2026.
+This is the expected behaviour as per epic SV-8582, read on 17 August 2026, and the Inventory Value report specification version 10 (S10-R7), read on 17 August 2026.
 Last checked against build v3.5-16cf83f on 8/6/2026.
 AUTOMATION: READY - EXPECT FAIL (SV-8823)</t>
         </is>
       </c>
       <c r="H50" s="2" t="inlineStr">
         <is>
-          <t>SV-8677 (IV spec v3 2026-07-29 Story 10 S10-R7 (+ context note))</t>
+          <t>SV-8677 (IV spec v10 2026-08-17 Story 10 S10-R7 (+ context note))</t>
         </is>
       </c>
       <c r="I50" s="2" t="inlineStr"/>
@@ -3186,14 +3157,14 @@
 - If it fails in a DIFFERENT way from what is described above, that is a NEW problem - please report it.
 - If it PASSES, the fix has shipped: tell the QA lead so the ticket can be closed and this note removed.
 ---
-This is the expected behaviour as per epic SV-8582, read on 11 August 2026, and Chris Ward's decision of 8/5/2026, recorded in his answers in this file: https://docs.google.com/spreadsheets/d/1x8cuYJlFsDHalVZZTh156_ZCq2gcOaGY/edit?usp=sharing&amp;ouid=106388879401921597782&amp;rtpof=true&amp;sd=true, read on 11 August 2026. Where the Inventory Value report specification version 5 (S10-R8, S10-R9), read on 11 August 2026, says something different, his decision is the later word and is the authority.
+This is the expected behaviour as per epic SV-8582, read on 17 August 2026, and Chris Ward's decision of 8/5/2026, recorded in his answers in this file: https://docs.google.com/spreadsheets/d/1x8cuYJlFsDHalVZZTh156_ZCq2gcOaGY/edit?usp=sharing&amp;ouid=106388879401921597782&amp;rtpof=true&amp;sd=true, read on 17 August 2026. Where the Inventory Value report specification version 10 (S10-R8, S10-R9), read on 17 August 2026, says something different, his decision is the later word and is the authority.
 Last checked against build v3.5-16cf83f on 8/6/2026.
 AUTOMATION: READY - EXPECT FAIL (SV-8818)</t>
         </is>
       </c>
       <c r="H51" s="2" t="inlineStr">
         <is>
-          <t>SV-8677 (IV spec v3 2026-07-29 Story 10 S10-R8; S10-R9)</t>
+          <t>SV-8677 (IV spec v10 2026-08-17 Story 10 S10-R8; S10-R9)</t>
         </is>
       </c>
       <c r="I51" s="2" t="inlineStr"/>
@@ -3241,14 +3212,14 @@
 - If it fails in a DIFFERENT way from what is described above, that is a NEW problem - please report it.
 - If it PASSES, the fix has shipped: tell the QA lead so the ticket can be closed and this note removed.
 ---
-This is the expected behaviour as per epic SV-8582, read on 11 August 2026, and the Inventory Value report specification version 5 (S10-R10), read on 11 August 2026.
+This is the expected behaviour as per epic SV-8582, read on 17 August 2026, and the Inventory Value report specification version 10 (S10-R10), read on 17 August 2026.
 Last checked against build v3.5-16cf83f on 8/6/2026.
 AUTOMATION: READY - EXPECT FAIL (SV-8818)</t>
         </is>
       </c>
       <c r="H52" s="2" t="inlineStr">
         <is>
-          <t>SV-8677 (IV spec v3 2026-07-29 Story 10 S10-R10 — S10-R10 CLOSES both file names verbatim; so the exact strings ARE the requirement)</t>
+          <t>SV-8677 (IV spec v10 2026-08-17 Story 10 S10-R10 — S10-R10 CLOSES both file names verbatim; so the exact strings ARE the requirement)</t>
         </is>
       </c>
       <c r="I52" s="2" t="inlineStr"/>
@@ -3290,19 +3261,17 @@
       </c>
       <c r="G53" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">1. The export contains the FULL filtered set — every qualifying row across all pages, not only the rows loaded in the browser.
+          <t>1. The export contains the FULL filtered set — every qualifying row across all pages, not only the rows loaded in the browser.
 2. Parts from the later pages are present.
 3. The export is generated server-side against the current filters, part search, and sort — it is not built from the rows currently in the browser.
 ---
-This is the expected behaviour as per epic SV-8582, read on 11 August 2026, and the Inventory Value report specification version 5 (S10-R11), read on 11 August 2026.
-Last checked against build v3.5-16cf83f on 8/5/2026.
-AUTOMATION: READY
-</t>
+This is the expected behaviour as per epic SV-8582, read on 17 August 2026, and the Inventory Value report specification version 10 (S10-R11), read on 17 August 2026.
+AUTOMATION: Not available on Build to test Yet - Last checked 8/17/2026</t>
         </is>
       </c>
       <c r="H53" s="2" t="inlineStr">
         <is>
-          <t>SV-8677 (IV spec v3 2026-07-29 Story 10 S10-R11)</t>
+          <t>SV-8677 (IV spec v10 2026-08-17 Story 10 S10-R11)</t>
         </is>
       </c>
       <c r="I53" s="2" t="inlineStr"/>
@@ -3345,7 +3314,7 @@
       <c r="G54" s="2" t="inlineStr">
         <is>
           <t>1. Neither the PDF nor the CSV is produced.
-2. The user sees the message: "This report is too large to export. Narrow the date range or filters, then try again." (a blocking notification; no file).
+2. The user sees the message: "This report is too large to export. Narrow the filters, then try again." (a blocking notification; no file).
 3. After narrowing the filters below the cap, the download works again.
 4. Note for the tester: on this environment the biggest view you can build is about 9,275 rows, which is under the cap, so you cannot make this message appear here. If the PDF fails with a plain error instead, that is the separate timeout problem - see the Inventory Value export-notification case.
 What you should see today: the spreadsheet download works and produces a file, but the PDF download of the same view fails with a server error and no file arrives. It depends on how much is in the view, not on which report - filtered down to one or two rows the PDF downloads normally, and on a full unfiltered view of several thousand rows it fails every time. This is a known problem and it is already reported - see https://shopview.atlassian.net/browse/SV-8818
@@ -3353,14 +3322,13 @@
 - If it fails in a DIFFERENT way from what is described above, that is a NEW problem - please report it.
 - If it PASSES, the fix has shipped: tell the QA lead so the ticket can be closed and this note removed.
 ---
-This is the expected behaviour as per epic SV-8582, read on 11 August 2026, and the Inventory Value report specification version 5 (S10-R12), read on 11 August 2026.
-Last checked against build v3.5-16cf83f on 8/6/2026.
+This is the expected behaviour as per epic SV-8582, read on 17 August 2026, and the Inventory Value report specification version 10 (S10-R12), read on 17 August 2026.
 AUTOMATION: READY - EXPECT FAIL (SV-8818)</t>
         </is>
       </c>
       <c r="H54" s="2" t="inlineStr">
         <is>
-          <t>SV-8677 (IV spec v3 2026-07-29 Story 10 S10-R12; §7 User Feedback Summary)</t>
+          <t>SV-8677 (IV spec v10 2026-08-17 Story 10 S10-R12; §7 User Feedback Summary)</t>
         </is>
       </c>
       <c r="I54" s="2" t="inlineStr"/>
@@ -3412,14 +3380,14 @@
 - If it fails in a DIFFERENT way from what is described above, that is a NEW problem - please report it.
 - If it PASSES, the fix has shipped: tell the QA lead so the ticket can be closed and this note removed.
 ---
-This is the expected behaviour as per epic SV-8582, read on 11 August 2026, and the Inventory Value report specification version 5 (S10-R13, S10-R14), read on 11 August 2026.
+This is the expected behaviour as per epic SV-8582, read on 17 August 2026, and the Inventory Value report specification version 10 (S10-R13, S10-R14), read on 17 August 2026.
 Last checked against build v3.5-16cf83f on 8/6/2026.
 AUTOMATION: READY - EXPECT FAIL (SV-8818)</t>
         </is>
       </c>
       <c r="H55" s="2" t="inlineStr">
         <is>
-          <t>SV-8677 (IV spec v3 2026-07-29 Story 10 S10-R13; S10-R14; §7 User Feedback Summary)</t>
+          <t>SV-8677 (IV spec v10 2026-08-17 Story 10 S10-R13; S10-R14; §7 User Feedback Summary)</t>
         </is>
       </c>
       <c r="I55" s="2" t="inlineStr"/>
@@ -3463,7 +3431,7 @@
       <c r="G56" s="2" t="inlineStr">
         <is>
           <t>1. The narrowed PDF downloads successfully.
-2. On the whole list the PDF either downloads successfully too, or is refused politely with the message "This report is too large to export. Narrow the date range or filters, then try again." Either of those is a pass.
+2. On the whole list the PDF either downloads successfully too, or is refused politely with the message "This report is too large to export. Narrow the filters, then try again." Either of those is a pass.
 3. The CSV of that same whole list downloads successfully and quickly.
 4. Once the view is narrowed the PDF works again.
 5. KNOWN PROBLEM at the time of writing: on the whole list the PDF did not download at all. After roughly half a minute a plain error appeared reading "An error occurred. We're sorry for this inconvenience, please try again a bit later later." If you still see that, mark this test Failed, note roughly how many rows were in the view, and refer to the reported problem — do not change the test.
@@ -3473,14 +3441,13 @@
 - If it fails in a DIFFERENT way from what is described above, that is a NEW problem - please report it.
 - If it PASSES, the fix has shipped: tell the QA lead so the ticket can be closed and this note removed.
 ---
-This is the expected behaviour as per epic SV-8582, read on 11 August 2026, and the Inventory Value report specification version 5 (S10-R11, S10-R12, S10-R14), read on 11 August 2026.
-Last checked against build v3.5-16cf83f on 8/6/2026.
+This is the expected behaviour as per epic SV-8582, read on 17 August 2026, and the Inventory Value report specification version 10 (S10-R11, S10-R12, S10-R14), read on 17 August 2026.
 AUTOMATION: READY - EXPECT FAIL (SV-8818)</t>
         </is>
       </c>
       <c r="H56" s="2" t="inlineStr">
         <is>
-          <t>SV-8677 (IV spec v3 2026-07-29 S10-R11; S10-R12; S10-R14 — the observed failure path is a roughly 30-second server-side timeout and not the S10-R12 row cap; observed on build v3.4.1-0ed4433)</t>
+          <t>SV-8677 (IV spec v10 2026-08-17 S10-R11; S10-R12; S10-R14 — the observed failure path is a roughly 30-second server-side timeout and not the S10-R12 row cap; observed on build v3.4.1-0ed4433)</t>
         </is>
       </c>
       <c r="I56" s="2" t="inlineStr"/>
@@ -3578,14 +3545,13 @@
           <t>1. The table has white column headers and white data cells, with no alternating row shading.
 2. The table sits on the standard soft blue-grey report backdrop.
 ---
-This is the expected behaviour as per epic SV-8582, read on 11 August 2026, and the Inventory Value report specification version 5 (S12-R1), read on 11 August 2026.
-Last checked against build v3.5-16cf83f on 8/6/2026.
-AUTOMATION: READY</t>
+This is the expected behaviour as per epic SV-8582, read on 17 August 2026, and the Inventory Value report specification version 10 (S12-R1), read on 17 August 2026.
+AUTOMATION: Not available on Build to test Yet - Last checked 8/17/2026</t>
         </is>
       </c>
       <c r="H58" s="2" t="inlineStr">
         <is>
-          <t>SV-8679 (IV spec v3 2026-07-29 Story 12 S12-R1)</t>
+          <t>SV-8679 (IV spec v10 2026-08-17 Story 12 S12-R1)</t>
         </is>
       </c>
       <c r="I58" s="2" t="inlineStr"/>
@@ -3629,14 +3595,13 @@
           <t>1. In the toolbar, the three-dot download menu sits leftmost in the action cluster, followed by the Column Selection control.
 2. The toolbar filters run, left to right: the date-range control, the part search, the Category filter, the Vendor filter, and the Location filter (rightmost).
 ---
-This is the expected behaviour as per epic SV-8582, read on 11 August 2026, and the Inventory Value report specification version 5 (S12-R2, S12-R3), read on 11 August 2026.
-Last checked against build v3.5-16cf83f on 8/6/2026.
-AUTOMATION: READY</t>
+This is the expected behaviour as per epic SV-8582, read on 17 August 2026, and the Inventory Value report specification version 10 (S12-R2, S12-R3), read on 17 August 2026.
+AUTOMATION: Not available on Build to test Yet - Last checked 8/17/2026</t>
         </is>
       </c>
       <c r="H59" s="2" t="inlineStr">
         <is>
-          <t>SV-8679 (IV spec v3 2026-07-29 Story 12 S12-R2; S12-R3)</t>
+          <t>SV-8679 (IV spec v10 2026-08-17 Story 12 S12-R2; S12-R3)</t>
         </is>
       </c>
       <c r="I59" s="2" t="inlineStr"/>
@@ -3686,14 +3651,14 @@
 - If it fails in a DIFFERENT way from what is described above, that is a NEW problem - please report it.
 - If it PASSES, the fix has shipped: tell the QA lead so the ticket can be closed and this note removed.
 ---
-This is the expected behaviour as per epic SV-8582, read on 11 August 2026, and the Inventory Value report specification version 5 (S12-R6), read on 11 August 2026.
+This is the expected behaviour as per epic SV-8582, read on 17 August 2026, and the Inventory Value report specification version 10 (S12-R6), read on 17 August 2026.
 Last checked against build v3.5-16cf83f on 8/6/2026.
 AUTOMATION: READY - EXPECT FAIL (SV-8932)</t>
         </is>
       </c>
       <c r="H60" s="2" t="inlineStr">
         <is>
-          <t>SV-8679 (IV spec v3 2026-07-29 Story 12 S12-R6)</t>
+          <t>SV-8679 (IV spec v10 2026-08-17 Story 12 S12-R6)</t>
         </is>
       </c>
       <c r="I60" s="2" t="inlineStr"/>
@@ -3739,14 +3704,13 @@
 2. In dark mode you can read the toolbar text and the cell text at a glance, and the "—" glyph in an empty Category or Vendor cell is clearly visible against the dark cell behind it — it does not disappear into the background.
 3. Note for the tester: you do not need to measure anything and you do not need any tool. Just say whether everything is easy to read in dark mode, and only report it if something is hard to see. (The exact colour values behind this are design-token values the design and engineering team check with their own tooling, not by hand.)
 ---
-This is the expected behaviour as per epic SV-8582, read on 11 August 2026, and the Inventory Value report specification version 5 (S12-R7), read on 11 August 2026.
-Last checked against build v3.5-16cf83f on 8/6/2026.
-AUTOMATION: READY</t>
+This is the expected behaviour as per epic SV-8582, read on 17 August 2026, and the Inventory Value report specification version 10 (S12-R7), read on 17 August 2026.
+AUTOMATION: Not available on Build to test Yet - Last checked 8/17/2026</t>
         </is>
       </c>
       <c r="H61" s="2" t="inlineStr">
         <is>
-          <t>SV-8679 (IV spec v3 2026-07-29 Story 12 S12-R7)</t>
+          <t>SV-8679 (IV spec v10 2026-08-17 Story 12 S12-R7)</t>
         </is>
       </c>
       <c r="I61" s="2" t="inlineStr"/>
@@ -3797,14 +3761,14 @@
 - If it fails in a DIFFERENT way from what is described above, that is a NEW problem - please report it.
 - If it PASSES, the fix has shipped: tell the QA lead so the ticket can be closed and this note removed.
 ---
-This is the expected behaviour as per epic SV-8582, read on 11 August 2026, and the Inventory Value report specification version 5 (S12-R8), read on 11 August 2026.
+This is the expected behaviour as per epic SV-8582, read on 17 August 2026, and the Inventory Value report specification version 10 (S12-R8), read on 17 August 2026.
 Last checked against build v3.5-16cf83f on 8/6/2026.
 AUTOMATION: READY - EXPECT FAIL (SV-8932)</t>
         </is>
       </c>
       <c r="H62" s="2" t="inlineStr">
         <is>
-          <t>SV-8679 (IV spec v3 2026-07-29 Story 12 S12-R8)</t>
+          <t>SV-8679 (IV spec v10 2026-08-17 Story 12 S12-R8)</t>
         </is>
       </c>
       <c r="I62" s="2" t="inlineStr"/>
@@ -3848,14 +3812,13 @@
         <is>
           <t>1. Each icon-only control carries an accessible name exposed to assistive technology (it is not announced as an unnamed button).
 ---
-This is the expected behaviour as per epic SV-8582, read on 11 August 2026, and the Inventory Value report specification version 5 (S12-R9), read on 11 August 2026.
-Last checked against build v3.5-16cf83f on 8/6/2026.
-AUTOMATION: READY</t>
+This is the expected behaviour as per epic SV-8582, read on 17 August 2026, and the Inventory Value report specification version 10 (S12-R9), read on 17 August 2026.
+AUTOMATION: Not available on Build to test Yet - Last checked 8/17/2026</t>
         </is>
       </c>
       <c r="H63" s="2" t="inlineStr">
         <is>
-          <t>SV-8679 (IV spec v3 2026-07-29 Story 12 S12-R9)</t>
+          <t>SV-8679 (IV spec v10 2026-08-17 Story 12 S12-R9)</t>
         </is>
       </c>
       <c r="I63" s="2" t="inlineStr"/>
@@ -3901,14 +3864,14 @@
 2. No additional report-specific permission is required — the specification allows the one ordinary reports access to cover all six of the new reports.
 3. Note for the tester: the specification allows ONE ordinary reports access for all six of these new reports and no per-report permission. If the build demands a separate report permission before this works, mark this Failed and report it — do not change the test.
 ---
-This is the expected behaviour as per epic SV-8582, read on 11 August 2026, and the Inventory Value report specification version 5 (Story 1 Prerequisites), read on 11 August 2026.
+This is the expected behaviour as per epic SV-8582, read on 17 August 2026, and the Inventory Value report specification version 10 (Story 1 Prerequisites), read on 17 August 2026.
 Last checked against build v3.5-16cf83f on 8/6/2026.
 AUTOMATION: HOLD - needs a second sign-in as a user holding only the ordinary reports access</t>
         </is>
       </c>
       <c r="H64" s="2" t="inlineStr">
         <is>
-          <t>SV-8668 (IV spec Story 1 Prerequisites — one reports permission for all six ruled by Chris Ward Q2=A + QA lead 2026-08-03 "ONE permission FOR NOW"; the IV prerequisite still names the inventory-reports permission — his spec edit owed)</t>
+          <t>SV-8668 (IV spec v10 2026-08-17 Story 1 Prerequisites — one reports permission for all six ruled by Chris Ward Q2=A + QA lead 2026-08-03 "ONE permission FOR NOW"; the IV prerequisite still names the inventory-reports permission — his spec edit owed)</t>
         </is>
       </c>
       <c r="I64" s="2" t="inlineStr"/>
@@ -3951,14 +3914,14 @@
         <is>
           <t>1. The report does not appear in the navigation for this user.
 ---
-This is the expected behaviour as per epic SV-8582, read on 11 August 2026, and the Inventory Value report specification version 5 (S1-N1), read on 11 August 2026.
+This is the expected behaviour as per epic SV-8582, read on 17 August 2026, and the Inventory Value report specification version 10 (S1-N1), read on 17 August 2026.
 Last checked against build v3.5-16cf83f on 8/6/2026.
 AUTOMATION: HOLD - needs a second sign-in as a user with no reports access</t>
         </is>
       </c>
       <c r="H65" s="2" t="inlineStr">
         <is>
-          <t>SV-8668 (IV spec Story 1 S1-N1 — the gate is the one ordinary reports access per Chris Ward Q2=A + QA lead 2026-08-03 "ONE permission FOR NOW")</t>
+          <t>SV-8668 (IV spec v10 2026-08-17 Story 1 S1-N1 — the gate is the one ordinary reports access per Chris Ward Q2=A + QA lead 2026-08-03 "ONE permission FOR NOW")</t>
         </is>
       </c>
       <c r="I65" s="2" t="inlineStr"/>
@@ -4006,14 +3969,14 @@
 2. Each row captures the part's identity (part, category, vendor), on-hand quantity, unit cost, unit sell, total cost, and total sell, stored to the cent.
 3. A location with no in-stock parts on the date simply has no rows for that date — this is valid, not an error.
 ---
-This is the expected behaviour as per epic SV-8582, read on 11 August 2026, and the Inventory Value report specification version 5 (S11-R1, S11-R4), read on 11 August 2026.
+This is the expected behaviour as per epic SV-8582, read on 17 August 2026, and the Inventory Value report specification version 10 (S11-R1, S11-R4), read on 17 August 2026.
 Last checked against build v3.5-16cf83f on 8/6/2026.
 AUTOMATION: HOLD - the nightly capture is a server-side job and its stored rows are not reachable from the application</t>
         </is>
       </c>
       <c r="H66" s="2" t="inlineStr">
         <is>
-          <t>SV-8678 (IV spec v3 2026-07-29 Story 11 S11-R1; S11-R4)</t>
+          <t>SV-8678 (IV spec v10 2026-08-17 Story 11 S11-R1; S11-R4)</t>
         </is>
       </c>
       <c r="I66" s="2" t="inlineStr"/>
@@ -4042,34 +4005,42 @@
       </c>
       <c r="E67" s="2" t="inlineStr">
         <is>
-          <t>1. ZZAUTOTEST parts with known quantities, costs, and sell resolutions (fixed price, matrix markup, and no-category fallback) are in stock and left UNCHANGED across the capture.
-2. A core-charge part and a zero-quantity part also exist.
-3. You can read the live report on the capture date and the stored rows afterward.
-4. To see the information this test asks for you need the browser's own developer tools: press F12 (or Ctrl+Shift+I; on a Mac Cmd+Option+I) and open the "Network" tab, then reload the page. There is nothing to install — it is built into Chrome, Edge and Firefox. Where a check also asks you to confirm what is stored on the server, ask a developer to read it back for you — that part cannot be seen from the browser.</t>
+          <t xml:space="preserve">&lt;ol&gt;
+&lt;li&gt;ZZAUTOTEST parts with known quantities, costs, and sell resolutions (fixed price, matrix markup, and no-category fallback) are in stock and left UNCHANGED across the capture.&lt;/li&gt;
+&lt;li&gt;A core-charge part and a zero-quantity part also exist.&lt;/li&gt;
+&lt;li&gt;You can read the live report on the capture date and the stored rows afterward.&lt;/li&gt;
+&lt;li&gt;To see the information this test asks for you need the browser's own developer tools: press F12 (or Ctrl+Shift+I; on a Mac Cmd+Option+I) and open the "Network" tab, then reload the page. There is nothing to install — it is built into Chrome, Edge and Firefox. Where a check also asks you to confirm what is stored on the server, ask a developer to read it back for you — that part cannot be seen from the browser.&lt;/li&gt;
+&lt;/ol&gt;
+</t>
         </is>
       </c>
       <c r="F67" s="2" t="inlineStr">
         <is>
-          <t>1. On the capture date, note the live report's rows and values for the seeded parts.
-2. After the overnight capture, read the same parts' captured rows.
-3. Look for the core-charge and zero-quantity parts among the captured rows.
-4. The next day, view the report as of the captured date and compare to the noted live values.</t>
+          <t xml:space="preserve">&lt;ol&gt;
+&lt;li&gt;On the capture date, note the live report's rows and values for the seeded parts.&lt;/li&gt;
+&lt;li&gt;After the overnight capture, read the same parts' captured rows.&lt;/li&gt;
+&lt;li&gt;Look for the core-charge and zero-quantity parts among the captured rows.&lt;/li&gt;
+&lt;li&gt;The next day, view the report as of the captured date and compare to the noted live values.&lt;/li&gt;
+&lt;/ol&gt;
+</t>
         </is>
       </c>
       <c r="G67" s="2" t="inlineStr">
         <is>
-          <t>1. The captured parts use the same in-stock, non-core scope as the live report (Story 2) — the core-charge and zero-quantity parts are NOT captured.
-2. The captured values use the same valuation as the live report (Story 3), including the sell-price fallback chain.
-3. A recorded day equals what the live report would have shown that day — the as-of view of the captured date matches the noted live values.
----
-This is the expected behaviour as per epic SV-8582, read on 11 August 2026, and the Inventory Value report specification version 5 (S11-R2), read on 11 August 2026.
-Last checked against build v3.5-16cf83f on 8/6/2026.
-AUTOMATION: HOLD - needs the stored nightly capture rows, which are not reachable from the application</t>
+          <t xml:space="preserve">&lt;ol&gt;
+&lt;li&gt;The captured parts use the same in-stock, non-core scope as the live report (Story 2) — the core-charge and zero-quantity parts are NOT captured.&lt;/li&gt;
+&lt;li&gt;The captured values use the same valuation as the live report (Story 3), including the sell-price fallback chain.&lt;/li&gt;
+&lt;li&gt;A recorded day equals what the live report would have shown that day — the as-of view of the captured date matches the noted live values.&lt;/li&gt;
+&lt;/ol&gt;
+&lt;hr /&gt;
+&lt;p&gt;This is the expected behaviour as per epic SV-8582, read on 11 August 2026, and the Inventory Value report specification version 5 (S11-R2), read on 11 August 2026.&lt;br /&gt;Last checked against build v3.5-16cf83f on 8/6/2026.&lt;/p&gt;
+&lt;p&gt;AUTOMATION: HOLD - needs the stored nightly capture rows, which are not reachable from the application&lt;/p&gt;
+</t>
         </is>
       </c>
       <c r="H67" s="2" t="inlineStr">
         <is>
-          <t>SV-8678 (IV spec v3 2026-07-29 Story 11 S11-R2; §2 Relationship to nightly history)</t>
+          <t>SV-8678 (IV spec v5 2026-08-07 Story 11 S11-R2; §2 Relationship to nightly history)</t>
         </is>
       </c>
       <c r="I67" s="2" t="inlineStr"/>
@@ -4119,14 +4090,14 @@
 5. A re-run always records current truth under the CURRENT date; it cannot reconstruct a past date.
 6. A past date's stored rows are unchanged by a current re-run.
 ---
-This is the expected behaviour as per epic SV-8582, read on 11 August 2026, and the Inventory Value report specification version 5 (S11-R3, S11-R5, S5-E1), read on 11 August 2026.
+This is the expected behaviour as per epic SV-8582, read on 17 August 2026, and the Inventory Value report specification version 10 (S11-R3, S11-R5, S5-E1), read on 17 August 2026.
 Last checked against build v3.5-16cf83f on 8/6/2026.
 AUTOMATION: HOLD - the nightly capture job cannot be re-run or inspected from the application</t>
         </is>
       </c>
       <c r="H68" s="2" t="inlineStr">
         <is>
-          <t>SV-8678 (IV spec v3 2026-07-29 Story 11 S11-R3; Story 11 S11-R5; Story 5 S5-E1)</t>
+          <t>SV-8678 (IV spec v10 2026-08-17 Story 11 S11-R3; Story 11 S11-R5; Story 5 S5-E1)</t>
         </is>
       </c>
       <c r="I68" s="2" t="inlineStr"/>
@@ -4169,20 +4140,19 @@
       </c>
       <c r="G69" s="2" t="inlineStr">
         <is>
-          <t>1. For ages 0–13 months (measured from the current date), every daily capture is kept — full daily per-part detail, covering the report's longest date preset (366 days / This Year / Last Year) entirely at daily resolution.
+          <t>1. For ages 0–13 months (measured from the current date), every daily capture is kept — full daily per-part detail, covering a full 13 months of selectable "as of" days entirely at daily resolution.
 2. For ages older than 13 months, only the last capture of each calendar month is retained; the other daily captures in that band are pruned.
 3. Pruning runs as part of, or alongside, the nightly capture.
 ---
 Note for the tester: this one needs records going back more than a year, and this test system only holds a few days of records so far. If there is nothing old enough to look at, mark this test BLOCKED - do not mark it failed, and do not raise it as a problem.
 ---
-This is the expected behaviour as per epic SV-8582, read on 11 August 2026, and the Inventory Value report specification version 5 (S11-R6), read on 11 August 2026.
-Last checked against build v3.5-16cf83f on 8/6/2026.
+This is the expected behaviour as per epic SV-8582, read on 17 August 2026, and the Inventory Value report specification version 10 (S11-R6), read on 17 August 2026.
 AUTOMATION: HOLD - retention pruning is a server-side job over stored history, not reachable from the application</t>
         </is>
       </c>
       <c r="H69" s="2" t="inlineStr">
         <is>
-          <t>SV-8678 (IV spec v3 2026-07-29 Story 11 S11-R6)</t>
+          <t>SV-8678 (IV spec v10 2026-08-17 Story 11 S11-R6)</t>
         </is>
       </c>
       <c r="I69" s="2" t="inlineStr"/>
@@ -4231,14 +4201,14 @@
 ---
 Note for the tester: this one needs records going back more than a year, and this test system only holds a few days of records so far. If there is nothing old enough to look at, mark this test BLOCKED - do not mark it failed, and do not raise it as a problem.
 ---
-This is the expected behaviour as per epic SV-8582, read on 11 August 2026, and the Inventory Value report specification version 5 (S11-E1, S11-R6, S5-R4, S5-R5, S5-N1), read on 11 August 2026.
+This is the expected behaviour as per epic SV-8582, read on 17 August 2026, and the Inventory Value report specification version 10 (S11-E1, S11-R6, S5-R4, S5-R5, S5-N1), read on 17 August 2026.
 Last checked against build v3.5-16cf83f on 8/6/2026.
 AUTOMATION: HOLD - needs a thinned history that this organisation does not have and cannot be produced from the application</t>
         </is>
       </c>
       <c r="H70" s="2" t="inlineStr">
         <is>
-          <t>SV-8678 (IV spec v3 2026-07-29 Story 11 S11-E1; S11-R6; Story 5 S5-R4; S5-R5; S5-N1)</t>
+          <t>SV-8678 (IV spec v10 2026-08-17 Story 11 S11-E1; S11-R6; Story 5 S5-R4; S5-R5; S5-N1)</t>
         </is>
       </c>
       <c r="I70" s="2" t="inlineStr"/>

</xml_diff>

<commit_message>
Report Suite demark: regenerate deliverables + docs (507/507 current)
Local source resync of the 3 demarked cases (plain text + new refs); id-map
re-merged (507 rows, 0 blank C-ids, refs 507/507); import regenerated (differs
from 8/17 in exactly the 3 rows; header sha256 unchanged vs peers; shredding
guard 0). CASES-TOUCHED + currency report updated: Report Suite = 507/507 current,
0 of 507 our cases carry raw markup (live census), 12 foreign untouched.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01AZ5XzKsK9wv7M41cSPaMyg
</commit_message>
<xml_diff>
--- a/testrail-import/Report-Suite_Inventory-Value-Report_testrail-import.xlsx
+++ b/testrail-import/Report-Suite_Inventory-Value-Report_testrail-import.xlsx
@@ -3011,43 +3011,36 @@
       </c>
       <c r="E49" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">&lt;ol&gt;
-&lt;li&gt;You are signed in to the ShopView App on a desktop browser.&lt;/li&gt;
-&lt;li&gt;The report is open with a non-default column selection, a Category or Vendor filter, a part search, and a non-default sort applied.&lt;/li&gt;
-&lt;/ol&gt;
-</t>
+          <t>1. You are signed in to the ShopView App on a desktop browser.
+2. The report is open with a non-default column selection, a Category or Vendor filter, a part search, and a non-default sort applied.</t>
         </is>
       </c>
       <c r="F49" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">&lt;ol&gt;
-&lt;li&gt;Download the current view as a CSV and open it.&lt;/li&gt;
-&lt;li&gt;Compare its columns and their order to the screen.&lt;/li&gt;
-&lt;li&gt;Compare its rows to the current filters, search, and sort.&lt;/li&gt;
-&lt;li&gt;Compare its totals row to the on-screen totals row.&lt;/li&gt;
-&lt;li&gt;Repeat the checks in the PDF.&lt;/li&gt;
-&lt;/ol&gt;
-</t>
+          <t>1. Download the current view as a CSV and open it.
+2. Compare its columns and their order to the screen.
+3. Compare its rows to the current filters, search, and sort.
+4. Compare its totals row to the on-screen totals row.
+5. Repeat the checks in the PDF.</t>
         </is>
       </c>
       <c r="G49" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">&lt;ol&gt;
-&lt;li&gt;Both downloads include only the columns currently shown, in the same left-to-right order as the screen, with Total Cost last.&lt;/li&gt;
-&lt;li&gt;Both downloads honor the current date, category, vendor, location, and part-search filters, and apply the current sort.&lt;/li&gt;
-&lt;li&gt;Both downloads include a totals row labeled "Totals" matching the on-screen totals (the full-filtered-set totals).&lt;/li&gt;
-&lt;li&gt;Each download (PDF and CSV) carries a "Locations:" line naming the location(s) the report was scoped to.&lt;/li&gt;
-&lt;li&gt;&lt;p&gt;Note for the tester: the files carry the Location column whenever it is showing on screen (it sits between Vendor and Qty).&lt;br /&gt;On this build the spreadsheet file ignores the columns you picked and puts them in a different order from the screen, so point 1 above will not match - record what you see and carry on.&lt;br /&gt;Known issue: the product does not currently do this. It has been filed for a fix here: &lt;a href="https://shopview.atlassian.net/browse/SV-8823"&gt;https://shopview.atlassian.net/browse/SV-8823&lt;/a&gt;&lt;/p&gt;&lt;/li&gt;
-&lt;/ol&gt;
-&lt;hr /&gt;
-&lt;p&gt;This is the expected behaviour as per epic SV-8582, read on 11 August 2026, and the Inventory Value report specification version 5 (S10-R3, S10-R4, S10-R5, S10-R6, S10-R15), read on 11 August 2026.&lt;br /&gt;Last checked against build v3.5-16cf83f on 8/6/2026.&lt;/p&gt;
-&lt;p&gt;AUTOMATION: READY&lt;/p&gt;
-</t>
+          <t>1. Both downloads include only the columns currently shown, in the same left-to-right order as the screen, with Total Cost last.
+2. Both downloads honor the current date, category, vendor, location, and part-search filters, and apply the current sort.
+3. Both downloads include a totals row labeled "Totals" matching the on-screen totals (the full-filtered-set totals).
+4. Each download (PDF and CSV) carries a "Locations:" line naming the location(s) the report was scoped to.
+5. Note for the tester: the files carry the Location column whenever it is showing on screen (it sits between Vendor and Qty).
+On this build the spreadsheet file ignores the columns you picked and puts them in a different order from the screen, so point 1 above will not match - record what you see and carry on.
+Known issue: the product does not currently do this. It has been filed for a fix here: https://shopview.atlassian.net/browse/SV-8823
+---
+This is the expected behaviour as per epic SV-8582 and story SV-8677, read on 18 August 2026, and the Inventory Value report specification version 10 (S10-R3, S10-R4, S10-R5, S10-R6, S10-R15), read on 18 August 2026.
+AUTOMATION: Not available on Build to test Yet - Last checked 8/17/2026</t>
         </is>
       </c>
       <c r="H49" s="2" t="inlineStr">
         <is>
-          <t>SV-8677 (IV spec v5 2026-08-07 Story 10 S10-R3; S10-R4; S10-R5; S10-R6; S10-R15 — downloads keep the shown columns and order; honour the filters; include the Totals row; S10-R15 = the "Locations:" line and the Location column when shown)</t>
+          <t>SV-8677 (IV spec v10 2026-08-18 Story 10 S10-R3; S10-R4; S10-R5; S10-R6; S10-R15 — downloads keep the shown columns and order; honour the filters; include the Totals row; S10-R15 = the "Locations:" line and the Location column when shown)</t>
         </is>
       </c>
       <c r="I49" s="2" t="inlineStr"/>
@@ -4005,42 +3998,33 @@
       </c>
       <c r="E67" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">&lt;ol&gt;
-&lt;li&gt;ZZAUTOTEST parts with known quantities, costs, and sell resolutions (fixed price, matrix markup, and no-category fallback) are in stock and left UNCHANGED across the capture.&lt;/li&gt;
-&lt;li&gt;A core-charge part and a zero-quantity part also exist.&lt;/li&gt;
-&lt;li&gt;You can read the live report on the capture date and the stored rows afterward.&lt;/li&gt;
-&lt;li&gt;To see the information this test asks for you need the browser's own developer tools: press F12 (or Ctrl+Shift+I; on a Mac Cmd+Option+I) and open the "Network" tab, then reload the page. There is nothing to install — it is built into Chrome, Edge and Firefox. Where a check also asks you to confirm what is stored on the server, ask a developer to read it back for you — that part cannot be seen from the browser.&lt;/li&gt;
-&lt;/ol&gt;
-</t>
+          <t>1. ZZAUTOTEST parts with known quantities, costs, and sell resolutions (fixed price, matrix markup, and no-category fallback) are in stock and left UNCHANGED across the capture.
+2. A core-charge part and a zero-quantity part also exist.
+3. You can read the live report on the capture date and the stored rows afterward.
+4. To see the information this test asks for you need the browser's own developer tools: press F12 (or Ctrl+Shift+I; on a Mac Cmd+Option+I) and open the "Network" tab, then reload the page. There is nothing to install — it is built into Chrome, Edge and Firefox. Where a check also asks you to confirm what is stored on the server, ask a developer to read it back for you — that part cannot be seen from the browser.</t>
         </is>
       </c>
       <c r="F67" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">&lt;ol&gt;
-&lt;li&gt;On the capture date, note the live report's rows and values for the seeded parts.&lt;/li&gt;
-&lt;li&gt;After the overnight capture, read the same parts' captured rows.&lt;/li&gt;
-&lt;li&gt;Look for the core-charge and zero-quantity parts among the captured rows.&lt;/li&gt;
-&lt;li&gt;The next day, view the report as of the captured date and compare to the noted live values.&lt;/li&gt;
-&lt;/ol&gt;
-</t>
+          <t>1. On the capture date, note the live report's rows and values for the seeded parts.
+2. After the overnight capture, read the same parts' captured rows.
+3. Look for the core-charge and zero-quantity parts among the captured rows.
+4. The next day, view the report as of the captured date and compare to the noted live values.</t>
         </is>
       </c>
       <c r="G67" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">&lt;ol&gt;
-&lt;li&gt;The captured parts use the same in-stock, non-core scope as the live report (Story 2) — the core-charge and zero-quantity parts are NOT captured.&lt;/li&gt;
-&lt;li&gt;The captured values use the same valuation as the live report (Story 3), including the sell-price fallback chain.&lt;/li&gt;
-&lt;li&gt;A recorded day equals what the live report would have shown that day — the as-of view of the captured date matches the noted live values.&lt;/li&gt;
-&lt;/ol&gt;
-&lt;hr /&gt;
-&lt;p&gt;This is the expected behaviour as per epic SV-8582, read on 11 August 2026, and the Inventory Value report specification version 5 (S11-R2), read on 11 August 2026.&lt;br /&gt;Last checked against build v3.5-16cf83f on 8/6/2026.&lt;/p&gt;
-&lt;p&gt;AUTOMATION: HOLD - needs the stored nightly capture rows, which are not reachable from the application&lt;/p&gt;
-</t>
+          <t>1. The captured parts use the same in-stock, non-core scope as the live report (Story 2) — the core-charge and zero-quantity parts are NOT captured.
+2. The captured values use the same valuation as the live report (Story 3), including the sell-price fallback chain.
+3. A recorded day equals what the live report would have shown that day — the as-of view of the captured date matches the noted live values.
+---
+This is the expected behaviour as per epic SV-8582 and story SV-8678, read on 18 August 2026, and the Inventory Value report specification version 10 (S11-R2), read on 18 August 2026.
+AUTOMATION: HOLD - needs the stored nightly capture rows, which are not reachable from the application</t>
         </is>
       </c>
       <c r="H67" s="2" t="inlineStr">
         <is>
-          <t>SV-8678 (IV spec v5 2026-08-07 Story 11 S11-R2; §2 Relationship to nightly history)</t>
+          <t>SV-8678 (IV spec v10 2026-08-18 Story 11 S11-R2; §2 Relationship to nightly history)</t>
         </is>
       </c>
       <c r="I67" s="2" t="inlineStr"/>

</xml_diff>

<commit_message>
Marker revert EXECUTED: restore correct AUTOMATION markers on 497 cases (metadata-only), sync local source + imports
- 497 live update_case reverts (marker line only): 430 -> READY, 22 -> READY - EXPECT FAIL, 45 -> HOLD
  (incl. 27 Automated reference-only cases as QA-lead-authorized metadata-only corrections)
- 2 Automated content-changed cases HELD (C30462, C30518) for the build-verify pass
- 5 local-only cases synced in local source (marker removed to match live)
- byte-verified: only the marker line changed; body/provenance/refs byte-identical (Rule 50)
- post-write live census: 497/497 clean, marker==prior, 0 anomalies; foreign cases untouched
- imports regenerated (shredding guard PASSED, header sha256==peers); id-maps byte-identical
- fix set independently re-derived from git baseline + live (Rule G), reconciled to the audit

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01AZ5XzKsK9wv7M41cSPaMyg
</commit_message>
<xml_diff>
--- a/testrail-import/Report-Suite_Inventory-Value-Report_testrail-import.xlsx
+++ b/testrail-import/Report-Suite_Inventory-Value-Report_testrail-import.xlsx
@@ -527,7 +527,7 @@
 2. Clicking it opens the Inventory Value report.
 ---
 This is the expected behaviour as per epic SV-8582, read on 17 August 2026, and the Inventory Value report specification version 10 (S1-R1), read on 17 August 2026.
-AUTOMATION: Not available on Build to test Yet - Last checked 8/17/2026</t>
+AUTOMATION: READY</t>
         </is>
       </c>
       <c r="H2" s="2" t="inlineStr">
@@ -686,7 +686,7 @@
 3. Note for the tester: on the build tested there were no numbered page controls on the screen - the rows loaded as you scrolled. That is a difference from the specification, which asks for the reports suite's standard page controls. Record what you see and carry on.
 ---
 This is the expected behaviour as per epic SV-8582, read on 17 August 2026, and the Inventory Value report specification version 10 (S1-R8), read on 17 August 2026.
-AUTOMATION: Not available on Build to test Yet - Last checked 8/17/2026</t>
+AUTOMATION: READY</t>
         </is>
       </c>
       <c r="H5" s="2" t="inlineStr">
@@ -795,7 +795,7 @@
 5. A part that has sat without movement for a long time still appears and is still counted — there is no dead-stock exclusion; how long stock has sat makes no difference.
 ---
 This is the expected behaviour as per epic SV-8582, read on 17 August 2026, and the Inventory Value report specification version 10 (S2-R1, S2-R2, S2-N1, S2-N2), read on 17 August 2026.
-AUTOMATION: Not available on Build to test Yet - Last checked 8/17/2026</t>
+AUTOMATION: READY</t>
         </is>
       </c>
       <c r="H7" s="2" t="inlineStr">
@@ -845,7 +845,7 @@
 2. The rows are NOT merged into one combined row; this is the documented v1 behavior.
 ---
 This is the expected behaviour as per epic SV-8582, read on 17 August 2026, and the Inventory Value report specification version 10 (S2-R3), read on 17 August 2026.
-AUTOMATION: Not available on Build to test Yet - Last checked 8/17/2026</t>
+AUTOMATION: READY</t>
         </is>
       </c>
       <c r="H8" s="2" t="inlineStr">
@@ -896,7 +896,7 @@
 2. The pricing-matrix markup is NOT applied when a fixed sell price is set — the fixed price wins.
 ---
 This is the expected behaviour as per epic SV-8582, read on 17 August 2026, and the Inventory Value report specification version 10 (S3-R5), read on 17 August 2026.
-AUTOMATION: Not available on Build to test Yet - Last checked 8/17/2026</t>
+AUTOMATION: READY</t>
         </is>
       </c>
       <c r="H9" s="2" t="inlineStr">
@@ -946,7 +946,7 @@
           <t>1. Unit Sell equals the shop's pricing-matrix markup on cost for that part's category (the same way the parts list resolves it).
 ---
 This is the expected behaviour as per epic SV-8582, read on 17 August 2026, and the Inventory Value report specification version 10 (S3-R5), read on 17 August 2026.
-AUTOMATION: Not available on Build to test Yet - Last checked 8/17/2026</t>
+AUTOMATION: READY</t>
         </is>
       </c>
       <c r="H10" s="2" t="inlineStr">
@@ -1053,7 +1053,7 @@
 2. Total Cost equals the part's on-hand quantity × Unit Cost, shown as US-dollar currency.
 ---
 This is the expected behaviour as per epic SV-8582, read on 17 August 2026, and the Inventory Value report specification version 10 (S3-R6, S3-R7), read on 17 August 2026.
-AUTOMATION: Not available on Build to test Yet - Last checked 8/17/2026</t>
+AUTOMATION: READY</t>
         </is>
       </c>
       <c r="H12" s="2" t="inlineStr">
@@ -1105,7 +1105,7 @@
 2. Margin is the extended (total) margin, not the per-unit difference.
 ---
 This is the expected behaviour as per epic SV-8582, read on 17 August 2026, and the Inventory Value report specification version 10 (S3-R8), read on 17 August 2026.
-AUTOMATION: Not available on Build to test Yet - Last checked 8/17/2026</t>
+AUTOMATION: READY</t>
         </is>
       </c>
       <c r="H13" s="2" t="inlineStr">
@@ -1157,7 +1157,7 @@
 3. Margin % shows "—" when Total Sell is zero or negative (the percentage is undefined).
 ---
 This is the expected behaviour as per epic SV-8582, read on 17 August 2026, and the Inventory Value report specification version 10 (S3-R9, S3-E3), read on 17 August 2026.
-AUTOMATION: Not available on Build to test Yet - Last checked 8/17/2026</t>
+AUTOMATION: READY</t>
         </is>
       </c>
       <c r="H14" s="2" t="inlineStr">
@@ -1209,7 +1209,7 @@
 3. Every other column is right-aligned. When it is on, the Location column appears between Vendor and Qty, and it is right-aligned like the other non-identity columns.The question is in the round-3 question sheet: https://raw.githubusercontent.com/bilalmuzamil-sketch/Manual-test-Cases/claude/slack-session-0sxnd9/build/report-suite/rulings-2026-08-05/Questions-for-Chris-Ward_Report-Suite_Round-3_2026-08-05.xlsx
 ---
 This is the expected behaviour as per epic SV-8582, read on 17 August 2026, and the Inventory Value report specification version 10 (S3-R1, S3-R2, S7-R6), read on 17 August 2026.
-AUTOMATION: Not available on Build to test Yet - Last checked 8/17/2026</t>
+AUTOMATION: READY</t>
         </is>
       </c>
       <c r="H15" s="2" t="inlineStr">
@@ -1261,7 +1261,7 @@
 3. Money values show a leading "$", two decimal places, and thousands separators (for example "$1,234.56"); a negative value shows a leading minus before the "$" ("-$1,234.56"); a genuine zero shows "$0.00".
 ---
 This is the expected behaviour as per epic SV-8582, read on 17 August 2026, and the Inventory Value report specification version 10 (S3-R3, S3-R4, S3-R5, S3-R10), read on 17 August 2026.
-AUTOMATION: Not available on Build to test Yet - Last checked 8/17/2026</t>
+AUTOMATION: READY</t>
         </is>
       </c>
       <c r="H16" s="2" t="inlineStr">
@@ -1312,7 +1312,7 @@
 3. It stays fixed to the right edge while the other columns scroll underneath.
 ---
 This is the expected behaviour as per epic SV-8582, read on 17 August 2026, and the Inventory Value report specification version 10 (S3-R11, S12-R4), read on 17 August 2026.
-AUTOMATION: Not available on Build to test Yet - Last checked 8/17/2026</t>
+AUTOMATION: READY</t>
         </is>
       </c>
       <c r="H17" s="2" t="inlineStr">
@@ -1364,7 +1364,7 @@
 Known issue: the product does not currently do this. It has been filed for a fix here: https://shopview.atlassian.net/browse/SV-8927
 ---
 This is the expected behaviour as per epic SV-8582, read on 17 August 2026, and the Inventory Value report specification version 10 (S3-R12, S3-R13, S8-R3, S7-R6), read on 17 August 2026.
-AUTOMATION: Not available on Build to test Yet - Last checked 8/17/2026</t>
+AUTOMATION: READY</t>
         </is>
       </c>
       <c r="H18" s="2" t="inlineStr">
@@ -1417,7 +1417,7 @@
 4. Note for the tester: on this build a part cannot be saved without a category, so you will not find a part whose Category cell shows "—". Check the Vendor half only.
 ---
 This is the expected behaviour as per epic SV-8582, read on 17 August 2026, and the Inventory Value report specification version 10 (S3-R14, S3-E1, S3-E2), read on 17 August 2026.
-AUTOMATION: Not available on Build to test Yet - Last checked 8/17/2026</t>
+AUTOMATION: READY</t>
         </is>
       </c>
       <c r="H19" s="2" t="inlineStr">
@@ -1535,7 +1535,7 @@
 4. After each filter change the totals row recomputes on the server over the full filtered set, independent of which page is shown.
 ---
 This is the expected behaviour as per epic SV-8582, read on 17 August 2026, and the Inventory Value report specification version 10 (S4-R2, S4-R8, S6-R6), read on 17 August 2026.
-AUTOMATION: Not available on Build to test Yet - Last checked 8/17/2026</t>
+AUTOMATION: READY</t>
         </is>
       </c>
       <c r="H21" s="2" t="inlineStr">
@@ -1588,7 +1588,7 @@
 3. It shows "—" when the total Total Sell is zero or negative.
 ---
 This is the expected behaviour as per epic SV-8582, read on 17 August 2026, and the Inventory Value report specification version 10 (S4-R3), read on 17 August 2026.
-AUTOMATION: Not available on Build to test Yet - Last checked 8/17/2026</t>
+AUTOMATION: READY</t>
         </is>
       </c>
       <c r="H22" s="2" t="inlineStr">
@@ -1968,7 +1968,7 @@
 2. This forward-capture-only behavior is the documented v1 boundary, not a defect.
 ---
 This is the expected behaviour as per epic SV-8582, read on 17 August 2026, and the Inventory Value report specification version 10 (S5-E1), read on 17 August 2026.
-AUTOMATION: Not available on Build to test Yet - Last checked 8/17/2026</t>
+AUTOMATION: READY</t>
         </is>
       </c>
       <c r="H29" s="2" t="inlineStr">
@@ -2073,7 +2073,7 @@
 3. Selecting one or more vendors reloads the report to show only parts supplied by the selected vendors.
 ---
 This is the expected behaviour as per epic SV-8582, read on 17 August 2026, and the Inventory Value report specification version 10 (S6-R1, S6-R2, S6-R3, S6-R4), read on 17 August 2026.
-AUTOMATION: Not available on Build to test Yet - Last checked 8/17/2026</t>
+AUTOMATION: READY</t>
         </is>
       </c>
       <c r="H31" s="2" t="inlineStr">
@@ -2178,7 +2178,7 @@
 3. With the part search empty, no search narrowing is applied.
 ---
 This is the expected behaviour as per epic SV-8582, read on 17 August 2026, and the Inventory Value report specification version 10 (S6-R7), read on 17 August 2026.
-AUTOMATION: Not available on Build to test Yet - Last checked 8/17/2026</t>
+AUTOMATION: READY</t>
         </is>
       </c>
       <c r="H33" s="2" t="inlineStr">
@@ -2232,7 +2232,7 @@
 4. The search applies server-side (whole data set, first page returned); a no-match search shows the no-data message.
 ---
 This is the expected behaviour as per epic SV-8582, read on 17 August 2026, and the Inventory Value report specification version 10 (S6-R8, S6-R5), read on 17 August 2026.
-AUTOMATION: Not available on Build to test Yet - Last checked 8/17/2026</t>
+AUTOMATION: READY</t>
         </is>
       </c>
       <c r="H34" s="2" t="inlineStr">
@@ -2391,7 +2391,7 @@
 2. With both locations selected, parts from both appear (one row per part per location) and the totals cover both.
 ---
 This is the expected behaviour as per epic SV-8582, read on 17 August 2026, and the Inventory Value report specification version 10 (S7-R3), read on 17 August 2026.
-AUTOMATION: Not available on Build to test Yet - Last checked 8/17/2026</t>
+AUTOMATION: READY</t>
         </is>
       </c>
       <c r="H37" s="2" t="inlineStr">
@@ -2441,7 +2441,7 @@
 2. If the requested location set resolves to none the user can access, the report falls back to the user's currently active location.
 ---
 This is the expected behaviour as per epic SV-8582, read on 17 August 2026, and the Inventory Value report specification version 10 (S7-R4, S7-R5), read on 17 August 2026.
-AUTOMATION: Not available on Build to test Yet - Last checked 8/17/2026</t>
+AUTOMATION: READY</t>
         </is>
       </c>
       <c r="H38" s="2" t="inlineStr">
@@ -2554,7 +2554,7 @@
 Note for the tester: whether this column appears depends on how many locations your login can reach, not on how many you have currently selected. Someone who can reach only one location never sees it and never finds it in the column list. If it stays on screen after you narrow to a single location, that is correct.
 ---
 This is the expected behaviour as per epic SV-8582, read on 17 August 2026, and the Inventory Value report specification version 10 (S7-R6, S7-R7, S3-R1, S12-R10, S10-R15), read on 17 August 2026.
-AUTOMATION: Not available on Build to test Yet - Last checked 8/17/2026</t>
+AUTOMATION: READY</t>
         </is>
       </c>
       <c r="H40" s="2" t="inlineStr">
@@ -2606,7 +2606,7 @@
 3. The Total Cost column is always shown and cannot be turned off.
 ---
 This is the expected behaviour as per epic SV-8582, read on 17 August 2026, and the Inventory Value report specification version 10 (S8-R1, S8-R2), read on 17 August 2026.
-AUTOMATION: Not available on Build to test Yet - Last checked 8/17/2026</t>
+AUTOMATION: READY</t>
         </is>
       </c>
       <c r="H41" s="2" t="inlineStr">
@@ -2656,7 +2656,7 @@
 2. Total Cost is always the last column.
 ---
 This is the expected behaviour as per epic SV-8582, read on 17 August 2026, and the Inventory Value report specification version 10 (S8-R4, S3-R1, S7-R6), read on 17 August 2026. Chris Ward confirmed this on 8/5/2026 in his answers in this file: https://docs.google.com/spreadsheets/d/1x8cuYJlFsDHalVZZTh156_ZCq2gcOaGY/edit?usp=sharing&amp;ouid=106388879401921597782&amp;rtpof=true&amp;sd=true, read on 17 August 2026
-AUTOMATION: Not available on Build to test Yet - Last checked 8/17/2026</t>
+AUTOMATION: READY</t>
         </is>
       </c>
       <c r="H42" s="2" t="inlineStr">
@@ -2817,7 +2817,7 @@
 2. The order holds across pages (page 2 continues below page 1's lowest value) — the server applies the default order over the full set.
 ---
 This is the expected behaviour as per epic SV-8582, read on 17 August 2026, and the Inventory Value report specification version 10 (S9-R1), read on 17 August 2026.
-AUTOMATION: Not available on Build to test Yet - Last checked 8/17/2026</t>
+AUTOMATION: READY</t>
         </is>
       </c>
       <c r="H45" s="2" t="inlineStr">
@@ -2870,7 +2870,7 @@
 3. Only one column sorts at a time.
 ---
 This is the expected behaviour as per epic SV-8582, read on 17 August 2026, and the Inventory Value report specification version 10 (S9-R2), read on 17 August 2026.
-AUTOMATION: Not available on Build to test Yet - Last checked 8/17/2026</t>
+AUTOMATION: READY</t>
         </is>
       </c>
       <c r="H46" s="2" t="inlineStr">
@@ -2921,7 +2921,7 @@
 2. Text columns (Part #, Description, Category, Vendor) sort as text, case-insensitively ("apple" and "Apple" sort together).
 ---
 This is the expected behaviour as per epic SV-8582, read on 17 August 2026, and the Inventory Value report specification version 10 (S9-R3), read on 17 August 2026.
-AUTOMATION: Not available on Build to test Yet - Last checked 8/17/2026</t>
+AUTOMATION: READY</t>
         </is>
       </c>
       <c r="H47" s="2" t="inlineStr">
@@ -3035,7 +3035,7 @@
 Known issue: the product does not currently do this. It has been filed for a fix here: https://shopview.atlassian.net/browse/SV-8823
 ---
 This is the expected behaviour as per epic SV-8582 and story SV-8677, read on 18 August 2026, and the Inventory Value report specification version 10 (S10-R3, S10-R4, S10-R5, S10-R6, S10-R15), read on 18 August 2026.
-AUTOMATION: Not available on Build to test Yet - Last checked 8/17/2026</t>
+AUTOMATION: READY</t>
         </is>
       </c>
       <c r="H49" s="2" t="inlineStr">
@@ -3259,7 +3259,7 @@
 3. The export is generated server-side against the current filters, part search, and sort — it is not built from the rows currently in the browser.
 ---
 This is the expected behaviour as per epic SV-8582, read on 17 August 2026, and the Inventory Value report specification version 10 (S10-R11), read on 17 August 2026.
-AUTOMATION: Not available on Build to test Yet - Last checked 8/17/2026</t>
+AUTOMATION: READY</t>
         </is>
       </c>
       <c r="H53" s="2" t="inlineStr">
@@ -3539,7 +3539,7 @@
 2. The table sits on the standard soft blue-grey report backdrop.
 ---
 This is the expected behaviour as per epic SV-8582, read on 17 August 2026, and the Inventory Value report specification version 10 (S12-R1), read on 17 August 2026.
-AUTOMATION: Not available on Build to test Yet - Last checked 8/17/2026</t>
+AUTOMATION: READY</t>
         </is>
       </c>
       <c r="H58" s="2" t="inlineStr">
@@ -3589,7 +3589,7 @@
 2. The toolbar filters run, left to right: the date-range control, the part search, the Category filter, the Vendor filter, and the Location filter (rightmost).
 ---
 This is the expected behaviour as per epic SV-8582, read on 17 August 2026, and the Inventory Value report specification version 10 (S12-R2, S12-R3), read on 17 August 2026.
-AUTOMATION: Not available on Build to test Yet - Last checked 8/17/2026</t>
+AUTOMATION: READY</t>
         </is>
       </c>
       <c r="H59" s="2" t="inlineStr">
@@ -3698,7 +3698,7 @@
 3. Note for the tester: you do not need to measure anything and you do not need any tool. Just say whether everything is easy to read in dark mode, and only report it if something is hard to see. (The exact colour values behind this are design-token values the design and engineering team check with their own tooling, not by hand.)
 ---
 This is the expected behaviour as per epic SV-8582, read on 17 August 2026, and the Inventory Value report specification version 10 (S12-R7), read on 17 August 2026.
-AUTOMATION: Not available on Build to test Yet - Last checked 8/17/2026</t>
+AUTOMATION: READY</t>
         </is>
       </c>
       <c r="H61" s="2" t="inlineStr">
@@ -3806,7 +3806,7 @@
           <t>1. Each icon-only control carries an accessible name exposed to assistive technology (it is not announced as an unnamed button).
 ---
 This is the expected behaviour as per epic SV-8582, read on 17 August 2026, and the Inventory Value report specification version 10 (S12-R9), read on 17 August 2026.
-AUTOMATION: Not available on Build to test Yet - Last checked 8/17/2026</t>
+AUTOMATION: READY</t>
         </is>
       </c>
       <c r="H63" s="2" t="inlineStr">

</xml_diff>